<commit_message>
purchase bills failure fixes are updated
purchase bills failure fixes are updated
</commit_message>
<xml_diff>
--- a/testdata/DBfin.xlsx
+++ b/testdata/DBfin.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4507"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="2520" windowWidth="15405" windowHeight="6540" tabRatio="594" firstSheet="7" activeTab="8"/>
+    <workbookView xWindow="0" yWindow="2520" windowWidth="16695" windowHeight="6540" tabRatio="594" firstSheet="9" activeTab="12"/>
   </bookViews>
   <sheets>
     <sheet name="PurchaseBillsLocal" sheetId="1" r:id="rId1"/>
@@ -18,14 +18,15 @@
     <sheet name="purchaseBills_GRN" sheetId="9" r:id="rId9"/>
     <sheet name="PurchaseBills_ExAcc" sheetId="10" r:id="rId10"/>
     <sheet name="PurchaseBills_Ex_Grn_Igst" sheetId="11" r:id="rId11"/>
-    <sheet name="Sheet2" sheetId="12" r:id="rId12"/>
+    <sheet name="PurchaseBills_Interstate_Un" sheetId="12" r:id="rId12"/>
+    <sheet name="PurchaseBillsUTGST_Ureq" sheetId="13" r:id="rId13"/>
   </sheets>
   <calcPr calcId="125725"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="584" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="670" uniqueCount="62">
   <si>
     <t>Scenario  : Local Sales - Stock UOM and Sales UOM (Similar)   DOC NO :  SORD-2425-00089</t>
   </si>
@@ -221,7 +222,7 @@
   <numFmts count="3">
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="0.000"/>
-    <numFmt numFmtId="167" formatCode="0.0"/>
+    <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
   <fonts count="8">
     <font>
@@ -362,7 +363,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -480,13 +481,25 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="3" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Comma" xfId="2" builtinId="3"/>
@@ -812,68 +825,68 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:59" ht="18">
-      <c r="A1" s="55" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="55"/>
-      <c r="C1" s="55"/>
-      <c r="D1" s="55"/>
-      <c r="E1" s="55"/>
-      <c r="F1" s="55"/>
-      <c r="G1" s="55"/>
-      <c r="H1" s="55"/>
-      <c r="I1" s="55"/>
-      <c r="J1" s="55"/>
-      <c r="K1" s="55"/>
-      <c r="L1" s="55"/>
-      <c r="M1" s="55"/>
-      <c r="N1" s="55"/>
-      <c r="O1" s="55"/>
-      <c r="P1" s="55"/>
-      <c r="Q1" s="55"/>
-      <c r="R1" s="55"/>
-      <c r="S1" s="55"/>
-      <c r="T1" s="55"/>
-      <c r="U1" s="55"/>
-      <c r="V1" s="55"/>
-      <c r="W1" s="55"/>
-      <c r="X1" s="55"/>
-      <c r="Y1" s="55"/>
-      <c r="Z1" s="55"/>
-      <c r="AA1" s="55"/>
-      <c r="AB1" s="55"/>
-      <c r="AC1" s="55"/>
-      <c r="AD1" s="55" t="s">
-        <v>0</v>
-      </c>
-      <c r="AE1" s="55"/>
-      <c r="AF1" s="55"/>
-      <c r="AG1" s="55"/>
-      <c r="AH1" s="55"/>
-      <c r="AI1" s="55"/>
-      <c r="AJ1" s="55"/>
-      <c r="AK1" s="55"/>
-      <c r="AL1" s="55"/>
-      <c r="AM1" s="55"/>
-      <c r="AN1" s="55"/>
-      <c r="AO1" s="55"/>
-      <c r="AP1" s="55"/>
-      <c r="AQ1" s="55"/>
-      <c r="AR1" s="55"/>
-      <c r="AS1" s="55"/>
-      <c r="AT1" s="55"/>
-      <c r="AU1" s="55"/>
-      <c r="AV1" s="55"/>
-      <c r="AW1" s="55"/>
-      <c r="AX1" s="55"/>
-      <c r="AY1" s="55"/>
-      <c r="AZ1" s="55"/>
-      <c r="BA1" s="55"/>
-      <c r="BB1" s="55"/>
-      <c r="BC1" s="55"/>
-      <c r="BD1" s="55"/>
-      <c r="BE1" s="55"/>
-      <c r="BF1" s="55"/>
+      <c r="A1" s="60" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="60"/>
+      <c r="C1" s="60"/>
+      <c r="D1" s="60"/>
+      <c r="E1" s="60"/>
+      <c r="F1" s="60"/>
+      <c r="G1" s="60"/>
+      <c r="H1" s="60"/>
+      <c r="I1" s="60"/>
+      <c r="J1" s="60"/>
+      <c r="K1" s="60"/>
+      <c r="L1" s="60"/>
+      <c r="M1" s="60"/>
+      <c r="N1" s="60"/>
+      <c r="O1" s="60"/>
+      <c r="P1" s="60"/>
+      <c r="Q1" s="60"/>
+      <c r="R1" s="60"/>
+      <c r="S1" s="60"/>
+      <c r="T1" s="60"/>
+      <c r="U1" s="60"/>
+      <c r="V1" s="60"/>
+      <c r="W1" s="60"/>
+      <c r="X1" s="60"/>
+      <c r="Y1" s="60"/>
+      <c r="Z1" s="60"/>
+      <c r="AA1" s="60"/>
+      <c r="AB1" s="60"/>
+      <c r="AC1" s="60"/>
+      <c r="AD1" s="60" t="s">
+        <v>0</v>
+      </c>
+      <c r="AE1" s="60"/>
+      <c r="AF1" s="60"/>
+      <c r="AG1" s="60"/>
+      <c r="AH1" s="60"/>
+      <c r="AI1" s="60"/>
+      <c r="AJ1" s="60"/>
+      <c r="AK1" s="60"/>
+      <c r="AL1" s="60"/>
+      <c r="AM1" s="60"/>
+      <c r="AN1" s="60"/>
+      <c r="AO1" s="60"/>
+      <c r="AP1" s="60"/>
+      <c r="AQ1" s="60"/>
+      <c r="AR1" s="60"/>
+      <c r="AS1" s="60"/>
+      <c r="AT1" s="60"/>
+      <c r="AU1" s="60"/>
+      <c r="AV1" s="60"/>
+      <c r="AW1" s="60"/>
+      <c r="AX1" s="60"/>
+      <c r="AY1" s="60"/>
+      <c r="AZ1" s="60"/>
+      <c r="BA1" s="60"/>
+      <c r="BB1" s="60"/>
+      <c r="BC1" s="60"/>
+      <c r="BD1" s="60"/>
+      <c r="BE1" s="60"/>
+      <c r="BF1" s="60"/>
     </row>
     <row r="2" spans="1:59" ht="18">
       <c r="A2" s="23" t="s">
@@ -944,10 +957,10 @@
       <c r="BF2" s="38"/>
     </row>
     <row r="3" spans="1:59">
-      <c r="A3" s="56" t="s">
+      <c r="A3" s="61" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="56"/>
+      <c r="B3" s="61"/>
       <c r="C3" s="2"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -987,10 +1000,10 @@
       <c r="AA3" s="6"/>
       <c r="AB3" s="6"/>
       <c r="AC3" s="6"/>
-      <c r="AD3" s="56" t="s">
+      <c r="AD3" s="61" t="s">
         <v>3</v>
       </c>
-      <c r="AE3" s="56"/>
+      <c r="AE3" s="61"/>
       <c r="AF3" s="39"/>
       <c r="AG3" s="3">
         <v>1</v>
@@ -1467,38 +1480,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:33" ht="18">
-      <c r="A1" s="55" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="55"/>
-      <c r="C1" s="55"/>
-      <c r="D1" s="55"/>
-      <c r="E1" s="55"/>
-      <c r="F1" s="55"/>
-      <c r="G1" s="55"/>
-      <c r="H1" s="55"/>
-      <c r="I1" s="55"/>
-      <c r="J1" s="55"/>
-      <c r="K1" s="55"/>
-      <c r="L1" s="55"/>
-      <c r="M1" s="55"/>
-      <c r="N1" s="55"/>
-      <c r="O1" s="55"/>
-      <c r="P1" s="55"/>
-      <c r="Q1" s="55"/>
-      <c r="R1" s="55"/>
-      <c r="S1" s="55"/>
-      <c r="T1" s="55"/>
-      <c r="U1" s="55"/>
-      <c r="V1" s="55"/>
-      <c r="W1" s="55"/>
-      <c r="X1" s="55"/>
-      <c r="Y1" s="55"/>
-      <c r="Z1" s="55"/>
-      <c r="AA1" s="55"/>
-      <c r="AB1" s="55"/>
-      <c r="AC1" s="55"/>
-      <c r="AD1" s="55"/>
+      <c r="A1" s="60" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="60"/>
+      <c r="C1" s="60"/>
+      <c r="D1" s="60"/>
+      <c r="E1" s="60"/>
+      <c r="F1" s="60"/>
+      <c r="G1" s="60"/>
+      <c r="H1" s="60"/>
+      <c r="I1" s="60"/>
+      <c r="J1" s="60"/>
+      <c r="K1" s="60"/>
+      <c r="L1" s="60"/>
+      <c r="M1" s="60"/>
+      <c r="N1" s="60"/>
+      <c r="O1" s="60"/>
+      <c r="P1" s="60"/>
+      <c r="Q1" s="60"/>
+      <c r="R1" s="60"/>
+      <c r="S1" s="60"/>
+      <c r="T1" s="60"/>
+      <c r="U1" s="60"/>
+      <c r="V1" s="60"/>
+      <c r="W1" s="60"/>
+      <c r="X1" s="60"/>
+      <c r="Y1" s="60"/>
+      <c r="Z1" s="60"/>
+      <c r="AA1" s="60"/>
+      <c r="AB1" s="60"/>
+      <c r="AC1" s="60"/>
+      <c r="AD1" s="60"/>
     </row>
     <row r="2" spans="1:33" ht="18">
       <c r="A2" s="23" t="s">
@@ -1537,10 +1550,10 @@
       <c r="AD2" s="43"/>
     </row>
     <row r="3" spans="1:33" ht="15.75" thickBot="1">
-      <c r="A3" s="56" t="s">
+      <c r="A3" s="61" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="56"/>
+      <c r="B3" s="61"/>
       <c r="C3" s="44"/>
       <c r="D3" s="3">
         <v>2</v>
@@ -1728,17 +1741,14 @@
         <f>ROUND(K5*N5%,2)</f>
         <v>0</v>
       </c>
-      <c r="P5" s="8">
-        <f>J5-O5</f>
-        <v>500.5</v>
-      </c>
+      <c r="P5" s="8"/>
       <c r="Q5" s="8">
         <f>ROUND(L5*P5%,2)</f>
         <v>0</v>
       </c>
       <c r="R5" s="8">
         <f>P5-Q5</f>
-        <v>500.5</v>
+        <v>0</v>
       </c>
       <c r="S5" s="8">
         <f>ROUND(M5*R5%,2)</f>
@@ -2156,37 +2166,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:30" ht="18">
-      <c r="A1" s="55" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="55"/>
-      <c r="C1" s="55"/>
-      <c r="D1" s="55"/>
-      <c r="E1" s="55"/>
-      <c r="F1" s="55"/>
-      <c r="G1" s="55"/>
-      <c r="H1" s="55"/>
-      <c r="I1" s="55"/>
-      <c r="J1" s="55"/>
-      <c r="K1" s="55"/>
-      <c r="L1" s="55"/>
-      <c r="M1" s="55"/>
-      <c r="N1" s="55"/>
-      <c r="O1" s="55"/>
-      <c r="P1" s="55"/>
-      <c r="Q1" s="55"/>
-      <c r="R1" s="55"/>
-      <c r="S1" s="55"/>
-      <c r="T1" s="55"/>
-      <c r="U1" s="55"/>
-      <c r="V1" s="55"/>
-      <c r="W1" s="55"/>
-      <c r="X1" s="55"/>
-      <c r="Y1" s="55"/>
-      <c r="Z1" s="55"/>
-      <c r="AA1" s="55"/>
-      <c r="AB1" s="55"/>
-      <c r="AC1" s="55"/>
+      <c r="A1" s="60" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="60"/>
+      <c r="C1" s="60"/>
+      <c r="D1" s="60"/>
+      <c r="E1" s="60"/>
+      <c r="F1" s="60"/>
+      <c r="G1" s="60"/>
+      <c r="H1" s="60"/>
+      <c r="I1" s="60"/>
+      <c r="J1" s="60"/>
+      <c r="K1" s="60"/>
+      <c r="L1" s="60"/>
+      <c r="M1" s="60"/>
+      <c r="N1" s="60"/>
+      <c r="O1" s="60"/>
+      <c r="P1" s="60"/>
+      <c r="Q1" s="60"/>
+      <c r="R1" s="60"/>
+      <c r="S1" s="60"/>
+      <c r="T1" s="60"/>
+      <c r="U1" s="60"/>
+      <c r="V1" s="60"/>
+      <c r="W1" s="60"/>
+      <c r="X1" s="60"/>
+      <c r="Y1" s="60"/>
+      <c r="Z1" s="60"/>
+      <c r="AA1" s="60"/>
+      <c r="AB1" s="60"/>
+      <c r="AC1" s="60"/>
     </row>
     <row r="2" spans="1:30" ht="16.5" customHeight="1">
       <c r="A2" s="23" t="s">
@@ -2224,10 +2234,10 @@
       <c r="AC2" s="54"/>
     </row>
     <row r="3" spans="1:30">
-      <c r="A3" s="56" t="s">
+      <c r="A3" s="61" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="56"/>
+      <c r="B3" s="61"/>
       <c r="D3">
         <v>2</v>
       </c>
@@ -2403,17 +2413,14 @@
         <f>ROUND(J5*M5%,2)</f>
         <v>0</v>
       </c>
-      <c r="O5" s="8">
-        <f>I5-N5</f>
-        <v>500.5</v>
-      </c>
+      <c r="O5" s="8"/>
       <c r="P5" s="8">
         <f>ROUND(K5*O5%,2)</f>
         <v>0</v>
       </c>
       <c r="Q5" s="8">
         <f>O5-P5</f>
-        <v>500.5</v>
+        <v>0</v>
       </c>
       <c r="R5" s="8">
         <f>ROUND(L5*Q5%,2)</f>
@@ -2682,9 +2689,705 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
+  <dimension ref="A1:AC6"/>
   <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col min="2" max="2" width="20.5703125" customWidth="1"/>
+    <col min="4" max="4" width="29.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.28515625" customWidth="1"/>
+    <col min="6" max="6" width="16.28515625" customWidth="1"/>
+    <col min="7" max="7" width="24.42578125" customWidth="1"/>
+    <col min="8" max="8" width="20.28515625" customWidth="1"/>
+    <col min="9" max="9" width="20" customWidth="1"/>
+    <col min="13" max="13" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="13.7109375" customWidth="1"/>
+    <col min="18" max="18" width="13" customWidth="1"/>
+    <col min="19" max="19" width="14.42578125" customWidth="1"/>
+    <col min="20" max="20" width="18.42578125" customWidth="1"/>
+    <col min="21" max="21" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="10" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:29" ht="18">
+      <c r="A1" s="60" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="60"/>
+      <c r="C1" s="60"/>
+      <c r="D1" s="60"/>
+      <c r="E1" s="60"/>
+      <c r="F1" s="60"/>
+      <c r="G1" s="60"/>
+      <c r="H1" s="60"/>
+      <c r="I1" s="60"/>
+      <c r="J1" s="60"/>
+      <c r="K1" s="60"/>
+      <c r="L1" s="60"/>
+      <c r="M1" s="60"/>
+      <c r="N1" s="60"/>
+      <c r="O1" s="60"/>
+      <c r="P1" s="60"/>
+      <c r="Q1" s="60"/>
+      <c r="R1" s="60"/>
+      <c r="S1" s="60"/>
+      <c r="T1" s="60"/>
+      <c r="U1" s="60"/>
+      <c r="V1" s="60"/>
+      <c r="W1" s="60"/>
+      <c r="X1" s="60"/>
+      <c r="Y1" s="60"/>
+      <c r="Z1" s="60"/>
+      <c r="AA1" s="60"/>
+      <c r="AB1" s="60"/>
+      <c r="AC1" s="60"/>
+    </row>
+    <row r="2" spans="1:29" ht="18">
+      <c r="A2" s="23" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="23" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" s="56"/>
+      <c r="D2" s="56"/>
+      <c r="E2" s="56"/>
+      <c r="F2" s="56"/>
+      <c r="G2" s="56"/>
+      <c r="H2" s="56"/>
+      <c r="I2" s="56"/>
+      <c r="J2" s="56"/>
+      <c r="K2" s="56"/>
+      <c r="L2" s="56"/>
+      <c r="M2" s="56"/>
+      <c r="N2" s="56"/>
+      <c r="O2" s="56"/>
+      <c r="P2" s="56"/>
+      <c r="Q2" s="56"/>
+      <c r="R2" s="56"/>
+      <c r="S2" s="56"/>
+      <c r="T2" s="56"/>
+      <c r="U2" s="56"/>
+      <c r="V2" s="56"/>
+      <c r="W2" s="56"/>
+      <c r="X2" s="56"/>
+      <c r="Y2" s="56"/>
+      <c r="Z2" s="56"/>
+      <c r="AA2" s="56"/>
+      <c r="AB2" s="56"/>
+      <c r="AC2" s="56"/>
+    </row>
+    <row r="3" spans="1:29">
+      <c r="A3" s="61" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="61"/>
+      <c r="C3" s="57"/>
+      <c r="D3" s="3">
+        <v>2</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="F3" s="5"/>
+      <c r="G3" s="5"/>
+      <c r="H3" s="5"/>
+      <c r="I3" s="6"/>
+      <c r="J3" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="K3" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="L3" s="7"/>
+      <c r="M3" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="N3" s="7">
+        <v>1</v>
+      </c>
+      <c r="O3" s="7"/>
+      <c r="P3" s="7"/>
+      <c r="Q3" s="7"/>
+      <c r="R3" s="7"/>
+      <c r="S3" s="6"/>
+      <c r="T3" s="6"/>
+      <c r="U3" s="6"/>
+      <c r="V3" s="6"/>
+      <c r="W3" s="6"/>
+      <c r="X3" s="6"/>
+      <c r="Y3" s="6"/>
+      <c r="Z3" s="6"/>
+      <c r="AA3" s="6"/>
+      <c r="AB3" s="6"/>
+      <c r="AC3" s="6"/>
+    </row>
+    <row r="4" spans="1:29" ht="42.75">
+      <c r="A4" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="E4" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="F4" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="G4" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="H4" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="I4" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="J4" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="K4" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="L4" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="M4" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="N4" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="O4" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="P4" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q4" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="R4" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="S4" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="T4" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="U4" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="V4" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="W4" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="X4" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y4" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="Z4" s="16" t="s">
+        <v>30</v>
+      </c>
+      <c r="AA4" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="AB4" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="AC4" s="17" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="5" spans="1:29">
+      <c r="A5" s="9">
+        <v>1</v>
+      </c>
+      <c r="B5" s="27" t="s">
+        <v>41</v>
+      </c>
+      <c r="C5" s="9">
+        <v>0</v>
+      </c>
+      <c r="D5" s="27" t="s">
+        <v>42</v>
+      </c>
+      <c r="E5" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="F5" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="G5" s="24">
+        <v>1</v>
+      </c>
+      <c r="H5" s="9">
+        <v>2255</v>
+      </c>
+      <c r="I5" s="8">
+        <v>2255</v>
+      </c>
+      <c r="J5" s="25"/>
+      <c r="K5" s="25"/>
+      <c r="L5" s="25"/>
+      <c r="M5" s="8">
+        <v>2255</v>
+      </c>
+      <c r="N5" s="8">
+        <v>0</v>
+      </c>
+      <c r="O5" s="8">
+        <v>2255</v>
+      </c>
+      <c r="P5" s="8">
+        <v>0</v>
+      </c>
+      <c r="Q5" s="8">
+        <v>2255</v>
+      </c>
+      <c r="R5" s="8">
+        <v>0</v>
+      </c>
+      <c r="S5" s="26">
+        <v>0</v>
+      </c>
+      <c r="T5" s="26">
+        <v>0</v>
+      </c>
+      <c r="U5" s="8">
+        <f>(I5-S5)</f>
+        <v>2255</v>
+      </c>
+      <c r="V5" s="24">
+        <v>88363222</v>
+      </c>
+      <c r="W5" s="18">
+        <v>0.18</v>
+      </c>
+      <c r="X5" s="24">
+        <f>IF($D$3=1,ROUND(((U5*W5)/2),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="Y5" s="31">
+        <f>IF($D$3=1,ROUND(((U5*W5)/2),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="Z5" s="24">
+        <f>IF($D$3=2,ROUND(((U5*W5)),2),0)</f>
+        <v>405.9</v>
+      </c>
+      <c r="AA5" s="24">
+        <v>0</v>
+      </c>
+      <c r="AB5" s="24">
+        <f>X5+Y5+Z5</f>
+        <v>405.9</v>
+      </c>
+      <c r="AC5" s="24">
+        <f>U5</f>
+        <v>2255</v>
+      </c>
+    </row>
+    <row r="6" spans="1:29">
+      <c r="A6" s="19"/>
+      <c r="B6" s="19"/>
+      <c r="C6" s="19"/>
+      <c r="D6" s="19"/>
+      <c r="E6" s="19"/>
+      <c r="F6" s="19"/>
+      <c r="G6" s="20"/>
+      <c r="H6" s="21"/>
+      <c r="I6" s="21"/>
+      <c r="J6" s="22"/>
+      <c r="K6" s="22"/>
+      <c r="L6" s="22"/>
+      <c r="M6" s="21"/>
+      <c r="N6" s="21"/>
+      <c r="O6" s="21"/>
+      <c r="P6" s="21"/>
+      <c r="Q6" s="21"/>
+      <c r="R6" s="21"/>
+      <c r="S6" s="21"/>
+      <c r="T6" s="21"/>
+      <c r="U6" s="21"/>
+      <c r="V6" s="21"/>
+      <c r="W6" s="22"/>
+      <c r="X6" s="21"/>
+      <c r="Y6" s="21"/>
+      <c r="Z6" s="21"/>
+      <c r="AA6" s="21"/>
+      <c r="AB6" s="21"/>
+      <c r="AC6" s="21"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:AC1"/>
+    <mergeCell ref="A3:B3"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:AC6"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="2" max="2" width="20.5703125" customWidth="1"/>
+    <col min="4" max="4" width="29.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.28515625" customWidth="1"/>
+    <col min="6" max="6" width="16.28515625" customWidth="1"/>
+    <col min="7" max="7" width="24.42578125" customWidth="1"/>
+    <col min="8" max="8" width="20.28515625" customWidth="1"/>
+    <col min="9" max="9" width="20" customWidth="1"/>
+    <col min="13" max="13" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="13.7109375" customWidth="1"/>
+    <col min="18" max="18" width="13" customWidth="1"/>
+    <col min="19" max="19" width="14.42578125" customWidth="1"/>
+    <col min="20" max="20" width="18.42578125" customWidth="1"/>
+    <col min="21" max="21" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="10.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:29" ht="18">
+      <c r="A1" s="60" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="60"/>
+      <c r="C1" s="60"/>
+      <c r="D1" s="60"/>
+      <c r="E1" s="60"/>
+      <c r="F1" s="60"/>
+      <c r="G1" s="60"/>
+      <c r="H1" s="60"/>
+      <c r="I1" s="60"/>
+      <c r="J1" s="60"/>
+      <c r="K1" s="60"/>
+      <c r="L1" s="60"/>
+      <c r="M1" s="60"/>
+      <c r="N1" s="60"/>
+      <c r="O1" s="60"/>
+      <c r="P1" s="60"/>
+      <c r="Q1" s="60"/>
+      <c r="R1" s="60"/>
+      <c r="S1" s="60"/>
+      <c r="T1" s="60"/>
+      <c r="U1" s="60"/>
+      <c r="V1" s="60"/>
+      <c r="W1" s="60"/>
+      <c r="X1" s="60"/>
+      <c r="Y1" s="60"/>
+      <c r="Z1" s="60"/>
+      <c r="AA1" s="60"/>
+      <c r="AB1" s="60"/>
+      <c r="AC1" s="60"/>
+    </row>
+    <row r="2" spans="1:29" ht="18">
+      <c r="A2" s="23" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="23" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" s="58"/>
+      <c r="D2" s="58"/>
+      <c r="E2" s="58"/>
+      <c r="F2" s="58"/>
+      <c r="G2" s="58"/>
+      <c r="H2" s="58"/>
+      <c r="I2" s="58"/>
+      <c r="J2" s="58"/>
+      <c r="K2" s="58"/>
+      <c r="L2" s="58"/>
+      <c r="M2" s="58"/>
+      <c r="N2" s="58"/>
+      <c r="O2" s="58"/>
+      <c r="P2" s="58"/>
+      <c r="Q2" s="58"/>
+      <c r="R2" s="58"/>
+      <c r="S2" s="58"/>
+      <c r="T2" s="58"/>
+      <c r="U2" s="58"/>
+      <c r="V2" s="58"/>
+      <c r="W2" s="58"/>
+      <c r="X2" s="58"/>
+      <c r="Y2" s="58"/>
+      <c r="Z2" s="58"/>
+      <c r="AA2" s="58"/>
+      <c r="AB2" s="58"/>
+      <c r="AC2" s="58"/>
+    </row>
+    <row r="3" spans="1:29">
+      <c r="A3" s="61" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="61"/>
+      <c r="C3" s="59"/>
+      <c r="D3" s="3">
+        <v>4</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="F3" s="5"/>
+      <c r="G3" s="5"/>
+      <c r="H3" s="5"/>
+      <c r="I3" s="6"/>
+      <c r="J3" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="K3" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="L3" s="7"/>
+      <c r="M3" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="N3" s="7">
+        <v>1</v>
+      </c>
+      <c r="O3" s="7"/>
+      <c r="P3" s="7"/>
+      <c r="Q3" s="7"/>
+      <c r="R3" s="7"/>
+      <c r="S3" s="6"/>
+      <c r="T3" s="6"/>
+      <c r="U3" s="6"/>
+      <c r="V3" s="6"/>
+      <c r="W3" s="6"/>
+      <c r="X3" s="6"/>
+      <c r="Y3" s="6"/>
+      <c r="Z3" s="6"/>
+      <c r="AA3" s="6"/>
+      <c r="AB3" s="6"/>
+      <c r="AC3" s="6"/>
+    </row>
+    <row r="4" spans="1:29" ht="42.75">
+      <c r="A4" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="E4" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="F4" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="G4" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="H4" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="I4" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="J4" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="K4" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="L4" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="M4" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="N4" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="O4" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="P4" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q4" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="R4" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="S4" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="T4" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="U4" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="V4" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="W4" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="X4" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y4" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="Z4" s="16" t="s">
+        <v>30</v>
+      </c>
+      <c r="AA4" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="AB4" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="AC4" s="17" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="5" spans="1:29">
+      <c r="A5" s="9">
+        <v>1</v>
+      </c>
+      <c r="B5" s="27" t="s">
+        <v>41</v>
+      </c>
+      <c r="C5" s="9">
+        <v>0</v>
+      </c>
+      <c r="D5" s="27" t="s">
+        <v>42</v>
+      </c>
+      <c r="E5" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="F5" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="G5" s="24">
+        <v>1</v>
+      </c>
+      <c r="H5" s="9">
+        <v>2255</v>
+      </c>
+      <c r="I5" s="8">
+        <v>2255</v>
+      </c>
+      <c r="J5" s="25"/>
+      <c r="K5" s="25"/>
+      <c r="L5" s="25"/>
+      <c r="M5" s="8">
+        <v>2255</v>
+      </c>
+      <c r="N5" s="8">
+        <v>0</v>
+      </c>
+      <c r="O5" s="8">
+        <v>2255</v>
+      </c>
+      <c r="P5" s="8">
+        <v>0</v>
+      </c>
+      <c r="Q5" s="8">
+        <v>2255</v>
+      </c>
+      <c r="R5" s="8">
+        <v>0</v>
+      </c>
+      <c r="S5" s="26">
+        <v>0</v>
+      </c>
+      <c r="T5" s="26">
+        <v>0</v>
+      </c>
+      <c r="U5" s="8">
+        <f>(I5-S5)</f>
+        <v>2255</v>
+      </c>
+      <c r="V5" s="24">
+        <v>88363222</v>
+      </c>
+      <c r="W5" s="18">
+        <v>0.18</v>
+      </c>
+      <c r="X5" s="24">
+        <v>0</v>
+      </c>
+      <c r="Y5" s="24">
+        <f>IF($D$3=1,ROUND(((U5*W5)/2),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="Z5" s="24">
+        <f>IF($D$3=2,ROUND(((U5*W5)),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="AA5" s="24">
+        <v>0</v>
+      </c>
+      <c r="AB5" s="24">
+        <f>X5+Y5+Z5+AA5</f>
+        <v>0</v>
+      </c>
+      <c r="AC5" s="24">
+        <f>U5</f>
+        <v>2255</v>
+      </c>
+    </row>
+    <row r="6" spans="1:29">
+      <c r="A6" s="19"/>
+      <c r="B6" s="19"/>
+      <c r="C6" s="19"/>
+      <c r="D6" s="19"/>
+      <c r="E6" s="19"/>
+      <c r="F6" s="19"/>
+      <c r="G6" s="20"/>
+      <c r="H6" s="21"/>
+      <c r="I6" s="21"/>
+      <c r="J6" s="22"/>
+      <c r="K6" s="22"/>
+      <c r="L6" s="22"/>
+      <c r="M6" s="21"/>
+      <c r="N6" s="21"/>
+      <c r="O6" s="21"/>
+      <c r="P6" s="21"/>
+      <c r="Q6" s="21"/>
+      <c r="R6" s="21"/>
+      <c r="S6" s="21"/>
+      <c r="T6" s="21"/>
+      <c r="U6" s="21"/>
+      <c r="V6" s="21"/>
+      <c r="W6" s="22"/>
+      <c r="X6" s="21"/>
+      <c r="Y6" s="21"/>
+      <c r="Z6" s="21"/>
+      <c r="AA6" s="21"/>
+      <c r="AB6" s="21"/>
+      <c r="AC6" s="21"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:AC1"/>
+    <mergeCell ref="A3:B3"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -2717,68 +3420,68 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:58" ht="18">
-      <c r="A1" s="55" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="55"/>
-      <c r="C1" s="55"/>
-      <c r="D1" s="55"/>
-      <c r="E1" s="55"/>
-      <c r="F1" s="55"/>
-      <c r="G1" s="55"/>
-      <c r="H1" s="55"/>
-      <c r="I1" s="55"/>
-      <c r="J1" s="55"/>
-      <c r="K1" s="55"/>
-      <c r="L1" s="55"/>
-      <c r="M1" s="55"/>
-      <c r="N1" s="55"/>
-      <c r="O1" s="55"/>
-      <c r="P1" s="55"/>
-      <c r="Q1" s="55"/>
-      <c r="R1" s="55"/>
-      <c r="S1" s="55"/>
-      <c r="T1" s="55"/>
-      <c r="U1" s="55"/>
-      <c r="V1" s="55"/>
-      <c r="W1" s="55"/>
-      <c r="X1" s="55"/>
-      <c r="Y1" s="55"/>
-      <c r="Z1" s="55"/>
-      <c r="AA1" s="55"/>
-      <c r="AB1" s="55"/>
-      <c r="AC1" s="55"/>
-      <c r="AD1" s="55" t="s">
-        <v>0</v>
-      </c>
-      <c r="AE1" s="55"/>
-      <c r="AF1" s="55"/>
-      <c r="AG1" s="55"/>
-      <c r="AH1" s="55"/>
-      <c r="AI1" s="55"/>
-      <c r="AJ1" s="55"/>
-      <c r="AK1" s="55"/>
-      <c r="AL1" s="55"/>
-      <c r="AM1" s="55"/>
-      <c r="AN1" s="55"/>
-      <c r="AO1" s="55"/>
-      <c r="AP1" s="55"/>
-      <c r="AQ1" s="55"/>
-      <c r="AR1" s="55"/>
-      <c r="AS1" s="55"/>
-      <c r="AT1" s="55"/>
-      <c r="AU1" s="55"/>
-      <c r="AV1" s="55"/>
-      <c r="AW1" s="55"/>
-      <c r="AX1" s="55"/>
-      <c r="AY1" s="55"/>
-      <c r="AZ1" s="55"/>
-      <c r="BA1" s="55"/>
-      <c r="BB1" s="55"/>
-      <c r="BC1" s="55"/>
-      <c r="BD1" s="55"/>
-      <c r="BE1" s="55"/>
-      <c r="BF1" s="55"/>
+      <c r="A1" s="60" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="60"/>
+      <c r="C1" s="60"/>
+      <c r="D1" s="60"/>
+      <c r="E1" s="60"/>
+      <c r="F1" s="60"/>
+      <c r="G1" s="60"/>
+      <c r="H1" s="60"/>
+      <c r="I1" s="60"/>
+      <c r="J1" s="60"/>
+      <c r="K1" s="60"/>
+      <c r="L1" s="60"/>
+      <c r="M1" s="60"/>
+      <c r="N1" s="60"/>
+      <c r="O1" s="60"/>
+      <c r="P1" s="60"/>
+      <c r="Q1" s="60"/>
+      <c r="R1" s="60"/>
+      <c r="S1" s="60"/>
+      <c r="T1" s="60"/>
+      <c r="U1" s="60"/>
+      <c r="V1" s="60"/>
+      <c r="W1" s="60"/>
+      <c r="X1" s="60"/>
+      <c r="Y1" s="60"/>
+      <c r="Z1" s="60"/>
+      <c r="AA1" s="60"/>
+      <c r="AB1" s="60"/>
+      <c r="AC1" s="60"/>
+      <c r="AD1" s="60" t="s">
+        <v>0</v>
+      </c>
+      <c r="AE1" s="60"/>
+      <c r="AF1" s="60"/>
+      <c r="AG1" s="60"/>
+      <c r="AH1" s="60"/>
+      <c r="AI1" s="60"/>
+      <c r="AJ1" s="60"/>
+      <c r="AK1" s="60"/>
+      <c r="AL1" s="60"/>
+      <c r="AM1" s="60"/>
+      <c r="AN1" s="60"/>
+      <c r="AO1" s="60"/>
+      <c r="AP1" s="60"/>
+      <c r="AQ1" s="60"/>
+      <c r="AR1" s="60"/>
+      <c r="AS1" s="60"/>
+      <c r="AT1" s="60"/>
+      <c r="AU1" s="60"/>
+      <c r="AV1" s="60"/>
+      <c r="AW1" s="60"/>
+      <c r="AX1" s="60"/>
+      <c r="AY1" s="60"/>
+      <c r="AZ1" s="60"/>
+      <c r="BA1" s="60"/>
+      <c r="BB1" s="60"/>
+      <c r="BC1" s="60"/>
+      <c r="BD1" s="60"/>
+      <c r="BE1" s="60"/>
+      <c r="BF1" s="60"/>
     </row>
     <row r="2" spans="1:58" ht="18">
       <c r="A2" s="23" t="s">
@@ -2849,10 +3552,10 @@
       <c r="BF2" s="36"/>
     </row>
     <row r="3" spans="1:58">
-      <c r="A3" s="56" t="s">
+      <c r="A3" s="61" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="56"/>
+      <c r="B3" s="61"/>
       <c r="C3" s="29"/>
       <c r="D3" s="3">
         <v>2</v>
@@ -2892,10 +3595,10 @@
       <c r="AA3" s="6"/>
       <c r="AB3" s="6"/>
       <c r="AC3" s="6"/>
-      <c r="AD3" s="56" t="s">
+      <c r="AD3" s="61" t="s">
         <v>3</v>
       </c>
-      <c r="AE3" s="56"/>
+      <c r="AE3" s="61"/>
       <c r="AF3" s="37"/>
       <c r="AG3" s="3">
         <v>2</v>
@@ -3365,37 +4068,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="18">
-      <c r="A1" s="55" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="55"/>
-      <c r="C1" s="55"/>
-      <c r="D1" s="55"/>
-      <c r="E1" s="55"/>
-      <c r="F1" s="55"/>
-      <c r="G1" s="55"/>
-      <c r="H1" s="55"/>
-      <c r="I1" s="55"/>
-      <c r="J1" s="55"/>
-      <c r="K1" s="55"/>
-      <c r="L1" s="55"/>
-      <c r="M1" s="55"/>
-      <c r="N1" s="55"/>
-      <c r="O1" s="55"/>
-      <c r="P1" s="55"/>
-      <c r="Q1" s="55"/>
-      <c r="R1" s="55"/>
-      <c r="S1" s="55"/>
-      <c r="T1" s="55"/>
-      <c r="U1" s="55"/>
-      <c r="V1" s="55"/>
-      <c r="W1" s="55"/>
-      <c r="X1" s="55"/>
-      <c r="Y1" s="55"/>
-      <c r="Z1" s="55"/>
-      <c r="AA1" s="55"/>
-      <c r="AB1" s="55"/>
-      <c r="AC1" s="55"/>
+      <c r="A1" s="60" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="60"/>
+      <c r="C1" s="60"/>
+      <c r="D1" s="60"/>
+      <c r="E1" s="60"/>
+      <c r="F1" s="60"/>
+      <c r="G1" s="60"/>
+      <c r="H1" s="60"/>
+      <c r="I1" s="60"/>
+      <c r="J1" s="60"/>
+      <c r="K1" s="60"/>
+      <c r="L1" s="60"/>
+      <c r="M1" s="60"/>
+      <c r="N1" s="60"/>
+      <c r="O1" s="60"/>
+      <c r="P1" s="60"/>
+      <c r="Q1" s="60"/>
+      <c r="R1" s="60"/>
+      <c r="S1" s="60"/>
+      <c r="T1" s="60"/>
+      <c r="U1" s="60"/>
+      <c r="V1" s="60"/>
+      <c r="W1" s="60"/>
+      <c r="X1" s="60"/>
+      <c r="Y1" s="60"/>
+      <c r="Z1" s="60"/>
+      <c r="AA1" s="60"/>
+      <c r="AB1" s="60"/>
+      <c r="AC1" s="60"/>
     </row>
     <row r="2" spans="1:29" ht="18">
       <c r="A2" s="23" t="s">
@@ -3433,10 +4136,10 @@
       <c r="AC2" s="28"/>
     </row>
     <row r="3" spans="1:29">
-      <c r="A3" s="56" t="s">
+      <c r="A3" s="61" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="56"/>
+      <c r="B3" s="61"/>
       <c r="C3" s="29"/>
       <c r="D3" s="3">
         <v>4</v>
@@ -3647,13 +4350,13 @@
         <f>IF($D$3=4,ROUND(((U5*W5)/2),2),0)</f>
         <v>202.95</v>
       </c>
-      <c r="AB5" s="8">
-        <f>X5+Y5+Z5</f>
-        <v>202.95</v>
-      </c>
-      <c r="AC5" s="8">
+      <c r="AB5" s="24">
+        <f>X5+Y5+Z5+AA5</f>
+        <v>405.9</v>
+      </c>
+      <c r="AC5" s="24">
         <f>U5+AB5</f>
-        <v>2457.9499999999998</v>
+        <v>2660.9</v>
       </c>
     </row>
     <row r="6" spans="1:29">
@@ -3719,37 +4422,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="18">
-      <c r="A1" s="55" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="55"/>
-      <c r="C1" s="55"/>
-      <c r="D1" s="55"/>
-      <c r="E1" s="55"/>
-      <c r="F1" s="55"/>
-      <c r="G1" s="55"/>
-      <c r="H1" s="55"/>
-      <c r="I1" s="55"/>
-      <c r="J1" s="55"/>
-      <c r="K1" s="55"/>
-      <c r="L1" s="55"/>
-      <c r="M1" s="55"/>
-      <c r="N1" s="55"/>
-      <c r="O1" s="55"/>
-      <c r="P1" s="55"/>
-      <c r="Q1" s="55"/>
-      <c r="R1" s="55"/>
-      <c r="S1" s="55"/>
-      <c r="T1" s="55"/>
-      <c r="U1" s="55"/>
-      <c r="V1" s="55"/>
-      <c r="W1" s="55"/>
-      <c r="X1" s="55"/>
-      <c r="Y1" s="55"/>
-      <c r="Z1" s="55"/>
-      <c r="AA1" s="55"/>
-      <c r="AB1" s="55"/>
-      <c r="AC1" s="55"/>
+      <c r="A1" s="60" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="60"/>
+      <c r="C1" s="60"/>
+      <c r="D1" s="60"/>
+      <c r="E1" s="60"/>
+      <c r="F1" s="60"/>
+      <c r="G1" s="60"/>
+      <c r="H1" s="60"/>
+      <c r="I1" s="60"/>
+      <c r="J1" s="60"/>
+      <c r="K1" s="60"/>
+      <c r="L1" s="60"/>
+      <c r="M1" s="60"/>
+      <c r="N1" s="60"/>
+      <c r="O1" s="60"/>
+      <c r="P1" s="60"/>
+      <c r="Q1" s="60"/>
+      <c r="R1" s="60"/>
+      <c r="S1" s="60"/>
+      <c r="T1" s="60"/>
+      <c r="U1" s="60"/>
+      <c r="V1" s="60"/>
+      <c r="W1" s="60"/>
+      <c r="X1" s="60"/>
+      <c r="Y1" s="60"/>
+      <c r="Z1" s="60"/>
+      <c r="AA1" s="60"/>
+      <c r="AB1" s="60"/>
+      <c r="AC1" s="60"/>
     </row>
     <row r="2" spans="1:29" ht="18">
       <c r="A2" s="23" t="s">
@@ -3787,10 +4490,10 @@
       <c r="AC2" s="28"/>
     </row>
     <row r="3" spans="1:29">
-      <c r="A3" s="56" t="s">
+      <c r="A3" s="61" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="56"/>
+      <c r="B3" s="61"/>
       <c r="C3" s="29"/>
       <c r="D3" s="3">
         <v>3</v>
@@ -4072,37 +4775,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="18">
-      <c r="A1" s="55" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="55"/>
-      <c r="C1" s="55"/>
-      <c r="D1" s="55"/>
-      <c r="E1" s="55"/>
-      <c r="F1" s="55"/>
-      <c r="G1" s="55"/>
-      <c r="H1" s="55"/>
-      <c r="I1" s="55"/>
-      <c r="J1" s="55"/>
-      <c r="K1" s="55"/>
-      <c r="L1" s="55"/>
-      <c r="M1" s="55"/>
-      <c r="N1" s="55"/>
-      <c r="O1" s="55"/>
-      <c r="P1" s="55"/>
-      <c r="Q1" s="55"/>
-      <c r="R1" s="55"/>
-      <c r="S1" s="55"/>
-      <c r="T1" s="55"/>
-      <c r="U1" s="55"/>
-      <c r="V1" s="55"/>
-      <c r="W1" s="55"/>
-      <c r="X1" s="55"/>
-      <c r="Y1" s="55"/>
-      <c r="Z1" s="55"/>
-      <c r="AA1" s="55"/>
-      <c r="AB1" s="55"/>
-      <c r="AC1" s="55"/>
+      <c r="A1" s="60" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="60"/>
+      <c r="C1" s="60"/>
+      <c r="D1" s="60"/>
+      <c r="E1" s="60"/>
+      <c r="F1" s="60"/>
+      <c r="G1" s="60"/>
+      <c r="H1" s="60"/>
+      <c r="I1" s="60"/>
+      <c r="J1" s="60"/>
+      <c r="K1" s="60"/>
+      <c r="L1" s="60"/>
+      <c r="M1" s="60"/>
+      <c r="N1" s="60"/>
+      <c r="O1" s="60"/>
+      <c r="P1" s="60"/>
+      <c r="Q1" s="60"/>
+      <c r="R1" s="60"/>
+      <c r="S1" s="60"/>
+      <c r="T1" s="60"/>
+      <c r="U1" s="60"/>
+      <c r="V1" s="60"/>
+      <c r="W1" s="60"/>
+      <c r="X1" s="60"/>
+      <c r="Y1" s="60"/>
+      <c r="Z1" s="60"/>
+      <c r="AA1" s="60"/>
+      <c r="AB1" s="60"/>
+      <c r="AC1" s="60"/>
     </row>
     <row r="2" spans="1:29" ht="18">
       <c r="A2" s="23" t="s">
@@ -4140,10 +4843,10 @@
       <c r="AC2" s="28"/>
     </row>
     <row r="3" spans="1:29">
-      <c r="A3" s="56" t="s">
+      <c r="A3" s="61" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="56"/>
+      <c r="B3" s="61"/>
       <c r="C3" s="29"/>
       <c r="D3" s="3">
         <v>5</v>
@@ -4427,37 +5130,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="18">
-      <c r="A1" s="55" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="55"/>
-      <c r="C1" s="55"/>
-      <c r="D1" s="55"/>
-      <c r="E1" s="55"/>
-      <c r="F1" s="55"/>
-      <c r="G1" s="55"/>
-      <c r="H1" s="55"/>
-      <c r="I1" s="55"/>
-      <c r="J1" s="55"/>
-      <c r="K1" s="55"/>
-      <c r="L1" s="55"/>
-      <c r="M1" s="55"/>
-      <c r="N1" s="55"/>
-      <c r="O1" s="55"/>
-      <c r="P1" s="55"/>
-      <c r="Q1" s="55"/>
-      <c r="R1" s="55"/>
-      <c r="S1" s="55"/>
-      <c r="T1" s="55"/>
-      <c r="U1" s="55"/>
-      <c r="V1" s="55"/>
-      <c r="W1" s="55"/>
-      <c r="X1" s="55"/>
-      <c r="Y1" s="55"/>
-      <c r="Z1" s="55"/>
-      <c r="AA1" s="55"/>
-      <c r="AB1" s="55"/>
-      <c r="AC1" s="55"/>
+      <c r="A1" s="60" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="60"/>
+      <c r="C1" s="60"/>
+      <c r="D1" s="60"/>
+      <c r="E1" s="60"/>
+      <c r="F1" s="60"/>
+      <c r="G1" s="60"/>
+      <c r="H1" s="60"/>
+      <c r="I1" s="60"/>
+      <c r="J1" s="60"/>
+      <c r="K1" s="60"/>
+      <c r="L1" s="60"/>
+      <c r="M1" s="60"/>
+      <c r="N1" s="60"/>
+      <c r="O1" s="60"/>
+      <c r="P1" s="60"/>
+      <c r="Q1" s="60"/>
+      <c r="R1" s="60"/>
+      <c r="S1" s="60"/>
+      <c r="T1" s="60"/>
+      <c r="U1" s="60"/>
+      <c r="V1" s="60"/>
+      <c r="W1" s="60"/>
+      <c r="X1" s="60"/>
+      <c r="Y1" s="60"/>
+      <c r="Z1" s="60"/>
+      <c r="AA1" s="60"/>
+      <c r="AB1" s="60"/>
+      <c r="AC1" s="60"/>
     </row>
     <row r="2" spans="1:29" ht="18">
       <c r="A2" s="23" t="s">
@@ -4495,10 +5198,10 @@
       <c r="AC2" s="32"/>
     </row>
     <row r="3" spans="1:29">
-      <c r="A3" s="56" t="s">
+      <c r="A3" s="61" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="56"/>
+      <c r="B3" s="61"/>
       <c r="C3" s="33"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -4780,37 +5483,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="18">
-      <c r="A1" s="55" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="55"/>
-      <c r="C1" s="55"/>
-      <c r="D1" s="55"/>
-      <c r="E1" s="55"/>
-      <c r="F1" s="55"/>
-      <c r="G1" s="55"/>
-      <c r="H1" s="55"/>
-      <c r="I1" s="55"/>
-      <c r="J1" s="55"/>
-      <c r="K1" s="55"/>
-      <c r="L1" s="55"/>
-      <c r="M1" s="55"/>
-      <c r="N1" s="55"/>
-      <c r="O1" s="55"/>
-      <c r="P1" s="55"/>
-      <c r="Q1" s="55"/>
-      <c r="R1" s="55"/>
-      <c r="S1" s="55"/>
-      <c r="T1" s="55"/>
-      <c r="U1" s="55"/>
-      <c r="V1" s="55"/>
-      <c r="W1" s="55"/>
-      <c r="X1" s="55"/>
-      <c r="Y1" s="55"/>
-      <c r="Z1" s="55"/>
-      <c r="AA1" s="55"/>
-      <c r="AB1" s="55"/>
-      <c r="AC1" s="55"/>
+      <c r="A1" s="60" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="60"/>
+      <c r="C1" s="60"/>
+      <c r="D1" s="60"/>
+      <c r="E1" s="60"/>
+      <c r="F1" s="60"/>
+      <c r="G1" s="60"/>
+      <c r="H1" s="60"/>
+      <c r="I1" s="60"/>
+      <c r="J1" s="60"/>
+      <c r="K1" s="60"/>
+      <c r="L1" s="60"/>
+      <c r="M1" s="60"/>
+      <c r="N1" s="60"/>
+      <c r="O1" s="60"/>
+      <c r="P1" s="60"/>
+      <c r="Q1" s="60"/>
+      <c r="R1" s="60"/>
+      <c r="S1" s="60"/>
+      <c r="T1" s="60"/>
+      <c r="U1" s="60"/>
+      <c r="V1" s="60"/>
+      <c r="W1" s="60"/>
+      <c r="X1" s="60"/>
+      <c r="Y1" s="60"/>
+      <c r="Z1" s="60"/>
+      <c r="AA1" s="60"/>
+      <c r="AB1" s="60"/>
+      <c r="AC1" s="60"/>
     </row>
     <row r="2" spans="1:29" ht="18">
       <c r="A2" s="23" t="s">
@@ -4848,10 +5551,10 @@
       <c r="AC2" s="34"/>
     </row>
     <row r="3" spans="1:29">
-      <c r="A3" s="56" t="s">
+      <c r="A3" s="61" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="56"/>
+      <c r="B3" s="61"/>
       <c r="C3" s="35"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -5060,7 +5763,7 @@
       <c r="AA5" s="24">
         <v>0</v>
       </c>
-      <c r="AB5" s="8">
+      <c r="AB5" s="24">
         <f>X5+Y5+Z5</f>
         <v>405.9</v>
       </c>
@@ -5131,37 +5834,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="18">
-      <c r="A1" s="55" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="55"/>
-      <c r="C1" s="55"/>
-      <c r="D1" s="55"/>
-      <c r="E1" s="55"/>
-      <c r="F1" s="55"/>
-      <c r="G1" s="55"/>
-      <c r="H1" s="55"/>
-      <c r="I1" s="55"/>
-      <c r="J1" s="55"/>
-      <c r="K1" s="55"/>
-      <c r="L1" s="55"/>
-      <c r="M1" s="55"/>
-      <c r="N1" s="55"/>
-      <c r="O1" s="55"/>
-      <c r="P1" s="55"/>
-      <c r="Q1" s="55"/>
-      <c r="R1" s="55"/>
-      <c r="S1" s="55"/>
-      <c r="T1" s="55"/>
-      <c r="U1" s="55"/>
-      <c r="V1" s="55"/>
-      <c r="W1" s="55"/>
-      <c r="X1" s="55"/>
-      <c r="Y1" s="55"/>
-      <c r="Z1" s="55"/>
-      <c r="AA1" s="55"/>
-      <c r="AB1" s="55"/>
-      <c r="AC1" s="55"/>
+      <c r="A1" s="60" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="60"/>
+      <c r="C1" s="60"/>
+      <c r="D1" s="60"/>
+      <c r="E1" s="60"/>
+      <c r="F1" s="60"/>
+      <c r="G1" s="60"/>
+      <c r="H1" s="60"/>
+      <c r="I1" s="60"/>
+      <c r="J1" s="60"/>
+      <c r="K1" s="60"/>
+      <c r="L1" s="60"/>
+      <c r="M1" s="60"/>
+      <c r="N1" s="60"/>
+      <c r="O1" s="60"/>
+      <c r="P1" s="60"/>
+      <c r="Q1" s="60"/>
+      <c r="R1" s="60"/>
+      <c r="S1" s="60"/>
+      <c r="T1" s="60"/>
+      <c r="U1" s="60"/>
+      <c r="V1" s="60"/>
+      <c r="W1" s="60"/>
+      <c r="X1" s="60"/>
+      <c r="Y1" s="60"/>
+      <c r="Z1" s="60"/>
+      <c r="AA1" s="60"/>
+      <c r="AB1" s="60"/>
+      <c r="AC1" s="60"/>
     </row>
     <row r="2" spans="1:29" ht="18">
       <c r="A2" s="23" t="s">
@@ -5199,10 +5902,10 @@
       <c r="AC2" s="36"/>
     </row>
     <row r="3" spans="1:29">
-      <c r="A3" s="56" t="s">
+      <c r="A3" s="61" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="56"/>
+      <c r="B3" s="61"/>
       <c r="C3" s="37"/>
       <c r="D3" s="3">
         <v>2</v>
@@ -5358,7 +6061,7 @@
         <v>250.25</v>
       </c>
       <c r="I5" s="8">
-        <v>2255</v>
+        <v>500.5</v>
       </c>
       <c r="J5" s="25">
         <v>2.21</v>
@@ -5370,32 +6073,38 @@
         <v>2.5</v>
       </c>
       <c r="M5" s="8">
-        <v>2255</v>
+        <v>500.5</v>
       </c>
       <c r="N5" s="8">
-        <v>0</v>
+        <f>ROUND(J5*M5%,2)</f>
+        <v>11.06</v>
       </c>
       <c r="O5" s="8">
-        <v>2255</v>
+        <f>I5-N5</f>
+        <v>489.44</v>
       </c>
       <c r="P5" s="8">
-        <v>0</v>
+        <f>ROUND(K5*O5%,2)</f>
+        <v>8.76</v>
       </c>
       <c r="Q5" s="8">
-        <v>2255</v>
+        <f>O5-P5</f>
+        <v>480.68</v>
       </c>
       <c r="R5" s="8">
-        <v>0</v>
+        <f>ROUND(L5*Q5%,2)</f>
+        <v>12.02</v>
       </c>
       <c r="S5" s="26">
-        <v>0</v>
+        <f>N5+P5+R5</f>
+        <v>31.84</v>
       </c>
       <c r="T5" s="26">
         <v>0</v>
       </c>
       <c r="U5" s="8">
         <f>(I5-S5)</f>
-        <v>2255</v>
+        <v>468.66</v>
       </c>
       <c r="V5" s="24">
         <v>88363222</v>
@@ -5411,20 +6120,20 @@
         <f>IF($D$3=1,ROUND(((U5*W5)/2),2),0)</f>
         <v>0</v>
       </c>
-      <c r="Z5" s="24">
+      <c r="Z5" s="8">
         <f>IF($D$3=2,ROUND(((U5*W5)),2),0)</f>
-        <v>405.9</v>
+        <v>84.36</v>
       </c>
       <c r="AA5" s="24">
         <v>0</v>
       </c>
       <c r="AB5" s="24">
         <f>X5+Y5+Z5</f>
-        <v>405.9</v>
+        <v>84.36</v>
       </c>
       <c r="AC5" s="24">
         <f>U5+AB5</f>
-        <v>2660.9</v>
+        <v>553.02</v>
       </c>
     </row>
     <row r="6" spans="1:29">
@@ -5469,7 +6178,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AD7"/>
+  <dimension ref="A1:AE8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="20.5703125" customWidth="1"/>
@@ -5489,42 +6198,43 @@
     <col min="22" max="22" width="10.140625" bestFit="1" customWidth="1"/>
     <col min="26" max="26" width="10.5703125" bestFit="1" customWidth="1"/>
     <col min="30" max="30" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" ht="18">
-      <c r="A1" s="55" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="55"/>
-      <c r="C1" s="55"/>
-      <c r="D1" s="55"/>
-      <c r="E1" s="55"/>
-      <c r="F1" s="55"/>
-      <c r="G1" s="55"/>
-      <c r="H1" s="55"/>
-      <c r="I1" s="55"/>
-      <c r="J1" s="55"/>
-      <c r="K1" s="55"/>
-      <c r="L1" s="55"/>
-      <c r="M1" s="55"/>
-      <c r="N1" s="55"/>
-      <c r="O1" s="55"/>
-      <c r="P1" s="55"/>
-      <c r="Q1" s="55"/>
-      <c r="R1" s="55"/>
-      <c r="S1" s="55"/>
-      <c r="T1" s="55"/>
-      <c r="U1" s="55"/>
-      <c r="V1" s="55"/>
-      <c r="W1" s="55"/>
-      <c r="X1" s="55"/>
-      <c r="Y1" s="55"/>
-      <c r="Z1" s="55"/>
-      <c r="AA1" s="55"/>
-      <c r="AB1" s="55"/>
-      <c r="AC1" s="55"/>
-    </row>
-    <row r="2" spans="1:30" ht="16.5" customHeight="1">
+    <row r="1" spans="1:31" ht="18">
+      <c r="A1" s="60" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="60"/>
+      <c r="C1" s="60"/>
+      <c r="D1" s="60"/>
+      <c r="E1" s="60"/>
+      <c r="F1" s="60"/>
+      <c r="G1" s="60"/>
+      <c r="H1" s="60"/>
+      <c r="I1" s="60"/>
+      <c r="J1" s="60"/>
+      <c r="K1" s="60"/>
+      <c r="L1" s="60"/>
+      <c r="M1" s="60"/>
+      <c r="N1" s="60"/>
+      <c r="O1" s="60"/>
+      <c r="P1" s="60"/>
+      <c r="Q1" s="60"/>
+      <c r="R1" s="60"/>
+      <c r="S1" s="60"/>
+      <c r="T1" s="60"/>
+      <c r="U1" s="60"/>
+      <c r="V1" s="60"/>
+      <c r="W1" s="60"/>
+      <c r="X1" s="60"/>
+      <c r="Y1" s="60"/>
+      <c r="Z1" s="60"/>
+      <c r="AA1" s="60"/>
+      <c r="AB1" s="60"/>
+      <c r="AC1" s="60"/>
+    </row>
+    <row r="2" spans="1:31" ht="16.5" customHeight="1">
       <c r="A2" s="23" t="s">
         <v>1</v>
       </c>
@@ -5559,11 +6269,11 @@
       <c r="AB2" s="41"/>
       <c r="AC2" s="41"/>
     </row>
-    <row r="3" spans="1:30">
-      <c r="A3" s="56" t="s">
+    <row r="3" spans="1:31">
+      <c r="A3" s="61" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="56"/>
+      <c r="B3" s="61"/>
       <c r="D3">
         <v>2</v>
       </c>
@@ -5603,7 +6313,7 @@
       <c r="AB3" s="6"/>
       <c r="AC3" s="6"/>
     </row>
-    <row r="4" spans="1:30" ht="42.75">
+    <row r="4" spans="1:31" ht="42.75">
       <c r="A4" s="10" t="s">
         <v>8</v>
       </c>
@@ -5694,8 +6404,11 @@
       <c r="AD4" s="10" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="5" spans="1:30">
+      <c r="AE4" s="10" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="5" spans="1:31">
       <c r="A5" s="9">
         <v>1</v>
       </c>
@@ -5798,8 +6511,11 @@
       <c r="AD5" s="46" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="6" spans="1:30" ht="16.5" customHeight="1">
+      <c r="AE5" s="46" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="6" spans="1:31" ht="16.5" customHeight="1">
       <c r="A6" s="9">
         <v>2</v>
       </c>
@@ -5902,8 +6618,11 @@
       <c r="AD6" s="46" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="7" spans="1:30">
+      <c r="AE6" s="46" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="7" spans="1:31">
       <c r="A7" s="9">
         <v>3</v>
       </c>
@@ -5988,7 +6707,7 @@
         <f>IF($D$3=1,ROUND(((U7*W7)/2),2),0)</f>
         <v>0</v>
       </c>
-      <c r="Z7" s="57">
+      <c r="Z7" s="55">
         <f t="shared" si="6"/>
         <v>364.5</v>
       </c>
@@ -6006,6 +6725,12 @@
       <c r="AD7" s="46" t="s">
         <v>54</v>
       </c>
+      <c r="AE7" s="46" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="8" spans="1:31">
+      <c r="AE8" s="46"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
Purchase Bills For New Cases
Purchase Bills For New Cases
</commit_message>
<xml_diff>
--- a/testdata/DBfin.xlsx
+++ b/testdata/DBfin.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4507"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="2520" windowWidth="16695" windowHeight="6540" tabRatio="594" firstSheet="9" activeTab="12"/>
+    <workbookView xWindow="0" yWindow="2520" windowWidth="16695" windowHeight="6540" tabRatio="594" firstSheet="11" activeTab="13"/>
   </bookViews>
   <sheets>
     <sheet name="PurchaseBillsLocal" sheetId="1" r:id="rId1"/>
@@ -20,13 +20,14 @@
     <sheet name="PurchaseBills_Ex_Grn_Igst" sheetId="11" r:id="rId11"/>
     <sheet name="PurchaseBills_Interstate_Un" sheetId="12" r:id="rId12"/>
     <sheet name="PurchaseBillsUTGST_Ureq" sheetId="13" r:id="rId13"/>
+    <sheet name="PurchaseBills_Un_Regrd_Iter" sheetId="14" r:id="rId14"/>
   </sheets>
   <calcPr calcId="125725"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="670" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="741" uniqueCount="62">
   <si>
     <t>Scenario  : Local Sales - Stock UOM and Sales UOM (Similar)   DOC NO :  SORD-2425-00089</t>
   </si>
@@ -363,7 +364,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -482,6 +483,12 @@
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="165" fontId="3" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -825,68 +832,68 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:59" ht="18">
-      <c r="A1" s="60" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="60"/>
-      <c r="C1" s="60"/>
-      <c r="D1" s="60"/>
-      <c r="E1" s="60"/>
-      <c r="F1" s="60"/>
-      <c r="G1" s="60"/>
-      <c r="H1" s="60"/>
-      <c r="I1" s="60"/>
-      <c r="J1" s="60"/>
-      <c r="K1" s="60"/>
-      <c r="L1" s="60"/>
-      <c r="M1" s="60"/>
-      <c r="N1" s="60"/>
-      <c r="O1" s="60"/>
-      <c r="P1" s="60"/>
-      <c r="Q1" s="60"/>
-      <c r="R1" s="60"/>
-      <c r="S1" s="60"/>
-      <c r="T1" s="60"/>
-      <c r="U1" s="60"/>
-      <c r="V1" s="60"/>
-      <c r="W1" s="60"/>
-      <c r="X1" s="60"/>
-      <c r="Y1" s="60"/>
-      <c r="Z1" s="60"/>
-      <c r="AA1" s="60"/>
-      <c r="AB1" s="60"/>
-      <c r="AC1" s="60"/>
-      <c r="AD1" s="60" t="s">
-        <v>0</v>
-      </c>
-      <c r="AE1" s="60"/>
-      <c r="AF1" s="60"/>
-      <c r="AG1" s="60"/>
-      <c r="AH1" s="60"/>
-      <c r="AI1" s="60"/>
-      <c r="AJ1" s="60"/>
-      <c r="AK1" s="60"/>
-      <c r="AL1" s="60"/>
-      <c r="AM1" s="60"/>
-      <c r="AN1" s="60"/>
-      <c r="AO1" s="60"/>
-      <c r="AP1" s="60"/>
-      <c r="AQ1" s="60"/>
-      <c r="AR1" s="60"/>
-      <c r="AS1" s="60"/>
-      <c r="AT1" s="60"/>
-      <c r="AU1" s="60"/>
-      <c r="AV1" s="60"/>
-      <c r="AW1" s="60"/>
-      <c r="AX1" s="60"/>
-      <c r="AY1" s="60"/>
-      <c r="AZ1" s="60"/>
-      <c r="BA1" s="60"/>
-      <c r="BB1" s="60"/>
-      <c r="BC1" s="60"/>
-      <c r="BD1" s="60"/>
-      <c r="BE1" s="60"/>
-      <c r="BF1" s="60"/>
+      <c r="A1" s="62" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="62"/>
+      <c r="C1" s="62"/>
+      <c r="D1" s="62"/>
+      <c r="E1" s="62"/>
+      <c r="F1" s="62"/>
+      <c r="G1" s="62"/>
+      <c r="H1" s="62"/>
+      <c r="I1" s="62"/>
+      <c r="J1" s="62"/>
+      <c r="K1" s="62"/>
+      <c r="L1" s="62"/>
+      <c r="M1" s="62"/>
+      <c r="N1" s="62"/>
+      <c r="O1" s="62"/>
+      <c r="P1" s="62"/>
+      <c r="Q1" s="62"/>
+      <c r="R1" s="62"/>
+      <c r="S1" s="62"/>
+      <c r="T1" s="62"/>
+      <c r="U1" s="62"/>
+      <c r="V1" s="62"/>
+      <c r="W1" s="62"/>
+      <c r="X1" s="62"/>
+      <c r="Y1" s="62"/>
+      <c r="Z1" s="62"/>
+      <c r="AA1" s="62"/>
+      <c r="AB1" s="62"/>
+      <c r="AC1" s="62"/>
+      <c r="AD1" s="62" t="s">
+        <v>0</v>
+      </c>
+      <c r="AE1" s="62"/>
+      <c r="AF1" s="62"/>
+      <c r="AG1" s="62"/>
+      <c r="AH1" s="62"/>
+      <c r="AI1" s="62"/>
+      <c r="AJ1" s="62"/>
+      <c r="AK1" s="62"/>
+      <c r="AL1" s="62"/>
+      <c r="AM1" s="62"/>
+      <c r="AN1" s="62"/>
+      <c r="AO1" s="62"/>
+      <c r="AP1" s="62"/>
+      <c r="AQ1" s="62"/>
+      <c r="AR1" s="62"/>
+      <c r="AS1" s="62"/>
+      <c r="AT1" s="62"/>
+      <c r="AU1" s="62"/>
+      <c r="AV1" s="62"/>
+      <c r="AW1" s="62"/>
+      <c r="AX1" s="62"/>
+      <c r="AY1" s="62"/>
+      <c r="AZ1" s="62"/>
+      <c r="BA1" s="62"/>
+      <c r="BB1" s="62"/>
+      <c r="BC1" s="62"/>
+      <c r="BD1" s="62"/>
+      <c r="BE1" s="62"/>
+      <c r="BF1" s="62"/>
     </row>
     <row r="2" spans="1:59" ht="18">
       <c r="A2" s="23" t="s">
@@ -957,10 +964,10 @@
       <c r="BF2" s="38"/>
     </row>
     <row r="3" spans="1:59">
-      <c r="A3" s="61" t="s">
+      <c r="A3" s="63" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="61"/>
+      <c r="B3" s="63"/>
       <c r="C3" s="2"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -1000,10 +1007,10 @@
       <c r="AA3" s="6"/>
       <c r="AB3" s="6"/>
       <c r="AC3" s="6"/>
-      <c r="AD3" s="61" t="s">
+      <c r="AD3" s="63" t="s">
         <v>3</v>
       </c>
-      <c r="AE3" s="61"/>
+      <c r="AE3" s="63"/>
       <c r="AF3" s="39"/>
       <c r="AG3" s="3">
         <v>1</v>
@@ -1480,38 +1487,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:33" ht="18">
-      <c r="A1" s="60" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="60"/>
-      <c r="C1" s="60"/>
-      <c r="D1" s="60"/>
-      <c r="E1" s="60"/>
-      <c r="F1" s="60"/>
-      <c r="G1" s="60"/>
-      <c r="H1" s="60"/>
-      <c r="I1" s="60"/>
-      <c r="J1" s="60"/>
-      <c r="K1" s="60"/>
-      <c r="L1" s="60"/>
-      <c r="M1" s="60"/>
-      <c r="N1" s="60"/>
-      <c r="O1" s="60"/>
-      <c r="P1" s="60"/>
-      <c r="Q1" s="60"/>
-      <c r="R1" s="60"/>
-      <c r="S1" s="60"/>
-      <c r="T1" s="60"/>
-      <c r="U1" s="60"/>
-      <c r="V1" s="60"/>
-      <c r="W1" s="60"/>
-      <c r="X1" s="60"/>
-      <c r="Y1" s="60"/>
-      <c r="Z1" s="60"/>
-      <c r="AA1" s="60"/>
-      <c r="AB1" s="60"/>
-      <c r="AC1" s="60"/>
-      <c r="AD1" s="60"/>
+      <c r="A1" s="62" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="62"/>
+      <c r="C1" s="62"/>
+      <c r="D1" s="62"/>
+      <c r="E1" s="62"/>
+      <c r="F1" s="62"/>
+      <c r="G1" s="62"/>
+      <c r="H1" s="62"/>
+      <c r="I1" s="62"/>
+      <c r="J1" s="62"/>
+      <c r="K1" s="62"/>
+      <c r="L1" s="62"/>
+      <c r="M1" s="62"/>
+      <c r="N1" s="62"/>
+      <c r="O1" s="62"/>
+      <c r="P1" s="62"/>
+      <c r="Q1" s="62"/>
+      <c r="R1" s="62"/>
+      <c r="S1" s="62"/>
+      <c r="T1" s="62"/>
+      <c r="U1" s="62"/>
+      <c r="V1" s="62"/>
+      <c r="W1" s="62"/>
+      <c r="X1" s="62"/>
+      <c r="Y1" s="62"/>
+      <c r="Z1" s="62"/>
+      <c r="AA1" s="62"/>
+      <c r="AB1" s="62"/>
+      <c r="AC1" s="62"/>
+      <c r="AD1" s="62"/>
     </row>
     <row r="2" spans="1:33" ht="18">
       <c r="A2" s="23" t="s">
@@ -1550,10 +1557,10 @@
       <c r="AD2" s="43"/>
     </row>
     <row r="3" spans="1:33" ht="15.75" thickBot="1">
-      <c r="A3" s="61" t="s">
+      <c r="A3" s="63" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="61"/>
+      <c r="B3" s="63"/>
       <c r="C3" s="44"/>
       <c r="D3" s="3">
         <v>2</v>
@@ -2144,7 +2151,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AD7"/>
+  <dimension ref="A1:AE8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="20.5703125" customWidth="1"/>
@@ -2163,42 +2170,43 @@
     <col min="21" max="21" width="10.5703125" bestFit="1" customWidth="1"/>
     <col min="22" max="22" width="10.140625" bestFit="1" customWidth="1"/>
     <col min="30" max="30" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" ht="18">
-      <c r="A1" s="60" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="60"/>
-      <c r="C1" s="60"/>
-      <c r="D1" s="60"/>
-      <c r="E1" s="60"/>
-      <c r="F1" s="60"/>
-      <c r="G1" s="60"/>
-      <c r="H1" s="60"/>
-      <c r="I1" s="60"/>
-      <c r="J1" s="60"/>
-      <c r="K1" s="60"/>
-      <c r="L1" s="60"/>
-      <c r="M1" s="60"/>
-      <c r="N1" s="60"/>
-      <c r="O1" s="60"/>
-      <c r="P1" s="60"/>
-      <c r="Q1" s="60"/>
-      <c r="R1" s="60"/>
-      <c r="S1" s="60"/>
-      <c r="T1" s="60"/>
-      <c r="U1" s="60"/>
-      <c r="V1" s="60"/>
-      <c r="W1" s="60"/>
-      <c r="X1" s="60"/>
-      <c r="Y1" s="60"/>
-      <c r="Z1" s="60"/>
-      <c r="AA1" s="60"/>
-      <c r="AB1" s="60"/>
-      <c r="AC1" s="60"/>
-    </row>
-    <row r="2" spans="1:30" ht="16.5" customHeight="1">
+    <row r="1" spans="1:31" ht="18">
+      <c r="A1" s="62" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="62"/>
+      <c r="C1" s="62"/>
+      <c r="D1" s="62"/>
+      <c r="E1" s="62"/>
+      <c r="F1" s="62"/>
+      <c r="G1" s="62"/>
+      <c r="H1" s="62"/>
+      <c r="I1" s="62"/>
+      <c r="J1" s="62"/>
+      <c r="K1" s="62"/>
+      <c r="L1" s="62"/>
+      <c r="M1" s="62"/>
+      <c r="N1" s="62"/>
+      <c r="O1" s="62"/>
+      <c r="P1" s="62"/>
+      <c r="Q1" s="62"/>
+      <c r="R1" s="62"/>
+      <c r="S1" s="62"/>
+      <c r="T1" s="62"/>
+      <c r="U1" s="62"/>
+      <c r="V1" s="62"/>
+      <c r="W1" s="62"/>
+      <c r="X1" s="62"/>
+      <c r="Y1" s="62"/>
+      <c r="Z1" s="62"/>
+      <c r="AA1" s="62"/>
+      <c r="AB1" s="62"/>
+      <c r="AC1" s="62"/>
+    </row>
+    <row r="2" spans="1:31" ht="16.5" customHeight="1">
       <c r="A2" s="23" t="s">
         <v>1</v>
       </c>
@@ -2233,11 +2241,11 @@
       <c r="AB2" s="54"/>
       <c r="AC2" s="54"/>
     </row>
-    <row r="3" spans="1:30">
-      <c r="A3" s="61" t="s">
+    <row r="3" spans="1:31">
+      <c r="A3" s="63" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="61"/>
+      <c r="B3" s="63"/>
       <c r="D3">
         <v>2</v>
       </c>
@@ -2277,7 +2285,7 @@
       <c r="AB3" s="6"/>
       <c r="AC3" s="6"/>
     </row>
-    <row r="4" spans="1:30" ht="42.75">
+    <row r="4" spans="1:31" ht="42.75">
       <c r="A4" s="10" t="s">
         <v>8</v>
       </c>
@@ -2368,8 +2376,11 @@
       <c r="AD4" s="10" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="5" spans="1:30">
+      <c r="AE4" s="10" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="5" spans="1:31">
       <c r="A5" s="9">
         <v>1</v>
       </c>
@@ -2413,14 +2424,16 @@
         <f>ROUND(J5*M5%,2)</f>
         <v>0</v>
       </c>
-      <c r="O5" s="8"/>
+      <c r="O5" s="8">
+        <v>500.5</v>
+      </c>
       <c r="P5" s="8">
         <f>ROUND(K5*O5%,2)</f>
         <v>0</v>
       </c>
       <c r="Q5" s="8">
         <f>O5-P5</f>
-        <v>0</v>
+        <v>500.5</v>
       </c>
       <c r="R5" s="8">
         <f>ROUND(L5*Q5%,2)</f>
@@ -2469,8 +2482,11 @@
       <c r="AD5" s="46" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="6" spans="1:30" ht="16.5" customHeight="1">
+      <c r="AE5" s="46" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="6" spans="1:31" ht="16.5" customHeight="1">
       <c r="A6" s="9">
         <v>2</v>
       </c>
@@ -2573,8 +2589,11 @@
       <c r="AD6" s="46" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="7" spans="1:30">
+      <c r="AE6" s="46" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="7" spans="1:31">
       <c r="A7" s="9">
         <v>3</v>
       </c>
@@ -2677,6 +2696,12 @@
       <c r="AD7" s="46" t="s">
         <v>54</v>
       </c>
+      <c r="AE7" s="46" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="8" spans="1:31">
+      <c r="AE8" s="46"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2711,37 +2736,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="18">
-      <c r="A1" s="60" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="60"/>
-      <c r="C1" s="60"/>
-      <c r="D1" s="60"/>
-      <c r="E1" s="60"/>
-      <c r="F1" s="60"/>
-      <c r="G1" s="60"/>
-      <c r="H1" s="60"/>
-      <c r="I1" s="60"/>
-      <c r="J1" s="60"/>
-      <c r="K1" s="60"/>
-      <c r="L1" s="60"/>
-      <c r="M1" s="60"/>
-      <c r="N1" s="60"/>
-      <c r="O1" s="60"/>
-      <c r="P1" s="60"/>
-      <c r="Q1" s="60"/>
-      <c r="R1" s="60"/>
-      <c r="S1" s="60"/>
-      <c r="T1" s="60"/>
-      <c r="U1" s="60"/>
-      <c r="V1" s="60"/>
-      <c r="W1" s="60"/>
-      <c r="X1" s="60"/>
-      <c r="Y1" s="60"/>
-      <c r="Z1" s="60"/>
-      <c r="AA1" s="60"/>
-      <c r="AB1" s="60"/>
-      <c r="AC1" s="60"/>
+      <c r="A1" s="62" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="62"/>
+      <c r="C1" s="62"/>
+      <c r="D1" s="62"/>
+      <c r="E1" s="62"/>
+      <c r="F1" s="62"/>
+      <c r="G1" s="62"/>
+      <c r="H1" s="62"/>
+      <c r="I1" s="62"/>
+      <c r="J1" s="62"/>
+      <c r="K1" s="62"/>
+      <c r="L1" s="62"/>
+      <c r="M1" s="62"/>
+      <c r="N1" s="62"/>
+      <c r="O1" s="62"/>
+      <c r="P1" s="62"/>
+      <c r="Q1" s="62"/>
+      <c r="R1" s="62"/>
+      <c r="S1" s="62"/>
+      <c r="T1" s="62"/>
+      <c r="U1" s="62"/>
+      <c r="V1" s="62"/>
+      <c r="W1" s="62"/>
+      <c r="X1" s="62"/>
+      <c r="Y1" s="62"/>
+      <c r="Z1" s="62"/>
+      <c r="AA1" s="62"/>
+      <c r="AB1" s="62"/>
+      <c r="AC1" s="62"/>
     </row>
     <row r="2" spans="1:29" ht="18">
       <c r="A2" s="23" t="s">
@@ -2779,10 +2804,10 @@
       <c r="AC2" s="56"/>
     </row>
     <row r="3" spans="1:29">
-      <c r="A3" s="61" t="s">
+      <c r="A3" s="63" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="61"/>
+      <c r="B3" s="63"/>
       <c r="C3" s="57"/>
       <c r="D3" s="3">
         <v>2</v>
@@ -3063,37 +3088,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="18">
-      <c r="A1" s="60" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="60"/>
-      <c r="C1" s="60"/>
-      <c r="D1" s="60"/>
-      <c r="E1" s="60"/>
-      <c r="F1" s="60"/>
-      <c r="G1" s="60"/>
-      <c r="H1" s="60"/>
-      <c r="I1" s="60"/>
-      <c r="J1" s="60"/>
-      <c r="K1" s="60"/>
-      <c r="L1" s="60"/>
-      <c r="M1" s="60"/>
-      <c r="N1" s="60"/>
-      <c r="O1" s="60"/>
-      <c r="P1" s="60"/>
-      <c r="Q1" s="60"/>
-      <c r="R1" s="60"/>
-      <c r="S1" s="60"/>
-      <c r="T1" s="60"/>
-      <c r="U1" s="60"/>
-      <c r="V1" s="60"/>
-      <c r="W1" s="60"/>
-      <c r="X1" s="60"/>
-      <c r="Y1" s="60"/>
-      <c r="Z1" s="60"/>
-      <c r="AA1" s="60"/>
-      <c r="AB1" s="60"/>
-      <c r="AC1" s="60"/>
+      <c r="A1" s="62" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="62"/>
+      <c r="C1" s="62"/>
+      <c r="D1" s="62"/>
+      <c r="E1" s="62"/>
+      <c r="F1" s="62"/>
+      <c r="G1" s="62"/>
+      <c r="H1" s="62"/>
+      <c r="I1" s="62"/>
+      <c r="J1" s="62"/>
+      <c r="K1" s="62"/>
+      <c r="L1" s="62"/>
+      <c r="M1" s="62"/>
+      <c r="N1" s="62"/>
+      <c r="O1" s="62"/>
+      <c r="P1" s="62"/>
+      <c r="Q1" s="62"/>
+      <c r="R1" s="62"/>
+      <c r="S1" s="62"/>
+      <c r="T1" s="62"/>
+      <c r="U1" s="62"/>
+      <c r="V1" s="62"/>
+      <c r="W1" s="62"/>
+      <c r="X1" s="62"/>
+      <c r="Y1" s="62"/>
+      <c r="Z1" s="62"/>
+      <c r="AA1" s="62"/>
+      <c r="AB1" s="62"/>
+      <c r="AC1" s="62"/>
     </row>
     <row r="2" spans="1:29" ht="18">
       <c r="A2" s="23" t="s">
@@ -3131,10 +3156,10 @@
       <c r="AC2" s="58"/>
     </row>
     <row r="3" spans="1:29">
-      <c r="A3" s="61" t="s">
+      <c r="A3" s="63" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="61"/>
+      <c r="B3" s="63"/>
       <c r="C3" s="59"/>
       <c r="D3" s="3">
         <v>4</v>
@@ -3386,6 +3411,695 @@
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:AC1"/>
+    <mergeCell ref="A3:B3"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:AG8"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="2" max="2" width="20.5703125" customWidth="1"/>
+    <col min="4" max="4" width="29.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="29.140625" customWidth="1"/>
+    <col min="6" max="6" width="19.28515625" customWidth="1"/>
+    <col min="7" max="7" width="16.28515625" customWidth="1"/>
+    <col min="8" max="8" width="24.42578125" customWidth="1"/>
+    <col min="9" max="9" width="20.28515625" customWidth="1"/>
+    <col min="10" max="10" width="20" customWidth="1"/>
+    <col min="14" max="14" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="13.7109375" customWidth="1"/>
+    <col min="19" max="19" width="13" customWidth="1"/>
+    <col min="20" max="20" width="14.42578125" customWidth="1"/>
+    <col min="21" max="21" width="18.42578125" customWidth="1"/>
+    <col min="22" max="22" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="13.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:33" ht="18">
+      <c r="A1" s="62" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="62"/>
+      <c r="C1" s="62"/>
+      <c r="D1" s="62"/>
+      <c r="E1" s="62"/>
+      <c r="F1" s="62"/>
+      <c r="G1" s="62"/>
+      <c r="H1" s="62"/>
+      <c r="I1" s="62"/>
+      <c r="J1" s="62"/>
+      <c r="K1" s="62"/>
+      <c r="L1" s="62"/>
+      <c r="M1" s="62"/>
+      <c r="N1" s="62"/>
+      <c r="O1" s="62"/>
+      <c r="P1" s="62"/>
+      <c r="Q1" s="62"/>
+      <c r="R1" s="62"/>
+      <c r="S1" s="62"/>
+      <c r="T1" s="62"/>
+      <c r="U1" s="62"/>
+      <c r="V1" s="62"/>
+      <c r="W1" s="62"/>
+      <c r="X1" s="62"/>
+      <c r="Y1" s="62"/>
+      <c r="Z1" s="62"/>
+      <c r="AA1" s="62"/>
+      <c r="AB1" s="62"/>
+      <c r="AC1" s="62"/>
+      <c r="AD1" s="62"/>
+    </row>
+    <row r="2" spans="1:33" ht="18">
+      <c r="A2" s="23" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="23" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" s="60"/>
+      <c r="D2" s="60"/>
+      <c r="E2" s="60"/>
+      <c r="F2" s="60"/>
+      <c r="G2" s="60"/>
+      <c r="H2" s="60"/>
+      <c r="I2" s="60"/>
+      <c r="J2" s="60"/>
+      <c r="K2" s="60"/>
+      <c r="L2" s="60"/>
+      <c r="M2" s="60"/>
+      <c r="N2" s="60"/>
+      <c r="O2" s="60"/>
+      <c r="P2" s="60"/>
+      <c r="Q2" s="60"/>
+      <c r="R2" s="60"/>
+      <c r="S2" s="60"/>
+      <c r="T2" s="60"/>
+      <c r="U2" s="60"/>
+      <c r="V2" s="60"/>
+      <c r="W2" s="60"/>
+      <c r="X2" s="60"/>
+      <c r="Y2" s="60"/>
+      <c r="Z2" s="60"/>
+      <c r="AA2" s="60"/>
+      <c r="AB2" s="60"/>
+      <c r="AC2" s="60"/>
+      <c r="AD2" s="60"/>
+    </row>
+    <row r="3" spans="1:33" ht="15.75" thickBot="1">
+      <c r="A3" s="63" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="63"/>
+      <c r="C3" s="61"/>
+      <c r="D3" s="3">
+        <v>2</v>
+      </c>
+      <c r="E3" s="3"/>
+      <c r="F3" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="G3" s="5"/>
+      <c r="H3" s="5"/>
+      <c r="I3" s="5"/>
+      <c r="J3" s="6"/>
+      <c r="K3" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="L3" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="M3" s="7"/>
+      <c r="N3" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="O3" s="7">
+        <v>1</v>
+      </c>
+      <c r="P3" s="7"/>
+      <c r="Q3" s="7"/>
+      <c r="R3" s="7"/>
+      <c r="S3" s="7"/>
+      <c r="T3" s="6"/>
+      <c r="U3" s="6"/>
+      <c r="V3" s="6"/>
+      <c r="W3" s="6"/>
+      <c r="X3" s="6"/>
+      <c r="Y3" s="6"/>
+      <c r="Z3" s="6"/>
+      <c r="AA3" s="6"/>
+      <c r="AB3" s="6"/>
+      <c r="AC3" s="6"/>
+      <c r="AD3" s="6"/>
+    </row>
+    <row r="4" spans="1:33" ht="43.5" thickTop="1">
+      <c r="A4" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="E4" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="F4" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="G4" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="H4" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="I4" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="J4" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="K4" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="L4" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="M4" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="N4" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="O4" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="P4" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="Q4" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="R4" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="S4" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="T4" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="U4" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="V4" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="W4" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="X4" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y4" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z4" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="AA4" s="16" t="s">
+        <v>30</v>
+      </c>
+      <c r="AB4" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="AC4" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="AD4" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="AE4" s="51" t="s">
+        <v>58</v>
+      </c>
+      <c r="AF4" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="AG4" s="10" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="5" spans="1:33">
+      <c r="A5" s="9">
+        <v>1</v>
+      </c>
+      <c r="B5" s="27" t="s">
+        <v>44</v>
+      </c>
+      <c r="C5" s="9">
+        <v>0</v>
+      </c>
+      <c r="D5" s="27" t="s">
+        <v>44</v>
+      </c>
+      <c r="E5" s="27"/>
+      <c r="F5" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="G5" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="H5" s="24">
+        <v>2</v>
+      </c>
+      <c r="I5" s="9">
+        <v>250.25</v>
+      </c>
+      <c r="J5" s="8">
+        <v>500.5</v>
+      </c>
+      <c r="K5" s="25">
+        <v>0</v>
+      </c>
+      <c r="L5" s="25">
+        <v>0</v>
+      </c>
+      <c r="M5" s="25">
+        <v>0</v>
+      </c>
+      <c r="N5" s="8">
+        <v>500.5</v>
+      </c>
+      <c r="O5" s="8">
+        <f>ROUND(K5*N5%,2)</f>
+        <v>0</v>
+      </c>
+      <c r="P5" s="8">
+        <v>500.5</v>
+      </c>
+      <c r="Q5" s="8">
+        <f>ROUND(L5*P5%,2)</f>
+        <v>0</v>
+      </c>
+      <c r="R5" s="8">
+        <f>P5-Q5</f>
+        <v>500.5</v>
+      </c>
+      <c r="S5" s="8">
+        <f>ROUND(M5*R5%,2)</f>
+        <v>0</v>
+      </c>
+      <c r="T5" s="26">
+        <f>O5+Q5+S5</f>
+        <v>0</v>
+      </c>
+      <c r="U5" s="26">
+        <v>0</v>
+      </c>
+      <c r="V5" s="8">
+        <f>(J5-T5)</f>
+        <v>500.5</v>
+      </c>
+      <c r="W5" s="24">
+        <v>88363222</v>
+      </c>
+      <c r="X5" s="18">
+        <v>0.18</v>
+      </c>
+      <c r="Y5" s="24">
+        <f>IF($D$3=1,ROUND(((V5*X5)/2),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="Z5" s="24">
+        <f>IF($D$3=1,ROUND(((V5*X5)/2),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="AA5" s="24">
+        <f>IF($D$3=2,ROUND(((V5*X5)),2),0)</f>
+        <v>90.09</v>
+      </c>
+      <c r="AB5" s="24">
+        <v>0</v>
+      </c>
+      <c r="AC5" s="24">
+        <f>Y5+Z5+AA5</f>
+        <v>90.09</v>
+      </c>
+      <c r="AD5" s="24">
+        <f>V5+AC5</f>
+        <v>590.59</v>
+      </c>
+      <c r="AE5" s="52" t="s">
+        <v>57</v>
+      </c>
+      <c r="AF5" s="46" t="s">
+        <v>42</v>
+      </c>
+      <c r="AG5" s="46" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="6" spans="1:33" ht="16.5" customHeight="1">
+      <c r="A6" s="9">
+        <v>2</v>
+      </c>
+      <c r="B6" s="45" t="s">
+        <v>51</v>
+      </c>
+      <c r="C6" s="9">
+        <v>0</v>
+      </c>
+      <c r="D6" s="45" t="s">
+        <v>50</v>
+      </c>
+      <c r="E6" s="45"/>
+      <c r="F6" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="G6" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="H6" s="24">
+        <v>1</v>
+      </c>
+      <c r="I6" s="9">
+        <v>3458</v>
+      </c>
+      <c r="J6" s="8">
+        <v>3458</v>
+      </c>
+      <c r="K6" s="25">
+        <v>0</v>
+      </c>
+      <c r="L6" s="25">
+        <v>0</v>
+      </c>
+      <c r="M6" s="25">
+        <v>0</v>
+      </c>
+      <c r="N6" s="8">
+        <v>3458</v>
+      </c>
+      <c r="O6" s="8">
+        <f t="shared" ref="O6:O8" si="0">ROUND(K6*N6%,2)</f>
+        <v>0</v>
+      </c>
+      <c r="P6" s="8">
+        <f t="shared" ref="P6:P8" si="1">J6-O6</f>
+        <v>3458</v>
+      </c>
+      <c r="Q6" s="8">
+        <f t="shared" ref="Q6:Q8" si="2">ROUND(L6*P6%,2)</f>
+        <v>0</v>
+      </c>
+      <c r="R6" s="8">
+        <f t="shared" ref="R6:R8" si="3">P6-Q6</f>
+        <v>3458</v>
+      </c>
+      <c r="S6" s="8">
+        <f t="shared" ref="S6:S8" si="4">ROUND(M6*R6%,2)</f>
+        <v>0</v>
+      </c>
+      <c r="T6" s="26">
+        <f t="shared" ref="T6:T8" si="5">O6+Q6+S6</f>
+        <v>0</v>
+      </c>
+      <c r="U6" s="26">
+        <v>0</v>
+      </c>
+      <c r="V6" s="8">
+        <f>(J6-T6)</f>
+        <v>3458</v>
+      </c>
+      <c r="W6" s="24">
+        <v>88363222</v>
+      </c>
+      <c r="X6" s="18">
+        <v>0.18</v>
+      </c>
+      <c r="Y6" s="24">
+        <f>IF($D$3=1,ROUND(((V6*X6)/2),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="Z6" s="24">
+        <f>IF($D$3=1,ROUND(((V6*X6)/2),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="AA6" s="24">
+        <f>IF($D$3=2,ROUND(((V6*X6)),2),0)</f>
+        <v>622.44000000000005</v>
+      </c>
+      <c r="AB6" s="24">
+        <v>0</v>
+      </c>
+      <c r="AC6" s="24">
+        <f>Y6+Z6+AA6</f>
+        <v>622.44000000000005</v>
+      </c>
+      <c r="AD6" s="24">
+        <f>V6+AC6</f>
+        <v>4080.44</v>
+      </c>
+      <c r="AE6" s="53" t="s">
+        <v>57</v>
+      </c>
+      <c r="AF6" s="46" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG6" s="46" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="7" spans="1:33">
+      <c r="A7" s="46">
+        <v>4</v>
+      </c>
+      <c r="B7" s="46"/>
+      <c r="C7" s="46"/>
+      <c r="D7" s="46"/>
+      <c r="E7" s="46" t="s">
+        <v>56</v>
+      </c>
+      <c r="F7" s="47" t="s">
+        <v>33</v>
+      </c>
+      <c r="G7" s="47" t="s">
+        <v>33</v>
+      </c>
+      <c r="H7" s="48">
+        <v>1</v>
+      </c>
+      <c r="I7" s="47">
+        <v>609</v>
+      </c>
+      <c r="J7" s="49">
+        <v>609</v>
+      </c>
+      <c r="K7" s="46">
+        <v>0</v>
+      </c>
+      <c r="L7" s="46">
+        <v>0</v>
+      </c>
+      <c r="M7" s="46">
+        <v>0</v>
+      </c>
+      <c r="N7" s="50">
+        <v>609</v>
+      </c>
+      <c r="O7" s="8">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="P7" s="8">
+        <f t="shared" si="1"/>
+        <v>609</v>
+      </c>
+      <c r="Q7" s="8">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="R7" s="8">
+        <f t="shared" si="3"/>
+        <v>609</v>
+      </c>
+      <c r="S7" s="8">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="T7" s="26">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="U7" s="26">
+        <v>0</v>
+      </c>
+      <c r="V7" s="8">
+        <f>(J7-T7)</f>
+        <v>609</v>
+      </c>
+      <c r="W7" s="24">
+        <v>75052200</v>
+      </c>
+      <c r="X7" s="18">
+        <v>0.18</v>
+      </c>
+      <c r="Y7" s="24">
+        <f>IF($D$3=1,ROUND(((V7*X7)/2),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="Z7" s="24">
+        <f>IF($D$3=1,ROUND(((V7*X7)/2),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="AA7" s="24">
+        <f>IF($D$3=2,ROUND(((V7*X7)),2),0)</f>
+        <v>109.62</v>
+      </c>
+      <c r="AB7" s="24">
+        <v>0</v>
+      </c>
+      <c r="AC7" s="24">
+        <f>Y7+Z7+AA7</f>
+        <v>109.62</v>
+      </c>
+      <c r="AD7" s="24">
+        <f>V7+AC7</f>
+        <v>718.62</v>
+      </c>
+      <c r="AE7" s="52" t="s">
+        <v>59</v>
+      </c>
+      <c r="AF7" s="46">
+        <v>5050121000</v>
+      </c>
+      <c r="AG7" s="46" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="8" spans="1:33">
+      <c r="A8" s="9">
+        <v>3</v>
+      </c>
+      <c r="B8" s="27" t="s">
+        <v>52</v>
+      </c>
+      <c r="C8" s="9">
+        <v>0</v>
+      </c>
+      <c r="D8" s="27" t="s">
+        <v>52</v>
+      </c>
+      <c r="E8" s="27"/>
+      <c r="F8" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="G8" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="H8" s="24">
+        <v>3</v>
+      </c>
+      <c r="I8" s="9">
+        <v>675</v>
+      </c>
+      <c r="J8" s="8">
+        <v>2025</v>
+      </c>
+      <c r="K8" s="25">
+        <v>0</v>
+      </c>
+      <c r="L8" s="25">
+        <v>0</v>
+      </c>
+      <c r="M8" s="25">
+        <v>0</v>
+      </c>
+      <c r="N8" s="8">
+        <v>2025</v>
+      </c>
+      <c r="O8" s="8">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="P8" s="8">
+        <f t="shared" si="1"/>
+        <v>2025</v>
+      </c>
+      <c r="Q8" s="8">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="R8" s="8">
+        <f t="shared" si="3"/>
+        <v>2025</v>
+      </c>
+      <c r="S8" s="8">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="T8" s="26">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="U8" s="26">
+        <v>0</v>
+      </c>
+      <c r="V8" s="8">
+        <f>(J8-T8)</f>
+        <v>2025</v>
+      </c>
+      <c r="W8" s="24">
+        <v>88363222</v>
+      </c>
+      <c r="X8" s="18">
+        <v>0.18</v>
+      </c>
+      <c r="Y8" s="24">
+        <f>IF($D$3=1,ROUND(((V8*X8)/2),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="Z8" s="24">
+        <f>IF($D$3=1,ROUND(((V8*X8)/2),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="AA8" s="24">
+        <f>IF($D$3=2,ROUND(((V8*X8)),2),0)</f>
+        <v>364.5</v>
+      </c>
+      <c r="AB8" s="24">
+        <v>0</v>
+      </c>
+      <c r="AC8" s="24">
+        <f>Y8+Z8+AA8</f>
+        <v>364.5</v>
+      </c>
+      <c r="AD8" s="24">
+        <f>V8+AC8</f>
+        <v>2389.5</v>
+      </c>
+      <c r="AE8" s="53" t="s">
+        <v>57</v>
+      </c>
+      <c r="AF8" s="46" t="s">
+        <v>54</v>
+      </c>
+      <c r="AG8" s="46" t="s">
+        <v>61</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:AD1"/>
     <mergeCell ref="A3:B3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3420,68 +4134,68 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:58" ht="18">
-      <c r="A1" s="60" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="60"/>
-      <c r="C1" s="60"/>
-      <c r="D1" s="60"/>
-      <c r="E1" s="60"/>
-      <c r="F1" s="60"/>
-      <c r="G1" s="60"/>
-      <c r="H1" s="60"/>
-      <c r="I1" s="60"/>
-      <c r="J1" s="60"/>
-      <c r="K1" s="60"/>
-      <c r="L1" s="60"/>
-      <c r="M1" s="60"/>
-      <c r="N1" s="60"/>
-      <c r="O1" s="60"/>
-      <c r="P1" s="60"/>
-      <c r="Q1" s="60"/>
-      <c r="R1" s="60"/>
-      <c r="S1" s="60"/>
-      <c r="T1" s="60"/>
-      <c r="U1" s="60"/>
-      <c r="V1" s="60"/>
-      <c r="W1" s="60"/>
-      <c r="X1" s="60"/>
-      <c r="Y1" s="60"/>
-      <c r="Z1" s="60"/>
-      <c r="AA1" s="60"/>
-      <c r="AB1" s="60"/>
-      <c r="AC1" s="60"/>
-      <c r="AD1" s="60" t="s">
-        <v>0</v>
-      </c>
-      <c r="AE1" s="60"/>
-      <c r="AF1" s="60"/>
-      <c r="AG1" s="60"/>
-      <c r="AH1" s="60"/>
-      <c r="AI1" s="60"/>
-      <c r="AJ1" s="60"/>
-      <c r="AK1" s="60"/>
-      <c r="AL1" s="60"/>
-      <c r="AM1" s="60"/>
-      <c r="AN1" s="60"/>
-      <c r="AO1" s="60"/>
-      <c r="AP1" s="60"/>
-      <c r="AQ1" s="60"/>
-      <c r="AR1" s="60"/>
-      <c r="AS1" s="60"/>
-      <c r="AT1" s="60"/>
-      <c r="AU1" s="60"/>
-      <c r="AV1" s="60"/>
-      <c r="AW1" s="60"/>
-      <c r="AX1" s="60"/>
-      <c r="AY1" s="60"/>
-      <c r="AZ1" s="60"/>
-      <c r="BA1" s="60"/>
-      <c r="BB1" s="60"/>
-      <c r="BC1" s="60"/>
-      <c r="BD1" s="60"/>
-      <c r="BE1" s="60"/>
-      <c r="BF1" s="60"/>
+      <c r="A1" s="62" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="62"/>
+      <c r="C1" s="62"/>
+      <c r="D1" s="62"/>
+      <c r="E1" s="62"/>
+      <c r="F1" s="62"/>
+      <c r="G1" s="62"/>
+      <c r="H1" s="62"/>
+      <c r="I1" s="62"/>
+      <c r="J1" s="62"/>
+      <c r="K1" s="62"/>
+      <c r="L1" s="62"/>
+      <c r="M1" s="62"/>
+      <c r="N1" s="62"/>
+      <c r="O1" s="62"/>
+      <c r="P1" s="62"/>
+      <c r="Q1" s="62"/>
+      <c r="R1" s="62"/>
+      <c r="S1" s="62"/>
+      <c r="T1" s="62"/>
+      <c r="U1" s="62"/>
+      <c r="V1" s="62"/>
+      <c r="W1" s="62"/>
+      <c r="X1" s="62"/>
+      <c r="Y1" s="62"/>
+      <c r="Z1" s="62"/>
+      <c r="AA1" s="62"/>
+      <c r="AB1" s="62"/>
+      <c r="AC1" s="62"/>
+      <c r="AD1" s="62" t="s">
+        <v>0</v>
+      </c>
+      <c r="AE1" s="62"/>
+      <c r="AF1" s="62"/>
+      <c r="AG1" s="62"/>
+      <c r="AH1" s="62"/>
+      <c r="AI1" s="62"/>
+      <c r="AJ1" s="62"/>
+      <c r="AK1" s="62"/>
+      <c r="AL1" s="62"/>
+      <c r="AM1" s="62"/>
+      <c r="AN1" s="62"/>
+      <c r="AO1" s="62"/>
+      <c r="AP1" s="62"/>
+      <c r="AQ1" s="62"/>
+      <c r="AR1" s="62"/>
+      <c r="AS1" s="62"/>
+      <c r="AT1" s="62"/>
+      <c r="AU1" s="62"/>
+      <c r="AV1" s="62"/>
+      <c r="AW1" s="62"/>
+      <c r="AX1" s="62"/>
+      <c r="AY1" s="62"/>
+      <c r="AZ1" s="62"/>
+      <c r="BA1" s="62"/>
+      <c r="BB1" s="62"/>
+      <c r="BC1" s="62"/>
+      <c r="BD1" s="62"/>
+      <c r="BE1" s="62"/>
+      <c r="BF1" s="62"/>
     </row>
     <row r="2" spans="1:58" ht="18">
       <c r="A2" s="23" t="s">
@@ -3552,10 +4266,10 @@
       <c r="BF2" s="36"/>
     </row>
     <row r="3" spans="1:58">
-      <c r="A3" s="61" t="s">
+      <c r="A3" s="63" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="61"/>
+      <c r="B3" s="63"/>
       <c r="C3" s="29"/>
       <c r="D3" s="3">
         <v>2</v>
@@ -3595,10 +4309,10 @@
       <c r="AA3" s="6"/>
       <c r="AB3" s="6"/>
       <c r="AC3" s="6"/>
-      <c r="AD3" s="61" t="s">
+      <c r="AD3" s="63" t="s">
         <v>3</v>
       </c>
-      <c r="AE3" s="61"/>
+      <c r="AE3" s="63"/>
       <c r="AF3" s="37"/>
       <c r="AG3" s="3">
         <v>2</v>
@@ -4068,37 +4782,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="18">
-      <c r="A1" s="60" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="60"/>
-      <c r="C1" s="60"/>
-      <c r="D1" s="60"/>
-      <c r="E1" s="60"/>
-      <c r="F1" s="60"/>
-      <c r="G1" s="60"/>
-      <c r="H1" s="60"/>
-      <c r="I1" s="60"/>
-      <c r="J1" s="60"/>
-      <c r="K1" s="60"/>
-      <c r="L1" s="60"/>
-      <c r="M1" s="60"/>
-      <c r="N1" s="60"/>
-      <c r="O1" s="60"/>
-      <c r="P1" s="60"/>
-      <c r="Q1" s="60"/>
-      <c r="R1" s="60"/>
-      <c r="S1" s="60"/>
-      <c r="T1" s="60"/>
-      <c r="U1" s="60"/>
-      <c r="V1" s="60"/>
-      <c r="W1" s="60"/>
-      <c r="X1" s="60"/>
-      <c r="Y1" s="60"/>
-      <c r="Z1" s="60"/>
-      <c r="AA1" s="60"/>
-      <c r="AB1" s="60"/>
-      <c r="AC1" s="60"/>
+      <c r="A1" s="62" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="62"/>
+      <c r="C1" s="62"/>
+      <c r="D1" s="62"/>
+      <c r="E1" s="62"/>
+      <c r="F1" s="62"/>
+      <c r="G1" s="62"/>
+      <c r="H1" s="62"/>
+      <c r="I1" s="62"/>
+      <c r="J1" s="62"/>
+      <c r="K1" s="62"/>
+      <c r="L1" s="62"/>
+      <c r="M1" s="62"/>
+      <c r="N1" s="62"/>
+      <c r="O1" s="62"/>
+      <c r="P1" s="62"/>
+      <c r="Q1" s="62"/>
+      <c r="R1" s="62"/>
+      <c r="S1" s="62"/>
+      <c r="T1" s="62"/>
+      <c r="U1" s="62"/>
+      <c r="V1" s="62"/>
+      <c r="W1" s="62"/>
+      <c r="X1" s="62"/>
+      <c r="Y1" s="62"/>
+      <c r="Z1" s="62"/>
+      <c r="AA1" s="62"/>
+      <c r="AB1" s="62"/>
+      <c r="AC1" s="62"/>
     </row>
     <row r="2" spans="1:29" ht="18">
       <c r="A2" s="23" t="s">
@@ -4136,10 +4850,10 @@
       <c r="AC2" s="28"/>
     </row>
     <row r="3" spans="1:29">
-      <c r="A3" s="61" t="s">
+      <c r="A3" s="63" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="61"/>
+      <c r="B3" s="63"/>
       <c r="C3" s="29"/>
       <c r="D3" s="3">
         <v>4</v>
@@ -4422,37 +5136,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="18">
-      <c r="A1" s="60" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="60"/>
-      <c r="C1" s="60"/>
-      <c r="D1" s="60"/>
-      <c r="E1" s="60"/>
-      <c r="F1" s="60"/>
-      <c r="G1" s="60"/>
-      <c r="H1" s="60"/>
-      <c r="I1" s="60"/>
-      <c r="J1" s="60"/>
-      <c r="K1" s="60"/>
-      <c r="L1" s="60"/>
-      <c r="M1" s="60"/>
-      <c r="N1" s="60"/>
-      <c r="O1" s="60"/>
-      <c r="P1" s="60"/>
-      <c r="Q1" s="60"/>
-      <c r="R1" s="60"/>
-      <c r="S1" s="60"/>
-      <c r="T1" s="60"/>
-      <c r="U1" s="60"/>
-      <c r="V1" s="60"/>
-      <c r="W1" s="60"/>
-      <c r="X1" s="60"/>
-      <c r="Y1" s="60"/>
-      <c r="Z1" s="60"/>
-      <c r="AA1" s="60"/>
-      <c r="AB1" s="60"/>
-      <c r="AC1" s="60"/>
+      <c r="A1" s="62" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="62"/>
+      <c r="C1" s="62"/>
+      <c r="D1" s="62"/>
+      <c r="E1" s="62"/>
+      <c r="F1" s="62"/>
+      <c r="G1" s="62"/>
+      <c r="H1" s="62"/>
+      <c r="I1" s="62"/>
+      <c r="J1" s="62"/>
+      <c r="K1" s="62"/>
+      <c r="L1" s="62"/>
+      <c r="M1" s="62"/>
+      <c r="N1" s="62"/>
+      <c r="O1" s="62"/>
+      <c r="P1" s="62"/>
+      <c r="Q1" s="62"/>
+      <c r="R1" s="62"/>
+      <c r="S1" s="62"/>
+      <c r="T1" s="62"/>
+      <c r="U1" s="62"/>
+      <c r="V1" s="62"/>
+      <c r="W1" s="62"/>
+      <c r="X1" s="62"/>
+      <c r="Y1" s="62"/>
+      <c r="Z1" s="62"/>
+      <c r="AA1" s="62"/>
+      <c r="AB1" s="62"/>
+      <c r="AC1" s="62"/>
     </row>
     <row r="2" spans="1:29" ht="18">
       <c r="A2" s="23" t="s">
@@ -4490,10 +5204,10 @@
       <c r="AC2" s="28"/>
     </row>
     <row r="3" spans="1:29">
-      <c r="A3" s="61" t="s">
+      <c r="A3" s="63" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="61"/>
+      <c r="B3" s="63"/>
       <c r="C3" s="29"/>
       <c r="D3" s="3">
         <v>3</v>
@@ -4775,37 +5489,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="18">
-      <c r="A1" s="60" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="60"/>
-      <c r="C1" s="60"/>
-      <c r="D1" s="60"/>
-      <c r="E1" s="60"/>
-      <c r="F1" s="60"/>
-      <c r="G1" s="60"/>
-      <c r="H1" s="60"/>
-      <c r="I1" s="60"/>
-      <c r="J1" s="60"/>
-      <c r="K1" s="60"/>
-      <c r="L1" s="60"/>
-      <c r="M1" s="60"/>
-      <c r="N1" s="60"/>
-      <c r="O1" s="60"/>
-      <c r="P1" s="60"/>
-      <c r="Q1" s="60"/>
-      <c r="R1" s="60"/>
-      <c r="S1" s="60"/>
-      <c r="T1" s="60"/>
-      <c r="U1" s="60"/>
-      <c r="V1" s="60"/>
-      <c r="W1" s="60"/>
-      <c r="X1" s="60"/>
-      <c r="Y1" s="60"/>
-      <c r="Z1" s="60"/>
-      <c r="AA1" s="60"/>
-      <c r="AB1" s="60"/>
-      <c r="AC1" s="60"/>
+      <c r="A1" s="62" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="62"/>
+      <c r="C1" s="62"/>
+      <c r="D1" s="62"/>
+      <c r="E1" s="62"/>
+      <c r="F1" s="62"/>
+      <c r="G1" s="62"/>
+      <c r="H1" s="62"/>
+      <c r="I1" s="62"/>
+      <c r="J1" s="62"/>
+      <c r="K1" s="62"/>
+      <c r="L1" s="62"/>
+      <c r="M1" s="62"/>
+      <c r="N1" s="62"/>
+      <c r="O1" s="62"/>
+      <c r="P1" s="62"/>
+      <c r="Q1" s="62"/>
+      <c r="R1" s="62"/>
+      <c r="S1" s="62"/>
+      <c r="T1" s="62"/>
+      <c r="U1" s="62"/>
+      <c r="V1" s="62"/>
+      <c r="W1" s="62"/>
+      <c r="X1" s="62"/>
+      <c r="Y1" s="62"/>
+      <c r="Z1" s="62"/>
+      <c r="AA1" s="62"/>
+      <c r="AB1" s="62"/>
+      <c r="AC1" s="62"/>
     </row>
     <row r="2" spans="1:29" ht="18">
       <c r="A2" s="23" t="s">
@@ -4843,10 +5557,10 @@
       <c r="AC2" s="28"/>
     </row>
     <row r="3" spans="1:29">
-      <c r="A3" s="61" t="s">
+      <c r="A3" s="63" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="61"/>
+      <c r="B3" s="63"/>
       <c r="C3" s="29"/>
       <c r="D3" s="3">
         <v>5</v>
@@ -5130,37 +5844,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="18">
-      <c r="A1" s="60" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="60"/>
-      <c r="C1" s="60"/>
-      <c r="D1" s="60"/>
-      <c r="E1" s="60"/>
-      <c r="F1" s="60"/>
-      <c r="G1" s="60"/>
-      <c r="H1" s="60"/>
-      <c r="I1" s="60"/>
-      <c r="J1" s="60"/>
-      <c r="K1" s="60"/>
-      <c r="L1" s="60"/>
-      <c r="M1" s="60"/>
-      <c r="N1" s="60"/>
-      <c r="O1" s="60"/>
-      <c r="P1" s="60"/>
-      <c r="Q1" s="60"/>
-      <c r="R1" s="60"/>
-      <c r="S1" s="60"/>
-      <c r="T1" s="60"/>
-      <c r="U1" s="60"/>
-      <c r="V1" s="60"/>
-      <c r="W1" s="60"/>
-      <c r="X1" s="60"/>
-      <c r="Y1" s="60"/>
-      <c r="Z1" s="60"/>
-      <c r="AA1" s="60"/>
-      <c r="AB1" s="60"/>
-      <c r="AC1" s="60"/>
+      <c r="A1" s="62" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="62"/>
+      <c r="C1" s="62"/>
+      <c r="D1" s="62"/>
+      <c r="E1" s="62"/>
+      <c r="F1" s="62"/>
+      <c r="G1" s="62"/>
+      <c r="H1" s="62"/>
+      <c r="I1" s="62"/>
+      <c r="J1" s="62"/>
+      <c r="K1" s="62"/>
+      <c r="L1" s="62"/>
+      <c r="M1" s="62"/>
+      <c r="N1" s="62"/>
+      <c r="O1" s="62"/>
+      <c r="P1" s="62"/>
+      <c r="Q1" s="62"/>
+      <c r="R1" s="62"/>
+      <c r="S1" s="62"/>
+      <c r="T1" s="62"/>
+      <c r="U1" s="62"/>
+      <c r="V1" s="62"/>
+      <c r="W1" s="62"/>
+      <c r="X1" s="62"/>
+      <c r="Y1" s="62"/>
+      <c r="Z1" s="62"/>
+      <c r="AA1" s="62"/>
+      <c r="AB1" s="62"/>
+      <c r="AC1" s="62"/>
     </row>
     <row r="2" spans="1:29" ht="18">
       <c r="A2" s="23" t="s">
@@ -5198,10 +5912,10 @@
       <c r="AC2" s="32"/>
     </row>
     <row r="3" spans="1:29">
-      <c r="A3" s="61" t="s">
+      <c r="A3" s="63" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="61"/>
+      <c r="B3" s="63"/>
       <c r="C3" s="33"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -5483,37 +6197,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="18">
-      <c r="A1" s="60" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="60"/>
-      <c r="C1" s="60"/>
-      <c r="D1" s="60"/>
-      <c r="E1" s="60"/>
-      <c r="F1" s="60"/>
-      <c r="G1" s="60"/>
-      <c r="H1" s="60"/>
-      <c r="I1" s="60"/>
-      <c r="J1" s="60"/>
-      <c r="K1" s="60"/>
-      <c r="L1" s="60"/>
-      <c r="M1" s="60"/>
-      <c r="N1" s="60"/>
-      <c r="O1" s="60"/>
-      <c r="P1" s="60"/>
-      <c r="Q1" s="60"/>
-      <c r="R1" s="60"/>
-      <c r="S1" s="60"/>
-      <c r="T1" s="60"/>
-      <c r="U1" s="60"/>
-      <c r="V1" s="60"/>
-      <c r="W1" s="60"/>
-      <c r="X1" s="60"/>
-      <c r="Y1" s="60"/>
-      <c r="Z1" s="60"/>
-      <c r="AA1" s="60"/>
-      <c r="AB1" s="60"/>
-      <c r="AC1" s="60"/>
+      <c r="A1" s="62" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="62"/>
+      <c r="C1" s="62"/>
+      <c r="D1" s="62"/>
+      <c r="E1" s="62"/>
+      <c r="F1" s="62"/>
+      <c r="G1" s="62"/>
+      <c r="H1" s="62"/>
+      <c r="I1" s="62"/>
+      <c r="J1" s="62"/>
+      <c r="K1" s="62"/>
+      <c r="L1" s="62"/>
+      <c r="M1" s="62"/>
+      <c r="N1" s="62"/>
+      <c r="O1" s="62"/>
+      <c r="P1" s="62"/>
+      <c r="Q1" s="62"/>
+      <c r="R1" s="62"/>
+      <c r="S1" s="62"/>
+      <c r="T1" s="62"/>
+      <c r="U1" s="62"/>
+      <c r="V1" s="62"/>
+      <c r="W1" s="62"/>
+      <c r="X1" s="62"/>
+      <c r="Y1" s="62"/>
+      <c r="Z1" s="62"/>
+      <c r="AA1" s="62"/>
+      <c r="AB1" s="62"/>
+      <c r="AC1" s="62"/>
     </row>
     <row r="2" spans="1:29" ht="18">
       <c r="A2" s="23" t="s">
@@ -5551,10 +6265,10 @@
       <c r="AC2" s="34"/>
     </row>
     <row r="3" spans="1:29">
-      <c r="A3" s="61" t="s">
+      <c r="A3" s="63" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="61"/>
+      <c r="B3" s="63"/>
       <c r="C3" s="35"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -5834,37 +6548,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="18">
-      <c r="A1" s="60" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="60"/>
-      <c r="C1" s="60"/>
-      <c r="D1" s="60"/>
-      <c r="E1" s="60"/>
-      <c r="F1" s="60"/>
-      <c r="G1" s="60"/>
-      <c r="H1" s="60"/>
-      <c r="I1" s="60"/>
-      <c r="J1" s="60"/>
-      <c r="K1" s="60"/>
-      <c r="L1" s="60"/>
-      <c r="M1" s="60"/>
-      <c r="N1" s="60"/>
-      <c r="O1" s="60"/>
-      <c r="P1" s="60"/>
-      <c r="Q1" s="60"/>
-      <c r="R1" s="60"/>
-      <c r="S1" s="60"/>
-      <c r="T1" s="60"/>
-      <c r="U1" s="60"/>
-      <c r="V1" s="60"/>
-      <c r="W1" s="60"/>
-      <c r="X1" s="60"/>
-      <c r="Y1" s="60"/>
-      <c r="Z1" s="60"/>
-      <c r="AA1" s="60"/>
-      <c r="AB1" s="60"/>
-      <c r="AC1" s="60"/>
+      <c r="A1" s="62" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="62"/>
+      <c r="C1" s="62"/>
+      <c r="D1" s="62"/>
+      <c r="E1" s="62"/>
+      <c r="F1" s="62"/>
+      <c r="G1" s="62"/>
+      <c r="H1" s="62"/>
+      <c r="I1" s="62"/>
+      <c r="J1" s="62"/>
+      <c r="K1" s="62"/>
+      <c r="L1" s="62"/>
+      <c r="M1" s="62"/>
+      <c r="N1" s="62"/>
+      <c r="O1" s="62"/>
+      <c r="P1" s="62"/>
+      <c r="Q1" s="62"/>
+      <c r="R1" s="62"/>
+      <c r="S1" s="62"/>
+      <c r="T1" s="62"/>
+      <c r="U1" s="62"/>
+      <c r="V1" s="62"/>
+      <c r="W1" s="62"/>
+      <c r="X1" s="62"/>
+      <c r="Y1" s="62"/>
+      <c r="Z1" s="62"/>
+      <c r="AA1" s="62"/>
+      <c r="AB1" s="62"/>
+      <c r="AC1" s="62"/>
     </row>
     <row r="2" spans="1:29" ht="18">
       <c r="A2" s="23" t="s">
@@ -5902,10 +6616,10 @@
       <c r="AC2" s="36"/>
     </row>
     <row r="3" spans="1:29">
-      <c r="A3" s="61" t="s">
+      <c r="A3" s="63" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="61"/>
+      <c r="B3" s="63"/>
       <c r="C3" s="37"/>
       <c r="D3" s="3">
         <v>2</v>
@@ -6202,37 +6916,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:31" ht="18">
-      <c r="A1" s="60" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="60"/>
-      <c r="C1" s="60"/>
-      <c r="D1" s="60"/>
-      <c r="E1" s="60"/>
-      <c r="F1" s="60"/>
-      <c r="G1" s="60"/>
-      <c r="H1" s="60"/>
-      <c r="I1" s="60"/>
-      <c r="J1" s="60"/>
-      <c r="K1" s="60"/>
-      <c r="L1" s="60"/>
-      <c r="M1" s="60"/>
-      <c r="N1" s="60"/>
-      <c r="O1" s="60"/>
-      <c r="P1" s="60"/>
-      <c r="Q1" s="60"/>
-      <c r="R1" s="60"/>
-      <c r="S1" s="60"/>
-      <c r="T1" s="60"/>
-      <c r="U1" s="60"/>
-      <c r="V1" s="60"/>
-      <c r="W1" s="60"/>
-      <c r="X1" s="60"/>
-      <c r="Y1" s="60"/>
-      <c r="Z1" s="60"/>
-      <c r="AA1" s="60"/>
-      <c r="AB1" s="60"/>
-      <c r="AC1" s="60"/>
+      <c r="A1" s="62" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="62"/>
+      <c r="C1" s="62"/>
+      <c r="D1" s="62"/>
+      <c r="E1" s="62"/>
+      <c r="F1" s="62"/>
+      <c r="G1" s="62"/>
+      <c r="H1" s="62"/>
+      <c r="I1" s="62"/>
+      <c r="J1" s="62"/>
+      <c r="K1" s="62"/>
+      <c r="L1" s="62"/>
+      <c r="M1" s="62"/>
+      <c r="N1" s="62"/>
+      <c r="O1" s="62"/>
+      <c r="P1" s="62"/>
+      <c r="Q1" s="62"/>
+      <c r="R1" s="62"/>
+      <c r="S1" s="62"/>
+      <c r="T1" s="62"/>
+      <c r="U1" s="62"/>
+      <c r="V1" s="62"/>
+      <c r="W1" s="62"/>
+      <c r="X1" s="62"/>
+      <c r="Y1" s="62"/>
+      <c r="Z1" s="62"/>
+      <c r="AA1" s="62"/>
+      <c r="AB1" s="62"/>
+      <c r="AC1" s="62"/>
     </row>
     <row r="2" spans="1:31" ht="16.5" customHeight="1">
       <c r="A2" s="23" t="s">
@@ -6270,10 +6984,10 @@
       <c r="AC2" s="41"/>
     </row>
     <row r="3" spans="1:31">
-      <c r="A3" s="61" t="s">
+      <c r="A3" s="63" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="61"/>
+      <c r="B3" s="63"/>
       <c r="D3">
         <v>2</v>
       </c>

</xml_diff>

<commit_message>
PurchaseBills Fixes are Updated
PurchaseBills Fixes are Updated
</commit_message>
<xml_diff>
--- a/testdata/DBfin.xlsx
+++ b/testdata/DBfin.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4507"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="2520" windowWidth="16695" windowHeight="6540" tabRatio="594" firstSheet="11" activeTab="13"/>
+    <workbookView xWindow="0" yWindow="2520" windowWidth="16695" windowHeight="6540" tabRatio="594" firstSheet="12" activeTab="15"/>
   </bookViews>
   <sheets>
     <sheet name="PurchaseBillsLocal" sheetId="1" r:id="rId1"/>
@@ -21,13 +21,15 @@
     <sheet name="PurchaseBills_Interstate_Un" sheetId="12" r:id="rId12"/>
     <sheet name="PurchaseBillsUTGST_Ureq" sheetId="13" r:id="rId13"/>
     <sheet name="PurchaseBills_Un_Regrd_Iter" sheetId="14" r:id="rId14"/>
+    <sheet name="Purchasebills_UTGST_2" sheetId="15" r:id="rId15"/>
+    <sheet name="PurchaseBills_Rcm" sheetId="16" r:id="rId16"/>
   </sheets>
   <calcPr calcId="125725"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="741" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="865" uniqueCount="62">
   <si>
     <t>Scenario  : Local Sales - Stock UOM and Sales UOM (Similar)   DOC NO :  SORD-2425-00089</t>
   </si>
@@ -364,7 +366,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="64">
+  <cellXfs count="69">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -501,6 +503,19 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -832,68 +847,68 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:59" ht="18">
-      <c r="A1" s="62" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="62"/>
-      <c r="C1" s="62"/>
-      <c r="D1" s="62"/>
-      <c r="E1" s="62"/>
-      <c r="F1" s="62"/>
-      <c r="G1" s="62"/>
-      <c r="H1" s="62"/>
-      <c r="I1" s="62"/>
-      <c r="J1" s="62"/>
-      <c r="K1" s="62"/>
-      <c r="L1" s="62"/>
-      <c r="M1" s="62"/>
-      <c r="N1" s="62"/>
-      <c r="O1" s="62"/>
-      <c r="P1" s="62"/>
-      <c r="Q1" s="62"/>
-      <c r="R1" s="62"/>
-      <c r="S1" s="62"/>
-      <c r="T1" s="62"/>
-      <c r="U1" s="62"/>
-      <c r="V1" s="62"/>
-      <c r="W1" s="62"/>
-      <c r="X1" s="62"/>
-      <c r="Y1" s="62"/>
-      <c r="Z1" s="62"/>
-      <c r="AA1" s="62"/>
-      <c r="AB1" s="62"/>
-      <c r="AC1" s="62"/>
-      <c r="AD1" s="62" t="s">
-        <v>0</v>
-      </c>
-      <c r="AE1" s="62"/>
-      <c r="AF1" s="62"/>
-      <c r="AG1" s="62"/>
-      <c r="AH1" s="62"/>
-      <c r="AI1" s="62"/>
-      <c r="AJ1" s="62"/>
-      <c r="AK1" s="62"/>
-      <c r="AL1" s="62"/>
-      <c r="AM1" s="62"/>
-      <c r="AN1" s="62"/>
-      <c r="AO1" s="62"/>
-      <c r="AP1" s="62"/>
-      <c r="AQ1" s="62"/>
-      <c r="AR1" s="62"/>
-      <c r="AS1" s="62"/>
-      <c r="AT1" s="62"/>
-      <c r="AU1" s="62"/>
-      <c r="AV1" s="62"/>
-      <c r="AW1" s="62"/>
-      <c r="AX1" s="62"/>
-      <c r="AY1" s="62"/>
-      <c r="AZ1" s="62"/>
-      <c r="BA1" s="62"/>
-      <c r="BB1" s="62"/>
-      <c r="BC1" s="62"/>
-      <c r="BD1" s="62"/>
-      <c r="BE1" s="62"/>
-      <c r="BF1" s="62"/>
+      <c r="A1" s="67" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="67"/>
+      <c r="C1" s="67"/>
+      <c r="D1" s="67"/>
+      <c r="E1" s="67"/>
+      <c r="F1" s="67"/>
+      <c r="G1" s="67"/>
+      <c r="H1" s="67"/>
+      <c r="I1" s="67"/>
+      <c r="J1" s="67"/>
+      <c r="K1" s="67"/>
+      <c r="L1" s="67"/>
+      <c r="M1" s="67"/>
+      <c r="N1" s="67"/>
+      <c r="O1" s="67"/>
+      <c r="P1" s="67"/>
+      <c r="Q1" s="67"/>
+      <c r="R1" s="67"/>
+      <c r="S1" s="67"/>
+      <c r="T1" s="67"/>
+      <c r="U1" s="67"/>
+      <c r="V1" s="67"/>
+      <c r="W1" s="67"/>
+      <c r="X1" s="67"/>
+      <c r="Y1" s="67"/>
+      <c r="Z1" s="67"/>
+      <c r="AA1" s="67"/>
+      <c r="AB1" s="67"/>
+      <c r="AC1" s="67"/>
+      <c r="AD1" s="67" t="s">
+        <v>0</v>
+      </c>
+      <c r="AE1" s="67"/>
+      <c r="AF1" s="67"/>
+      <c r="AG1" s="67"/>
+      <c r="AH1" s="67"/>
+      <c r="AI1" s="67"/>
+      <c r="AJ1" s="67"/>
+      <c r="AK1" s="67"/>
+      <c r="AL1" s="67"/>
+      <c r="AM1" s="67"/>
+      <c r="AN1" s="67"/>
+      <c r="AO1" s="67"/>
+      <c r="AP1" s="67"/>
+      <c r="AQ1" s="67"/>
+      <c r="AR1" s="67"/>
+      <c r="AS1" s="67"/>
+      <c r="AT1" s="67"/>
+      <c r="AU1" s="67"/>
+      <c r="AV1" s="67"/>
+      <c r="AW1" s="67"/>
+      <c r="AX1" s="67"/>
+      <c r="AY1" s="67"/>
+      <c r="AZ1" s="67"/>
+      <c r="BA1" s="67"/>
+      <c r="BB1" s="67"/>
+      <c r="BC1" s="67"/>
+      <c r="BD1" s="67"/>
+      <c r="BE1" s="67"/>
+      <c r="BF1" s="67"/>
     </row>
     <row r="2" spans="1:59" ht="18">
       <c r="A2" s="23" t="s">
@@ -964,10 +979,10 @@
       <c r="BF2" s="38"/>
     </row>
     <row r="3" spans="1:59">
-      <c r="A3" s="63" t="s">
+      <c r="A3" s="68" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="63"/>
+      <c r="B3" s="68"/>
       <c r="C3" s="2"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -1007,10 +1022,10 @@
       <c r="AA3" s="6"/>
       <c r="AB3" s="6"/>
       <c r="AC3" s="6"/>
-      <c r="AD3" s="63" t="s">
+      <c r="AD3" s="68" t="s">
         <v>3</v>
       </c>
-      <c r="AE3" s="63"/>
+      <c r="AE3" s="68"/>
       <c r="AF3" s="39"/>
       <c r="AG3" s="3">
         <v>1</v>
@@ -1487,38 +1502,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:33" ht="18">
-      <c r="A1" s="62" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="62"/>
-      <c r="C1" s="62"/>
-      <c r="D1" s="62"/>
-      <c r="E1" s="62"/>
-      <c r="F1" s="62"/>
-      <c r="G1" s="62"/>
-      <c r="H1" s="62"/>
-      <c r="I1" s="62"/>
-      <c r="J1" s="62"/>
-      <c r="K1" s="62"/>
-      <c r="L1" s="62"/>
-      <c r="M1" s="62"/>
-      <c r="N1" s="62"/>
-      <c r="O1" s="62"/>
-      <c r="P1" s="62"/>
-      <c r="Q1" s="62"/>
-      <c r="R1" s="62"/>
-      <c r="S1" s="62"/>
-      <c r="T1" s="62"/>
-      <c r="U1" s="62"/>
-      <c r="V1" s="62"/>
-      <c r="W1" s="62"/>
-      <c r="X1" s="62"/>
-      <c r="Y1" s="62"/>
-      <c r="Z1" s="62"/>
-      <c r="AA1" s="62"/>
-      <c r="AB1" s="62"/>
-      <c r="AC1" s="62"/>
-      <c r="AD1" s="62"/>
+      <c r="A1" s="67" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="67"/>
+      <c r="C1" s="67"/>
+      <c r="D1" s="67"/>
+      <c r="E1" s="67"/>
+      <c r="F1" s="67"/>
+      <c r="G1" s="67"/>
+      <c r="H1" s="67"/>
+      <c r="I1" s="67"/>
+      <c r="J1" s="67"/>
+      <c r="K1" s="67"/>
+      <c r="L1" s="67"/>
+      <c r="M1" s="67"/>
+      <c r="N1" s="67"/>
+      <c r="O1" s="67"/>
+      <c r="P1" s="67"/>
+      <c r="Q1" s="67"/>
+      <c r="R1" s="67"/>
+      <c r="S1" s="67"/>
+      <c r="T1" s="67"/>
+      <c r="U1" s="67"/>
+      <c r="V1" s="67"/>
+      <c r="W1" s="67"/>
+      <c r="X1" s="67"/>
+      <c r="Y1" s="67"/>
+      <c r="Z1" s="67"/>
+      <c r="AA1" s="67"/>
+      <c r="AB1" s="67"/>
+      <c r="AC1" s="67"/>
+      <c r="AD1" s="67"/>
     </row>
     <row r="2" spans="1:33" ht="18">
       <c r="A2" s="23" t="s">
@@ -1557,10 +1572,10 @@
       <c r="AD2" s="43"/>
     </row>
     <row r="3" spans="1:33" ht="15.75" thickBot="1">
-      <c r="A3" s="63" t="s">
+      <c r="A3" s="68" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="63"/>
+      <c r="B3" s="68"/>
       <c r="C3" s="44"/>
       <c r="D3" s="3">
         <v>2</v>
@@ -2174,37 +2189,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:31" ht="18">
-      <c r="A1" s="62" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="62"/>
-      <c r="C1" s="62"/>
-      <c r="D1" s="62"/>
-      <c r="E1" s="62"/>
-      <c r="F1" s="62"/>
-      <c r="G1" s="62"/>
-      <c r="H1" s="62"/>
-      <c r="I1" s="62"/>
-      <c r="J1" s="62"/>
-      <c r="K1" s="62"/>
-      <c r="L1" s="62"/>
-      <c r="M1" s="62"/>
-      <c r="N1" s="62"/>
-      <c r="O1" s="62"/>
-      <c r="P1" s="62"/>
-      <c r="Q1" s="62"/>
-      <c r="R1" s="62"/>
-      <c r="S1" s="62"/>
-      <c r="T1" s="62"/>
-      <c r="U1" s="62"/>
-      <c r="V1" s="62"/>
-      <c r="W1" s="62"/>
-      <c r="X1" s="62"/>
-      <c r="Y1" s="62"/>
-      <c r="Z1" s="62"/>
-      <c r="AA1" s="62"/>
-      <c r="AB1" s="62"/>
-      <c r="AC1" s="62"/>
+      <c r="A1" s="67" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="67"/>
+      <c r="C1" s="67"/>
+      <c r="D1" s="67"/>
+      <c r="E1" s="67"/>
+      <c r="F1" s="67"/>
+      <c r="G1" s="67"/>
+      <c r="H1" s="67"/>
+      <c r="I1" s="67"/>
+      <c r="J1" s="67"/>
+      <c r="K1" s="67"/>
+      <c r="L1" s="67"/>
+      <c r="M1" s="67"/>
+      <c r="N1" s="67"/>
+      <c r="O1" s="67"/>
+      <c r="P1" s="67"/>
+      <c r="Q1" s="67"/>
+      <c r="R1" s="67"/>
+      <c r="S1" s="67"/>
+      <c r="T1" s="67"/>
+      <c r="U1" s="67"/>
+      <c r="V1" s="67"/>
+      <c r="W1" s="67"/>
+      <c r="X1" s="67"/>
+      <c r="Y1" s="67"/>
+      <c r="Z1" s="67"/>
+      <c r="AA1" s="67"/>
+      <c r="AB1" s="67"/>
+      <c r="AC1" s="67"/>
     </row>
     <row r="2" spans="1:31" ht="16.5" customHeight="1">
       <c r="A2" s="23" t="s">
@@ -2242,10 +2257,10 @@
       <c r="AC2" s="54"/>
     </row>
     <row r="3" spans="1:31">
-      <c r="A3" s="63" t="s">
+      <c r="A3" s="68" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="63"/>
+      <c r="B3" s="68"/>
       <c r="D3">
         <v>2</v>
       </c>
@@ -2736,37 +2751,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="18">
-      <c r="A1" s="62" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="62"/>
-      <c r="C1" s="62"/>
-      <c r="D1" s="62"/>
-      <c r="E1" s="62"/>
-      <c r="F1" s="62"/>
-      <c r="G1" s="62"/>
-      <c r="H1" s="62"/>
-      <c r="I1" s="62"/>
-      <c r="J1" s="62"/>
-      <c r="K1" s="62"/>
-      <c r="L1" s="62"/>
-      <c r="M1" s="62"/>
-      <c r="N1" s="62"/>
-      <c r="O1" s="62"/>
-      <c r="P1" s="62"/>
-      <c r="Q1" s="62"/>
-      <c r="R1" s="62"/>
-      <c r="S1" s="62"/>
-      <c r="T1" s="62"/>
-      <c r="U1" s="62"/>
-      <c r="V1" s="62"/>
-      <c r="W1" s="62"/>
-      <c r="X1" s="62"/>
-      <c r="Y1" s="62"/>
-      <c r="Z1" s="62"/>
-      <c r="AA1" s="62"/>
-      <c r="AB1" s="62"/>
-      <c r="AC1" s="62"/>
+      <c r="A1" s="67" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="67"/>
+      <c r="C1" s="67"/>
+      <c r="D1" s="67"/>
+      <c r="E1" s="67"/>
+      <c r="F1" s="67"/>
+      <c r="G1" s="67"/>
+      <c r="H1" s="67"/>
+      <c r="I1" s="67"/>
+      <c r="J1" s="67"/>
+      <c r="K1" s="67"/>
+      <c r="L1" s="67"/>
+      <c r="M1" s="67"/>
+      <c r="N1" s="67"/>
+      <c r="O1" s="67"/>
+      <c r="P1" s="67"/>
+      <c r="Q1" s="67"/>
+      <c r="R1" s="67"/>
+      <c r="S1" s="67"/>
+      <c r="T1" s="67"/>
+      <c r="U1" s="67"/>
+      <c r="V1" s="67"/>
+      <c r="W1" s="67"/>
+      <c r="X1" s="67"/>
+      <c r="Y1" s="67"/>
+      <c r="Z1" s="67"/>
+      <c r="AA1" s="67"/>
+      <c r="AB1" s="67"/>
+      <c r="AC1" s="67"/>
     </row>
     <row r="2" spans="1:29" ht="18">
       <c r="A2" s="23" t="s">
@@ -2804,10 +2819,10 @@
       <c r="AC2" s="56"/>
     </row>
     <row r="3" spans="1:29">
-      <c r="A3" s="63" t="s">
+      <c r="A3" s="68" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="63"/>
+      <c r="B3" s="68"/>
       <c r="C3" s="57"/>
       <c r="D3" s="3">
         <v>2</v>
@@ -3088,37 +3103,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="18">
-      <c r="A1" s="62" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="62"/>
-      <c r="C1" s="62"/>
-      <c r="D1" s="62"/>
-      <c r="E1" s="62"/>
-      <c r="F1" s="62"/>
-      <c r="G1" s="62"/>
-      <c r="H1" s="62"/>
-      <c r="I1" s="62"/>
-      <c r="J1" s="62"/>
-      <c r="K1" s="62"/>
-      <c r="L1" s="62"/>
-      <c r="M1" s="62"/>
-      <c r="N1" s="62"/>
-      <c r="O1" s="62"/>
-      <c r="P1" s="62"/>
-      <c r="Q1" s="62"/>
-      <c r="R1" s="62"/>
-      <c r="S1" s="62"/>
-      <c r="T1" s="62"/>
-      <c r="U1" s="62"/>
-      <c r="V1" s="62"/>
-      <c r="W1" s="62"/>
-      <c r="X1" s="62"/>
-      <c r="Y1" s="62"/>
-      <c r="Z1" s="62"/>
-      <c r="AA1" s="62"/>
-      <c r="AB1" s="62"/>
-      <c r="AC1" s="62"/>
+      <c r="A1" s="67" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="67"/>
+      <c r="C1" s="67"/>
+      <c r="D1" s="67"/>
+      <c r="E1" s="67"/>
+      <c r="F1" s="67"/>
+      <c r="G1" s="67"/>
+      <c r="H1" s="67"/>
+      <c r="I1" s="67"/>
+      <c r="J1" s="67"/>
+      <c r="K1" s="67"/>
+      <c r="L1" s="67"/>
+      <c r="M1" s="67"/>
+      <c r="N1" s="67"/>
+      <c r="O1" s="67"/>
+      <c r="P1" s="67"/>
+      <c r="Q1" s="67"/>
+      <c r="R1" s="67"/>
+      <c r="S1" s="67"/>
+      <c r="T1" s="67"/>
+      <c r="U1" s="67"/>
+      <c r="V1" s="67"/>
+      <c r="W1" s="67"/>
+      <c r="X1" s="67"/>
+      <c r="Y1" s="67"/>
+      <c r="Z1" s="67"/>
+      <c r="AA1" s="67"/>
+      <c r="AB1" s="67"/>
+      <c r="AC1" s="67"/>
     </row>
     <row r="2" spans="1:29" ht="18">
       <c r="A2" s="23" t="s">
@@ -3156,10 +3171,10 @@
       <c r="AC2" s="58"/>
     </row>
     <row r="3" spans="1:29">
-      <c r="A3" s="63" t="s">
+      <c r="A3" s="68" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="63"/>
+      <c r="B3" s="68"/>
       <c r="C3" s="59"/>
       <c r="D3" s="3">
         <v>4</v>
@@ -3355,7 +3370,7 @@
         <v>0.18</v>
       </c>
       <c r="X5" s="24">
-        <v>0</v>
+        <v>203</v>
       </c>
       <c r="Y5" s="24">
         <f>IF($D$3=1,ROUND(((U5*W5)/2),2),0)</f>
@@ -3366,11 +3381,11 @@
         <v>0</v>
       </c>
       <c r="AA5" s="24">
-        <v>0</v>
+        <v>203</v>
       </c>
       <c r="AB5" s="24">
         <f>X5+Y5+Z5+AA5</f>
-        <v>0</v>
+        <v>406</v>
       </c>
       <c r="AC5" s="24">
         <f>U5</f>
@@ -3442,38 +3457,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:33" ht="18">
-      <c r="A1" s="62" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="62"/>
-      <c r="C1" s="62"/>
-      <c r="D1" s="62"/>
-      <c r="E1" s="62"/>
-      <c r="F1" s="62"/>
-      <c r="G1" s="62"/>
-      <c r="H1" s="62"/>
-      <c r="I1" s="62"/>
-      <c r="J1" s="62"/>
-      <c r="K1" s="62"/>
-      <c r="L1" s="62"/>
-      <c r="M1" s="62"/>
-      <c r="N1" s="62"/>
-      <c r="O1" s="62"/>
-      <c r="P1" s="62"/>
-      <c r="Q1" s="62"/>
-      <c r="R1" s="62"/>
-      <c r="S1" s="62"/>
-      <c r="T1" s="62"/>
-      <c r="U1" s="62"/>
-      <c r="V1" s="62"/>
-      <c r="W1" s="62"/>
-      <c r="X1" s="62"/>
-      <c r="Y1" s="62"/>
-      <c r="Z1" s="62"/>
-      <c r="AA1" s="62"/>
-      <c r="AB1" s="62"/>
-      <c r="AC1" s="62"/>
-      <c r="AD1" s="62"/>
+      <c r="A1" s="67" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="67"/>
+      <c r="C1" s="67"/>
+      <c r="D1" s="67"/>
+      <c r="E1" s="67"/>
+      <c r="F1" s="67"/>
+      <c r="G1" s="67"/>
+      <c r="H1" s="67"/>
+      <c r="I1" s="67"/>
+      <c r="J1" s="67"/>
+      <c r="K1" s="67"/>
+      <c r="L1" s="67"/>
+      <c r="M1" s="67"/>
+      <c r="N1" s="67"/>
+      <c r="O1" s="67"/>
+      <c r="P1" s="67"/>
+      <c r="Q1" s="67"/>
+      <c r="R1" s="67"/>
+      <c r="S1" s="67"/>
+      <c r="T1" s="67"/>
+      <c r="U1" s="67"/>
+      <c r="V1" s="67"/>
+      <c r="W1" s="67"/>
+      <c r="X1" s="67"/>
+      <c r="Y1" s="67"/>
+      <c r="Z1" s="67"/>
+      <c r="AA1" s="67"/>
+      <c r="AB1" s="67"/>
+      <c r="AC1" s="67"/>
+      <c r="AD1" s="67"/>
     </row>
     <row r="2" spans="1:33" ht="18">
       <c r="A2" s="23" t="s">
@@ -3512,10 +3527,10 @@
       <c r="AD2" s="60"/>
     </row>
     <row r="3" spans="1:33" ht="15.75" thickBot="1">
-      <c r="A3" s="63" t="s">
+      <c r="A3" s="68" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="63"/>
+      <c r="B3" s="68"/>
       <c r="C3" s="61"/>
       <c r="D3" s="3">
         <v>2</v>
@@ -4103,6 +4118,1017 @@
     <mergeCell ref="A3:B3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:AC6"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="2" max="2" width="20.5703125" customWidth="1"/>
+    <col min="4" max="4" width="29.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.28515625" customWidth="1"/>
+    <col min="6" max="6" width="16.28515625" customWidth="1"/>
+    <col min="7" max="7" width="24.42578125" customWidth="1"/>
+    <col min="8" max="8" width="20.28515625" customWidth="1"/>
+    <col min="9" max="9" width="20" customWidth="1"/>
+    <col min="13" max="13" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="13.7109375" customWidth="1"/>
+    <col min="18" max="18" width="13" customWidth="1"/>
+    <col min="19" max="19" width="14.42578125" customWidth="1"/>
+    <col min="20" max="20" width="18.42578125" customWidth="1"/>
+    <col min="21" max="21" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="10.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:29" ht="18">
+      <c r="A1" s="67" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="67"/>
+      <c r="C1" s="67"/>
+      <c r="D1" s="67"/>
+      <c r="E1" s="67"/>
+      <c r="F1" s="67"/>
+      <c r="G1" s="67"/>
+      <c r="H1" s="67"/>
+      <c r="I1" s="67"/>
+      <c r="J1" s="67"/>
+      <c r="K1" s="67"/>
+      <c r="L1" s="67"/>
+      <c r="M1" s="67"/>
+      <c r="N1" s="67"/>
+      <c r="O1" s="67"/>
+      <c r="P1" s="67"/>
+      <c r="Q1" s="67"/>
+      <c r="R1" s="67"/>
+      <c r="S1" s="67"/>
+      <c r="T1" s="67"/>
+      <c r="U1" s="67"/>
+      <c r="V1" s="67"/>
+      <c r="W1" s="67"/>
+      <c r="X1" s="67"/>
+      <c r="Y1" s="67"/>
+      <c r="Z1" s="67"/>
+      <c r="AA1" s="67"/>
+      <c r="AB1" s="67"/>
+      <c r="AC1" s="67"/>
+    </row>
+    <row r="2" spans="1:29" ht="18">
+      <c r="A2" s="23" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="23" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" s="62"/>
+      <c r="D2" s="62"/>
+      <c r="E2" s="62"/>
+      <c r="F2" s="62"/>
+      <c r="G2" s="62"/>
+      <c r="H2" s="62"/>
+      <c r="I2" s="62"/>
+      <c r="J2" s="62"/>
+      <c r="K2" s="62"/>
+      <c r="L2" s="62"/>
+      <c r="M2" s="62"/>
+      <c r="N2" s="62"/>
+      <c r="O2" s="62"/>
+      <c r="P2" s="62"/>
+      <c r="Q2" s="62"/>
+      <c r="R2" s="62"/>
+      <c r="S2" s="62"/>
+      <c r="T2" s="62"/>
+      <c r="U2" s="62"/>
+      <c r="V2" s="62"/>
+      <c r="W2" s="62"/>
+      <c r="X2" s="62"/>
+      <c r="Y2" s="62"/>
+      <c r="Z2" s="62"/>
+      <c r="AA2" s="62"/>
+      <c r="AB2" s="62"/>
+      <c r="AC2" s="62"/>
+    </row>
+    <row r="3" spans="1:29">
+      <c r="A3" s="68" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="68"/>
+      <c r="C3" s="63"/>
+      <c r="D3" s="3">
+        <v>4</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="F3" s="5"/>
+      <c r="G3" s="5"/>
+      <c r="H3" s="5"/>
+      <c r="I3" s="6"/>
+      <c r="J3" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="K3" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="L3" s="7"/>
+      <c r="M3" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="N3" s="7">
+        <v>1</v>
+      </c>
+      <c r="O3" s="7"/>
+      <c r="P3" s="7"/>
+      <c r="Q3" s="7"/>
+      <c r="R3" s="7"/>
+      <c r="S3" s="6"/>
+      <c r="T3" s="6"/>
+      <c r="U3" s="6"/>
+      <c r="V3" s="6"/>
+      <c r="W3" s="6"/>
+      <c r="X3" s="6"/>
+      <c r="Y3" s="6"/>
+      <c r="Z3" s="6"/>
+      <c r="AA3" s="6"/>
+      <c r="AB3" s="6"/>
+      <c r="AC3" s="6"/>
+    </row>
+    <row r="4" spans="1:29" ht="42.75">
+      <c r="A4" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="E4" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="F4" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="G4" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="H4" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="I4" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="J4" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="K4" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="L4" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="M4" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="N4" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="O4" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="P4" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q4" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="R4" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="S4" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="T4" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="U4" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="V4" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="W4" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="X4" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y4" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="Z4" s="16" t="s">
+        <v>30</v>
+      </c>
+      <c r="AA4" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="AB4" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="AC4" s="17" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="5" spans="1:29">
+      <c r="A5" s="9">
+        <v>1</v>
+      </c>
+      <c r="B5" s="27" t="s">
+        <v>41</v>
+      </c>
+      <c r="C5" s="9">
+        <v>0</v>
+      </c>
+      <c r="D5" s="27" t="s">
+        <v>42</v>
+      </c>
+      <c r="E5" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="F5" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="G5" s="24">
+        <v>1</v>
+      </c>
+      <c r="H5" s="9">
+        <v>2255</v>
+      </c>
+      <c r="I5" s="8">
+        <v>2255</v>
+      </c>
+      <c r="J5" s="25"/>
+      <c r="K5" s="25"/>
+      <c r="L5" s="25"/>
+      <c r="M5" s="8">
+        <v>2255</v>
+      </c>
+      <c r="N5" s="8">
+        <v>0</v>
+      </c>
+      <c r="O5" s="8">
+        <v>2255</v>
+      </c>
+      <c r="P5" s="8">
+        <v>0</v>
+      </c>
+      <c r="Q5" s="8">
+        <v>2255</v>
+      </c>
+      <c r="R5" s="8">
+        <v>0</v>
+      </c>
+      <c r="S5" s="26">
+        <v>0</v>
+      </c>
+      <c r="T5" s="26">
+        <v>0</v>
+      </c>
+      <c r="U5" s="8">
+        <f>(I5-S5)</f>
+        <v>2255</v>
+      </c>
+      <c r="V5" s="24">
+        <v>88363222</v>
+      </c>
+      <c r="W5" s="18">
+        <v>0.18</v>
+      </c>
+      <c r="X5" s="24">
+        <v>203</v>
+      </c>
+      <c r="Y5" s="24">
+        <f>IF($D$3=1,ROUND(((U5*W5)/2),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="Z5" s="24">
+        <f>IF($D$3=2,ROUND(((U5*W5)),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="AA5" s="24">
+        <v>203</v>
+      </c>
+      <c r="AB5" s="24">
+        <f>X5+Y5+Z5+AA5</f>
+        <v>406</v>
+      </c>
+      <c r="AC5" s="24">
+        <f>U5</f>
+        <v>2255</v>
+      </c>
+    </row>
+    <row r="6" spans="1:29">
+      <c r="A6" s="19"/>
+      <c r="B6" s="19"/>
+      <c r="C6" s="19"/>
+      <c r="D6" s="19"/>
+      <c r="E6" s="19"/>
+      <c r="F6" s="19"/>
+      <c r="G6" s="20"/>
+      <c r="H6" s="21"/>
+      <c r="I6" s="21"/>
+      <c r="J6" s="22"/>
+      <c r="K6" s="22"/>
+      <c r="L6" s="22"/>
+      <c r="M6" s="21"/>
+      <c r="N6" s="21"/>
+      <c r="O6" s="21"/>
+      <c r="P6" s="21"/>
+      <c r="Q6" s="21"/>
+      <c r="R6" s="21"/>
+      <c r="S6" s="21"/>
+      <c r="T6" s="21"/>
+      <c r="U6" s="21"/>
+      <c r="V6" s="21"/>
+      <c r="W6" s="22"/>
+      <c r="X6" s="21"/>
+      <c r="Y6" s="21"/>
+      <c r="Z6" s="21"/>
+      <c r="AA6" s="21"/>
+      <c r="AB6" s="21"/>
+      <c r="AC6" s="21"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:AC1"/>
+    <mergeCell ref="A3:B3"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:BG6"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="2" max="2" width="20.5703125" customWidth="1"/>
+    <col min="4" max="4" width="29.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.28515625" customWidth="1"/>
+    <col min="6" max="6" width="16.28515625" customWidth="1"/>
+    <col min="7" max="7" width="24.42578125" customWidth="1"/>
+    <col min="8" max="8" width="20.28515625" customWidth="1"/>
+    <col min="9" max="9" width="20" customWidth="1"/>
+    <col min="13" max="13" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="13.7109375" customWidth="1"/>
+    <col min="18" max="18" width="13" customWidth="1"/>
+    <col min="19" max="19" width="14.42578125" customWidth="1"/>
+    <col min="20" max="20" width="18.42578125" customWidth="1"/>
+    <col min="21" max="21" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="10" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="14" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="50" max="50" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="51" max="51" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="10" bestFit="1" customWidth="1"/>
+    <col min="59" max="59" width="15.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:59" ht="18">
+      <c r="A1" s="67" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="67"/>
+      <c r="C1" s="67"/>
+      <c r="D1" s="67"/>
+      <c r="E1" s="67"/>
+      <c r="F1" s="67"/>
+      <c r="G1" s="67"/>
+      <c r="H1" s="67"/>
+      <c r="I1" s="67"/>
+      <c r="J1" s="67"/>
+      <c r="K1" s="67"/>
+      <c r="L1" s="67"/>
+      <c r="M1" s="67"/>
+      <c r="N1" s="67"/>
+      <c r="O1" s="67"/>
+      <c r="P1" s="67"/>
+      <c r="Q1" s="67"/>
+      <c r="R1" s="67"/>
+      <c r="S1" s="67"/>
+      <c r="T1" s="67"/>
+      <c r="U1" s="67"/>
+      <c r="V1" s="67"/>
+      <c r="W1" s="67"/>
+      <c r="X1" s="67"/>
+      <c r="Y1" s="67"/>
+      <c r="Z1" s="67"/>
+      <c r="AA1" s="67"/>
+      <c r="AB1" s="67"/>
+      <c r="AC1" s="67"/>
+      <c r="AD1" s="67" t="s">
+        <v>0</v>
+      </c>
+      <c r="AE1" s="67"/>
+      <c r="AF1" s="67"/>
+      <c r="AG1" s="67"/>
+      <c r="AH1" s="67"/>
+      <c r="AI1" s="67"/>
+      <c r="AJ1" s="67"/>
+      <c r="AK1" s="67"/>
+      <c r="AL1" s="67"/>
+      <c r="AM1" s="67"/>
+      <c r="AN1" s="67"/>
+      <c r="AO1" s="67"/>
+      <c r="AP1" s="67"/>
+      <c r="AQ1" s="67"/>
+      <c r="AR1" s="67"/>
+      <c r="AS1" s="67"/>
+      <c r="AT1" s="67"/>
+      <c r="AU1" s="67"/>
+      <c r="AV1" s="67"/>
+      <c r="AW1" s="67"/>
+      <c r="AX1" s="67"/>
+      <c r="AY1" s="67"/>
+      <c r="AZ1" s="67"/>
+      <c r="BA1" s="67"/>
+      <c r="BB1" s="67"/>
+      <c r="BC1" s="67"/>
+      <c r="BD1" s="67"/>
+      <c r="BE1" s="67"/>
+      <c r="BF1" s="67"/>
+    </row>
+    <row r="2" spans="1:59" ht="18">
+      <c r="A2" s="23" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="23" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" s="64"/>
+      <c r="D2" s="64"/>
+      <c r="E2" s="64"/>
+      <c r="F2" s="64"/>
+      <c r="G2" s="64"/>
+      <c r="H2" s="64"/>
+      <c r="I2" s="64"/>
+      <c r="J2" s="64"/>
+      <c r="K2" s="64"/>
+      <c r="L2" s="64"/>
+      <c r="M2" s="64"/>
+      <c r="N2" s="64"/>
+      <c r="O2" s="64"/>
+      <c r="P2" s="64"/>
+      <c r="Q2" s="64"/>
+      <c r="R2" s="64"/>
+      <c r="S2" s="64"/>
+      <c r="T2" s="64"/>
+      <c r="U2" s="64"/>
+      <c r="V2" s="64"/>
+      <c r="W2" s="64"/>
+      <c r="X2" s="64"/>
+      <c r="Y2" s="64"/>
+      <c r="Z2" s="64"/>
+      <c r="AA2" s="64"/>
+      <c r="AB2" s="64"/>
+      <c r="AC2" s="64"/>
+      <c r="AD2" s="23" t="s">
+        <v>1</v>
+      </c>
+      <c r="AE2" s="23" t="s">
+        <v>2</v>
+      </c>
+      <c r="AF2" s="64"/>
+      <c r="AG2" s="64"/>
+      <c r="AH2" s="64"/>
+      <c r="AI2" s="64"/>
+      <c r="AJ2" s="64"/>
+      <c r="AK2" s="64"/>
+      <c r="AL2" s="64"/>
+      <c r="AM2" s="64"/>
+      <c r="AN2" s="64"/>
+      <c r="AO2" s="64"/>
+      <c r="AP2" s="64"/>
+      <c r="AQ2" s="64"/>
+      <c r="AR2" s="64"/>
+      <c r="AS2" s="64"/>
+      <c r="AT2" s="64"/>
+      <c r="AU2" s="64"/>
+      <c r="AV2" s="64"/>
+      <c r="AW2" s="64"/>
+      <c r="AX2" s="64"/>
+      <c r="AY2" s="64"/>
+      <c r="AZ2" s="64"/>
+      <c r="BA2" s="64"/>
+      <c r="BB2" s="64"/>
+      <c r="BC2" s="64"/>
+      <c r="BD2" s="64"/>
+      <c r="BE2" s="64"/>
+      <c r="BF2" s="64"/>
+    </row>
+    <row r="3" spans="1:59">
+      <c r="A3" s="68" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="68"/>
+      <c r="C3" s="65"/>
+      <c r="D3" s="3">
+        <v>1</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="F3" s="5"/>
+      <c r="G3" s="5"/>
+      <c r="H3" s="5"/>
+      <c r="I3" s="6"/>
+      <c r="J3" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="K3" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="L3" s="7"/>
+      <c r="M3" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="N3" s="7">
+        <v>1</v>
+      </c>
+      <c r="O3" s="7"/>
+      <c r="P3" s="7"/>
+      <c r="Q3" s="7"/>
+      <c r="R3" s="7"/>
+      <c r="S3" s="6"/>
+      <c r="T3" s="6"/>
+      <c r="U3" s="6"/>
+      <c r="V3" s="6"/>
+      <c r="W3" s="6"/>
+      <c r="X3" s="6"/>
+      <c r="Y3" s="6"/>
+      <c r="Z3" s="6"/>
+      <c r="AA3" s="6"/>
+      <c r="AB3" s="6"/>
+      <c r="AC3" s="6"/>
+      <c r="AD3" s="68" t="s">
+        <v>3</v>
+      </c>
+      <c r="AE3" s="68"/>
+      <c r="AF3" s="65"/>
+      <c r="AG3" s="3">
+        <v>2</v>
+      </c>
+      <c r="AH3" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="AI3" s="5"/>
+      <c r="AJ3" s="5"/>
+      <c r="AK3" s="5"/>
+      <c r="AL3" s="6"/>
+      <c r="AM3" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="AN3" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="AO3" s="7"/>
+      <c r="AP3" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="AQ3" s="7">
+        <v>1</v>
+      </c>
+      <c r="AR3" s="7"/>
+      <c r="AS3" s="7"/>
+      <c r="AT3" s="7"/>
+      <c r="AU3" s="7"/>
+      <c r="AV3" s="6"/>
+      <c r="AW3" s="6"/>
+      <c r="AX3" s="6"/>
+      <c r="AY3" s="6"/>
+      <c r="AZ3" s="6"/>
+      <c r="BA3" s="6"/>
+      <c r="BB3" s="6"/>
+      <c r="BC3" s="6"/>
+      <c r="BD3" s="6"/>
+      <c r="BE3" s="6"/>
+      <c r="BF3" s="6"/>
+    </row>
+    <row r="4" spans="1:59" ht="42.75">
+      <c r="A4" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="E4" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="F4" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="G4" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="H4" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="I4" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="J4" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="K4" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="L4" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="M4" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="N4" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="O4" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="P4" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q4" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="R4" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="S4" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="T4" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="U4" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="V4" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="W4" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="X4" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y4" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="Z4" s="16" t="s">
+        <v>30</v>
+      </c>
+      <c r="AA4" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="AB4" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="AC4" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="AD4" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="AE4" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="AF4" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="AG4" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="AH4" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="AI4" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="AJ4" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="AK4" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="AL4" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="AM4" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="AN4" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="AO4" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="AP4" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="AQ4" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="AR4" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="AS4" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="AT4" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="AU4" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="AV4" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="AW4" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="AX4" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="AY4" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="AZ4" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="BA4" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="BB4" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="BC4" s="16" t="s">
+        <v>30</v>
+      </c>
+      <c r="BD4" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="BE4" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="BF4" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="BG4" s="17" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="5" spans="1:59">
+      <c r="A5" s="9">
+        <v>1</v>
+      </c>
+      <c r="B5" s="27" t="s">
+        <v>41</v>
+      </c>
+      <c r="C5" s="9">
+        <v>0</v>
+      </c>
+      <c r="D5" s="27" t="s">
+        <v>42</v>
+      </c>
+      <c r="E5" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="F5" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="G5" s="24">
+        <v>1</v>
+      </c>
+      <c r="H5" s="9">
+        <v>2255</v>
+      </c>
+      <c r="I5" s="8">
+        <v>2255</v>
+      </c>
+      <c r="J5" s="25"/>
+      <c r="K5" s="25"/>
+      <c r="L5" s="25"/>
+      <c r="M5" s="8">
+        <v>2255</v>
+      </c>
+      <c r="N5" s="8">
+        <v>0</v>
+      </c>
+      <c r="O5" s="8">
+        <v>2255</v>
+      </c>
+      <c r="P5" s="8">
+        <v>0</v>
+      </c>
+      <c r="Q5" s="8">
+        <v>2255</v>
+      </c>
+      <c r="R5" s="8">
+        <v>0</v>
+      </c>
+      <c r="S5" s="26">
+        <v>0</v>
+      </c>
+      <c r="T5" s="26">
+        <v>0</v>
+      </c>
+      <c r="U5" s="8">
+        <f>(I5-S5)</f>
+        <v>2255</v>
+      </c>
+      <c r="V5" s="24">
+        <v>88363222</v>
+      </c>
+      <c r="W5" s="18">
+        <v>0.18</v>
+      </c>
+      <c r="X5" s="24">
+        <f>IF($D$3=1,ROUND(((U5*W5)/2),2),0)</f>
+        <v>202.95</v>
+      </c>
+      <c r="Y5" s="31">
+        <f>IF($D$3=1,ROUND(((U5*W5)/2),2),0)</f>
+        <v>202.95</v>
+      </c>
+      <c r="Z5" s="24">
+        <v>0</v>
+      </c>
+      <c r="AA5" s="24">
+        <v>0</v>
+      </c>
+      <c r="AB5" s="8">
+        <f>X5+Y5+Z5</f>
+        <v>405.9</v>
+      </c>
+      <c r="AC5" s="24">
+        <f>U5+AB5</f>
+        <v>2660.9</v>
+      </c>
+      <c r="AD5" s="9">
+        <v>1</v>
+      </c>
+      <c r="AE5" s="27" t="s">
+        <v>44</v>
+      </c>
+      <c r="AF5" s="9">
+        <v>0</v>
+      </c>
+      <c r="AG5" s="27" t="s">
+        <v>44</v>
+      </c>
+      <c r="AH5" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="AI5" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="AJ5" s="24">
+        <v>2</v>
+      </c>
+      <c r="AK5" s="9">
+        <v>250.25</v>
+      </c>
+      <c r="AL5" s="8">
+        <v>500.5</v>
+      </c>
+      <c r="AM5" s="25">
+        <v>2.21</v>
+      </c>
+      <c r="AN5" s="25">
+        <v>1.79</v>
+      </c>
+      <c r="AO5" s="25">
+        <v>2.5</v>
+      </c>
+      <c r="AP5" s="8">
+        <v>500.5</v>
+      </c>
+      <c r="AQ5" s="8">
+        <f>ROUND(AM5*AP5%,2)</f>
+        <v>11.06</v>
+      </c>
+      <c r="AR5" s="8">
+        <f>AL5-AQ5</f>
+        <v>489.44</v>
+      </c>
+      <c r="AS5" s="8">
+        <f>ROUND(AN5*AR5%,2)</f>
+        <v>8.76</v>
+      </c>
+      <c r="AT5" s="8">
+        <f>AR5-AS5</f>
+        <v>480.68</v>
+      </c>
+      <c r="AU5" s="40">
+        <f>ROUND(AO5*AT5%,2)</f>
+        <v>12.02</v>
+      </c>
+      <c r="AV5" s="26">
+        <f>AQ5+AS5+AU5</f>
+        <v>31.84</v>
+      </c>
+      <c r="AW5" s="26">
+        <v>0</v>
+      </c>
+      <c r="AX5" s="8">
+        <f>(AL5-AV5)</f>
+        <v>468.66</v>
+      </c>
+      <c r="AY5" s="24">
+        <v>88363222</v>
+      </c>
+      <c r="AZ5" s="18">
+        <v>0.18</v>
+      </c>
+      <c r="BA5" s="31">
+        <v>0</v>
+      </c>
+      <c r="BB5" s="31">
+        <v>0</v>
+      </c>
+      <c r="BC5" s="66">
+        <v>84.36</v>
+      </c>
+      <c r="BD5" s="24">
+        <v>0</v>
+      </c>
+      <c r="BE5" s="8">
+        <f>BA5+BB5+BC5</f>
+        <v>84.36</v>
+      </c>
+      <c r="BF5" s="24">
+        <f>AX5+BE5</f>
+        <v>553.02</v>
+      </c>
+      <c r="BG5" s="24">
+        <f>BF5-BE5</f>
+        <v>468.65999999999997</v>
+      </c>
+    </row>
+    <row r="6" spans="1:59">
+      <c r="A6" s="19"/>
+      <c r="B6" s="19"/>
+      <c r="C6" s="19"/>
+      <c r="D6" s="19"/>
+      <c r="E6" s="19"/>
+      <c r="F6" s="19"/>
+      <c r="G6" s="20"/>
+      <c r="H6" s="21"/>
+      <c r="I6" s="21"/>
+      <c r="J6" s="22"/>
+      <c r="K6" s="22"/>
+      <c r="L6" s="22"/>
+      <c r="M6" s="21"/>
+      <c r="N6" s="21"/>
+      <c r="O6" s="21"/>
+      <c r="P6" s="21"/>
+      <c r="Q6" s="21"/>
+      <c r="R6" s="21"/>
+      <c r="S6" s="21"/>
+      <c r="T6" s="21"/>
+      <c r="U6" s="21"/>
+      <c r="V6" s="21"/>
+      <c r="W6" s="22"/>
+      <c r="X6" s="21"/>
+      <c r="Y6" s="21"/>
+      <c r="Z6" s="21"/>
+      <c r="AA6" s="21"/>
+      <c r="AB6" s="21"/>
+      <c r="AC6" s="21"/>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A1:AC1"/>
+    <mergeCell ref="AD1:BF1"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="AD3:AE3"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -4134,68 +5160,68 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:58" ht="18">
-      <c r="A1" s="62" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="62"/>
-      <c r="C1" s="62"/>
-      <c r="D1" s="62"/>
-      <c r="E1" s="62"/>
-      <c r="F1" s="62"/>
-      <c r="G1" s="62"/>
-      <c r="H1" s="62"/>
-      <c r="I1" s="62"/>
-      <c r="J1" s="62"/>
-      <c r="K1" s="62"/>
-      <c r="L1" s="62"/>
-      <c r="M1" s="62"/>
-      <c r="N1" s="62"/>
-      <c r="O1" s="62"/>
-      <c r="P1" s="62"/>
-      <c r="Q1" s="62"/>
-      <c r="R1" s="62"/>
-      <c r="S1" s="62"/>
-      <c r="T1" s="62"/>
-      <c r="U1" s="62"/>
-      <c r="V1" s="62"/>
-      <c r="W1" s="62"/>
-      <c r="X1" s="62"/>
-      <c r="Y1" s="62"/>
-      <c r="Z1" s="62"/>
-      <c r="AA1" s="62"/>
-      <c r="AB1" s="62"/>
-      <c r="AC1" s="62"/>
-      <c r="AD1" s="62" t="s">
-        <v>0</v>
-      </c>
-      <c r="AE1" s="62"/>
-      <c r="AF1" s="62"/>
-      <c r="AG1" s="62"/>
-      <c r="AH1" s="62"/>
-      <c r="AI1" s="62"/>
-      <c r="AJ1" s="62"/>
-      <c r="AK1" s="62"/>
-      <c r="AL1" s="62"/>
-      <c r="AM1" s="62"/>
-      <c r="AN1" s="62"/>
-      <c r="AO1" s="62"/>
-      <c r="AP1" s="62"/>
-      <c r="AQ1" s="62"/>
-      <c r="AR1" s="62"/>
-      <c r="AS1" s="62"/>
-      <c r="AT1" s="62"/>
-      <c r="AU1" s="62"/>
-      <c r="AV1" s="62"/>
-      <c r="AW1" s="62"/>
-      <c r="AX1" s="62"/>
-      <c r="AY1" s="62"/>
-      <c r="AZ1" s="62"/>
-      <c r="BA1" s="62"/>
-      <c r="BB1" s="62"/>
-      <c r="BC1" s="62"/>
-      <c r="BD1" s="62"/>
-      <c r="BE1" s="62"/>
-      <c r="BF1" s="62"/>
+      <c r="A1" s="67" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="67"/>
+      <c r="C1" s="67"/>
+      <c r="D1" s="67"/>
+      <c r="E1" s="67"/>
+      <c r="F1" s="67"/>
+      <c r="G1" s="67"/>
+      <c r="H1" s="67"/>
+      <c r="I1" s="67"/>
+      <c r="J1" s="67"/>
+      <c r="K1" s="67"/>
+      <c r="L1" s="67"/>
+      <c r="M1" s="67"/>
+      <c r="N1" s="67"/>
+      <c r="O1" s="67"/>
+      <c r="P1" s="67"/>
+      <c r="Q1" s="67"/>
+      <c r="R1" s="67"/>
+      <c r="S1" s="67"/>
+      <c r="T1" s="67"/>
+      <c r="U1" s="67"/>
+      <c r="V1" s="67"/>
+      <c r="W1" s="67"/>
+      <c r="X1" s="67"/>
+      <c r="Y1" s="67"/>
+      <c r="Z1" s="67"/>
+      <c r="AA1" s="67"/>
+      <c r="AB1" s="67"/>
+      <c r="AC1" s="67"/>
+      <c r="AD1" s="67" t="s">
+        <v>0</v>
+      </c>
+      <c r="AE1" s="67"/>
+      <c r="AF1" s="67"/>
+      <c r="AG1" s="67"/>
+      <c r="AH1" s="67"/>
+      <c r="AI1" s="67"/>
+      <c r="AJ1" s="67"/>
+      <c r="AK1" s="67"/>
+      <c r="AL1" s="67"/>
+      <c r="AM1" s="67"/>
+      <c r="AN1" s="67"/>
+      <c r="AO1" s="67"/>
+      <c r="AP1" s="67"/>
+      <c r="AQ1" s="67"/>
+      <c r="AR1" s="67"/>
+      <c r="AS1" s="67"/>
+      <c r="AT1" s="67"/>
+      <c r="AU1" s="67"/>
+      <c r="AV1" s="67"/>
+      <c r="AW1" s="67"/>
+      <c r="AX1" s="67"/>
+      <c r="AY1" s="67"/>
+      <c r="AZ1" s="67"/>
+      <c r="BA1" s="67"/>
+      <c r="BB1" s="67"/>
+      <c r="BC1" s="67"/>
+      <c r="BD1" s="67"/>
+      <c r="BE1" s="67"/>
+      <c r="BF1" s="67"/>
     </row>
     <row r="2" spans="1:58" ht="18">
       <c r="A2" s="23" t="s">
@@ -4266,10 +5292,10 @@
       <c r="BF2" s="36"/>
     </row>
     <row r="3" spans="1:58">
-      <c r="A3" s="63" t="s">
+      <c r="A3" s="68" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="63"/>
+      <c r="B3" s="68"/>
       <c r="C3" s="29"/>
       <c r="D3" s="3">
         <v>2</v>
@@ -4309,10 +5335,10 @@
       <c r="AA3" s="6"/>
       <c r="AB3" s="6"/>
       <c r="AC3" s="6"/>
-      <c r="AD3" s="63" t="s">
+      <c r="AD3" s="68" t="s">
         <v>3</v>
       </c>
-      <c r="AE3" s="63"/>
+      <c r="AE3" s="68"/>
       <c r="AF3" s="37"/>
       <c r="AG3" s="3">
         <v>2</v>
@@ -4782,37 +5808,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="18">
-      <c r="A1" s="62" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="62"/>
-      <c r="C1" s="62"/>
-      <c r="D1" s="62"/>
-      <c r="E1" s="62"/>
-      <c r="F1" s="62"/>
-      <c r="G1" s="62"/>
-      <c r="H1" s="62"/>
-      <c r="I1" s="62"/>
-      <c r="J1" s="62"/>
-      <c r="K1" s="62"/>
-      <c r="L1" s="62"/>
-      <c r="M1" s="62"/>
-      <c r="N1" s="62"/>
-      <c r="O1" s="62"/>
-      <c r="P1" s="62"/>
-      <c r="Q1" s="62"/>
-      <c r="R1" s="62"/>
-      <c r="S1" s="62"/>
-      <c r="T1" s="62"/>
-      <c r="U1" s="62"/>
-      <c r="V1" s="62"/>
-      <c r="W1" s="62"/>
-      <c r="X1" s="62"/>
-      <c r="Y1" s="62"/>
-      <c r="Z1" s="62"/>
-      <c r="AA1" s="62"/>
-      <c r="AB1" s="62"/>
-      <c r="AC1" s="62"/>
+      <c r="A1" s="67" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="67"/>
+      <c r="C1" s="67"/>
+      <c r="D1" s="67"/>
+      <c r="E1" s="67"/>
+      <c r="F1" s="67"/>
+      <c r="G1" s="67"/>
+      <c r="H1" s="67"/>
+      <c r="I1" s="67"/>
+      <c r="J1" s="67"/>
+      <c r="K1" s="67"/>
+      <c r="L1" s="67"/>
+      <c r="M1" s="67"/>
+      <c r="N1" s="67"/>
+      <c r="O1" s="67"/>
+      <c r="P1" s="67"/>
+      <c r="Q1" s="67"/>
+      <c r="R1" s="67"/>
+      <c r="S1" s="67"/>
+      <c r="T1" s="67"/>
+      <c r="U1" s="67"/>
+      <c r="V1" s="67"/>
+      <c r="W1" s="67"/>
+      <c r="X1" s="67"/>
+      <c r="Y1" s="67"/>
+      <c r="Z1" s="67"/>
+      <c r="AA1" s="67"/>
+      <c r="AB1" s="67"/>
+      <c r="AC1" s="67"/>
     </row>
     <row r="2" spans="1:29" ht="18">
       <c r="A2" s="23" t="s">
@@ -4850,10 +5876,10 @@
       <c r="AC2" s="28"/>
     </row>
     <row r="3" spans="1:29">
-      <c r="A3" s="63" t="s">
+      <c r="A3" s="68" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="63"/>
+      <c r="B3" s="68"/>
       <c r="C3" s="29"/>
       <c r="D3" s="3">
         <v>4</v>
@@ -5136,37 +6162,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="18">
-      <c r="A1" s="62" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="62"/>
-      <c r="C1" s="62"/>
-      <c r="D1" s="62"/>
-      <c r="E1" s="62"/>
-      <c r="F1" s="62"/>
-      <c r="G1" s="62"/>
-      <c r="H1" s="62"/>
-      <c r="I1" s="62"/>
-      <c r="J1" s="62"/>
-      <c r="K1" s="62"/>
-      <c r="L1" s="62"/>
-      <c r="M1" s="62"/>
-      <c r="N1" s="62"/>
-      <c r="O1" s="62"/>
-      <c r="P1" s="62"/>
-      <c r="Q1" s="62"/>
-      <c r="R1" s="62"/>
-      <c r="S1" s="62"/>
-      <c r="T1" s="62"/>
-      <c r="U1" s="62"/>
-      <c r="V1" s="62"/>
-      <c r="W1" s="62"/>
-      <c r="X1" s="62"/>
-      <c r="Y1" s="62"/>
-      <c r="Z1" s="62"/>
-      <c r="AA1" s="62"/>
-      <c r="AB1" s="62"/>
-      <c r="AC1" s="62"/>
+      <c r="A1" s="67" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="67"/>
+      <c r="C1" s="67"/>
+      <c r="D1" s="67"/>
+      <c r="E1" s="67"/>
+      <c r="F1" s="67"/>
+      <c r="G1" s="67"/>
+      <c r="H1" s="67"/>
+      <c r="I1" s="67"/>
+      <c r="J1" s="67"/>
+      <c r="K1" s="67"/>
+      <c r="L1" s="67"/>
+      <c r="M1" s="67"/>
+      <c r="N1" s="67"/>
+      <c r="O1" s="67"/>
+      <c r="P1" s="67"/>
+      <c r="Q1" s="67"/>
+      <c r="R1" s="67"/>
+      <c r="S1" s="67"/>
+      <c r="T1" s="67"/>
+      <c r="U1" s="67"/>
+      <c r="V1" s="67"/>
+      <c r="W1" s="67"/>
+      <c r="X1" s="67"/>
+      <c r="Y1" s="67"/>
+      <c r="Z1" s="67"/>
+      <c r="AA1" s="67"/>
+      <c r="AB1" s="67"/>
+      <c r="AC1" s="67"/>
     </row>
     <row r="2" spans="1:29" ht="18">
       <c r="A2" s="23" t="s">
@@ -5204,10 +6230,10 @@
       <c r="AC2" s="28"/>
     </row>
     <row r="3" spans="1:29">
-      <c r="A3" s="63" t="s">
+      <c r="A3" s="68" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="63"/>
+      <c r="B3" s="68"/>
       <c r="C3" s="29"/>
       <c r="D3" s="3">
         <v>3</v>
@@ -5489,37 +6515,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="18">
-      <c r="A1" s="62" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="62"/>
-      <c r="C1" s="62"/>
-      <c r="D1" s="62"/>
-      <c r="E1" s="62"/>
-      <c r="F1" s="62"/>
-      <c r="G1" s="62"/>
-      <c r="H1" s="62"/>
-      <c r="I1" s="62"/>
-      <c r="J1" s="62"/>
-      <c r="K1" s="62"/>
-      <c r="L1" s="62"/>
-      <c r="M1" s="62"/>
-      <c r="N1" s="62"/>
-      <c r="O1" s="62"/>
-      <c r="P1" s="62"/>
-      <c r="Q1" s="62"/>
-      <c r="R1" s="62"/>
-      <c r="S1" s="62"/>
-      <c r="T1" s="62"/>
-      <c r="U1" s="62"/>
-      <c r="V1" s="62"/>
-      <c r="W1" s="62"/>
-      <c r="X1" s="62"/>
-      <c r="Y1" s="62"/>
-      <c r="Z1" s="62"/>
-      <c r="AA1" s="62"/>
-      <c r="AB1" s="62"/>
-      <c r="AC1" s="62"/>
+      <c r="A1" s="67" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="67"/>
+      <c r="C1" s="67"/>
+      <c r="D1" s="67"/>
+      <c r="E1" s="67"/>
+      <c r="F1" s="67"/>
+      <c r="G1" s="67"/>
+      <c r="H1" s="67"/>
+      <c r="I1" s="67"/>
+      <c r="J1" s="67"/>
+      <c r="K1" s="67"/>
+      <c r="L1" s="67"/>
+      <c r="M1" s="67"/>
+      <c r="N1" s="67"/>
+      <c r="O1" s="67"/>
+      <c r="P1" s="67"/>
+      <c r="Q1" s="67"/>
+      <c r="R1" s="67"/>
+      <c r="S1" s="67"/>
+      <c r="T1" s="67"/>
+      <c r="U1" s="67"/>
+      <c r="V1" s="67"/>
+      <c r="W1" s="67"/>
+      <c r="X1" s="67"/>
+      <c r="Y1" s="67"/>
+      <c r="Z1" s="67"/>
+      <c r="AA1" s="67"/>
+      <c r="AB1" s="67"/>
+      <c r="AC1" s="67"/>
     </row>
     <row r="2" spans="1:29" ht="18">
       <c r="A2" s="23" t="s">
@@ -5557,10 +6583,10 @@
       <c r="AC2" s="28"/>
     </row>
     <row r="3" spans="1:29">
-      <c r="A3" s="63" t="s">
+      <c r="A3" s="68" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="63"/>
+      <c r="B3" s="68"/>
       <c r="C3" s="29"/>
       <c r="D3" s="3">
         <v>5</v>
@@ -5844,37 +6870,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="18">
-      <c r="A1" s="62" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="62"/>
-      <c r="C1" s="62"/>
-      <c r="D1" s="62"/>
-      <c r="E1" s="62"/>
-      <c r="F1" s="62"/>
-      <c r="G1" s="62"/>
-      <c r="H1" s="62"/>
-      <c r="I1" s="62"/>
-      <c r="J1" s="62"/>
-      <c r="K1" s="62"/>
-      <c r="L1" s="62"/>
-      <c r="M1" s="62"/>
-      <c r="N1" s="62"/>
-      <c r="O1" s="62"/>
-      <c r="P1" s="62"/>
-      <c r="Q1" s="62"/>
-      <c r="R1" s="62"/>
-      <c r="S1" s="62"/>
-      <c r="T1" s="62"/>
-      <c r="U1" s="62"/>
-      <c r="V1" s="62"/>
-      <c r="W1" s="62"/>
-      <c r="X1" s="62"/>
-      <c r="Y1" s="62"/>
-      <c r="Z1" s="62"/>
-      <c r="AA1" s="62"/>
-      <c r="AB1" s="62"/>
-      <c r="AC1" s="62"/>
+      <c r="A1" s="67" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="67"/>
+      <c r="C1" s="67"/>
+      <c r="D1" s="67"/>
+      <c r="E1" s="67"/>
+      <c r="F1" s="67"/>
+      <c r="G1" s="67"/>
+      <c r="H1" s="67"/>
+      <c r="I1" s="67"/>
+      <c r="J1" s="67"/>
+      <c r="K1" s="67"/>
+      <c r="L1" s="67"/>
+      <c r="M1" s="67"/>
+      <c r="N1" s="67"/>
+      <c r="O1" s="67"/>
+      <c r="P1" s="67"/>
+      <c r="Q1" s="67"/>
+      <c r="R1" s="67"/>
+      <c r="S1" s="67"/>
+      <c r="T1" s="67"/>
+      <c r="U1" s="67"/>
+      <c r="V1" s="67"/>
+      <c r="W1" s="67"/>
+      <c r="X1" s="67"/>
+      <c r="Y1" s="67"/>
+      <c r="Z1" s="67"/>
+      <c r="AA1" s="67"/>
+      <c r="AB1" s="67"/>
+      <c r="AC1" s="67"/>
     </row>
     <row r="2" spans="1:29" ht="18">
       <c r="A2" s="23" t="s">
@@ -5912,10 +6938,10 @@
       <c r="AC2" s="32"/>
     </row>
     <row r="3" spans="1:29">
-      <c r="A3" s="63" t="s">
+      <c r="A3" s="68" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="63"/>
+      <c r="B3" s="68"/>
       <c r="C3" s="33"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -6197,37 +7223,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="18">
-      <c r="A1" s="62" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="62"/>
-      <c r="C1" s="62"/>
-      <c r="D1" s="62"/>
-      <c r="E1" s="62"/>
-      <c r="F1" s="62"/>
-      <c r="G1" s="62"/>
-      <c r="H1" s="62"/>
-      <c r="I1" s="62"/>
-      <c r="J1" s="62"/>
-      <c r="K1" s="62"/>
-      <c r="L1" s="62"/>
-      <c r="M1" s="62"/>
-      <c r="N1" s="62"/>
-      <c r="O1" s="62"/>
-      <c r="P1" s="62"/>
-      <c r="Q1" s="62"/>
-      <c r="R1" s="62"/>
-      <c r="S1" s="62"/>
-      <c r="T1" s="62"/>
-      <c r="U1" s="62"/>
-      <c r="V1" s="62"/>
-      <c r="W1" s="62"/>
-      <c r="X1" s="62"/>
-      <c r="Y1" s="62"/>
-      <c r="Z1" s="62"/>
-      <c r="AA1" s="62"/>
-      <c r="AB1" s="62"/>
-      <c r="AC1" s="62"/>
+      <c r="A1" s="67" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="67"/>
+      <c r="C1" s="67"/>
+      <c r="D1" s="67"/>
+      <c r="E1" s="67"/>
+      <c r="F1" s="67"/>
+      <c r="G1" s="67"/>
+      <c r="H1" s="67"/>
+      <c r="I1" s="67"/>
+      <c r="J1" s="67"/>
+      <c r="K1" s="67"/>
+      <c r="L1" s="67"/>
+      <c r="M1" s="67"/>
+      <c r="N1" s="67"/>
+      <c r="O1" s="67"/>
+      <c r="P1" s="67"/>
+      <c r="Q1" s="67"/>
+      <c r="R1" s="67"/>
+      <c r="S1" s="67"/>
+      <c r="T1" s="67"/>
+      <c r="U1" s="67"/>
+      <c r="V1" s="67"/>
+      <c r="W1" s="67"/>
+      <c r="X1" s="67"/>
+      <c r="Y1" s="67"/>
+      <c r="Z1" s="67"/>
+      <c r="AA1" s="67"/>
+      <c r="AB1" s="67"/>
+      <c r="AC1" s="67"/>
     </row>
     <row r="2" spans="1:29" ht="18">
       <c r="A2" s="23" t="s">
@@ -6265,10 +7291,10 @@
       <c r="AC2" s="34"/>
     </row>
     <row r="3" spans="1:29">
-      <c r="A3" s="63" t="s">
+      <c r="A3" s="68" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="63"/>
+      <c r="B3" s="68"/>
       <c r="C3" s="35"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -6548,37 +7574,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="18">
-      <c r="A1" s="62" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="62"/>
-      <c r="C1" s="62"/>
-      <c r="D1" s="62"/>
-      <c r="E1" s="62"/>
-      <c r="F1" s="62"/>
-      <c r="G1" s="62"/>
-      <c r="H1" s="62"/>
-      <c r="I1" s="62"/>
-      <c r="J1" s="62"/>
-      <c r="K1" s="62"/>
-      <c r="L1" s="62"/>
-      <c r="M1" s="62"/>
-      <c r="N1" s="62"/>
-      <c r="O1" s="62"/>
-      <c r="P1" s="62"/>
-      <c r="Q1" s="62"/>
-      <c r="R1" s="62"/>
-      <c r="S1" s="62"/>
-      <c r="T1" s="62"/>
-      <c r="U1" s="62"/>
-      <c r="V1" s="62"/>
-      <c r="W1" s="62"/>
-      <c r="X1" s="62"/>
-      <c r="Y1" s="62"/>
-      <c r="Z1" s="62"/>
-      <c r="AA1" s="62"/>
-      <c r="AB1" s="62"/>
-      <c r="AC1" s="62"/>
+      <c r="A1" s="67" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="67"/>
+      <c r="C1" s="67"/>
+      <c r="D1" s="67"/>
+      <c r="E1" s="67"/>
+      <c r="F1" s="67"/>
+      <c r="G1" s="67"/>
+      <c r="H1" s="67"/>
+      <c r="I1" s="67"/>
+      <c r="J1" s="67"/>
+      <c r="K1" s="67"/>
+      <c r="L1" s="67"/>
+      <c r="M1" s="67"/>
+      <c r="N1" s="67"/>
+      <c r="O1" s="67"/>
+      <c r="P1" s="67"/>
+      <c r="Q1" s="67"/>
+      <c r="R1" s="67"/>
+      <c r="S1" s="67"/>
+      <c r="T1" s="67"/>
+      <c r="U1" s="67"/>
+      <c r="V1" s="67"/>
+      <c r="W1" s="67"/>
+      <c r="X1" s="67"/>
+      <c r="Y1" s="67"/>
+      <c r="Z1" s="67"/>
+      <c r="AA1" s="67"/>
+      <c r="AB1" s="67"/>
+      <c r="AC1" s="67"/>
     </row>
     <row r="2" spans="1:29" ht="18">
       <c r="A2" s="23" t="s">
@@ -6616,10 +7642,10 @@
       <c r="AC2" s="36"/>
     </row>
     <row r="3" spans="1:29">
-      <c r="A3" s="63" t="s">
+      <c r="A3" s="68" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="63"/>
+      <c r="B3" s="68"/>
       <c r="C3" s="37"/>
       <c r="D3" s="3">
         <v>2</v>
@@ -6916,37 +7942,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:31" ht="18">
-      <c r="A1" s="62" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="62"/>
-      <c r="C1" s="62"/>
-      <c r="D1" s="62"/>
-      <c r="E1" s="62"/>
-      <c r="F1" s="62"/>
-      <c r="G1" s="62"/>
-      <c r="H1" s="62"/>
-      <c r="I1" s="62"/>
-      <c r="J1" s="62"/>
-      <c r="K1" s="62"/>
-      <c r="L1" s="62"/>
-      <c r="M1" s="62"/>
-      <c r="N1" s="62"/>
-      <c r="O1" s="62"/>
-      <c r="P1" s="62"/>
-      <c r="Q1" s="62"/>
-      <c r="R1" s="62"/>
-      <c r="S1" s="62"/>
-      <c r="T1" s="62"/>
-      <c r="U1" s="62"/>
-      <c r="V1" s="62"/>
-      <c r="W1" s="62"/>
-      <c r="X1" s="62"/>
-      <c r="Y1" s="62"/>
-      <c r="Z1" s="62"/>
-      <c r="AA1" s="62"/>
-      <c r="AB1" s="62"/>
-      <c r="AC1" s="62"/>
+      <c r="A1" s="67" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="67"/>
+      <c r="C1" s="67"/>
+      <c r="D1" s="67"/>
+      <c r="E1" s="67"/>
+      <c r="F1" s="67"/>
+      <c r="G1" s="67"/>
+      <c r="H1" s="67"/>
+      <c r="I1" s="67"/>
+      <c r="J1" s="67"/>
+      <c r="K1" s="67"/>
+      <c r="L1" s="67"/>
+      <c r="M1" s="67"/>
+      <c r="N1" s="67"/>
+      <c r="O1" s="67"/>
+      <c r="P1" s="67"/>
+      <c r="Q1" s="67"/>
+      <c r="R1" s="67"/>
+      <c r="S1" s="67"/>
+      <c r="T1" s="67"/>
+      <c r="U1" s="67"/>
+      <c r="V1" s="67"/>
+      <c r="W1" s="67"/>
+      <c r="X1" s="67"/>
+      <c r="Y1" s="67"/>
+      <c r="Z1" s="67"/>
+      <c r="AA1" s="67"/>
+      <c r="AB1" s="67"/>
+      <c r="AC1" s="67"/>
     </row>
     <row r="2" spans="1:31" ht="16.5" customHeight="1">
       <c r="A2" s="23" t="s">
@@ -6984,10 +8010,10 @@
       <c r="AC2" s="41"/>
     </row>
     <row r="3" spans="1:31">
-      <c r="A3" s="63" t="s">
+      <c r="A3" s="68" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="63"/>
+      <c r="B3" s="68"/>
       <c r="D3">
         <v>2</v>
       </c>

</xml_diff>

<commit_message>
Failure Fixes And Purchase Bills New Cases
Failure Fixes And Purchase Bills New Cases
</commit_message>
<xml_diff>
--- a/testdata/DBfin.xlsx
+++ b/testdata/DBfin.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4507"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="2520" windowWidth="16695" windowHeight="6540" tabRatio="594" firstSheet="12" activeTab="15"/>
+    <workbookView xWindow="0" yWindow="2520" windowWidth="16695" windowHeight="6540" tabRatio="594" firstSheet="13" activeTab="16"/>
   </bookViews>
   <sheets>
     <sheet name="PurchaseBillsLocal" sheetId="1" r:id="rId1"/>
@@ -23,13 +23,14 @@
     <sheet name="PurchaseBills_Un_Regrd_Iter" sheetId="14" r:id="rId14"/>
     <sheet name="Purchasebills_UTGST_2" sheetId="15" r:id="rId15"/>
     <sheet name="PurchaseBills_Rcm" sheetId="16" r:id="rId16"/>
+    <sheet name="Purchase_Bills_In_Updated_2" sheetId="17" r:id="rId17"/>
   </sheets>
   <calcPr calcId="125725"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="865" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="931" uniqueCount="62">
   <si>
     <t>Scenario  : Local Sales - Stock UOM and Sales UOM (Similar)   DOC NO :  SORD-2425-00089</t>
   </si>
@@ -366,7 +367,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="69">
+  <cellXfs count="71">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -516,6 +517,12 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -847,68 +854,68 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:59" ht="18">
-      <c r="A1" s="67" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="67"/>
-      <c r="C1" s="67"/>
-      <c r="D1" s="67"/>
-      <c r="E1" s="67"/>
-      <c r="F1" s="67"/>
-      <c r="G1" s="67"/>
-      <c r="H1" s="67"/>
-      <c r="I1" s="67"/>
-      <c r="J1" s="67"/>
-      <c r="K1" s="67"/>
-      <c r="L1" s="67"/>
-      <c r="M1" s="67"/>
-      <c r="N1" s="67"/>
-      <c r="O1" s="67"/>
-      <c r="P1" s="67"/>
-      <c r="Q1" s="67"/>
-      <c r="R1" s="67"/>
-      <c r="S1" s="67"/>
-      <c r="T1" s="67"/>
-      <c r="U1" s="67"/>
-      <c r="V1" s="67"/>
-      <c r="W1" s="67"/>
-      <c r="X1" s="67"/>
-      <c r="Y1" s="67"/>
-      <c r="Z1" s="67"/>
-      <c r="AA1" s="67"/>
-      <c r="AB1" s="67"/>
-      <c r="AC1" s="67"/>
-      <c r="AD1" s="67" t="s">
-        <v>0</v>
-      </c>
-      <c r="AE1" s="67"/>
-      <c r="AF1" s="67"/>
-      <c r="AG1" s="67"/>
-      <c r="AH1" s="67"/>
-      <c r="AI1" s="67"/>
-      <c r="AJ1" s="67"/>
-      <c r="AK1" s="67"/>
-      <c r="AL1" s="67"/>
-      <c r="AM1" s="67"/>
-      <c r="AN1" s="67"/>
-      <c r="AO1" s="67"/>
-      <c r="AP1" s="67"/>
-      <c r="AQ1" s="67"/>
-      <c r="AR1" s="67"/>
-      <c r="AS1" s="67"/>
-      <c r="AT1" s="67"/>
-      <c r="AU1" s="67"/>
-      <c r="AV1" s="67"/>
-      <c r="AW1" s="67"/>
-      <c r="AX1" s="67"/>
-      <c r="AY1" s="67"/>
-      <c r="AZ1" s="67"/>
-      <c r="BA1" s="67"/>
-      <c r="BB1" s="67"/>
-      <c r="BC1" s="67"/>
-      <c r="BD1" s="67"/>
-      <c r="BE1" s="67"/>
-      <c r="BF1" s="67"/>
+      <c r="A1" s="69" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="69"/>
+      <c r="C1" s="69"/>
+      <c r="D1" s="69"/>
+      <c r="E1" s="69"/>
+      <c r="F1" s="69"/>
+      <c r="G1" s="69"/>
+      <c r="H1" s="69"/>
+      <c r="I1" s="69"/>
+      <c r="J1" s="69"/>
+      <c r="K1" s="69"/>
+      <c r="L1" s="69"/>
+      <c r="M1" s="69"/>
+      <c r="N1" s="69"/>
+      <c r="O1" s="69"/>
+      <c r="P1" s="69"/>
+      <c r="Q1" s="69"/>
+      <c r="R1" s="69"/>
+      <c r="S1" s="69"/>
+      <c r="T1" s="69"/>
+      <c r="U1" s="69"/>
+      <c r="V1" s="69"/>
+      <c r="W1" s="69"/>
+      <c r="X1" s="69"/>
+      <c r="Y1" s="69"/>
+      <c r="Z1" s="69"/>
+      <c r="AA1" s="69"/>
+      <c r="AB1" s="69"/>
+      <c r="AC1" s="69"/>
+      <c r="AD1" s="69" t="s">
+        <v>0</v>
+      </c>
+      <c r="AE1" s="69"/>
+      <c r="AF1" s="69"/>
+      <c r="AG1" s="69"/>
+      <c r="AH1" s="69"/>
+      <c r="AI1" s="69"/>
+      <c r="AJ1" s="69"/>
+      <c r="AK1" s="69"/>
+      <c r="AL1" s="69"/>
+      <c r="AM1" s="69"/>
+      <c r="AN1" s="69"/>
+      <c r="AO1" s="69"/>
+      <c r="AP1" s="69"/>
+      <c r="AQ1" s="69"/>
+      <c r="AR1" s="69"/>
+      <c r="AS1" s="69"/>
+      <c r="AT1" s="69"/>
+      <c r="AU1" s="69"/>
+      <c r="AV1" s="69"/>
+      <c r="AW1" s="69"/>
+      <c r="AX1" s="69"/>
+      <c r="AY1" s="69"/>
+      <c r="AZ1" s="69"/>
+      <c r="BA1" s="69"/>
+      <c r="BB1" s="69"/>
+      <c r="BC1" s="69"/>
+      <c r="BD1" s="69"/>
+      <c r="BE1" s="69"/>
+      <c r="BF1" s="69"/>
     </row>
     <row r="2" spans="1:59" ht="18">
       <c r="A2" s="23" t="s">
@@ -979,10 +986,10 @@
       <c r="BF2" s="38"/>
     </row>
     <row r="3" spans="1:59">
-      <c r="A3" s="68" t="s">
+      <c r="A3" s="70" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="68"/>
+      <c r="B3" s="70"/>
       <c r="C3" s="2"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -1022,10 +1029,10 @@
       <c r="AA3" s="6"/>
       <c r="AB3" s="6"/>
       <c r="AC3" s="6"/>
-      <c r="AD3" s="68" t="s">
+      <c r="AD3" s="70" t="s">
         <v>3</v>
       </c>
-      <c r="AE3" s="68"/>
+      <c r="AE3" s="70"/>
       <c r="AF3" s="39"/>
       <c r="AG3" s="3">
         <v>1</v>
@@ -1502,38 +1509,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:33" ht="18">
-      <c r="A1" s="67" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="67"/>
-      <c r="C1" s="67"/>
-      <c r="D1" s="67"/>
-      <c r="E1" s="67"/>
-      <c r="F1" s="67"/>
-      <c r="G1" s="67"/>
-      <c r="H1" s="67"/>
-      <c r="I1" s="67"/>
-      <c r="J1" s="67"/>
-      <c r="K1" s="67"/>
-      <c r="L1" s="67"/>
-      <c r="M1" s="67"/>
-      <c r="N1" s="67"/>
-      <c r="O1" s="67"/>
-      <c r="P1" s="67"/>
-      <c r="Q1" s="67"/>
-      <c r="R1" s="67"/>
-      <c r="S1" s="67"/>
-      <c r="T1" s="67"/>
-      <c r="U1" s="67"/>
-      <c r="V1" s="67"/>
-      <c r="W1" s="67"/>
-      <c r="X1" s="67"/>
-      <c r="Y1" s="67"/>
-      <c r="Z1" s="67"/>
-      <c r="AA1" s="67"/>
-      <c r="AB1" s="67"/>
-      <c r="AC1" s="67"/>
-      <c r="AD1" s="67"/>
+      <c r="A1" s="69" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="69"/>
+      <c r="C1" s="69"/>
+      <c r="D1" s="69"/>
+      <c r="E1" s="69"/>
+      <c r="F1" s="69"/>
+      <c r="G1" s="69"/>
+      <c r="H1" s="69"/>
+      <c r="I1" s="69"/>
+      <c r="J1" s="69"/>
+      <c r="K1" s="69"/>
+      <c r="L1" s="69"/>
+      <c r="M1" s="69"/>
+      <c r="N1" s="69"/>
+      <c r="O1" s="69"/>
+      <c r="P1" s="69"/>
+      <c r="Q1" s="69"/>
+      <c r="R1" s="69"/>
+      <c r="S1" s="69"/>
+      <c r="T1" s="69"/>
+      <c r="U1" s="69"/>
+      <c r="V1" s="69"/>
+      <c r="W1" s="69"/>
+      <c r="X1" s="69"/>
+      <c r="Y1" s="69"/>
+      <c r="Z1" s="69"/>
+      <c r="AA1" s="69"/>
+      <c r="AB1" s="69"/>
+      <c r="AC1" s="69"/>
+      <c r="AD1" s="69"/>
     </row>
     <row r="2" spans="1:33" ht="18">
       <c r="A2" s="23" t="s">
@@ -1572,10 +1579,10 @@
       <c r="AD2" s="43"/>
     </row>
     <row r="3" spans="1:33" ht="15.75" thickBot="1">
-      <c r="A3" s="68" t="s">
+      <c r="A3" s="70" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="68"/>
+      <c r="B3" s="70"/>
       <c r="C3" s="44"/>
       <c r="D3" s="3">
         <v>2</v>
@@ -1801,7 +1808,7 @@
         <f>IF($D$3=1,ROUND(((V5*X5)/2),2),0)</f>
         <v>0</v>
       </c>
-      <c r="AA5" s="24">
+      <c r="AA5" s="8">
         <f>IF($D$3=2,ROUND(((V5*X5)),2),0)</f>
         <v>90.09</v>
       </c>
@@ -1812,7 +1819,7 @@
         <f>Y5+Z5+AA5</f>
         <v>90.09</v>
       </c>
-      <c r="AD5" s="24">
+      <c r="AD5" s="8">
         <f>V5+AC5</f>
         <v>590.59</v>
       </c>
@@ -1912,7 +1919,7 @@
         <f>IF($D$3=1,ROUND(((V6*X6)/2),2),0)</f>
         <v>0</v>
       </c>
-      <c r="AA6" s="24">
+      <c r="AA6" s="8">
         <f>IF($D$3=2,ROUND(((V6*X6)),2),0)</f>
         <v>622.44000000000005</v>
       </c>
@@ -1923,7 +1930,7 @@
         <f>Y6+Z6+AA6</f>
         <v>622.44000000000005</v>
       </c>
-      <c r="AD6" s="24">
+      <c r="AD6" s="8">
         <f>V6+AC6</f>
         <v>4080.44</v>
       </c>
@@ -2019,7 +2026,7 @@
         <f>IF($D$3=1,ROUND(((V7*X7)/2),2),0)</f>
         <v>0</v>
       </c>
-      <c r="AA7" s="24">
+      <c r="AA7" s="8">
         <f>IF($D$3=2,ROUND(((V7*X7)),2),0)</f>
         <v>109.62</v>
       </c>
@@ -2030,7 +2037,7 @@
         <f>Y7+Z7+AA7</f>
         <v>109.62</v>
       </c>
-      <c r="AD7" s="24">
+      <c r="AD7" s="8">
         <f>V7+AC7</f>
         <v>718.62</v>
       </c>
@@ -2130,7 +2137,7 @@
         <f>IF($D$3=1,ROUND(((V8*X8)/2),2),0)</f>
         <v>0</v>
       </c>
-      <c r="AA8" s="24">
+      <c r="AA8" s="8">
         <f>IF($D$3=2,ROUND(((V8*X8)),2),0)</f>
         <v>364.5</v>
       </c>
@@ -2141,7 +2148,7 @@
         <f>Y8+Z8+AA8</f>
         <v>364.5</v>
       </c>
-      <c r="AD8" s="24">
+      <c r="AD8" s="8">
         <f>V8+AC8</f>
         <v>2389.5</v>
       </c>
@@ -2189,37 +2196,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:31" ht="18">
-      <c r="A1" s="67" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="67"/>
-      <c r="C1" s="67"/>
-      <c r="D1" s="67"/>
-      <c r="E1" s="67"/>
-      <c r="F1" s="67"/>
-      <c r="G1" s="67"/>
-      <c r="H1" s="67"/>
-      <c r="I1" s="67"/>
-      <c r="J1" s="67"/>
-      <c r="K1" s="67"/>
-      <c r="L1" s="67"/>
-      <c r="M1" s="67"/>
-      <c r="N1" s="67"/>
-      <c r="O1" s="67"/>
-      <c r="P1" s="67"/>
-      <c r="Q1" s="67"/>
-      <c r="R1" s="67"/>
-      <c r="S1" s="67"/>
-      <c r="T1" s="67"/>
-      <c r="U1" s="67"/>
-      <c r="V1" s="67"/>
-      <c r="W1" s="67"/>
-      <c r="X1" s="67"/>
-      <c r="Y1" s="67"/>
-      <c r="Z1" s="67"/>
-      <c r="AA1" s="67"/>
-      <c r="AB1" s="67"/>
-      <c r="AC1" s="67"/>
+      <c r="A1" s="69" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="69"/>
+      <c r="C1" s="69"/>
+      <c r="D1" s="69"/>
+      <c r="E1" s="69"/>
+      <c r="F1" s="69"/>
+      <c r="G1" s="69"/>
+      <c r="H1" s="69"/>
+      <c r="I1" s="69"/>
+      <c r="J1" s="69"/>
+      <c r="K1" s="69"/>
+      <c r="L1" s="69"/>
+      <c r="M1" s="69"/>
+      <c r="N1" s="69"/>
+      <c r="O1" s="69"/>
+      <c r="P1" s="69"/>
+      <c r="Q1" s="69"/>
+      <c r="R1" s="69"/>
+      <c r="S1" s="69"/>
+      <c r="T1" s="69"/>
+      <c r="U1" s="69"/>
+      <c r="V1" s="69"/>
+      <c r="W1" s="69"/>
+      <c r="X1" s="69"/>
+      <c r="Y1" s="69"/>
+      <c r="Z1" s="69"/>
+      <c r="AA1" s="69"/>
+      <c r="AB1" s="69"/>
+      <c r="AC1" s="69"/>
     </row>
     <row r="2" spans="1:31" ht="16.5" customHeight="1">
       <c r="A2" s="23" t="s">
@@ -2257,10 +2264,10 @@
       <c r="AC2" s="54"/>
     </row>
     <row r="3" spans="1:31">
-      <c r="A3" s="68" t="s">
+      <c r="A3" s="70" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="68"/>
+      <c r="B3" s="70"/>
       <c r="D3">
         <v>2</v>
       </c>
@@ -2751,37 +2758,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="18">
-      <c r="A1" s="67" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="67"/>
-      <c r="C1" s="67"/>
-      <c r="D1" s="67"/>
-      <c r="E1" s="67"/>
-      <c r="F1" s="67"/>
-      <c r="G1" s="67"/>
-      <c r="H1" s="67"/>
-      <c r="I1" s="67"/>
-      <c r="J1" s="67"/>
-      <c r="K1" s="67"/>
-      <c r="L1" s="67"/>
-      <c r="M1" s="67"/>
-      <c r="N1" s="67"/>
-      <c r="O1" s="67"/>
-      <c r="P1" s="67"/>
-      <c r="Q1" s="67"/>
-      <c r="R1" s="67"/>
-      <c r="S1" s="67"/>
-      <c r="T1" s="67"/>
-      <c r="U1" s="67"/>
-      <c r="V1" s="67"/>
-      <c r="W1" s="67"/>
-      <c r="X1" s="67"/>
-      <c r="Y1" s="67"/>
-      <c r="Z1" s="67"/>
-      <c r="AA1" s="67"/>
-      <c r="AB1" s="67"/>
-      <c r="AC1" s="67"/>
+      <c r="A1" s="69" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="69"/>
+      <c r="C1" s="69"/>
+      <c r="D1" s="69"/>
+      <c r="E1" s="69"/>
+      <c r="F1" s="69"/>
+      <c r="G1" s="69"/>
+      <c r="H1" s="69"/>
+      <c r="I1" s="69"/>
+      <c r="J1" s="69"/>
+      <c r="K1" s="69"/>
+      <c r="L1" s="69"/>
+      <c r="M1" s="69"/>
+      <c r="N1" s="69"/>
+      <c r="O1" s="69"/>
+      <c r="P1" s="69"/>
+      <c r="Q1" s="69"/>
+      <c r="R1" s="69"/>
+      <c r="S1" s="69"/>
+      <c r="T1" s="69"/>
+      <c r="U1" s="69"/>
+      <c r="V1" s="69"/>
+      <c r="W1" s="69"/>
+      <c r="X1" s="69"/>
+      <c r="Y1" s="69"/>
+      <c r="Z1" s="69"/>
+      <c r="AA1" s="69"/>
+      <c r="AB1" s="69"/>
+      <c r="AC1" s="69"/>
     </row>
     <row r="2" spans="1:29" ht="18">
       <c r="A2" s="23" t="s">
@@ -2819,10 +2826,10 @@
       <c r="AC2" s="56"/>
     </row>
     <row r="3" spans="1:29">
-      <c r="A3" s="68" t="s">
+      <c r="A3" s="70" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="68"/>
+      <c r="B3" s="70"/>
       <c r="C3" s="57"/>
       <c r="D3" s="3">
         <v>2</v>
@@ -3103,37 +3110,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="18">
-      <c r="A1" s="67" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="67"/>
-      <c r="C1" s="67"/>
-      <c r="D1" s="67"/>
-      <c r="E1" s="67"/>
-      <c r="F1" s="67"/>
-      <c r="G1" s="67"/>
-      <c r="H1" s="67"/>
-      <c r="I1" s="67"/>
-      <c r="J1" s="67"/>
-      <c r="K1" s="67"/>
-      <c r="L1" s="67"/>
-      <c r="M1" s="67"/>
-      <c r="N1" s="67"/>
-      <c r="O1" s="67"/>
-      <c r="P1" s="67"/>
-      <c r="Q1" s="67"/>
-      <c r="R1" s="67"/>
-      <c r="S1" s="67"/>
-      <c r="T1" s="67"/>
-      <c r="U1" s="67"/>
-      <c r="V1" s="67"/>
-      <c r="W1" s="67"/>
-      <c r="X1" s="67"/>
-      <c r="Y1" s="67"/>
-      <c r="Z1" s="67"/>
-      <c r="AA1" s="67"/>
-      <c r="AB1" s="67"/>
-      <c r="AC1" s="67"/>
+      <c r="A1" s="69" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="69"/>
+      <c r="C1" s="69"/>
+      <c r="D1" s="69"/>
+      <c r="E1" s="69"/>
+      <c r="F1" s="69"/>
+      <c r="G1" s="69"/>
+      <c r="H1" s="69"/>
+      <c r="I1" s="69"/>
+      <c r="J1" s="69"/>
+      <c r="K1" s="69"/>
+      <c r="L1" s="69"/>
+      <c r="M1" s="69"/>
+      <c r="N1" s="69"/>
+      <c r="O1" s="69"/>
+      <c r="P1" s="69"/>
+      <c r="Q1" s="69"/>
+      <c r="R1" s="69"/>
+      <c r="S1" s="69"/>
+      <c r="T1" s="69"/>
+      <c r="U1" s="69"/>
+      <c r="V1" s="69"/>
+      <c r="W1" s="69"/>
+      <c r="X1" s="69"/>
+      <c r="Y1" s="69"/>
+      <c r="Z1" s="69"/>
+      <c r="AA1" s="69"/>
+      <c r="AB1" s="69"/>
+      <c r="AC1" s="69"/>
     </row>
     <row r="2" spans="1:29" ht="18">
       <c r="A2" s="23" t="s">
@@ -3171,10 +3178,10 @@
       <c r="AC2" s="58"/>
     </row>
     <row r="3" spans="1:29">
-      <c r="A3" s="68" t="s">
+      <c r="A3" s="70" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="68"/>
+      <c r="B3" s="70"/>
       <c r="C3" s="59"/>
       <c r="D3" s="3">
         <v>4</v>
@@ -3457,38 +3464,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:33" ht="18">
-      <c r="A1" s="67" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="67"/>
-      <c r="C1" s="67"/>
-      <c r="D1" s="67"/>
-      <c r="E1" s="67"/>
-      <c r="F1" s="67"/>
-      <c r="G1" s="67"/>
-      <c r="H1" s="67"/>
-      <c r="I1" s="67"/>
-      <c r="J1" s="67"/>
-      <c r="K1" s="67"/>
-      <c r="L1" s="67"/>
-      <c r="M1" s="67"/>
-      <c r="N1" s="67"/>
-      <c r="O1" s="67"/>
-      <c r="P1" s="67"/>
-      <c r="Q1" s="67"/>
-      <c r="R1" s="67"/>
-      <c r="S1" s="67"/>
-      <c r="T1" s="67"/>
-      <c r="U1" s="67"/>
-      <c r="V1" s="67"/>
-      <c r="W1" s="67"/>
-      <c r="X1" s="67"/>
-      <c r="Y1" s="67"/>
-      <c r="Z1" s="67"/>
-      <c r="AA1" s="67"/>
-      <c r="AB1" s="67"/>
-      <c r="AC1" s="67"/>
-      <c r="AD1" s="67"/>
+      <c r="A1" s="69" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="69"/>
+      <c r="C1" s="69"/>
+      <c r="D1" s="69"/>
+      <c r="E1" s="69"/>
+      <c r="F1" s="69"/>
+      <c r="G1" s="69"/>
+      <c r="H1" s="69"/>
+      <c r="I1" s="69"/>
+      <c r="J1" s="69"/>
+      <c r="K1" s="69"/>
+      <c r="L1" s="69"/>
+      <c r="M1" s="69"/>
+      <c r="N1" s="69"/>
+      <c r="O1" s="69"/>
+      <c r="P1" s="69"/>
+      <c r="Q1" s="69"/>
+      <c r="R1" s="69"/>
+      <c r="S1" s="69"/>
+      <c r="T1" s="69"/>
+      <c r="U1" s="69"/>
+      <c r="V1" s="69"/>
+      <c r="W1" s="69"/>
+      <c r="X1" s="69"/>
+      <c r="Y1" s="69"/>
+      <c r="Z1" s="69"/>
+      <c r="AA1" s="69"/>
+      <c r="AB1" s="69"/>
+      <c r="AC1" s="69"/>
+      <c r="AD1" s="69"/>
     </row>
     <row r="2" spans="1:33" ht="18">
       <c r="A2" s="23" t="s">
@@ -3527,10 +3534,10 @@
       <c r="AD2" s="60"/>
     </row>
     <row r="3" spans="1:33" ht="15.75" thickBot="1">
-      <c r="A3" s="68" t="s">
+      <c r="A3" s="70" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="68"/>
+      <c r="B3" s="70"/>
       <c r="C3" s="61"/>
       <c r="D3" s="3">
         <v>2</v>
@@ -4143,37 +4150,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="18">
-      <c r="A1" s="67" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="67"/>
-      <c r="C1" s="67"/>
-      <c r="D1" s="67"/>
-      <c r="E1" s="67"/>
-      <c r="F1" s="67"/>
-      <c r="G1" s="67"/>
-      <c r="H1" s="67"/>
-      <c r="I1" s="67"/>
-      <c r="J1" s="67"/>
-      <c r="K1" s="67"/>
-      <c r="L1" s="67"/>
-      <c r="M1" s="67"/>
-      <c r="N1" s="67"/>
-      <c r="O1" s="67"/>
-      <c r="P1" s="67"/>
-      <c r="Q1" s="67"/>
-      <c r="R1" s="67"/>
-      <c r="S1" s="67"/>
-      <c r="T1" s="67"/>
-      <c r="U1" s="67"/>
-      <c r="V1" s="67"/>
-      <c r="W1" s="67"/>
-      <c r="X1" s="67"/>
-      <c r="Y1" s="67"/>
-      <c r="Z1" s="67"/>
-      <c r="AA1" s="67"/>
-      <c r="AB1" s="67"/>
-      <c r="AC1" s="67"/>
+      <c r="A1" s="69" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="69"/>
+      <c r="C1" s="69"/>
+      <c r="D1" s="69"/>
+      <c r="E1" s="69"/>
+      <c r="F1" s="69"/>
+      <c r="G1" s="69"/>
+      <c r="H1" s="69"/>
+      <c r="I1" s="69"/>
+      <c r="J1" s="69"/>
+      <c r="K1" s="69"/>
+      <c r="L1" s="69"/>
+      <c r="M1" s="69"/>
+      <c r="N1" s="69"/>
+      <c r="O1" s="69"/>
+      <c r="P1" s="69"/>
+      <c r="Q1" s="69"/>
+      <c r="R1" s="69"/>
+      <c r="S1" s="69"/>
+      <c r="T1" s="69"/>
+      <c r="U1" s="69"/>
+      <c r="V1" s="69"/>
+      <c r="W1" s="69"/>
+      <c r="X1" s="69"/>
+      <c r="Y1" s="69"/>
+      <c r="Z1" s="69"/>
+      <c r="AA1" s="69"/>
+      <c r="AB1" s="69"/>
+      <c r="AC1" s="69"/>
     </row>
     <row r="2" spans="1:29" ht="18">
       <c r="A2" s="23" t="s">
@@ -4211,10 +4218,10 @@
       <c r="AC2" s="62"/>
     </row>
     <row r="3" spans="1:29">
-      <c r="A3" s="68" t="s">
+      <c r="A3" s="70" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="68"/>
+      <c r="B3" s="70"/>
       <c r="C3" s="63"/>
       <c r="D3" s="3">
         <v>4</v>
@@ -4503,68 +4510,68 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:59" ht="18">
-      <c r="A1" s="67" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="67"/>
-      <c r="C1" s="67"/>
-      <c r="D1" s="67"/>
-      <c r="E1" s="67"/>
-      <c r="F1" s="67"/>
-      <c r="G1" s="67"/>
-      <c r="H1" s="67"/>
-      <c r="I1" s="67"/>
-      <c r="J1" s="67"/>
-      <c r="K1" s="67"/>
-      <c r="L1" s="67"/>
-      <c r="M1" s="67"/>
-      <c r="N1" s="67"/>
-      <c r="O1" s="67"/>
-      <c r="P1" s="67"/>
-      <c r="Q1" s="67"/>
-      <c r="R1" s="67"/>
-      <c r="S1" s="67"/>
-      <c r="T1" s="67"/>
-      <c r="U1" s="67"/>
-      <c r="V1" s="67"/>
-      <c r="W1" s="67"/>
-      <c r="X1" s="67"/>
-      <c r="Y1" s="67"/>
-      <c r="Z1" s="67"/>
-      <c r="AA1" s="67"/>
-      <c r="AB1" s="67"/>
-      <c r="AC1" s="67"/>
-      <c r="AD1" s="67" t="s">
-        <v>0</v>
-      </c>
-      <c r="AE1" s="67"/>
-      <c r="AF1" s="67"/>
-      <c r="AG1" s="67"/>
-      <c r="AH1" s="67"/>
-      <c r="AI1" s="67"/>
-      <c r="AJ1" s="67"/>
-      <c r="AK1" s="67"/>
-      <c r="AL1" s="67"/>
-      <c r="AM1" s="67"/>
-      <c r="AN1" s="67"/>
-      <c r="AO1" s="67"/>
-      <c r="AP1" s="67"/>
-      <c r="AQ1" s="67"/>
-      <c r="AR1" s="67"/>
-      <c r="AS1" s="67"/>
-      <c r="AT1" s="67"/>
-      <c r="AU1" s="67"/>
-      <c r="AV1" s="67"/>
-      <c r="AW1" s="67"/>
-      <c r="AX1" s="67"/>
-      <c r="AY1" s="67"/>
-      <c r="AZ1" s="67"/>
-      <c r="BA1" s="67"/>
-      <c r="BB1" s="67"/>
-      <c r="BC1" s="67"/>
-      <c r="BD1" s="67"/>
-      <c r="BE1" s="67"/>
-      <c r="BF1" s="67"/>
+      <c r="A1" s="69" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="69"/>
+      <c r="C1" s="69"/>
+      <c r="D1" s="69"/>
+      <c r="E1" s="69"/>
+      <c r="F1" s="69"/>
+      <c r="G1" s="69"/>
+      <c r="H1" s="69"/>
+      <c r="I1" s="69"/>
+      <c r="J1" s="69"/>
+      <c r="K1" s="69"/>
+      <c r="L1" s="69"/>
+      <c r="M1" s="69"/>
+      <c r="N1" s="69"/>
+      <c r="O1" s="69"/>
+      <c r="P1" s="69"/>
+      <c r="Q1" s="69"/>
+      <c r="R1" s="69"/>
+      <c r="S1" s="69"/>
+      <c r="T1" s="69"/>
+      <c r="U1" s="69"/>
+      <c r="V1" s="69"/>
+      <c r="W1" s="69"/>
+      <c r="X1" s="69"/>
+      <c r="Y1" s="69"/>
+      <c r="Z1" s="69"/>
+      <c r="AA1" s="69"/>
+      <c r="AB1" s="69"/>
+      <c r="AC1" s="69"/>
+      <c r="AD1" s="69" t="s">
+        <v>0</v>
+      </c>
+      <c r="AE1" s="69"/>
+      <c r="AF1" s="69"/>
+      <c r="AG1" s="69"/>
+      <c r="AH1" s="69"/>
+      <c r="AI1" s="69"/>
+      <c r="AJ1" s="69"/>
+      <c r="AK1" s="69"/>
+      <c r="AL1" s="69"/>
+      <c r="AM1" s="69"/>
+      <c r="AN1" s="69"/>
+      <c r="AO1" s="69"/>
+      <c r="AP1" s="69"/>
+      <c r="AQ1" s="69"/>
+      <c r="AR1" s="69"/>
+      <c r="AS1" s="69"/>
+      <c r="AT1" s="69"/>
+      <c r="AU1" s="69"/>
+      <c r="AV1" s="69"/>
+      <c r="AW1" s="69"/>
+      <c r="AX1" s="69"/>
+      <c r="AY1" s="69"/>
+      <c r="AZ1" s="69"/>
+      <c r="BA1" s="69"/>
+      <c r="BB1" s="69"/>
+      <c r="BC1" s="69"/>
+      <c r="BD1" s="69"/>
+      <c r="BE1" s="69"/>
+      <c r="BF1" s="69"/>
     </row>
     <row r="2" spans="1:59" ht="18">
       <c r="A2" s="23" t="s">
@@ -4635,10 +4642,10 @@
       <c r="BF2" s="64"/>
     </row>
     <row r="3" spans="1:59">
-      <c r="A3" s="68" t="s">
+      <c r="A3" s="70" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="68"/>
+      <c r="B3" s="70"/>
       <c r="C3" s="65"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -4678,10 +4685,10 @@
       <c r="AA3" s="6"/>
       <c r="AB3" s="6"/>
       <c r="AC3" s="6"/>
-      <c r="AD3" s="68" t="s">
+      <c r="AD3" s="70" t="s">
         <v>3</v>
       </c>
-      <c r="AE3" s="68"/>
+      <c r="AE3" s="70"/>
       <c r="AF3" s="65"/>
       <c r="AG3" s="3">
         <v>2</v>
@@ -5129,6 +5136,674 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:AF8"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="2" max="2" width="20.5703125" customWidth="1"/>
+    <col min="4" max="4" width="29.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="29.140625" customWidth="1"/>
+    <col min="6" max="6" width="19.28515625" customWidth="1"/>
+    <col min="7" max="7" width="16.28515625" customWidth="1"/>
+    <col min="8" max="8" width="24.42578125" customWidth="1"/>
+    <col min="9" max="9" width="20.28515625" customWidth="1"/>
+    <col min="10" max="10" width="20" customWidth="1"/>
+    <col min="14" max="14" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="13.7109375" customWidth="1"/>
+    <col min="19" max="19" width="13" customWidth="1"/>
+    <col min="20" max="20" width="14.42578125" customWidth="1"/>
+    <col min="21" max="21" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="13.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:32" ht="18">
+      <c r="A1" s="69" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="69"/>
+      <c r="C1" s="69"/>
+      <c r="D1" s="69"/>
+      <c r="E1" s="69"/>
+      <c r="F1" s="69"/>
+      <c r="G1" s="69"/>
+      <c r="H1" s="69"/>
+      <c r="I1" s="69"/>
+      <c r="J1" s="69"/>
+      <c r="K1" s="69"/>
+      <c r="L1" s="69"/>
+      <c r="M1" s="69"/>
+      <c r="N1" s="69"/>
+      <c r="O1" s="69"/>
+      <c r="P1" s="69"/>
+      <c r="Q1" s="69"/>
+      <c r="R1" s="69"/>
+      <c r="S1" s="69"/>
+      <c r="T1" s="69"/>
+      <c r="U1" s="69"/>
+      <c r="V1" s="69"/>
+      <c r="W1" s="69"/>
+      <c r="X1" s="69"/>
+      <c r="Y1" s="69"/>
+      <c r="Z1" s="69"/>
+      <c r="AA1" s="69"/>
+      <c r="AB1" s="69"/>
+      <c r="AC1" s="69"/>
+    </row>
+    <row r="2" spans="1:32" ht="18">
+      <c r="A2" s="23" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="23" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" s="67"/>
+      <c r="D2" s="67"/>
+      <c r="E2" s="67"/>
+      <c r="F2" s="67"/>
+      <c r="G2" s="67"/>
+      <c r="H2" s="67"/>
+      <c r="I2" s="67"/>
+      <c r="J2" s="67"/>
+      <c r="K2" s="67"/>
+      <c r="L2" s="67"/>
+      <c r="M2" s="67"/>
+      <c r="N2" s="67"/>
+      <c r="O2" s="67"/>
+      <c r="P2" s="67"/>
+      <c r="Q2" s="67"/>
+      <c r="R2" s="67"/>
+      <c r="S2" s="67"/>
+      <c r="T2" s="67"/>
+      <c r="U2" s="67"/>
+      <c r="V2" s="67"/>
+      <c r="W2" s="67"/>
+      <c r="X2" s="67"/>
+      <c r="Y2" s="67"/>
+      <c r="Z2" s="67"/>
+      <c r="AA2" s="67"/>
+      <c r="AB2" s="67"/>
+      <c r="AC2" s="67"/>
+    </row>
+    <row r="3" spans="1:32" ht="15.75" thickBot="1">
+      <c r="A3" s="70" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="70"/>
+      <c r="C3" s="68"/>
+      <c r="D3" s="3">
+        <v>2</v>
+      </c>
+      <c r="E3" s="3"/>
+      <c r="F3" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="G3" s="5"/>
+      <c r="H3" s="5"/>
+      <c r="I3" s="5"/>
+      <c r="J3" s="6"/>
+      <c r="K3" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="L3" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="M3" s="7"/>
+      <c r="N3" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="O3" s="7">
+        <v>1</v>
+      </c>
+      <c r="P3" s="7"/>
+      <c r="Q3" s="7"/>
+      <c r="R3" s="7"/>
+      <c r="S3" s="7"/>
+      <c r="T3" s="6"/>
+      <c r="U3" s="6"/>
+      <c r="V3" s="6"/>
+      <c r="W3" s="6"/>
+      <c r="X3" s="6"/>
+      <c r="Y3" s="6"/>
+      <c r="Z3" s="6"/>
+      <c r="AA3" s="6"/>
+      <c r="AB3" s="6"/>
+      <c r="AC3" s="6"/>
+    </row>
+    <row r="4" spans="1:32" ht="43.5" thickTop="1">
+      <c r="A4" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="E4" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="F4" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="G4" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="H4" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="I4" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="J4" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="K4" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="L4" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="M4" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="N4" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="O4" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="P4" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="Q4" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="R4" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="S4" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="T4" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="U4" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="V4" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="W4" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="X4" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y4" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="Z4" s="16" t="s">
+        <v>30</v>
+      </c>
+      <c r="AA4" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="AB4" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="AC4" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="AD4" s="51" t="s">
+        <v>58</v>
+      </c>
+      <c r="AE4" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="AF4" s="10" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="5" spans="1:32">
+      <c r="A5" s="9">
+        <v>1</v>
+      </c>
+      <c r="B5" s="27" t="s">
+        <v>44</v>
+      </c>
+      <c r="C5" s="9">
+        <v>0</v>
+      </c>
+      <c r="D5" s="27" t="s">
+        <v>44</v>
+      </c>
+      <c r="E5" s="27"/>
+      <c r="F5" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="G5" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="H5" s="24">
+        <v>2</v>
+      </c>
+      <c r="I5" s="9">
+        <v>250.25</v>
+      </c>
+      <c r="J5" s="8">
+        <v>500.5</v>
+      </c>
+      <c r="K5" s="25">
+        <v>0</v>
+      </c>
+      <c r="L5" s="25">
+        <v>0</v>
+      </c>
+      <c r="M5" s="25">
+        <v>0</v>
+      </c>
+      <c r="N5" s="8">
+        <v>500.5</v>
+      </c>
+      <c r="O5" s="8">
+        <f>ROUND(K5*N5%,2)</f>
+        <v>0</v>
+      </c>
+      <c r="P5" s="8"/>
+      <c r="Q5" s="8">
+        <f>ROUND(L5*P5%,2)</f>
+        <v>0</v>
+      </c>
+      <c r="R5" s="8">
+        <f>P5-Q5</f>
+        <v>0</v>
+      </c>
+      <c r="S5" s="8">
+        <f>ROUND(M5*R5%,2)</f>
+        <v>0</v>
+      </c>
+      <c r="T5" s="26">
+        <f>O5+Q5+S5</f>
+        <v>0</v>
+      </c>
+      <c r="U5" s="8">
+        <f>(J5-T5)</f>
+        <v>500.5</v>
+      </c>
+      <c r="V5" s="24">
+        <v>88363222</v>
+      </c>
+      <c r="W5" s="18">
+        <v>0.18</v>
+      </c>
+      <c r="X5" s="24">
+        <f>IF($D$3=1,ROUND(((U5*W5)/2),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="Y5" s="24">
+        <f>IF($D$3=1,ROUND(((U5*W5)/2),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="Z5" s="8">
+        <f>IF($D$3=2,ROUND(((U5*W5)),2),0)</f>
+        <v>90.09</v>
+      </c>
+      <c r="AA5" s="24">
+        <v>0</v>
+      </c>
+      <c r="AB5" s="24">
+        <f>X5+Y5+Z5</f>
+        <v>90.09</v>
+      </c>
+      <c r="AC5" s="8">
+        <f>U5+AB5</f>
+        <v>590.59</v>
+      </c>
+      <c r="AD5" s="52" t="s">
+        <v>57</v>
+      </c>
+      <c r="AE5" s="46" t="s">
+        <v>42</v>
+      </c>
+      <c r="AF5" s="46" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="6" spans="1:32" ht="16.5" customHeight="1">
+      <c r="A6" s="9">
+        <v>2</v>
+      </c>
+      <c r="B6" s="45" t="s">
+        <v>51</v>
+      </c>
+      <c r="C6" s="9">
+        <v>0</v>
+      </c>
+      <c r="D6" s="45" t="s">
+        <v>50</v>
+      </c>
+      <c r="E6" s="45"/>
+      <c r="F6" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="G6" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="H6" s="24">
+        <v>1</v>
+      </c>
+      <c r="I6" s="9">
+        <v>3458</v>
+      </c>
+      <c r="J6" s="8">
+        <v>3458</v>
+      </c>
+      <c r="K6" s="25">
+        <v>0</v>
+      </c>
+      <c r="L6" s="25">
+        <v>0</v>
+      </c>
+      <c r="M6" s="25">
+        <v>0</v>
+      </c>
+      <c r="N6" s="8">
+        <v>3458</v>
+      </c>
+      <c r="O6" s="8">
+        <f t="shared" ref="O6:O8" si="0">ROUND(K6*N6%,2)</f>
+        <v>0</v>
+      </c>
+      <c r="P6" s="8">
+        <f t="shared" ref="P6:P8" si="1">J6-O6</f>
+        <v>3458</v>
+      </c>
+      <c r="Q6" s="8">
+        <f t="shared" ref="Q6:Q8" si="2">ROUND(L6*P6%,2)</f>
+        <v>0</v>
+      </c>
+      <c r="R6" s="8">
+        <f t="shared" ref="R6:R8" si="3">P6-Q6</f>
+        <v>3458</v>
+      </c>
+      <c r="S6" s="8">
+        <f t="shared" ref="S6:S8" si="4">ROUND(M6*R6%,2)</f>
+        <v>0</v>
+      </c>
+      <c r="T6" s="26">
+        <f t="shared" ref="T6:T8" si="5">O6+Q6+S6</f>
+        <v>0</v>
+      </c>
+      <c r="U6" s="8">
+        <f>(J6-T6)</f>
+        <v>3458</v>
+      </c>
+      <c r="V6" s="24">
+        <v>88363222</v>
+      </c>
+      <c r="W6" s="18">
+        <v>0.18</v>
+      </c>
+      <c r="X6" s="24">
+        <f>IF($D$3=1,ROUND(((U6*W6)/2),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="Y6" s="24">
+        <f>IF($D$3=1,ROUND(((U6*W6)/2),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="Z6" s="8">
+        <f>IF($D$3=2,ROUND(((U6*W6)),2),0)</f>
+        <v>622.44000000000005</v>
+      </c>
+      <c r="AA6" s="24">
+        <v>0</v>
+      </c>
+      <c r="AB6" s="24">
+        <f>X6+Y6+Z6</f>
+        <v>622.44000000000005</v>
+      </c>
+      <c r="AC6" s="8">
+        <f>U6+AB6</f>
+        <v>4080.44</v>
+      </c>
+      <c r="AD6" s="53" t="s">
+        <v>57</v>
+      </c>
+      <c r="AE6" s="46" t="s">
+        <v>53</v>
+      </c>
+      <c r="AF6" s="46" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="7" spans="1:32">
+      <c r="A7" s="46">
+        <v>4</v>
+      </c>
+      <c r="B7" s="46"/>
+      <c r="C7" s="46"/>
+      <c r="D7" s="46"/>
+      <c r="E7" s="46" t="s">
+        <v>56</v>
+      </c>
+      <c r="F7" s="47" t="s">
+        <v>33</v>
+      </c>
+      <c r="G7" s="47" t="s">
+        <v>33</v>
+      </c>
+      <c r="H7" s="48">
+        <v>1</v>
+      </c>
+      <c r="I7" s="47">
+        <v>609</v>
+      </c>
+      <c r="J7" s="49">
+        <v>609</v>
+      </c>
+      <c r="K7" s="46">
+        <v>0</v>
+      </c>
+      <c r="L7" s="46">
+        <v>0</v>
+      </c>
+      <c r="M7" s="46">
+        <v>0</v>
+      </c>
+      <c r="N7" s="50">
+        <v>609</v>
+      </c>
+      <c r="O7" s="8">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="P7" s="8">
+        <f t="shared" si="1"/>
+        <v>609</v>
+      </c>
+      <c r="Q7" s="8">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="R7" s="8">
+        <f t="shared" si="3"/>
+        <v>609</v>
+      </c>
+      <c r="S7" s="8">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="T7" s="26">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="U7" s="8">
+        <f>(J7-T7)</f>
+        <v>609</v>
+      </c>
+      <c r="V7" s="24">
+        <v>75052200</v>
+      </c>
+      <c r="W7" s="18">
+        <v>0.18</v>
+      </c>
+      <c r="X7" s="24">
+        <f>IF($D$3=1,ROUND(((U7*W7)/2),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="Y7" s="24">
+        <f>IF($D$3=1,ROUND(((U7*W7)/2),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="Z7" s="8">
+        <f>IF($D$3=2,ROUND(((U7*W7)),2),0)</f>
+        <v>109.62</v>
+      </c>
+      <c r="AA7" s="24">
+        <v>0</v>
+      </c>
+      <c r="AB7" s="24">
+        <f>X7+Y7+Z7</f>
+        <v>109.62</v>
+      </c>
+      <c r="AC7" s="8">
+        <f>U7+AB7</f>
+        <v>718.62</v>
+      </c>
+      <c r="AD7" s="52" t="s">
+        <v>59</v>
+      </c>
+      <c r="AE7" s="46">
+        <v>5050121000</v>
+      </c>
+      <c r="AF7" s="46" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="8" spans="1:32">
+      <c r="A8" s="9">
+        <v>3</v>
+      </c>
+      <c r="B8" s="27" t="s">
+        <v>52</v>
+      </c>
+      <c r="C8" s="9">
+        <v>0</v>
+      </c>
+      <c r="D8" s="27" t="s">
+        <v>52</v>
+      </c>
+      <c r="E8" s="27"/>
+      <c r="F8" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="G8" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="H8" s="24">
+        <v>3</v>
+      </c>
+      <c r="I8" s="9">
+        <v>675</v>
+      </c>
+      <c r="J8" s="8">
+        <v>2025</v>
+      </c>
+      <c r="K8" s="25">
+        <v>0</v>
+      </c>
+      <c r="L8" s="25">
+        <v>0</v>
+      </c>
+      <c r="M8" s="25">
+        <v>0</v>
+      </c>
+      <c r="N8" s="8">
+        <v>2025</v>
+      </c>
+      <c r="O8" s="8">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="P8" s="8">
+        <f t="shared" si="1"/>
+        <v>2025</v>
+      </c>
+      <c r="Q8" s="8">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="R8" s="8">
+        <f t="shared" si="3"/>
+        <v>2025</v>
+      </c>
+      <c r="S8" s="8">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="T8" s="26">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="U8" s="8">
+        <f>(J8-T8)</f>
+        <v>2025</v>
+      </c>
+      <c r="V8" s="24">
+        <v>88363222</v>
+      </c>
+      <c r="W8" s="18">
+        <v>0.18</v>
+      </c>
+      <c r="X8" s="24">
+        <f>IF($D$3=1,ROUND(((U8*W8)/2),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="Y8" s="24">
+        <f>IF($D$3=1,ROUND(((U8*W8)/2),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="Z8" s="55">
+        <f>IF($D$3=2,ROUND(((U8*W8)),2),0)</f>
+        <v>364.5</v>
+      </c>
+      <c r="AA8" s="24">
+        <v>0</v>
+      </c>
+      <c r="AB8" s="24">
+        <f>X8+Y8+Z8</f>
+        <v>364.5</v>
+      </c>
+      <c r="AC8" s="8">
+        <f>U8+AB8</f>
+        <v>2389.5</v>
+      </c>
+      <c r="AD8" s="53" t="s">
+        <v>57</v>
+      </c>
+      <c r="AE8" s="46" t="s">
+        <v>54</v>
+      </c>
+      <c r="AF8" s="46" t="s">
+        <v>61</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:AC1"/>
+    <mergeCell ref="A3:B3"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -5160,68 +5835,68 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:58" ht="18">
-      <c r="A1" s="67" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="67"/>
-      <c r="C1" s="67"/>
-      <c r="D1" s="67"/>
-      <c r="E1" s="67"/>
-      <c r="F1" s="67"/>
-      <c r="G1" s="67"/>
-      <c r="H1" s="67"/>
-      <c r="I1" s="67"/>
-      <c r="J1" s="67"/>
-      <c r="K1" s="67"/>
-      <c r="L1" s="67"/>
-      <c r="M1" s="67"/>
-      <c r="N1" s="67"/>
-      <c r="O1" s="67"/>
-      <c r="P1" s="67"/>
-      <c r="Q1" s="67"/>
-      <c r="R1" s="67"/>
-      <c r="S1" s="67"/>
-      <c r="T1" s="67"/>
-      <c r="U1" s="67"/>
-      <c r="V1" s="67"/>
-      <c r="W1" s="67"/>
-      <c r="X1" s="67"/>
-      <c r="Y1" s="67"/>
-      <c r="Z1" s="67"/>
-      <c r="AA1" s="67"/>
-      <c r="AB1" s="67"/>
-      <c r="AC1" s="67"/>
-      <c r="AD1" s="67" t="s">
-        <v>0</v>
-      </c>
-      <c r="AE1" s="67"/>
-      <c r="AF1" s="67"/>
-      <c r="AG1" s="67"/>
-      <c r="AH1" s="67"/>
-      <c r="AI1" s="67"/>
-      <c r="AJ1" s="67"/>
-      <c r="AK1" s="67"/>
-      <c r="AL1" s="67"/>
-      <c r="AM1" s="67"/>
-      <c r="AN1" s="67"/>
-      <c r="AO1" s="67"/>
-      <c r="AP1" s="67"/>
-      <c r="AQ1" s="67"/>
-      <c r="AR1" s="67"/>
-      <c r="AS1" s="67"/>
-      <c r="AT1" s="67"/>
-      <c r="AU1" s="67"/>
-      <c r="AV1" s="67"/>
-      <c r="AW1" s="67"/>
-      <c r="AX1" s="67"/>
-      <c r="AY1" s="67"/>
-      <c r="AZ1" s="67"/>
-      <c r="BA1" s="67"/>
-      <c r="BB1" s="67"/>
-      <c r="BC1" s="67"/>
-      <c r="BD1" s="67"/>
-      <c r="BE1" s="67"/>
-      <c r="BF1" s="67"/>
+      <c r="A1" s="69" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="69"/>
+      <c r="C1" s="69"/>
+      <c r="D1" s="69"/>
+      <c r="E1" s="69"/>
+      <c r="F1" s="69"/>
+      <c r="G1" s="69"/>
+      <c r="H1" s="69"/>
+      <c r="I1" s="69"/>
+      <c r="J1" s="69"/>
+      <c r="K1" s="69"/>
+      <c r="L1" s="69"/>
+      <c r="M1" s="69"/>
+      <c r="N1" s="69"/>
+      <c r="O1" s="69"/>
+      <c r="P1" s="69"/>
+      <c r="Q1" s="69"/>
+      <c r="R1" s="69"/>
+      <c r="S1" s="69"/>
+      <c r="T1" s="69"/>
+      <c r="U1" s="69"/>
+      <c r="V1" s="69"/>
+      <c r="W1" s="69"/>
+      <c r="X1" s="69"/>
+      <c r="Y1" s="69"/>
+      <c r="Z1" s="69"/>
+      <c r="AA1" s="69"/>
+      <c r="AB1" s="69"/>
+      <c r="AC1" s="69"/>
+      <c r="AD1" s="69" t="s">
+        <v>0</v>
+      </c>
+      <c r="AE1" s="69"/>
+      <c r="AF1" s="69"/>
+      <c r="AG1" s="69"/>
+      <c r="AH1" s="69"/>
+      <c r="AI1" s="69"/>
+      <c r="AJ1" s="69"/>
+      <c r="AK1" s="69"/>
+      <c r="AL1" s="69"/>
+      <c r="AM1" s="69"/>
+      <c r="AN1" s="69"/>
+      <c r="AO1" s="69"/>
+      <c r="AP1" s="69"/>
+      <c r="AQ1" s="69"/>
+      <c r="AR1" s="69"/>
+      <c r="AS1" s="69"/>
+      <c r="AT1" s="69"/>
+      <c r="AU1" s="69"/>
+      <c r="AV1" s="69"/>
+      <c r="AW1" s="69"/>
+      <c r="AX1" s="69"/>
+      <c r="AY1" s="69"/>
+      <c r="AZ1" s="69"/>
+      <c r="BA1" s="69"/>
+      <c r="BB1" s="69"/>
+      <c r="BC1" s="69"/>
+      <c r="BD1" s="69"/>
+      <c r="BE1" s="69"/>
+      <c r="BF1" s="69"/>
     </row>
     <row r="2" spans="1:58" ht="18">
       <c r="A2" s="23" t="s">
@@ -5292,10 +5967,10 @@
       <c r="BF2" s="36"/>
     </row>
     <row r="3" spans="1:58">
-      <c r="A3" s="68" t="s">
+      <c r="A3" s="70" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="68"/>
+      <c r="B3" s="70"/>
       <c r="C3" s="29"/>
       <c r="D3" s="3">
         <v>2</v>
@@ -5335,10 +6010,10 @@
       <c r="AA3" s="6"/>
       <c r="AB3" s="6"/>
       <c r="AC3" s="6"/>
-      <c r="AD3" s="68" t="s">
+      <c r="AD3" s="70" t="s">
         <v>3</v>
       </c>
-      <c r="AE3" s="68"/>
+      <c r="AE3" s="70"/>
       <c r="AF3" s="37"/>
       <c r="AG3" s="3">
         <v>2</v>
@@ -5808,37 +6483,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="18">
-      <c r="A1" s="67" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="67"/>
-      <c r="C1" s="67"/>
-      <c r="D1" s="67"/>
-      <c r="E1" s="67"/>
-      <c r="F1" s="67"/>
-      <c r="G1" s="67"/>
-      <c r="H1" s="67"/>
-      <c r="I1" s="67"/>
-      <c r="J1" s="67"/>
-      <c r="K1" s="67"/>
-      <c r="L1" s="67"/>
-      <c r="M1" s="67"/>
-      <c r="N1" s="67"/>
-      <c r="O1" s="67"/>
-      <c r="P1" s="67"/>
-      <c r="Q1" s="67"/>
-      <c r="R1" s="67"/>
-      <c r="S1" s="67"/>
-      <c r="T1" s="67"/>
-      <c r="U1" s="67"/>
-      <c r="V1" s="67"/>
-      <c r="W1" s="67"/>
-      <c r="X1" s="67"/>
-      <c r="Y1" s="67"/>
-      <c r="Z1" s="67"/>
-      <c r="AA1" s="67"/>
-      <c r="AB1" s="67"/>
-      <c r="AC1" s="67"/>
+      <c r="A1" s="69" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="69"/>
+      <c r="C1" s="69"/>
+      <c r="D1" s="69"/>
+      <c r="E1" s="69"/>
+      <c r="F1" s="69"/>
+      <c r="G1" s="69"/>
+      <c r="H1" s="69"/>
+      <c r="I1" s="69"/>
+      <c r="J1" s="69"/>
+      <c r="K1" s="69"/>
+      <c r="L1" s="69"/>
+      <c r="M1" s="69"/>
+      <c r="N1" s="69"/>
+      <c r="O1" s="69"/>
+      <c r="P1" s="69"/>
+      <c r="Q1" s="69"/>
+      <c r="R1" s="69"/>
+      <c r="S1" s="69"/>
+      <c r="T1" s="69"/>
+      <c r="U1" s="69"/>
+      <c r="V1" s="69"/>
+      <c r="W1" s="69"/>
+      <c r="X1" s="69"/>
+      <c r="Y1" s="69"/>
+      <c r="Z1" s="69"/>
+      <c r="AA1" s="69"/>
+      <c r="AB1" s="69"/>
+      <c r="AC1" s="69"/>
     </row>
     <row r="2" spans="1:29" ht="18">
       <c r="A2" s="23" t="s">
@@ -5876,10 +6551,10 @@
       <c r="AC2" s="28"/>
     </row>
     <row r="3" spans="1:29">
-      <c r="A3" s="68" t="s">
+      <c r="A3" s="70" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="68"/>
+      <c r="B3" s="70"/>
       <c r="C3" s="29"/>
       <c r="D3" s="3">
         <v>4</v>
@@ -6162,37 +6837,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="18">
-      <c r="A1" s="67" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="67"/>
-      <c r="C1" s="67"/>
-      <c r="D1" s="67"/>
-      <c r="E1" s="67"/>
-      <c r="F1" s="67"/>
-      <c r="G1" s="67"/>
-      <c r="H1" s="67"/>
-      <c r="I1" s="67"/>
-      <c r="J1" s="67"/>
-      <c r="K1" s="67"/>
-      <c r="L1" s="67"/>
-      <c r="M1" s="67"/>
-      <c r="N1" s="67"/>
-      <c r="O1" s="67"/>
-      <c r="P1" s="67"/>
-      <c r="Q1" s="67"/>
-      <c r="R1" s="67"/>
-      <c r="S1" s="67"/>
-      <c r="T1" s="67"/>
-      <c r="U1" s="67"/>
-      <c r="V1" s="67"/>
-      <c r="W1" s="67"/>
-      <c r="X1" s="67"/>
-      <c r="Y1" s="67"/>
-      <c r="Z1" s="67"/>
-      <c r="AA1" s="67"/>
-      <c r="AB1" s="67"/>
-      <c r="AC1" s="67"/>
+      <c r="A1" s="69" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="69"/>
+      <c r="C1" s="69"/>
+      <c r="D1" s="69"/>
+      <c r="E1" s="69"/>
+      <c r="F1" s="69"/>
+      <c r="G1" s="69"/>
+      <c r="H1" s="69"/>
+      <c r="I1" s="69"/>
+      <c r="J1" s="69"/>
+      <c r="K1" s="69"/>
+      <c r="L1" s="69"/>
+      <c r="M1" s="69"/>
+      <c r="N1" s="69"/>
+      <c r="O1" s="69"/>
+      <c r="P1" s="69"/>
+      <c r="Q1" s="69"/>
+      <c r="R1" s="69"/>
+      <c r="S1" s="69"/>
+      <c r="T1" s="69"/>
+      <c r="U1" s="69"/>
+      <c r="V1" s="69"/>
+      <c r="W1" s="69"/>
+      <c r="X1" s="69"/>
+      <c r="Y1" s="69"/>
+      <c r="Z1" s="69"/>
+      <c r="AA1" s="69"/>
+      <c r="AB1" s="69"/>
+      <c r="AC1" s="69"/>
     </row>
     <row r="2" spans="1:29" ht="18">
       <c r="A2" s="23" t="s">
@@ -6230,10 +6905,10 @@
       <c r="AC2" s="28"/>
     </row>
     <row r="3" spans="1:29">
-      <c r="A3" s="68" t="s">
+      <c r="A3" s="70" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="68"/>
+      <c r="B3" s="70"/>
       <c r="C3" s="29"/>
       <c r="D3" s="3">
         <v>3</v>
@@ -6515,37 +7190,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="18">
-      <c r="A1" s="67" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="67"/>
-      <c r="C1" s="67"/>
-      <c r="D1" s="67"/>
-      <c r="E1" s="67"/>
-      <c r="F1" s="67"/>
-      <c r="G1" s="67"/>
-      <c r="H1" s="67"/>
-      <c r="I1" s="67"/>
-      <c r="J1" s="67"/>
-      <c r="K1" s="67"/>
-      <c r="L1" s="67"/>
-      <c r="M1" s="67"/>
-      <c r="N1" s="67"/>
-      <c r="O1" s="67"/>
-      <c r="P1" s="67"/>
-      <c r="Q1" s="67"/>
-      <c r="R1" s="67"/>
-      <c r="S1" s="67"/>
-      <c r="T1" s="67"/>
-      <c r="U1" s="67"/>
-      <c r="V1" s="67"/>
-      <c r="W1" s="67"/>
-      <c r="X1" s="67"/>
-      <c r="Y1" s="67"/>
-      <c r="Z1" s="67"/>
-      <c r="AA1" s="67"/>
-      <c r="AB1" s="67"/>
-      <c r="AC1" s="67"/>
+      <c r="A1" s="69" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="69"/>
+      <c r="C1" s="69"/>
+      <c r="D1" s="69"/>
+      <c r="E1" s="69"/>
+      <c r="F1" s="69"/>
+      <c r="G1" s="69"/>
+      <c r="H1" s="69"/>
+      <c r="I1" s="69"/>
+      <c r="J1" s="69"/>
+      <c r="K1" s="69"/>
+      <c r="L1" s="69"/>
+      <c r="M1" s="69"/>
+      <c r="N1" s="69"/>
+      <c r="O1" s="69"/>
+      <c r="P1" s="69"/>
+      <c r="Q1" s="69"/>
+      <c r="R1" s="69"/>
+      <c r="S1" s="69"/>
+      <c r="T1" s="69"/>
+      <c r="U1" s="69"/>
+      <c r="V1" s="69"/>
+      <c r="W1" s="69"/>
+      <c r="X1" s="69"/>
+      <c r="Y1" s="69"/>
+      <c r="Z1" s="69"/>
+      <c r="AA1" s="69"/>
+      <c r="AB1" s="69"/>
+      <c r="AC1" s="69"/>
     </row>
     <row r="2" spans="1:29" ht="18">
       <c r="A2" s="23" t="s">
@@ -6583,10 +7258,10 @@
       <c r="AC2" s="28"/>
     </row>
     <row r="3" spans="1:29">
-      <c r="A3" s="68" t="s">
+      <c r="A3" s="70" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="68"/>
+      <c r="B3" s="70"/>
       <c r="C3" s="29"/>
       <c r="D3" s="3">
         <v>5</v>
@@ -6870,37 +7545,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="18">
-      <c r="A1" s="67" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="67"/>
-      <c r="C1" s="67"/>
-      <c r="D1" s="67"/>
-      <c r="E1" s="67"/>
-      <c r="F1" s="67"/>
-      <c r="G1" s="67"/>
-      <c r="H1" s="67"/>
-      <c r="I1" s="67"/>
-      <c r="J1" s="67"/>
-      <c r="K1" s="67"/>
-      <c r="L1" s="67"/>
-      <c r="M1" s="67"/>
-      <c r="N1" s="67"/>
-      <c r="O1" s="67"/>
-      <c r="P1" s="67"/>
-      <c r="Q1" s="67"/>
-      <c r="R1" s="67"/>
-      <c r="S1" s="67"/>
-      <c r="T1" s="67"/>
-      <c r="U1" s="67"/>
-      <c r="V1" s="67"/>
-      <c r="W1" s="67"/>
-      <c r="X1" s="67"/>
-      <c r="Y1" s="67"/>
-      <c r="Z1" s="67"/>
-      <c r="AA1" s="67"/>
-      <c r="AB1" s="67"/>
-      <c r="AC1" s="67"/>
+      <c r="A1" s="69" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="69"/>
+      <c r="C1" s="69"/>
+      <c r="D1" s="69"/>
+      <c r="E1" s="69"/>
+      <c r="F1" s="69"/>
+      <c r="G1" s="69"/>
+      <c r="H1" s="69"/>
+      <c r="I1" s="69"/>
+      <c r="J1" s="69"/>
+      <c r="K1" s="69"/>
+      <c r="L1" s="69"/>
+      <c r="M1" s="69"/>
+      <c r="N1" s="69"/>
+      <c r="O1" s="69"/>
+      <c r="P1" s="69"/>
+      <c r="Q1" s="69"/>
+      <c r="R1" s="69"/>
+      <c r="S1" s="69"/>
+      <c r="T1" s="69"/>
+      <c r="U1" s="69"/>
+      <c r="V1" s="69"/>
+      <c r="W1" s="69"/>
+      <c r="X1" s="69"/>
+      <c r="Y1" s="69"/>
+      <c r="Z1" s="69"/>
+      <c r="AA1" s="69"/>
+      <c r="AB1" s="69"/>
+      <c r="AC1" s="69"/>
     </row>
     <row r="2" spans="1:29" ht="18">
       <c r="A2" s="23" t="s">
@@ -6938,10 +7613,10 @@
       <c r="AC2" s="32"/>
     </row>
     <row r="3" spans="1:29">
-      <c r="A3" s="68" t="s">
+      <c r="A3" s="70" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="68"/>
+      <c r="B3" s="70"/>
       <c r="C3" s="33"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -7223,37 +7898,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="18">
-      <c r="A1" s="67" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="67"/>
-      <c r="C1" s="67"/>
-      <c r="D1" s="67"/>
-      <c r="E1" s="67"/>
-      <c r="F1" s="67"/>
-      <c r="G1" s="67"/>
-      <c r="H1" s="67"/>
-      <c r="I1" s="67"/>
-      <c r="J1" s="67"/>
-      <c r="K1" s="67"/>
-      <c r="L1" s="67"/>
-      <c r="M1" s="67"/>
-      <c r="N1" s="67"/>
-      <c r="O1" s="67"/>
-      <c r="P1" s="67"/>
-      <c r="Q1" s="67"/>
-      <c r="R1" s="67"/>
-      <c r="S1" s="67"/>
-      <c r="T1" s="67"/>
-      <c r="U1" s="67"/>
-      <c r="V1" s="67"/>
-      <c r="W1" s="67"/>
-      <c r="X1" s="67"/>
-      <c r="Y1" s="67"/>
-      <c r="Z1" s="67"/>
-      <c r="AA1" s="67"/>
-      <c r="AB1" s="67"/>
-      <c r="AC1" s="67"/>
+      <c r="A1" s="69" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="69"/>
+      <c r="C1" s="69"/>
+      <c r="D1" s="69"/>
+      <c r="E1" s="69"/>
+      <c r="F1" s="69"/>
+      <c r="G1" s="69"/>
+      <c r="H1" s="69"/>
+      <c r="I1" s="69"/>
+      <c r="J1" s="69"/>
+      <c r="K1" s="69"/>
+      <c r="L1" s="69"/>
+      <c r="M1" s="69"/>
+      <c r="N1" s="69"/>
+      <c r="O1" s="69"/>
+      <c r="P1" s="69"/>
+      <c r="Q1" s="69"/>
+      <c r="R1" s="69"/>
+      <c r="S1" s="69"/>
+      <c r="T1" s="69"/>
+      <c r="U1" s="69"/>
+      <c r="V1" s="69"/>
+      <c r="W1" s="69"/>
+      <c r="X1" s="69"/>
+      <c r="Y1" s="69"/>
+      <c r="Z1" s="69"/>
+      <c r="AA1" s="69"/>
+      <c r="AB1" s="69"/>
+      <c r="AC1" s="69"/>
     </row>
     <row r="2" spans="1:29" ht="18">
       <c r="A2" s="23" t="s">
@@ -7291,10 +7966,10 @@
       <c r="AC2" s="34"/>
     </row>
     <row r="3" spans="1:29">
-      <c r="A3" s="68" t="s">
+      <c r="A3" s="70" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="68"/>
+      <c r="B3" s="70"/>
       <c r="C3" s="35"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -7574,37 +8249,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="18">
-      <c r="A1" s="67" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="67"/>
-      <c r="C1" s="67"/>
-      <c r="D1" s="67"/>
-      <c r="E1" s="67"/>
-      <c r="F1" s="67"/>
-      <c r="G1" s="67"/>
-      <c r="H1" s="67"/>
-      <c r="I1" s="67"/>
-      <c r="J1" s="67"/>
-      <c r="K1" s="67"/>
-      <c r="L1" s="67"/>
-      <c r="M1" s="67"/>
-      <c r="N1" s="67"/>
-      <c r="O1" s="67"/>
-      <c r="P1" s="67"/>
-      <c r="Q1" s="67"/>
-      <c r="R1" s="67"/>
-      <c r="S1" s="67"/>
-      <c r="T1" s="67"/>
-      <c r="U1" s="67"/>
-      <c r="V1" s="67"/>
-      <c r="W1" s="67"/>
-      <c r="X1" s="67"/>
-      <c r="Y1" s="67"/>
-      <c r="Z1" s="67"/>
-      <c r="AA1" s="67"/>
-      <c r="AB1" s="67"/>
-      <c r="AC1" s="67"/>
+      <c r="A1" s="69" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="69"/>
+      <c r="C1" s="69"/>
+      <c r="D1" s="69"/>
+      <c r="E1" s="69"/>
+      <c r="F1" s="69"/>
+      <c r="G1" s="69"/>
+      <c r="H1" s="69"/>
+      <c r="I1" s="69"/>
+      <c r="J1" s="69"/>
+      <c r="K1" s="69"/>
+      <c r="L1" s="69"/>
+      <c r="M1" s="69"/>
+      <c r="N1" s="69"/>
+      <c r="O1" s="69"/>
+      <c r="P1" s="69"/>
+      <c r="Q1" s="69"/>
+      <c r="R1" s="69"/>
+      <c r="S1" s="69"/>
+      <c r="T1" s="69"/>
+      <c r="U1" s="69"/>
+      <c r="V1" s="69"/>
+      <c r="W1" s="69"/>
+      <c r="X1" s="69"/>
+      <c r="Y1" s="69"/>
+      <c r="Z1" s="69"/>
+      <c r="AA1" s="69"/>
+      <c r="AB1" s="69"/>
+      <c r="AC1" s="69"/>
     </row>
     <row r="2" spans="1:29" ht="18">
       <c r="A2" s="23" t="s">
@@ -7642,10 +8317,10 @@
       <c r="AC2" s="36"/>
     </row>
     <row r="3" spans="1:29">
-      <c r="A3" s="68" t="s">
+      <c r="A3" s="70" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="68"/>
+      <c r="B3" s="70"/>
       <c r="C3" s="37"/>
       <c r="D3" s="3">
         <v>2</v>
@@ -7942,37 +8617,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:31" ht="18">
-      <c r="A1" s="67" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="67"/>
-      <c r="C1" s="67"/>
-      <c r="D1" s="67"/>
-      <c r="E1" s="67"/>
-      <c r="F1" s="67"/>
-      <c r="G1" s="67"/>
-      <c r="H1" s="67"/>
-      <c r="I1" s="67"/>
-      <c r="J1" s="67"/>
-      <c r="K1" s="67"/>
-      <c r="L1" s="67"/>
-      <c r="M1" s="67"/>
-      <c r="N1" s="67"/>
-      <c r="O1" s="67"/>
-      <c r="P1" s="67"/>
-      <c r="Q1" s="67"/>
-      <c r="R1" s="67"/>
-      <c r="S1" s="67"/>
-      <c r="T1" s="67"/>
-      <c r="U1" s="67"/>
-      <c r="V1" s="67"/>
-      <c r="W1" s="67"/>
-      <c r="X1" s="67"/>
-      <c r="Y1" s="67"/>
-      <c r="Z1" s="67"/>
-      <c r="AA1" s="67"/>
-      <c r="AB1" s="67"/>
-      <c r="AC1" s="67"/>
+      <c r="A1" s="69" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="69"/>
+      <c r="C1" s="69"/>
+      <c r="D1" s="69"/>
+      <c r="E1" s="69"/>
+      <c r="F1" s="69"/>
+      <c r="G1" s="69"/>
+      <c r="H1" s="69"/>
+      <c r="I1" s="69"/>
+      <c r="J1" s="69"/>
+      <c r="K1" s="69"/>
+      <c r="L1" s="69"/>
+      <c r="M1" s="69"/>
+      <c r="N1" s="69"/>
+      <c r="O1" s="69"/>
+      <c r="P1" s="69"/>
+      <c r="Q1" s="69"/>
+      <c r="R1" s="69"/>
+      <c r="S1" s="69"/>
+      <c r="T1" s="69"/>
+      <c r="U1" s="69"/>
+      <c r="V1" s="69"/>
+      <c r="W1" s="69"/>
+      <c r="X1" s="69"/>
+      <c r="Y1" s="69"/>
+      <c r="Z1" s="69"/>
+      <c r="AA1" s="69"/>
+      <c r="AB1" s="69"/>
+      <c r="AC1" s="69"/>
     </row>
     <row r="2" spans="1:31" ht="16.5" customHeight="1">
       <c r="A2" s="23" t="s">
@@ -8010,10 +8685,10 @@
       <c r="AC2" s="41"/>
     </row>
     <row r="3" spans="1:31">
-      <c r="A3" s="68" t="s">
+      <c r="A3" s="70" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="68"/>
+      <c r="B3" s="70"/>
       <c r="D3">
         <v>2</v>
       </c>

</xml_diff>

<commit_message>
Fixes for PurchaseBills Scenarios
Fixes for PurchaseBills Scenarios
</commit_message>
<xml_diff>
--- a/testdata/DBfin.xlsx
+++ b/testdata/DBfin.xlsx
@@ -1,10 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4507"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="2520" windowWidth="15240" windowHeight="6540" tabRatio="849" firstSheet="16" activeTab="20"/>
+    <workbookView xWindow="0" yWindow="2520" windowWidth="15240" windowHeight="6540" tabRatio="849" firstSheet="20" activeTab="25"/>
   </bookViews>
   <sheets>
     <sheet name="PurchaseBillsLocal" sheetId="1" r:id="rId1"/>
@@ -32,13 +32,14 @@
     <sheet name="Purchasebills_Adj_unregrd" sheetId="22" r:id="rId23"/>
     <sheet name="PurchaseBills_Banks" sheetId="23" r:id="rId24"/>
     <sheet name="PurchaseBills_Import" sheetId="24" r:id="rId25"/>
+    <sheet name="PurchaseBills_IGST_Validation_2" sheetId="26" r:id="rId26"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="125725"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1356" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1425" uniqueCount="114">
   <si>
     <t>Scenario  : Local Sales - Stock UOM and Sales UOM (Similar)   DOC NO :  SORD-2425-00089</t>
   </si>
@@ -373,17 +374,26 @@
   <si>
     <t>PSV INDUSTRIES (AP)</t>
   </si>
+  <si>
+    <t>NULL</t>
+  </si>
+  <si>
+    <t>Process Flow</t>
+  </si>
+  <si>
+    <t>null</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="165" formatCode="0.000"/>
-    <numFmt numFmtId="166" formatCode="0.0"/>
+    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="0.000"/>
+    <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -454,6 +464,14 @@
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="7">
@@ -558,9 +576,9 @@
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="85">
+  <cellXfs count="90">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -607,7 +625,7 @@
     </xf>
     <xf numFmtId="10" fontId="3" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="10" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1"/>
@@ -651,11 +669,11 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -678,7 +696,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="166" fontId="3" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -755,6 +773,19 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -1087,68 +1118,68 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:59" ht="18">
-      <c r="A1" s="83" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="83"/>
-      <c r="C1" s="83"/>
-      <c r="D1" s="83"/>
-      <c r="E1" s="83"/>
-      <c r="F1" s="83"/>
-      <c r="G1" s="83"/>
-      <c r="H1" s="83"/>
-      <c r="I1" s="83"/>
-      <c r="J1" s="83"/>
-      <c r="K1" s="83"/>
-      <c r="L1" s="83"/>
-      <c r="M1" s="83"/>
-      <c r="N1" s="83"/>
-      <c r="O1" s="83"/>
-      <c r="P1" s="83"/>
-      <c r="Q1" s="83"/>
-      <c r="R1" s="83"/>
-      <c r="S1" s="83"/>
-      <c r="T1" s="83"/>
-      <c r="U1" s="83"/>
-      <c r="V1" s="83"/>
-      <c r="W1" s="83"/>
-      <c r="X1" s="83"/>
-      <c r="Y1" s="83"/>
-      <c r="Z1" s="83"/>
-      <c r="AA1" s="83"/>
-      <c r="AB1" s="83"/>
-      <c r="AC1" s="83"/>
-      <c r="AD1" s="83" t="s">
-        <v>0</v>
-      </c>
-      <c r="AE1" s="83"/>
-      <c r="AF1" s="83"/>
-      <c r="AG1" s="83"/>
-      <c r="AH1" s="83"/>
-      <c r="AI1" s="83"/>
-      <c r="AJ1" s="83"/>
-      <c r="AK1" s="83"/>
-      <c r="AL1" s="83"/>
-      <c r="AM1" s="83"/>
-      <c r="AN1" s="83"/>
-      <c r="AO1" s="83"/>
-      <c r="AP1" s="83"/>
-      <c r="AQ1" s="83"/>
-      <c r="AR1" s="83"/>
-      <c r="AS1" s="83"/>
-      <c r="AT1" s="83"/>
-      <c r="AU1" s="83"/>
-      <c r="AV1" s="83"/>
-      <c r="AW1" s="83"/>
-      <c r="AX1" s="83"/>
-      <c r="AY1" s="83"/>
-      <c r="AZ1" s="83"/>
-      <c r="BA1" s="83"/>
-      <c r="BB1" s="83"/>
-      <c r="BC1" s="83"/>
-      <c r="BD1" s="83"/>
-      <c r="BE1" s="83"/>
-      <c r="BF1" s="83"/>
+      <c r="A1" s="88" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="88"/>
+      <c r="C1" s="88"/>
+      <c r="D1" s="88"/>
+      <c r="E1" s="88"/>
+      <c r="F1" s="88"/>
+      <c r="G1" s="88"/>
+      <c r="H1" s="88"/>
+      <c r="I1" s="88"/>
+      <c r="J1" s="88"/>
+      <c r="K1" s="88"/>
+      <c r="L1" s="88"/>
+      <c r="M1" s="88"/>
+      <c r="N1" s="88"/>
+      <c r="O1" s="88"/>
+      <c r="P1" s="88"/>
+      <c r="Q1" s="88"/>
+      <c r="R1" s="88"/>
+      <c r="S1" s="88"/>
+      <c r="T1" s="88"/>
+      <c r="U1" s="88"/>
+      <c r="V1" s="88"/>
+      <c r="W1" s="88"/>
+      <c r="X1" s="88"/>
+      <c r="Y1" s="88"/>
+      <c r="Z1" s="88"/>
+      <c r="AA1" s="88"/>
+      <c r="AB1" s="88"/>
+      <c r="AC1" s="88"/>
+      <c r="AD1" s="88" t="s">
+        <v>0</v>
+      </c>
+      <c r="AE1" s="88"/>
+      <c r="AF1" s="88"/>
+      <c r="AG1" s="88"/>
+      <c r="AH1" s="88"/>
+      <c r="AI1" s="88"/>
+      <c r="AJ1" s="88"/>
+      <c r="AK1" s="88"/>
+      <c r="AL1" s="88"/>
+      <c r="AM1" s="88"/>
+      <c r="AN1" s="88"/>
+      <c r="AO1" s="88"/>
+      <c r="AP1" s="88"/>
+      <c r="AQ1" s="88"/>
+      <c r="AR1" s="88"/>
+      <c r="AS1" s="88"/>
+      <c r="AT1" s="88"/>
+      <c r="AU1" s="88"/>
+      <c r="AV1" s="88"/>
+      <c r="AW1" s="88"/>
+      <c r="AX1" s="88"/>
+      <c r="AY1" s="88"/>
+      <c r="AZ1" s="88"/>
+      <c r="BA1" s="88"/>
+      <c r="BB1" s="88"/>
+      <c r="BC1" s="88"/>
+      <c r="BD1" s="88"/>
+      <c r="BE1" s="88"/>
+      <c r="BF1" s="88"/>
     </row>
     <row r="2" spans="1:59" ht="18">
       <c r="A2" s="23" t="s">
@@ -1219,10 +1250,10 @@
       <c r="BF2" s="38"/>
     </row>
     <row r="3" spans="1:59">
-      <c r="A3" s="84" t="s">
+      <c r="A3" s="89" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="84"/>
+      <c r="B3" s="89"/>
       <c r="C3" s="2"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -1262,10 +1293,10 @@
       <c r="AA3" s="6"/>
       <c r="AB3" s="6"/>
       <c r="AC3" s="6"/>
-      <c r="AD3" s="84" t="s">
+      <c r="AD3" s="89" t="s">
         <v>3</v>
       </c>
-      <c r="AE3" s="84"/>
+      <c r="AE3" s="89"/>
       <c r="AF3" s="39"/>
       <c r="AG3" s="3">
         <v>1</v>
@@ -1743,38 +1774,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:33" ht="18">
-      <c r="A1" s="83" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="83"/>
-      <c r="C1" s="83"/>
-      <c r="D1" s="83"/>
-      <c r="E1" s="83"/>
-      <c r="F1" s="83"/>
-      <c r="G1" s="83"/>
-      <c r="H1" s="83"/>
-      <c r="I1" s="83"/>
-      <c r="J1" s="83"/>
-      <c r="K1" s="83"/>
-      <c r="L1" s="83"/>
-      <c r="M1" s="83"/>
-      <c r="N1" s="83"/>
-      <c r="O1" s="83"/>
-      <c r="P1" s="83"/>
-      <c r="Q1" s="83"/>
-      <c r="R1" s="83"/>
-      <c r="S1" s="83"/>
-      <c r="T1" s="83"/>
-      <c r="U1" s="83"/>
-      <c r="V1" s="83"/>
-      <c r="W1" s="83"/>
-      <c r="X1" s="83"/>
-      <c r="Y1" s="83"/>
-      <c r="Z1" s="83"/>
-      <c r="AA1" s="83"/>
-      <c r="AB1" s="83"/>
-      <c r="AC1" s="83"/>
-      <c r="AD1" s="83"/>
+      <c r="A1" s="88" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="88"/>
+      <c r="C1" s="88"/>
+      <c r="D1" s="88"/>
+      <c r="E1" s="88"/>
+      <c r="F1" s="88"/>
+      <c r="G1" s="88"/>
+      <c r="H1" s="88"/>
+      <c r="I1" s="88"/>
+      <c r="J1" s="88"/>
+      <c r="K1" s="88"/>
+      <c r="L1" s="88"/>
+      <c r="M1" s="88"/>
+      <c r="N1" s="88"/>
+      <c r="O1" s="88"/>
+      <c r="P1" s="88"/>
+      <c r="Q1" s="88"/>
+      <c r="R1" s="88"/>
+      <c r="S1" s="88"/>
+      <c r="T1" s="88"/>
+      <c r="U1" s="88"/>
+      <c r="V1" s="88"/>
+      <c r="W1" s="88"/>
+      <c r="X1" s="88"/>
+      <c r="Y1" s="88"/>
+      <c r="Z1" s="88"/>
+      <c r="AA1" s="88"/>
+      <c r="AB1" s="88"/>
+      <c r="AC1" s="88"/>
+      <c r="AD1" s="88"/>
     </row>
     <row r="2" spans="1:33" ht="18">
       <c r="A2" s="23" t="s">
@@ -1813,10 +1844,10 @@
       <c r="AD2" s="43"/>
     </row>
     <row r="3" spans="1:33" ht="15.75" thickBot="1">
-      <c r="A3" s="84" t="s">
+      <c r="A3" s="89" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="84"/>
+      <c r="B3" s="89"/>
       <c r="C3" s="44"/>
       <c r="D3" s="3">
         <v>2</v>
@@ -2042,7 +2073,7 @@
         <f>IF($D$3=1,ROUND(((V5*X5)/2),2),0)</f>
         <v>0</v>
       </c>
-      <c r="AA5" s="24">
+      <c r="AA5" s="8">
         <f>IF($D$3=2,ROUND(((V5*X5)),2),0)</f>
         <v>90.09</v>
       </c>
@@ -2153,8 +2184,8 @@
         <f>IF($D$3=1,ROUND(((V6*X6)/2),2),0)</f>
         <v>0</v>
       </c>
-      <c r="AA6" s="24">
-        <f>IF($D$3=2,ROUND(((V6*X6)),2),0)</f>
+      <c r="AA6" s="8">
+        <f t="shared" ref="AA6:AA8" si="6">IF($D$3=2,ROUND(((V6*X6)),2),0)</f>
         <v>622.44000000000005</v>
       </c>
       <c r="AB6" s="24">
@@ -2216,27 +2247,27 @@
         <v>609</v>
       </c>
       <c r="O7" s="8">
-        <f t="shared" ref="O7" si="6">ROUND(K7*N7%,2)</f>
+        <f t="shared" ref="O7" si="7">ROUND(K7*N7%,2)</f>
         <v>0</v>
       </c>
       <c r="P7" s="8">
-        <f t="shared" ref="P7" si="7">J7-O7</f>
+        <f t="shared" ref="P7" si="8">J7-O7</f>
         <v>609</v>
       </c>
       <c r="Q7" s="8">
-        <f t="shared" ref="Q7" si="8">ROUND(L7*P7%,2)</f>
+        <f t="shared" ref="Q7" si="9">ROUND(L7*P7%,2)</f>
         <v>0</v>
       </c>
       <c r="R7" s="8">
-        <f t="shared" ref="R7" si="9">P7-Q7</f>
+        <f t="shared" ref="R7" si="10">P7-Q7</f>
         <v>609</v>
       </c>
       <c r="S7" s="8">
-        <f t="shared" ref="S7" si="10">ROUND(M7*R7%,2)</f>
+        <f t="shared" ref="S7" si="11">ROUND(M7*R7%,2)</f>
         <v>0</v>
       </c>
       <c r="T7" s="26">
-        <f t="shared" ref="T7" si="11">O7+Q7+S7</f>
+        <f t="shared" ref="T7" si="12">O7+Q7+S7</f>
         <v>0</v>
       </c>
       <c r="U7" s="26">
@@ -2250,7 +2281,7 @@
         <v>75052200</v>
       </c>
       <c r="X7" s="18">
-        <v>0.18</v>
+        <v>0.05</v>
       </c>
       <c r="Y7" s="24">
         <f>IF($D$3=1,ROUND(((V7*X7)/2),2),0)</f>
@@ -2260,20 +2291,20 @@
         <f>IF($D$3=1,ROUND(((V7*X7)/2),2),0)</f>
         <v>0</v>
       </c>
-      <c r="AA7" s="24">
-        <f>IF($D$3=2,ROUND(((V7*X7)),2),0)</f>
-        <v>109.62</v>
+      <c r="AA7" s="8">
+        <f t="shared" si="6"/>
+        <v>30.45</v>
       </c>
       <c r="AB7" s="24">
         <v>0</v>
       </c>
       <c r="AC7" s="24">
         <f>Y7+Z7+AA7</f>
-        <v>109.62</v>
+        <v>30.45</v>
       </c>
       <c r="AD7" s="24">
         <f>V7+AC7</f>
-        <v>718.62</v>
+        <v>639.45000000000005</v>
       </c>
       <c r="AE7" s="52" t="s">
         <v>59</v>
@@ -2371,8 +2402,8 @@
         <f>IF($D$3=1,ROUND(((V8*X8)/2),2),0)</f>
         <v>0</v>
       </c>
-      <c r="AA8" s="24">
-        <f>IF($D$3=2,ROUND(((V8*X8)),2),0)</f>
+      <c r="AA8" s="55">
+        <f t="shared" si="6"/>
         <v>364.5</v>
       </c>
       <c r="AB8" s="24">
@@ -2430,37 +2461,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:31" ht="18">
-      <c r="A1" s="83" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="83"/>
-      <c r="C1" s="83"/>
-      <c r="D1" s="83"/>
-      <c r="E1" s="83"/>
-      <c r="F1" s="83"/>
-      <c r="G1" s="83"/>
-      <c r="H1" s="83"/>
-      <c r="I1" s="83"/>
-      <c r="J1" s="83"/>
-      <c r="K1" s="83"/>
-      <c r="L1" s="83"/>
-      <c r="M1" s="83"/>
-      <c r="N1" s="83"/>
-      <c r="O1" s="83"/>
-      <c r="P1" s="83"/>
-      <c r="Q1" s="83"/>
-      <c r="R1" s="83"/>
-      <c r="S1" s="83"/>
-      <c r="T1" s="83"/>
-      <c r="U1" s="83"/>
-      <c r="V1" s="83"/>
-      <c r="W1" s="83"/>
-      <c r="X1" s="83"/>
-      <c r="Y1" s="83"/>
-      <c r="Z1" s="83"/>
-      <c r="AA1" s="83"/>
-      <c r="AB1" s="83"/>
-      <c r="AC1" s="83"/>
+      <c r="A1" s="88" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="88"/>
+      <c r="C1" s="88"/>
+      <c r="D1" s="88"/>
+      <c r="E1" s="88"/>
+      <c r="F1" s="88"/>
+      <c r="G1" s="88"/>
+      <c r="H1" s="88"/>
+      <c r="I1" s="88"/>
+      <c r="J1" s="88"/>
+      <c r="K1" s="88"/>
+      <c r="L1" s="88"/>
+      <c r="M1" s="88"/>
+      <c r="N1" s="88"/>
+      <c r="O1" s="88"/>
+      <c r="P1" s="88"/>
+      <c r="Q1" s="88"/>
+      <c r="R1" s="88"/>
+      <c r="S1" s="88"/>
+      <c r="T1" s="88"/>
+      <c r="U1" s="88"/>
+      <c r="V1" s="88"/>
+      <c r="W1" s="88"/>
+      <c r="X1" s="88"/>
+      <c r="Y1" s="88"/>
+      <c r="Z1" s="88"/>
+      <c r="AA1" s="88"/>
+      <c r="AB1" s="88"/>
+      <c r="AC1" s="88"/>
     </row>
     <row r="2" spans="1:31" ht="16.5" customHeight="1">
       <c r="A2" s="23" t="s">
@@ -2498,10 +2529,10 @@
       <c r="AC2" s="54"/>
     </row>
     <row r="3" spans="1:31">
-      <c r="A3" s="84" t="s">
+      <c r="A3" s="89" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="84"/>
+      <c r="B3" s="89"/>
       <c r="D3">
         <v>2</v>
       </c>
@@ -2992,37 +3023,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="18">
-      <c r="A1" s="83" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="83"/>
-      <c r="C1" s="83"/>
-      <c r="D1" s="83"/>
-      <c r="E1" s="83"/>
-      <c r="F1" s="83"/>
-      <c r="G1" s="83"/>
-      <c r="H1" s="83"/>
-      <c r="I1" s="83"/>
-      <c r="J1" s="83"/>
-      <c r="K1" s="83"/>
-      <c r="L1" s="83"/>
-      <c r="M1" s="83"/>
-      <c r="N1" s="83"/>
-      <c r="O1" s="83"/>
-      <c r="P1" s="83"/>
-      <c r="Q1" s="83"/>
-      <c r="R1" s="83"/>
-      <c r="S1" s="83"/>
-      <c r="T1" s="83"/>
-      <c r="U1" s="83"/>
-      <c r="V1" s="83"/>
-      <c r="W1" s="83"/>
-      <c r="X1" s="83"/>
-      <c r="Y1" s="83"/>
-      <c r="Z1" s="83"/>
-      <c r="AA1" s="83"/>
-      <c r="AB1" s="83"/>
-      <c r="AC1" s="83"/>
+      <c r="A1" s="88" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="88"/>
+      <c r="C1" s="88"/>
+      <c r="D1" s="88"/>
+      <c r="E1" s="88"/>
+      <c r="F1" s="88"/>
+      <c r="G1" s="88"/>
+      <c r="H1" s="88"/>
+      <c r="I1" s="88"/>
+      <c r="J1" s="88"/>
+      <c r="K1" s="88"/>
+      <c r="L1" s="88"/>
+      <c r="M1" s="88"/>
+      <c r="N1" s="88"/>
+      <c r="O1" s="88"/>
+      <c r="P1" s="88"/>
+      <c r="Q1" s="88"/>
+      <c r="R1" s="88"/>
+      <c r="S1" s="88"/>
+      <c r="T1" s="88"/>
+      <c r="U1" s="88"/>
+      <c r="V1" s="88"/>
+      <c r="W1" s="88"/>
+      <c r="X1" s="88"/>
+      <c r="Y1" s="88"/>
+      <c r="Z1" s="88"/>
+      <c r="AA1" s="88"/>
+      <c r="AB1" s="88"/>
+      <c r="AC1" s="88"/>
     </row>
     <row r="2" spans="1:29" ht="18">
       <c r="A2" s="23" t="s">
@@ -3060,10 +3091,10 @@
       <c r="AC2" s="56"/>
     </row>
     <row r="3" spans="1:29">
-      <c r="A3" s="84" t="s">
+      <c r="A3" s="89" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="84"/>
+      <c r="B3" s="89"/>
       <c r="C3" s="57"/>
       <c r="D3" s="3">
         <v>2</v>
@@ -3344,37 +3375,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="18">
-      <c r="A1" s="83" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="83"/>
-      <c r="C1" s="83"/>
-      <c r="D1" s="83"/>
-      <c r="E1" s="83"/>
-      <c r="F1" s="83"/>
-      <c r="G1" s="83"/>
-      <c r="H1" s="83"/>
-      <c r="I1" s="83"/>
-      <c r="J1" s="83"/>
-      <c r="K1" s="83"/>
-      <c r="L1" s="83"/>
-      <c r="M1" s="83"/>
-      <c r="N1" s="83"/>
-      <c r="O1" s="83"/>
-      <c r="P1" s="83"/>
-      <c r="Q1" s="83"/>
-      <c r="R1" s="83"/>
-      <c r="S1" s="83"/>
-      <c r="T1" s="83"/>
-      <c r="U1" s="83"/>
-      <c r="V1" s="83"/>
-      <c r="W1" s="83"/>
-      <c r="X1" s="83"/>
-      <c r="Y1" s="83"/>
-      <c r="Z1" s="83"/>
-      <c r="AA1" s="83"/>
-      <c r="AB1" s="83"/>
-      <c r="AC1" s="83"/>
+      <c r="A1" s="88" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="88"/>
+      <c r="C1" s="88"/>
+      <c r="D1" s="88"/>
+      <c r="E1" s="88"/>
+      <c r="F1" s="88"/>
+      <c r="G1" s="88"/>
+      <c r="H1" s="88"/>
+      <c r="I1" s="88"/>
+      <c r="J1" s="88"/>
+      <c r="K1" s="88"/>
+      <c r="L1" s="88"/>
+      <c r="M1" s="88"/>
+      <c r="N1" s="88"/>
+      <c r="O1" s="88"/>
+      <c r="P1" s="88"/>
+      <c r="Q1" s="88"/>
+      <c r="R1" s="88"/>
+      <c r="S1" s="88"/>
+      <c r="T1" s="88"/>
+      <c r="U1" s="88"/>
+      <c r="V1" s="88"/>
+      <c r="W1" s="88"/>
+      <c r="X1" s="88"/>
+      <c r="Y1" s="88"/>
+      <c r="Z1" s="88"/>
+      <c r="AA1" s="88"/>
+      <c r="AB1" s="88"/>
+      <c r="AC1" s="88"/>
     </row>
     <row r="2" spans="1:29" ht="18">
       <c r="A2" s="23" t="s">
@@ -3412,10 +3443,10 @@
       <c r="AC2" s="58"/>
     </row>
     <row r="3" spans="1:29">
-      <c r="A3" s="84" t="s">
+      <c r="A3" s="89" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="84"/>
+      <c r="B3" s="89"/>
       <c r="C3" s="59"/>
       <c r="D3" s="3">
         <v>4</v>
@@ -3698,38 +3729,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:33" ht="18">
-      <c r="A1" s="83" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="83"/>
-      <c r="C1" s="83"/>
-      <c r="D1" s="83"/>
-      <c r="E1" s="83"/>
-      <c r="F1" s="83"/>
-      <c r="G1" s="83"/>
-      <c r="H1" s="83"/>
-      <c r="I1" s="83"/>
-      <c r="J1" s="83"/>
-      <c r="K1" s="83"/>
-      <c r="L1" s="83"/>
-      <c r="M1" s="83"/>
-      <c r="N1" s="83"/>
-      <c r="O1" s="83"/>
-      <c r="P1" s="83"/>
-      <c r="Q1" s="83"/>
-      <c r="R1" s="83"/>
-      <c r="S1" s="83"/>
-      <c r="T1" s="83"/>
-      <c r="U1" s="83"/>
-      <c r="V1" s="83"/>
-      <c r="W1" s="83"/>
-      <c r="X1" s="83"/>
-      <c r="Y1" s="83"/>
-      <c r="Z1" s="83"/>
-      <c r="AA1" s="83"/>
-      <c r="AB1" s="83"/>
-      <c r="AC1" s="83"/>
-      <c r="AD1" s="83"/>
+      <c r="A1" s="88" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="88"/>
+      <c r="C1" s="88"/>
+      <c r="D1" s="88"/>
+      <c r="E1" s="88"/>
+      <c r="F1" s="88"/>
+      <c r="G1" s="88"/>
+      <c r="H1" s="88"/>
+      <c r="I1" s="88"/>
+      <c r="J1" s="88"/>
+      <c r="K1" s="88"/>
+      <c r="L1" s="88"/>
+      <c r="M1" s="88"/>
+      <c r="N1" s="88"/>
+      <c r="O1" s="88"/>
+      <c r="P1" s="88"/>
+      <c r="Q1" s="88"/>
+      <c r="R1" s="88"/>
+      <c r="S1" s="88"/>
+      <c r="T1" s="88"/>
+      <c r="U1" s="88"/>
+      <c r="V1" s="88"/>
+      <c r="W1" s="88"/>
+      <c r="X1" s="88"/>
+      <c r="Y1" s="88"/>
+      <c r="Z1" s="88"/>
+      <c r="AA1" s="88"/>
+      <c r="AB1" s="88"/>
+      <c r="AC1" s="88"/>
+      <c r="AD1" s="88"/>
     </row>
     <row r="2" spans="1:33" ht="18">
       <c r="A2" s="23" t="s">
@@ -3768,10 +3799,10 @@
       <c r="AD2" s="60"/>
     </row>
     <row r="3" spans="1:33" ht="15.75" thickBot="1">
-      <c r="A3" s="84" t="s">
+      <c r="A3" s="89" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="84"/>
+      <c r="B3" s="89"/>
       <c r="C3" s="61"/>
       <c r="D3" s="3">
         <v>2</v>
@@ -4207,7 +4238,7 @@
         <v>75052200</v>
       </c>
       <c r="X7" s="18">
-        <v>0.18</v>
+        <v>0.05</v>
       </c>
       <c r="Y7" s="24">
         <f>IF($D$3=1,ROUND(((V7*X7)/2),2),0)</f>
@@ -4219,18 +4250,18 @@
       </c>
       <c r="AA7" s="24">
         <f>IF($D$3=2,ROUND(((V7*X7)),2),0)</f>
-        <v>109.62</v>
+        <v>30.45</v>
       </c>
       <c r="AB7" s="24">
         <v>0</v>
       </c>
       <c r="AC7" s="24">
         <f>Y7+Z7+AA7</f>
-        <v>109.62</v>
+        <v>30.45</v>
       </c>
       <c r="AD7" s="24">
         <f>V7+AC7</f>
-        <v>718.62</v>
+        <v>639.45000000000005</v>
       </c>
       <c r="AE7" s="52" t="s">
         <v>59</v>
@@ -4384,37 +4415,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="18">
-      <c r="A1" s="83" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="83"/>
-      <c r="C1" s="83"/>
-      <c r="D1" s="83"/>
-      <c r="E1" s="83"/>
-      <c r="F1" s="83"/>
-      <c r="G1" s="83"/>
-      <c r="H1" s="83"/>
-      <c r="I1" s="83"/>
-      <c r="J1" s="83"/>
-      <c r="K1" s="83"/>
-      <c r="L1" s="83"/>
-      <c r="M1" s="83"/>
-      <c r="N1" s="83"/>
-      <c r="O1" s="83"/>
-      <c r="P1" s="83"/>
-      <c r="Q1" s="83"/>
-      <c r="R1" s="83"/>
-      <c r="S1" s="83"/>
-      <c r="T1" s="83"/>
-      <c r="U1" s="83"/>
-      <c r="V1" s="83"/>
-      <c r="W1" s="83"/>
-      <c r="X1" s="83"/>
-      <c r="Y1" s="83"/>
-      <c r="Z1" s="83"/>
-      <c r="AA1" s="83"/>
-      <c r="AB1" s="83"/>
-      <c r="AC1" s="83"/>
+      <c r="A1" s="88" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="88"/>
+      <c r="C1" s="88"/>
+      <c r="D1" s="88"/>
+      <c r="E1" s="88"/>
+      <c r="F1" s="88"/>
+      <c r="G1" s="88"/>
+      <c r="H1" s="88"/>
+      <c r="I1" s="88"/>
+      <c r="J1" s="88"/>
+      <c r="K1" s="88"/>
+      <c r="L1" s="88"/>
+      <c r="M1" s="88"/>
+      <c r="N1" s="88"/>
+      <c r="O1" s="88"/>
+      <c r="P1" s="88"/>
+      <c r="Q1" s="88"/>
+      <c r="R1" s="88"/>
+      <c r="S1" s="88"/>
+      <c r="T1" s="88"/>
+      <c r="U1" s="88"/>
+      <c r="V1" s="88"/>
+      <c r="W1" s="88"/>
+      <c r="X1" s="88"/>
+      <c r="Y1" s="88"/>
+      <c r="Z1" s="88"/>
+      <c r="AA1" s="88"/>
+      <c r="AB1" s="88"/>
+      <c r="AC1" s="88"/>
     </row>
     <row r="2" spans="1:29" ht="18">
       <c r="A2" s="23" t="s">
@@ -4452,10 +4483,10 @@
       <c r="AC2" s="62"/>
     </row>
     <row r="3" spans="1:29">
-      <c r="A3" s="84" t="s">
+      <c r="A3" s="89" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="84"/>
+      <c r="B3" s="89"/>
       <c r="C3" s="63"/>
       <c r="D3" s="3">
         <v>4</v>
@@ -4744,68 +4775,68 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:59" ht="18">
-      <c r="A1" s="83" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="83"/>
-      <c r="C1" s="83"/>
-      <c r="D1" s="83"/>
-      <c r="E1" s="83"/>
-      <c r="F1" s="83"/>
-      <c r="G1" s="83"/>
-      <c r="H1" s="83"/>
-      <c r="I1" s="83"/>
-      <c r="J1" s="83"/>
-      <c r="K1" s="83"/>
-      <c r="L1" s="83"/>
-      <c r="M1" s="83"/>
-      <c r="N1" s="83"/>
-      <c r="O1" s="83"/>
-      <c r="P1" s="83"/>
-      <c r="Q1" s="83"/>
-      <c r="R1" s="83"/>
-      <c r="S1" s="83"/>
-      <c r="T1" s="83"/>
-      <c r="U1" s="83"/>
-      <c r="V1" s="83"/>
-      <c r="W1" s="83"/>
-      <c r="X1" s="83"/>
-      <c r="Y1" s="83"/>
-      <c r="Z1" s="83"/>
-      <c r="AA1" s="83"/>
-      <c r="AB1" s="83"/>
-      <c r="AC1" s="83"/>
-      <c r="AD1" s="83" t="s">
-        <v>0</v>
-      </c>
-      <c r="AE1" s="83"/>
-      <c r="AF1" s="83"/>
-      <c r="AG1" s="83"/>
-      <c r="AH1" s="83"/>
-      <c r="AI1" s="83"/>
-      <c r="AJ1" s="83"/>
-      <c r="AK1" s="83"/>
-      <c r="AL1" s="83"/>
-      <c r="AM1" s="83"/>
-      <c r="AN1" s="83"/>
-      <c r="AO1" s="83"/>
-      <c r="AP1" s="83"/>
-      <c r="AQ1" s="83"/>
-      <c r="AR1" s="83"/>
-      <c r="AS1" s="83"/>
-      <c r="AT1" s="83"/>
-      <c r="AU1" s="83"/>
-      <c r="AV1" s="83"/>
-      <c r="AW1" s="83"/>
-      <c r="AX1" s="83"/>
-      <c r="AY1" s="83"/>
-      <c r="AZ1" s="83"/>
-      <c r="BA1" s="83"/>
-      <c r="BB1" s="83"/>
-      <c r="BC1" s="83"/>
-      <c r="BD1" s="83"/>
-      <c r="BE1" s="83"/>
-      <c r="BF1" s="83"/>
+      <c r="A1" s="88" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="88"/>
+      <c r="C1" s="88"/>
+      <c r="D1" s="88"/>
+      <c r="E1" s="88"/>
+      <c r="F1" s="88"/>
+      <c r="G1" s="88"/>
+      <c r="H1" s="88"/>
+      <c r="I1" s="88"/>
+      <c r="J1" s="88"/>
+      <c r="K1" s="88"/>
+      <c r="L1" s="88"/>
+      <c r="M1" s="88"/>
+      <c r="N1" s="88"/>
+      <c r="O1" s="88"/>
+      <c r="P1" s="88"/>
+      <c r="Q1" s="88"/>
+      <c r="R1" s="88"/>
+      <c r="S1" s="88"/>
+      <c r="T1" s="88"/>
+      <c r="U1" s="88"/>
+      <c r="V1" s="88"/>
+      <c r="W1" s="88"/>
+      <c r="X1" s="88"/>
+      <c r="Y1" s="88"/>
+      <c r="Z1" s="88"/>
+      <c r="AA1" s="88"/>
+      <c r="AB1" s="88"/>
+      <c r="AC1" s="88"/>
+      <c r="AD1" s="88" t="s">
+        <v>0</v>
+      </c>
+      <c r="AE1" s="88"/>
+      <c r="AF1" s="88"/>
+      <c r="AG1" s="88"/>
+      <c r="AH1" s="88"/>
+      <c r="AI1" s="88"/>
+      <c r="AJ1" s="88"/>
+      <c r="AK1" s="88"/>
+      <c r="AL1" s="88"/>
+      <c r="AM1" s="88"/>
+      <c r="AN1" s="88"/>
+      <c r="AO1" s="88"/>
+      <c r="AP1" s="88"/>
+      <c r="AQ1" s="88"/>
+      <c r="AR1" s="88"/>
+      <c r="AS1" s="88"/>
+      <c r="AT1" s="88"/>
+      <c r="AU1" s="88"/>
+      <c r="AV1" s="88"/>
+      <c r="AW1" s="88"/>
+      <c r="AX1" s="88"/>
+      <c r="AY1" s="88"/>
+      <c r="AZ1" s="88"/>
+      <c r="BA1" s="88"/>
+      <c r="BB1" s="88"/>
+      <c r="BC1" s="88"/>
+      <c r="BD1" s="88"/>
+      <c r="BE1" s="88"/>
+      <c r="BF1" s="88"/>
     </row>
     <row r="2" spans="1:59" ht="18">
       <c r="A2" s="23" t="s">
@@ -4876,10 +4907,10 @@
       <c r="BF2" s="64"/>
     </row>
     <row r="3" spans="1:59">
-      <c r="A3" s="84" t="s">
+      <c r="A3" s="89" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="84"/>
+      <c r="B3" s="89"/>
       <c r="C3" s="65"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -4919,10 +4950,10 @@
       <c r="AA3" s="6"/>
       <c r="AB3" s="6"/>
       <c r="AC3" s="6"/>
-      <c r="AD3" s="84" t="s">
+      <c r="AD3" s="89" t="s">
         <v>3</v>
       </c>
-      <c r="AE3" s="84"/>
+      <c r="AE3" s="89"/>
       <c r="AF3" s="65"/>
       <c r="AG3" s="3">
         <v>2</v>
@@ -5404,68 +5435,68 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:59" ht="18">
-      <c r="A1" s="83" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="83"/>
-      <c r="C1" s="83"/>
-      <c r="D1" s="83"/>
-      <c r="E1" s="83"/>
-      <c r="F1" s="83"/>
-      <c r="G1" s="83"/>
-      <c r="H1" s="83"/>
-      <c r="I1" s="83"/>
-      <c r="J1" s="83"/>
-      <c r="K1" s="83"/>
-      <c r="L1" s="83"/>
-      <c r="M1" s="83"/>
-      <c r="N1" s="83"/>
-      <c r="O1" s="83"/>
-      <c r="P1" s="83"/>
-      <c r="Q1" s="83"/>
-      <c r="R1" s="83"/>
-      <c r="S1" s="83"/>
-      <c r="T1" s="83"/>
-      <c r="U1" s="83"/>
-      <c r="V1" s="83"/>
-      <c r="W1" s="83"/>
-      <c r="X1" s="83"/>
-      <c r="Y1" s="83"/>
-      <c r="Z1" s="83"/>
-      <c r="AA1" s="83"/>
-      <c r="AB1" s="83"/>
-      <c r="AC1" s="83"/>
-      <c r="AD1" s="83" t="s">
-        <v>0</v>
-      </c>
-      <c r="AE1" s="83"/>
-      <c r="AF1" s="83"/>
-      <c r="AG1" s="83"/>
-      <c r="AH1" s="83"/>
-      <c r="AI1" s="83"/>
-      <c r="AJ1" s="83"/>
-      <c r="AK1" s="83"/>
-      <c r="AL1" s="83"/>
-      <c r="AM1" s="83"/>
-      <c r="AN1" s="83"/>
-      <c r="AO1" s="83"/>
-      <c r="AP1" s="83"/>
-      <c r="AQ1" s="83"/>
-      <c r="AR1" s="83"/>
-      <c r="AS1" s="83"/>
-      <c r="AT1" s="83"/>
-      <c r="AU1" s="83"/>
-      <c r="AV1" s="83"/>
-      <c r="AW1" s="83"/>
-      <c r="AX1" s="83"/>
-      <c r="AY1" s="83"/>
-      <c r="AZ1" s="83"/>
-      <c r="BA1" s="83"/>
-      <c r="BB1" s="83"/>
-      <c r="BC1" s="83"/>
-      <c r="BD1" s="83"/>
-      <c r="BE1" s="83"/>
-      <c r="BF1" s="83"/>
+      <c r="A1" s="88" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="88"/>
+      <c r="C1" s="88"/>
+      <c r="D1" s="88"/>
+      <c r="E1" s="88"/>
+      <c r="F1" s="88"/>
+      <c r="G1" s="88"/>
+      <c r="H1" s="88"/>
+      <c r="I1" s="88"/>
+      <c r="J1" s="88"/>
+      <c r="K1" s="88"/>
+      <c r="L1" s="88"/>
+      <c r="M1" s="88"/>
+      <c r="N1" s="88"/>
+      <c r="O1" s="88"/>
+      <c r="P1" s="88"/>
+      <c r="Q1" s="88"/>
+      <c r="R1" s="88"/>
+      <c r="S1" s="88"/>
+      <c r="T1" s="88"/>
+      <c r="U1" s="88"/>
+      <c r="V1" s="88"/>
+      <c r="W1" s="88"/>
+      <c r="X1" s="88"/>
+      <c r="Y1" s="88"/>
+      <c r="Z1" s="88"/>
+      <c r="AA1" s="88"/>
+      <c r="AB1" s="88"/>
+      <c r="AC1" s="88"/>
+      <c r="AD1" s="88" t="s">
+        <v>0</v>
+      </c>
+      <c r="AE1" s="88"/>
+      <c r="AF1" s="88"/>
+      <c r="AG1" s="88"/>
+      <c r="AH1" s="88"/>
+      <c r="AI1" s="88"/>
+      <c r="AJ1" s="88"/>
+      <c r="AK1" s="88"/>
+      <c r="AL1" s="88"/>
+      <c r="AM1" s="88"/>
+      <c r="AN1" s="88"/>
+      <c r="AO1" s="88"/>
+      <c r="AP1" s="88"/>
+      <c r="AQ1" s="88"/>
+      <c r="AR1" s="88"/>
+      <c r="AS1" s="88"/>
+      <c r="AT1" s="88"/>
+      <c r="AU1" s="88"/>
+      <c r="AV1" s="88"/>
+      <c r="AW1" s="88"/>
+      <c r="AX1" s="88"/>
+      <c r="AY1" s="88"/>
+      <c r="AZ1" s="88"/>
+      <c r="BA1" s="88"/>
+      <c r="BB1" s="88"/>
+      <c r="BC1" s="88"/>
+      <c r="BD1" s="88"/>
+      <c r="BE1" s="88"/>
+      <c r="BF1" s="88"/>
     </row>
     <row r="2" spans="1:59" ht="18">
       <c r="A2" s="23" t="s">
@@ -5536,10 +5567,10 @@
       <c r="BF2" s="67"/>
     </row>
     <row r="3" spans="1:59">
-      <c r="A3" s="84" t="s">
+      <c r="A3" s="89" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="84"/>
+      <c r="B3" s="89"/>
       <c r="C3" s="68"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -5579,10 +5610,10 @@
       <c r="AA3" s="6"/>
       <c r="AB3" s="6"/>
       <c r="AC3" s="6"/>
-      <c r="AD3" s="84" t="s">
+      <c r="AD3" s="89" t="s">
         <v>3</v>
       </c>
-      <c r="AE3" s="84"/>
+      <c r="AE3" s="89"/>
       <c r="AF3" s="68"/>
       <c r="AG3" s="3">
         <v>2</v>
@@ -6057,38 +6088,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:33" ht="18">
-      <c r="A1" s="83" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="83"/>
-      <c r="C1" s="83"/>
-      <c r="D1" s="83"/>
-      <c r="E1" s="83"/>
-      <c r="F1" s="83"/>
-      <c r="G1" s="83"/>
-      <c r="H1" s="83"/>
-      <c r="I1" s="83"/>
-      <c r="J1" s="83"/>
-      <c r="K1" s="83"/>
-      <c r="L1" s="83"/>
-      <c r="M1" s="83"/>
-      <c r="N1" s="83"/>
-      <c r="O1" s="83"/>
-      <c r="P1" s="83"/>
-      <c r="Q1" s="83"/>
-      <c r="R1" s="83"/>
-      <c r="S1" s="83"/>
-      <c r="T1" s="83"/>
-      <c r="U1" s="83"/>
-      <c r="V1" s="83"/>
-      <c r="W1" s="83"/>
-      <c r="X1" s="83"/>
-      <c r="Y1" s="83"/>
-      <c r="Z1" s="83"/>
-      <c r="AA1" s="83"/>
-      <c r="AB1" s="83"/>
-      <c r="AC1" s="83"/>
-      <c r="AD1" s="83"/>
+      <c r="A1" s="88" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="88"/>
+      <c r="C1" s="88"/>
+      <c r="D1" s="88"/>
+      <c r="E1" s="88"/>
+      <c r="F1" s="88"/>
+      <c r="G1" s="88"/>
+      <c r="H1" s="88"/>
+      <c r="I1" s="88"/>
+      <c r="J1" s="88"/>
+      <c r="K1" s="88"/>
+      <c r="L1" s="88"/>
+      <c r="M1" s="88"/>
+      <c r="N1" s="88"/>
+      <c r="O1" s="88"/>
+      <c r="P1" s="88"/>
+      <c r="Q1" s="88"/>
+      <c r="R1" s="88"/>
+      <c r="S1" s="88"/>
+      <c r="T1" s="88"/>
+      <c r="U1" s="88"/>
+      <c r="V1" s="88"/>
+      <c r="W1" s="88"/>
+      <c r="X1" s="88"/>
+      <c r="Y1" s="88"/>
+      <c r="Z1" s="88"/>
+      <c r="AA1" s="88"/>
+      <c r="AB1" s="88"/>
+      <c r="AC1" s="88"/>
+      <c r="AD1" s="88"/>
     </row>
     <row r="2" spans="1:33" ht="18">
       <c r="A2" s="23" t="s">
@@ -6127,10 +6158,10 @@
       <c r="AD2" s="70"/>
     </row>
     <row r="3" spans="1:33" ht="15.75" thickBot="1">
-      <c r="A3" s="84" t="s">
+      <c r="A3" s="89" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="84"/>
+      <c r="B3" s="89"/>
       <c r="C3" s="71"/>
       <c r="D3" s="3">
         <v>3</v>
@@ -6980,68 +7011,68 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:58" ht="18">
-      <c r="A1" s="83" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="83"/>
-      <c r="C1" s="83"/>
-      <c r="D1" s="83"/>
-      <c r="E1" s="83"/>
-      <c r="F1" s="83"/>
-      <c r="G1" s="83"/>
-      <c r="H1" s="83"/>
-      <c r="I1" s="83"/>
-      <c r="J1" s="83"/>
-      <c r="K1" s="83"/>
-      <c r="L1" s="83"/>
-      <c r="M1" s="83"/>
-      <c r="N1" s="83"/>
-      <c r="O1" s="83"/>
-      <c r="P1" s="83"/>
-      <c r="Q1" s="83"/>
-      <c r="R1" s="83"/>
-      <c r="S1" s="83"/>
-      <c r="T1" s="83"/>
-      <c r="U1" s="83"/>
-      <c r="V1" s="83"/>
-      <c r="W1" s="83"/>
-      <c r="X1" s="83"/>
-      <c r="Y1" s="83"/>
-      <c r="Z1" s="83"/>
-      <c r="AA1" s="83"/>
-      <c r="AB1" s="83"/>
-      <c r="AC1" s="83"/>
-      <c r="AD1" s="83" t="s">
-        <v>0</v>
-      </c>
-      <c r="AE1" s="83"/>
-      <c r="AF1" s="83"/>
-      <c r="AG1" s="83"/>
-      <c r="AH1" s="83"/>
-      <c r="AI1" s="83"/>
-      <c r="AJ1" s="83"/>
-      <c r="AK1" s="83"/>
-      <c r="AL1" s="83"/>
-      <c r="AM1" s="83"/>
-      <c r="AN1" s="83"/>
-      <c r="AO1" s="83"/>
-      <c r="AP1" s="83"/>
-      <c r="AQ1" s="83"/>
-      <c r="AR1" s="83"/>
-      <c r="AS1" s="83"/>
-      <c r="AT1" s="83"/>
-      <c r="AU1" s="83"/>
-      <c r="AV1" s="83"/>
-      <c r="AW1" s="83"/>
-      <c r="AX1" s="83"/>
-      <c r="AY1" s="83"/>
-      <c r="AZ1" s="83"/>
-      <c r="BA1" s="83"/>
-      <c r="BB1" s="83"/>
-      <c r="BC1" s="83"/>
-      <c r="BD1" s="83"/>
-      <c r="BE1" s="83"/>
-      <c r="BF1" s="83"/>
+      <c r="A1" s="88" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="88"/>
+      <c r="C1" s="88"/>
+      <c r="D1" s="88"/>
+      <c r="E1" s="88"/>
+      <c r="F1" s="88"/>
+      <c r="G1" s="88"/>
+      <c r="H1" s="88"/>
+      <c r="I1" s="88"/>
+      <c r="J1" s="88"/>
+      <c r="K1" s="88"/>
+      <c r="L1" s="88"/>
+      <c r="M1" s="88"/>
+      <c r="N1" s="88"/>
+      <c r="O1" s="88"/>
+      <c r="P1" s="88"/>
+      <c r="Q1" s="88"/>
+      <c r="R1" s="88"/>
+      <c r="S1" s="88"/>
+      <c r="T1" s="88"/>
+      <c r="U1" s="88"/>
+      <c r="V1" s="88"/>
+      <c r="W1" s="88"/>
+      <c r="X1" s="88"/>
+      <c r="Y1" s="88"/>
+      <c r="Z1" s="88"/>
+      <c r="AA1" s="88"/>
+      <c r="AB1" s="88"/>
+      <c r="AC1" s="88"/>
+      <c r="AD1" s="88" t="s">
+        <v>0</v>
+      </c>
+      <c r="AE1" s="88"/>
+      <c r="AF1" s="88"/>
+      <c r="AG1" s="88"/>
+      <c r="AH1" s="88"/>
+      <c r="AI1" s="88"/>
+      <c r="AJ1" s="88"/>
+      <c r="AK1" s="88"/>
+      <c r="AL1" s="88"/>
+      <c r="AM1" s="88"/>
+      <c r="AN1" s="88"/>
+      <c r="AO1" s="88"/>
+      <c r="AP1" s="88"/>
+      <c r="AQ1" s="88"/>
+      <c r="AR1" s="88"/>
+      <c r="AS1" s="88"/>
+      <c r="AT1" s="88"/>
+      <c r="AU1" s="88"/>
+      <c r="AV1" s="88"/>
+      <c r="AW1" s="88"/>
+      <c r="AX1" s="88"/>
+      <c r="AY1" s="88"/>
+      <c r="AZ1" s="88"/>
+      <c r="BA1" s="88"/>
+      <c r="BB1" s="88"/>
+      <c r="BC1" s="88"/>
+      <c r="BD1" s="88"/>
+      <c r="BE1" s="88"/>
+      <c r="BF1" s="88"/>
     </row>
     <row r="2" spans="1:58" ht="18">
       <c r="A2" s="23" t="s">
@@ -7112,10 +7143,10 @@
       <c r="BF2" s="36"/>
     </row>
     <row r="3" spans="1:58">
-      <c r="A3" s="84" t="s">
+      <c r="A3" s="89" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="84"/>
+      <c r="B3" s="89"/>
       <c r="C3" s="29"/>
       <c r="D3" s="3">
         <v>2</v>
@@ -7155,10 +7186,10 @@
       <c r="AA3" s="6"/>
       <c r="AB3" s="6"/>
       <c r="AC3" s="6"/>
-      <c r="AD3" s="84" t="s">
+      <c r="AD3" s="89" t="s">
         <v>3</v>
       </c>
-      <c r="AE3" s="84"/>
+      <c r="AE3" s="89"/>
       <c r="AF3" s="37"/>
       <c r="AG3" s="3">
         <v>2</v>
@@ -7608,7 +7639,7 @@
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AF8"/>
+  <dimension ref="A1:AG12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="20.5703125" customWidth="1"/>
@@ -7630,47 +7661,50 @@
     <col min="32" max="32" width="13.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:32" ht="18">
-      <c r="A1" s="83" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="83"/>
-      <c r="C1" s="83"/>
-      <c r="D1" s="83"/>
-      <c r="E1" s="83"/>
-      <c r="F1" s="83"/>
-      <c r="G1" s="83"/>
-      <c r="H1" s="83"/>
-      <c r="I1" s="83"/>
-      <c r="J1" s="83"/>
-      <c r="K1" s="83"/>
-      <c r="L1" s="83"/>
-      <c r="M1" s="83"/>
-      <c r="N1" s="83"/>
-      <c r="O1" s="83"/>
-      <c r="P1" s="83"/>
-      <c r="Q1" s="83"/>
-      <c r="R1" s="83"/>
-      <c r="S1" s="83"/>
-      <c r="T1" s="83"/>
-      <c r="U1" s="83"/>
-      <c r="V1" s="83"/>
-      <c r="W1" s="83"/>
-      <c r="X1" s="83"/>
-      <c r="Y1" s="83"/>
-      <c r="Z1" s="83"/>
-      <c r="AA1" s="83"/>
-      <c r="AB1" s="83"/>
-      <c r="AC1" s="83"/>
-    </row>
-    <row r="2" spans="1:32" ht="18">
-      <c r="A2" s="23" t="s">
+    <row r="1" spans="1:33" ht="23.25">
+      <c r="A1" s="84" t="s">
+        <v>112</v>
+      </c>
+      <c r="B1" s="88" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="88"/>
+      <c r="D1" s="88"/>
+      <c r="E1" s="88"/>
+      <c r="F1" s="88"/>
+      <c r="G1" s="88"/>
+      <c r="H1" s="88"/>
+      <c r="I1" s="88"/>
+      <c r="J1" s="88"/>
+      <c r="K1" s="88"/>
+      <c r="L1" s="88"/>
+      <c r="M1" s="88"/>
+      <c r="N1" s="88"/>
+      <c r="O1" s="88"/>
+      <c r="P1" s="88"/>
+      <c r="Q1" s="88"/>
+      <c r="R1" s="88"/>
+      <c r="S1" s="88"/>
+      <c r="T1" s="88"/>
+      <c r="U1" s="88"/>
+      <c r="V1" s="88"/>
+      <c r="W1" s="88"/>
+      <c r="X1" s="88"/>
+      <c r="Y1" s="88"/>
+      <c r="Z1" s="88"/>
+      <c r="AA1" s="88"/>
+      <c r="AB1" s="88"/>
+      <c r="AC1" s="88"/>
+      <c r="AD1" s="88"/>
+    </row>
+    <row r="2" spans="1:33" ht="18">
+      <c r="A2" s="85"/>
+      <c r="B2" s="23" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="23" t="s">
+      <c r="C2" s="23" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="79"/>
       <c r="D2" s="79"/>
       <c r="E2" s="79"/>
       <c r="F2" s="79"/>
@@ -7697,41 +7731,42 @@
       <c r="AA2" s="79"/>
       <c r="AB2" s="79"/>
       <c r="AC2" s="79"/>
-    </row>
-    <row r="3" spans="1:32" ht="15.75" thickBot="1">
-      <c r="A3" s="84" t="s">
+      <c r="AD2" s="79"/>
+    </row>
+    <row r="3" spans="1:33" ht="15.75" thickBot="1">
+      <c r="A3" s="85"/>
+      <c r="B3" s="89" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="84"/>
-      <c r="C3" s="3">
+      <c r="C3" s="89"/>
+      <c r="D3" s="3">
         <v>2</v>
       </c>
-      <c r="D3" s="3"/>
-      <c r="E3" s="4" t="s">
+      <c r="E3" s="3"/>
+      <c r="F3" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F3" s="5"/>
       <c r="G3" s="5"/>
       <c r="H3" s="5"/>
-      <c r="I3" s="6"/>
-      <c r="J3" s="7" t="s">
+      <c r="I3" s="5"/>
+      <c r="J3" s="6"/>
+      <c r="K3" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="K3" s="7" t="s">
+      <c r="L3" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="L3" s="7"/>
-      <c r="M3" s="7" t="s">
+      <c r="M3" s="7"/>
+      <c r="N3" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="N3" s="7">
+      <c r="O3" s="7">
         <v>1</v>
       </c>
-      <c r="O3" s="7"/>
       <c r="P3" s="7"/>
       <c r="Q3" s="7"/>
       <c r="R3" s="7"/>
-      <c r="S3" s="6"/>
+      <c r="S3" s="7"/>
       <c r="T3" s="6"/>
       <c r="U3" s="6"/>
       <c r="V3" s="6"/>
@@ -7742,536 +7777,556 @@
       <c r="AA3" s="6"/>
       <c r="AB3" s="6"/>
       <c r="AC3" s="6"/>
-    </row>
-    <row r="4" spans="1:32" ht="43.5" thickTop="1">
+      <c r="AD3" s="6"/>
+    </row>
+    <row r="4" spans="1:33" ht="29.25" thickTop="1">
       <c r="A4" s="10" t="s">
+        <v>113</v>
+      </c>
+      <c r="B4" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="10" t="s">
+      <c r="C4" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="C4" s="11" t="s">
+      <c r="D4" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="D4" s="11" t="s">
+      <c r="E4" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="E4" s="10" t="s">
+      <c r="F4" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="F4" s="10" t="s">
+      <c r="G4" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="G4" s="12" t="s">
+      <c r="H4" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="H4" s="10" t="s">
+      <c r="I4" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="I4" s="10" t="s">
+      <c r="J4" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="J4" s="13" t="s">
+      <c r="K4" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="K4" s="13" t="s">
+      <c r="L4" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="L4" s="13" t="s">
+      <c r="M4" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="M4" s="14" t="s">
+      <c r="N4" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="N4" s="14" t="s">
+      <c r="O4" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="O4" s="14" t="s">
+      <c r="P4" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="P4" s="14" t="s">
+      <c r="Q4" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="Q4" s="15" t="s">
+      <c r="R4" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="R4" s="14" t="s">
+      <c r="S4" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="S4" s="13" t="s">
+      <c r="T4" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="T4" s="13" t="s">
+      <c r="U4" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="U4" s="10" t="s">
+      <c r="V4" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="V4" s="10" t="s">
+      <c r="W4" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="W4" s="16" t="s">
+      <c r="X4" s="16" t="s">
         <v>27</v>
       </c>
-      <c r="X4" s="16" t="s">
+      <c r="Y4" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="Y4" s="16" t="s">
+      <c r="Z4" s="16" t="s">
         <v>29</v>
       </c>
-      <c r="Z4" s="16" t="s">
+      <c r="AA4" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="AA4" s="16" t="s">
+      <c r="AB4" s="16" t="s">
         <v>37</v>
       </c>
-      <c r="AB4" s="16" t="s">
+      <c r="AC4" s="16" t="s">
         <v>31</v>
       </c>
-      <c r="AC4" s="17" t="s">
+      <c r="AD4" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="AD4" s="51" t="s">
+      <c r="AE4" s="51" t="s">
         <v>58</v>
       </c>
-      <c r="AE4" s="10" t="s">
+      <c r="AF4" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="AF4" s="10" t="s">
+      <c r="AG4" s="10" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="5" spans="1:32">
-      <c r="A5" s="9">
+    <row r="5" spans="1:33">
+      <c r="A5" s="86"/>
+      <c r="B5" s="9">
         <v>1</v>
-      </c>
-      <c r="B5" s="27" t="s">
-        <v>44</v>
       </c>
       <c r="C5" s="27" t="s">
         <v>44</v>
       </c>
-      <c r="D5" s="27"/>
-      <c r="E5" s="9" t="s">
-        <v>33</v>
-      </c>
+      <c r="D5" s="27" t="s">
+        <v>44</v>
+      </c>
+      <c r="E5" s="27"/>
       <c r="F5" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="G5" s="24">
+      <c r="G5" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="H5" s="24">
         <v>2</v>
       </c>
-      <c r="H5" s="9">
+      <c r="I5" s="9">
         <v>250.25</v>
       </c>
-      <c r="I5" s="8">
+      <c r="J5" s="8">
         <v>500.5</v>
       </c>
-      <c r="J5" s="25">
-        <v>0</v>
-      </c>
       <c r="K5" s="25">
         <v>0</v>
       </c>
       <c r="L5" s="25">
         <v>0</v>
       </c>
-      <c r="M5" s="8">
+      <c r="M5" s="25">
+        <v>0</v>
+      </c>
+      <c r="N5" s="8">
         <v>500.5</v>
       </c>
-      <c r="N5" s="8">
-        <f>ROUND(J5*M5%,2)</f>
-        <v>0</v>
-      </c>
-      <c r="O5" s="8"/>
-      <c r="P5" s="8">
-        <f>ROUND(K5*O5%,2)</f>
-        <v>0</v>
-      </c>
+      <c r="O5" s="8">
+        <f>ROUND(K5*N5%,2)</f>
+        <v>0</v>
+      </c>
+      <c r="P5" s="8"/>
       <c r="Q5" s="8">
-        <f>O5-P5</f>
+        <f>ROUND(L5*P5%,2)</f>
         <v>0</v>
       </c>
       <c r="R5" s="8">
-        <f>ROUND(L5*Q5%,2)</f>
-        <v>0</v>
-      </c>
-      <c r="S5" s="26">
-        <f>N5+P5+R5</f>
+        <f>P5-Q5</f>
+        <v>0</v>
+      </c>
+      <c r="S5" s="8">
+        <f>ROUND(M5*R5%,2)</f>
         <v>0</v>
       </c>
       <c r="T5" s="26">
-        <v>0</v>
-      </c>
-      <c r="U5" s="8">
-        <f>(I5-S5)</f>
+        <f>O5+Q5+S5</f>
+        <v>0</v>
+      </c>
+      <c r="U5" s="26">
+        <v>0</v>
+      </c>
+      <c r="V5" s="8">
+        <f>(J5-T5)</f>
         <v>500.5</v>
       </c>
-      <c r="V5" s="24">
+      <c r="W5" s="24">
         <v>88363222</v>
       </c>
-      <c r="W5" s="18">
+      <c r="X5" s="18">
         <v>0.18</v>
       </c>
-      <c r="X5" s="24">
-        <f>IF($C$3=1,ROUND(((U5*W5)/2),2),0)</f>
-        <v>0</v>
-      </c>
       <c r="Y5" s="24">
-        <f>IF($C$3=1,ROUND(((U5*W5)/2),2),0)</f>
+        <f>IF($D$3=1,ROUND(((V5*X5)/2),2),0)</f>
         <v>0</v>
       </c>
       <c r="Z5" s="24">
-        <f>IF($C$3=2,ROUND(((U5*W5)),2),0)</f>
+        <f>IF($D$3=1,ROUND(((V5*X5)/2),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="AA5" s="24">
+        <f>IF($D$3=2,ROUND(((V5*X5)),2),0)</f>
         <v>90.09</v>
       </c>
-      <c r="AA5" s="24">
-        <v>0</v>
-      </c>
       <c r="AB5" s="24">
-        <f>X5+Y5+Z5</f>
+        <v>0</v>
+      </c>
+      <c r="AC5" s="24">
+        <f>Y5+Z5+AA5</f>
         <v>90.09</v>
       </c>
-      <c r="AC5" s="24">
-        <f>U5+AB5</f>
+      <c r="AD5" s="24">
+        <f>V5+AC5</f>
         <v>590.59</v>
       </c>
-      <c r="AD5" s="52" t="s">
+      <c r="AE5" s="52" t="s">
         <v>57</v>
       </c>
-      <c r="AE5" s="46" t="s">
+      <c r="AF5" s="46" t="s">
         <v>42</v>
       </c>
-      <c r="AF5" s="46" t="s">
+      <c r="AG5" s="46" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="6" spans="1:32" ht="16.5" customHeight="1">
-      <c r="A6" s="9">
+    <row r="6" spans="1:33" ht="16.5" customHeight="1">
+      <c r="A6" s="86"/>
+      <c r="B6" s="9">
         <v>2</v>
       </c>
-      <c r="B6" s="45" t="s">
+      <c r="C6" s="45" t="s">
         <v>51</v>
       </c>
-      <c r="C6" s="45" t="s">
+      <c r="D6" s="45" t="s">
         <v>50</v>
       </c>
-      <c r="D6" s="45"/>
-      <c r="E6" s="9" t="s">
-        <v>33</v>
-      </c>
+      <c r="E6" s="45"/>
       <c r="F6" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="G6" s="24">
+      <c r="G6" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="H6" s="24">
         <v>1</v>
       </c>
-      <c r="H6" s="9">
+      <c r="I6" s="9">
         <v>3458</v>
       </c>
-      <c r="I6" s="8">
+      <c r="J6" s="8">
         <v>3458</v>
       </c>
-      <c r="J6" s="25">
-        <v>0</v>
-      </c>
       <c r="K6" s="25">
         <v>0</v>
       </c>
       <c r="L6" s="25">
         <v>0</v>
       </c>
-      <c r="M6" s="8">
+      <c r="M6" s="25">
+        <v>0</v>
+      </c>
+      <c r="N6" s="8">
         <v>3458</v>
       </c>
-      <c r="N6" s="8">
-        <f t="shared" ref="N6:N8" si="0">ROUND(J6*M6%,2)</f>
-        <v>0</v>
-      </c>
       <c r="O6" s="8">
-        <f t="shared" ref="O6:O8" si="1">I6-N6</f>
+        <f t="shared" ref="O6:O8" si="0">ROUND(K6*N6%,2)</f>
+        <v>0</v>
+      </c>
+      <c r="P6" s="8">
+        <f t="shared" ref="P6:P8" si="1">J6-O6</f>
         <v>3458</v>
       </c>
-      <c r="P6" s="8">
-        <f t="shared" ref="P6:P8" si="2">ROUND(K6*O6%,2)</f>
-        <v>0</v>
-      </c>
       <c r="Q6" s="8">
-        <f t="shared" ref="Q6:Q8" si="3">O6-P6</f>
+        <f t="shared" ref="Q6:Q8" si="2">ROUND(L6*P6%,2)</f>
+        <v>0</v>
+      </c>
+      <c r="R6" s="8">
+        <f t="shared" ref="R6:R8" si="3">P6-Q6</f>
         <v>3458</v>
       </c>
-      <c r="R6" s="8">
-        <f t="shared" ref="R6:R8" si="4">ROUND(L6*Q6%,2)</f>
-        <v>0</v>
-      </c>
-      <c r="S6" s="26">
-        <f t="shared" ref="S6:S8" si="5">N6+P6+R6</f>
+      <c r="S6" s="8">
+        <f t="shared" ref="S6:S8" si="4">ROUND(M6*R6%,2)</f>
         <v>0</v>
       </c>
       <c r="T6" s="26">
-        <v>0</v>
-      </c>
-      <c r="U6" s="8">
-        <f>(I6-S6)</f>
+        <f t="shared" ref="T6:T8" si="5">O6+Q6+S6</f>
+        <v>0</v>
+      </c>
+      <c r="U6" s="26">
+        <v>0</v>
+      </c>
+      <c r="V6" s="8">
+        <f>(J6-T6)</f>
         <v>3458</v>
       </c>
-      <c r="V6" s="24">
+      <c r="W6" s="24">
         <v>88363222</v>
       </c>
-      <c r="W6" s="18">
+      <c r="X6" s="18">
         <v>0.18</v>
       </c>
-      <c r="X6" s="24">
-        <f>IF($C$3=1,ROUND(((U6*W6)/2),2),0)</f>
-        <v>0</v>
-      </c>
       <c r="Y6" s="24">
-        <f>IF($C$3=1,ROUND(((U6*W6)/2),2),0)</f>
+        <f>IF($D$3=1,ROUND(((V6*X6)/2),2),0)</f>
         <v>0</v>
       </c>
       <c r="Z6" s="24">
-        <f>IF($C$3=2,ROUND(((U6*W6)),2),0)</f>
+        <f>IF($D$3=1,ROUND(((V6*X6)/2),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="AA6" s="24">
+        <f>IF($D$3=2,ROUND(((V6*X6)),2),0)</f>
         <v>622.44000000000005</v>
       </c>
-      <c r="AA6" s="24">
-        <v>0</v>
-      </c>
       <c r="AB6" s="24">
-        <f>X6+Y6+Z6</f>
+        <v>0</v>
+      </c>
+      <c r="AC6" s="24">
+        <f>Y6+Z6+AA6</f>
         <v>622.44000000000005</v>
       </c>
-      <c r="AC6" s="24">
-        <f>U6+AB6</f>
+      <c r="AD6" s="24">
+        <f>V6+AC6</f>
         <v>4080.44</v>
       </c>
-      <c r="AD6" s="53" t="s">
+      <c r="AE6" s="53" t="s">
         <v>57</v>
       </c>
-      <c r="AE6" s="46" t="s">
+      <c r="AF6" s="46" t="s">
         <v>53</v>
       </c>
-      <c r="AF6" s="46" t="s">
+      <c r="AG6" s="46" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="7" spans="1:32">
-      <c r="A7" s="46">
+    <row r="7" spans="1:33">
+      <c r="A7" s="86"/>
+      <c r="B7" s="46">
         <v>4</v>
       </c>
-      <c r="B7" s="46"/>
       <c r="C7" s="46"/>
-      <c r="D7" s="46" t="s">
+      <c r="D7" s="46"/>
+      <c r="E7" s="46" t="s">
         <v>56</v>
-      </c>
-      <c r="E7" s="47" t="s">
-        <v>33</v>
       </c>
       <c r="F7" s="47" t="s">
         <v>33</v>
       </c>
-      <c r="G7" s="48">
+      <c r="G7" s="47" t="s">
+        <v>33</v>
+      </c>
+      <c r="H7" s="48">
         <v>1</v>
       </c>
-      <c r="H7" s="47">
+      <c r="I7" s="47">
         <v>609</v>
       </c>
-      <c r="I7" s="49">
+      <c r="J7" s="49">
         <v>609</v>
       </c>
-      <c r="J7" s="46">
-        <v>0</v>
-      </c>
       <c r="K7" s="46">
         <v>0</v>
       </c>
       <c r="L7" s="46">
         <v>0</v>
       </c>
-      <c r="M7" s="50">
+      <c r="M7" s="46">
+        <v>0</v>
+      </c>
+      <c r="N7" s="50">
         <v>609</v>
       </c>
-      <c r="N7" s="8">
+      <c r="O7" s="8">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="O7" s="8">
+      <c r="P7" s="8">
         <f t="shared" si="1"/>
         <v>609</v>
       </c>
-      <c r="P7" s="8">
+      <c r="Q7" s="8">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="Q7" s="8">
+      <c r="R7" s="8">
         <f t="shared" si="3"/>
         <v>609</v>
       </c>
-      <c r="R7" s="8">
+      <c r="S7" s="8">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="S7" s="26">
+      <c r="T7" s="26">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="T7" s="26">
-        <v>0</v>
-      </c>
-      <c r="U7" s="8">
-        <f>(I7-S7)</f>
+      <c r="U7" s="26">
+        <v>0</v>
+      </c>
+      <c r="V7" s="8">
+        <f>(J7-T7)</f>
         <v>609</v>
       </c>
-      <c r="V7" s="24">
+      <c r="W7" s="24">
         <v>75052200</v>
       </c>
-      <c r="W7" s="18">
-        <v>0.18</v>
-      </c>
-      <c r="X7" s="24">
-        <f>IF($C$3=1,ROUND(((U7*W7)/2),2),0)</f>
-        <v>0</v>
+      <c r="X7" s="18">
+        <v>0.05</v>
       </c>
       <c r="Y7" s="24">
-        <f>IF($C$3=1,ROUND(((U7*W7)/2),2),0)</f>
+        <f>IF($D$3=1,ROUND(((V7*X7)/2),2),0)</f>
         <v>0</v>
       </c>
       <c r="Z7" s="24">
-        <f>IF($C$3=2,ROUND(((U7*W7)),2),0)</f>
-        <v>109.62</v>
+        <f>IF($D$3=1,ROUND(((V7*X7)/2),2),0)</f>
+        <v>0</v>
       </c>
       <c r="AA7" s="24">
-        <v>0</v>
+        <f>IF($D$3=2,ROUND(((V7*X7)),2),0)</f>
+        <v>30.45</v>
       </c>
       <c r="AB7" s="24">
-        <f>X7+Y7+Z7</f>
-        <v>109.62</v>
+        <v>0</v>
       </c>
       <c r="AC7" s="24">
-        <f>U7+AB7</f>
-        <v>718.62</v>
-      </c>
-      <c r="AD7" s="52" t="s">
+        <f>Y7+Z7+AA7</f>
+        <v>30.45</v>
+      </c>
+      <c r="AD7" s="24">
+        <f>V7+AC7</f>
+        <v>639.45000000000005</v>
+      </c>
+      <c r="AE7" s="52" t="s">
         <v>59</v>
       </c>
-      <c r="AE7" s="46">
+      <c r="AF7" s="46">
         <v>5050121000</v>
       </c>
-      <c r="AF7" s="46" t="s">
+      <c r="AG7" s="46" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="8" spans="1:32">
-      <c r="A8" s="9">
+    <row r="8" spans="1:33">
+      <c r="A8" s="86"/>
+      <c r="B8" s="9">
         <v>3</v>
-      </c>
-      <c r="B8" s="27" t="s">
-        <v>52</v>
       </c>
       <c r="C8" s="27" t="s">
         <v>52</v>
       </c>
-      <c r="D8" s="27"/>
-      <c r="E8" s="9" t="s">
-        <v>33</v>
-      </c>
+      <c r="D8" s="27" t="s">
+        <v>52</v>
+      </c>
+      <c r="E8" s="27"/>
       <c r="F8" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="G8" s="24">
+      <c r="G8" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="H8" s="24">
         <v>3</v>
       </c>
-      <c r="H8" s="9">
+      <c r="I8" s="9">
         <v>675</v>
       </c>
-      <c r="I8" s="8">
+      <c r="J8" s="8">
         <v>2025</v>
       </c>
-      <c r="J8" s="25">
-        <v>0</v>
-      </c>
       <c r="K8" s="25">
         <v>0</v>
       </c>
       <c r="L8" s="25">
         <v>0</v>
       </c>
-      <c r="M8" s="8">
+      <c r="M8" s="25">
+        <v>0</v>
+      </c>
+      <c r="N8" s="8">
         <v>2025</v>
       </c>
-      <c r="N8" s="8">
+      <c r="O8" s="8">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="O8" s="8">
+      <c r="P8" s="8">
         <f t="shared" si="1"/>
         <v>2025</v>
       </c>
-      <c r="P8" s="8">
+      <c r="Q8" s="8">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="Q8" s="8">
+      <c r="R8" s="8">
         <f t="shared" si="3"/>
         <v>2025</v>
       </c>
-      <c r="R8" s="8">
+      <c r="S8" s="8">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="S8" s="26">
+      <c r="T8" s="26">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="T8" s="26">
-        <v>0</v>
-      </c>
-      <c r="U8" s="8">
-        <f>(I8-S8)</f>
+      <c r="U8" s="26">
+        <v>0</v>
+      </c>
+      <c r="V8" s="8">
+        <f>(J8-T8)</f>
         <v>2025</v>
       </c>
-      <c r="V8" s="24">
+      <c r="W8" s="24">
         <v>88363222</v>
       </c>
-      <c r="W8" s="18">
+      <c r="X8" s="18">
         <v>0.18</v>
       </c>
-      <c r="X8" s="24">
-        <f>IF($C$3=1,ROUND(((U8*W8)/2),2),0)</f>
-        <v>0</v>
-      </c>
       <c r="Y8" s="24">
-        <f>IF($C$3=1,ROUND(((U8*W8)/2),2),0)</f>
+        <f>IF($D$3=1,ROUND(((V8*X8)/2),2),0)</f>
         <v>0</v>
       </c>
       <c r="Z8" s="24">
-        <f>IF($C$3=2,ROUND(((U8*W8)),2),0)</f>
+        <f>IF($D$3=1,ROUND(((V8*X8)/2),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="AA8" s="24">
+        <f>IF($D$3=2,ROUND(((V8*X8)),2),0)</f>
         <v>364.5</v>
       </c>
-      <c r="AA8" s="24">
-        <v>0</v>
-      </c>
       <c r="AB8" s="24">
-        <f>X8+Y8+Z8</f>
+        <v>0</v>
+      </c>
+      <c r="AC8" s="24">
+        <f>Y8+Z8+AA8</f>
         <v>364.5</v>
       </c>
-      <c r="AC8" s="24">
-        <f>U8+AB8</f>
+      <c r="AD8" s="24">
+        <f>V8+AC8</f>
         <v>2389.5</v>
       </c>
-      <c r="AD8" s="53" t="s">
+      <c r="AE8" s="53" t="s">
         <v>57</v>
       </c>
-      <c r="AE8" s="46" t="s">
+      <c r="AF8" s="46" t="s">
         <v>54</v>
       </c>
-      <c r="AF8" s="46" t="s">
+      <c r="AG8" s="46" t="s">
         <v>61</v>
       </c>
+    </row>
+    <row r="9" spans="1:33">
+      <c r="A9" s="85"/>
+    </row>
+    <row r="10" spans="1:33">
+      <c r="A10" s="85"/>
+    </row>
+    <row r="11" spans="1:33">
+      <c r="A11" s="85"/>
+    </row>
+    <row r="12" spans="1:33">
+      <c r="A12" s="85"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:AC1"/>
-    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="B1:AD1"/>
+    <mergeCell ref="B3:C3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -8994,36 +9049,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:31" ht="18">
-      <c r="A1" s="83" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="83"/>
-      <c r="C1" s="83"/>
-      <c r="D1" s="83"/>
-      <c r="E1" s="83"/>
-      <c r="F1" s="83"/>
-      <c r="G1" s="83"/>
-      <c r="H1" s="83"/>
-      <c r="I1" s="83"/>
-      <c r="J1" s="83"/>
-      <c r="K1" s="83"/>
-      <c r="L1" s="83"/>
-      <c r="M1" s="83"/>
-      <c r="N1" s="83"/>
-      <c r="O1" s="83"/>
-      <c r="P1" s="83"/>
-      <c r="Q1" s="83"/>
-      <c r="R1" s="83"/>
-      <c r="S1" s="83"/>
-      <c r="T1" s="83"/>
-      <c r="U1" s="83"/>
-      <c r="V1" s="83"/>
-      <c r="W1" s="83"/>
-      <c r="X1" s="83"/>
-      <c r="Y1" s="83"/>
-      <c r="Z1" s="83"/>
-      <c r="AA1" s="83"/>
-      <c r="AB1" s="83"/>
+      <c r="A1" s="88" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="88"/>
+      <c r="C1" s="88"/>
+      <c r="D1" s="88"/>
+      <c r="E1" s="88"/>
+      <c r="F1" s="88"/>
+      <c r="G1" s="88"/>
+      <c r="H1" s="88"/>
+      <c r="I1" s="88"/>
+      <c r="J1" s="88"/>
+      <c r="K1" s="88"/>
+      <c r="L1" s="88"/>
+      <c r="M1" s="88"/>
+      <c r="N1" s="88"/>
+      <c r="O1" s="88"/>
+      <c r="P1" s="88"/>
+      <c r="Q1" s="88"/>
+      <c r="R1" s="88"/>
+      <c r="S1" s="88"/>
+      <c r="T1" s="88"/>
+      <c r="U1" s="88"/>
+      <c r="V1" s="88"/>
+      <c r="W1" s="88"/>
+      <c r="X1" s="88"/>
+      <c r="Y1" s="88"/>
+      <c r="Z1" s="88"/>
+      <c r="AA1" s="88"/>
+      <c r="AB1" s="88"/>
     </row>
     <row r="2" spans="1:31" ht="18">
       <c r="A2" s="23" t="s">
@@ -9060,10 +9115,10 @@
       <c r="AB2" s="80"/>
     </row>
     <row r="3" spans="1:31" ht="15.75" thickBot="1">
-      <c r="A3" s="84" t="s">
+      <c r="A3" s="89" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="84"/>
+      <c r="B3" s="89"/>
       <c r="C3" s="81"/>
       <c r="D3" s="3">
         <v>2</v>
@@ -9851,6 +9906,679 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:AF8"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="2" max="2" width="20.5703125" customWidth="1"/>
+    <col min="3" max="3" width="29.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="29.140625" customWidth="1"/>
+    <col min="5" max="5" width="19.28515625" customWidth="1"/>
+    <col min="6" max="6" width="16.28515625" customWidth="1"/>
+    <col min="7" max="7" width="24.42578125" customWidth="1"/>
+    <col min="8" max="8" width="20.28515625" customWidth="1"/>
+    <col min="9" max="9" width="20" customWidth="1"/>
+    <col min="13" max="13" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="13.7109375" customWidth="1"/>
+    <col min="18" max="18" width="13" customWidth="1"/>
+    <col min="19" max="19" width="14.42578125" customWidth="1"/>
+    <col min="20" max="20" width="18.42578125" customWidth="1"/>
+    <col min="21" max="21" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="13.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:32" ht="18">
+      <c r="A1" s="88" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="88"/>
+      <c r="C1" s="88"/>
+      <c r="D1" s="88"/>
+      <c r="E1" s="88"/>
+      <c r="F1" s="88"/>
+      <c r="G1" s="88"/>
+      <c r="H1" s="88"/>
+      <c r="I1" s="88"/>
+      <c r="J1" s="88"/>
+      <c r="K1" s="88"/>
+      <c r="L1" s="88"/>
+      <c r="M1" s="88"/>
+      <c r="N1" s="88"/>
+      <c r="O1" s="88"/>
+      <c r="P1" s="88"/>
+      <c r="Q1" s="88"/>
+      <c r="R1" s="88"/>
+      <c r="S1" s="88"/>
+      <c r="T1" s="88"/>
+      <c r="U1" s="88"/>
+      <c r="V1" s="88"/>
+      <c r="W1" s="88"/>
+      <c r="X1" s="88"/>
+      <c r="Y1" s="88"/>
+      <c r="Z1" s="88"/>
+      <c r="AA1" s="88"/>
+      <c r="AB1" s="88"/>
+      <c r="AC1" s="88"/>
+    </row>
+    <row r="2" spans="1:32" ht="18">
+      <c r="A2" s="23" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="23" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" s="87"/>
+      <c r="D2" s="87"/>
+      <c r="E2" s="87"/>
+      <c r="F2" s="87"/>
+      <c r="G2" s="87"/>
+      <c r="H2" s="87"/>
+      <c r="I2" s="87"/>
+      <c r="J2" s="87"/>
+      <c r="K2" s="87"/>
+      <c r="L2" s="87"/>
+      <c r="M2" s="87"/>
+      <c r="N2" s="87"/>
+      <c r="O2" s="87"/>
+      <c r="P2" s="87"/>
+      <c r="Q2" s="87"/>
+      <c r="R2" s="87"/>
+      <c r="S2" s="87"/>
+      <c r="T2" s="87"/>
+      <c r="U2" s="87"/>
+      <c r="V2" s="87"/>
+      <c r="W2" s="87"/>
+      <c r="X2" s="87"/>
+      <c r="Y2" s="87"/>
+      <c r="Z2" s="87"/>
+      <c r="AA2" s="87"/>
+      <c r="AB2" s="87"/>
+      <c r="AC2" s="87"/>
+    </row>
+    <row r="3" spans="1:32" ht="15.75" thickBot="1">
+      <c r="A3" s="89" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="89"/>
+      <c r="C3" s="3">
+        <v>2</v>
+      </c>
+      <c r="D3" s="3"/>
+      <c r="E3" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="F3" s="5"/>
+      <c r="G3" s="5"/>
+      <c r="H3" s="5"/>
+      <c r="I3" s="6"/>
+      <c r="J3" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="K3" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="L3" s="7"/>
+      <c r="M3" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="N3" s="7">
+        <v>1</v>
+      </c>
+      <c r="O3" s="7"/>
+      <c r="P3" s="7"/>
+      <c r="Q3" s="7"/>
+      <c r="R3" s="7"/>
+      <c r="S3" s="6"/>
+      <c r="T3" s="6"/>
+      <c r="U3" s="6"/>
+      <c r="V3" s="6"/>
+      <c r="W3" s="6"/>
+      <c r="X3" s="6"/>
+      <c r="Y3" s="6"/>
+      <c r="Z3" s="6"/>
+      <c r="AA3" s="6"/>
+      <c r="AB3" s="6"/>
+      <c r="AC3" s="6"/>
+    </row>
+    <row r="4" spans="1:32" ht="43.5" thickTop="1">
+      <c r="A4" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="D4" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="E4" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="F4" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="G4" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="H4" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="I4" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="J4" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="K4" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="L4" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="M4" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="N4" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="O4" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="P4" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q4" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="R4" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="S4" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="T4" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="U4" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="V4" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="W4" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="X4" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y4" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="Z4" s="16" t="s">
+        <v>30</v>
+      </c>
+      <c r="AA4" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="AB4" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="AC4" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="AD4" s="51" t="s">
+        <v>58</v>
+      </c>
+      <c r="AE4" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="AF4" s="10" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="5" spans="1:32">
+      <c r="A5" s="9">
+        <v>1</v>
+      </c>
+      <c r="B5" s="27" t="s">
+        <v>44</v>
+      </c>
+      <c r="C5" s="27" t="s">
+        <v>44</v>
+      </c>
+      <c r="D5" s="27"/>
+      <c r="E5" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="F5" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="G5" s="24">
+        <v>2</v>
+      </c>
+      <c r="H5" s="9">
+        <v>250.25</v>
+      </c>
+      <c r="I5" s="8">
+        <v>500.5</v>
+      </c>
+      <c r="J5" s="25">
+        <v>0</v>
+      </c>
+      <c r="K5" s="25">
+        <v>0</v>
+      </c>
+      <c r="L5" s="25">
+        <v>0</v>
+      </c>
+      <c r="M5" s="8">
+        <v>500.5</v>
+      </c>
+      <c r="N5" s="8">
+        <f>ROUND(J5*M5%,2)</f>
+        <v>0</v>
+      </c>
+      <c r="O5" s="8">
+        <v>500.5</v>
+      </c>
+      <c r="P5" s="8">
+        <f>ROUND(K5*O5%,2)</f>
+        <v>0</v>
+      </c>
+      <c r="Q5" s="8">
+        <f>O5-P5</f>
+        <v>500.5</v>
+      </c>
+      <c r="R5" s="8">
+        <f>ROUND(L5*Q5%,2)</f>
+        <v>0</v>
+      </c>
+      <c r="S5" s="26">
+        <f>N5+P5+R5</f>
+        <v>0</v>
+      </c>
+      <c r="T5" s="26">
+        <v>0</v>
+      </c>
+      <c r="U5" s="8">
+        <f>(I5-S5)</f>
+        <v>500.5</v>
+      </c>
+      <c r="V5" s="24">
+        <v>88363222</v>
+      </c>
+      <c r="W5" s="18">
+        <v>0.18</v>
+      </c>
+      <c r="X5" s="24">
+        <f>IF($C$3=1,ROUND(((U5*W5)/2),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="Y5" s="24">
+        <f>IF($C$3=1,ROUND(((U5*W5)/2),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="Z5" s="24">
+        <f>IF($C$3=2,ROUND(((U5*W5)),2),0)</f>
+        <v>90.09</v>
+      </c>
+      <c r="AA5" s="24">
+        <v>0</v>
+      </c>
+      <c r="AB5" s="24">
+        <f>X5+Y5+Z5</f>
+        <v>90.09</v>
+      </c>
+      <c r="AC5" s="24">
+        <f>U5+AB5</f>
+        <v>590.59</v>
+      </c>
+      <c r="AD5" s="52" t="s">
+        <v>57</v>
+      </c>
+      <c r="AE5" s="46" t="s">
+        <v>42</v>
+      </c>
+      <c r="AF5" s="46" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="6" spans="1:32" ht="16.5" customHeight="1">
+      <c r="A6" s="9">
+        <v>2</v>
+      </c>
+      <c r="B6" s="45" t="s">
+        <v>51</v>
+      </c>
+      <c r="C6" s="45" t="s">
+        <v>50</v>
+      </c>
+      <c r="D6" s="45"/>
+      <c r="E6" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="F6" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="G6" s="24">
+        <v>1</v>
+      </c>
+      <c r="H6" s="9">
+        <v>3458</v>
+      </c>
+      <c r="I6" s="8">
+        <v>3458</v>
+      </c>
+      <c r="J6" s="25">
+        <v>0</v>
+      </c>
+      <c r="K6" s="25">
+        <v>0</v>
+      </c>
+      <c r="L6" s="25">
+        <v>0</v>
+      </c>
+      <c r="M6" s="8">
+        <v>3458</v>
+      </c>
+      <c r="N6" s="8">
+        <f t="shared" ref="N6:N8" si="0">ROUND(J6*M6%,2)</f>
+        <v>0</v>
+      </c>
+      <c r="O6" s="8">
+        <f t="shared" ref="O6:O8" si="1">I6-N6</f>
+        <v>3458</v>
+      </c>
+      <c r="P6" s="8">
+        <f t="shared" ref="P6:P8" si="2">ROUND(K6*O6%,2)</f>
+        <v>0</v>
+      </c>
+      <c r="Q6" s="8">
+        <f t="shared" ref="Q6:Q8" si="3">O6-P6</f>
+        <v>3458</v>
+      </c>
+      <c r="R6" s="8">
+        <f t="shared" ref="R6:R8" si="4">ROUND(L6*Q6%,2)</f>
+        <v>0</v>
+      </c>
+      <c r="S6" s="26">
+        <f t="shared" ref="S6:S8" si="5">N6+P6+R6</f>
+        <v>0</v>
+      </c>
+      <c r="T6" s="26">
+        <v>0</v>
+      </c>
+      <c r="U6" s="8">
+        <f>(I6-S6)</f>
+        <v>3458</v>
+      </c>
+      <c r="V6" s="24">
+        <v>88363222</v>
+      </c>
+      <c r="W6" s="18">
+        <v>0.18</v>
+      </c>
+      <c r="X6" s="24">
+        <f>IF($C$3=1,ROUND(((U6*W6)/2),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="Y6" s="24">
+        <f>IF($C$3=1,ROUND(((U6*W6)/2),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="Z6" s="24">
+        <f>IF($C$3=2,ROUND(((U6*W6)),2),0)</f>
+        <v>622.44000000000005</v>
+      </c>
+      <c r="AA6" s="24">
+        <v>0</v>
+      </c>
+      <c r="AB6" s="24">
+        <f>X6+Y6+Z6</f>
+        <v>622.44000000000005</v>
+      </c>
+      <c r="AC6" s="24">
+        <f>U6+AB6</f>
+        <v>4080.44</v>
+      </c>
+      <c r="AD6" s="53" t="s">
+        <v>57</v>
+      </c>
+      <c r="AE6" s="46" t="s">
+        <v>53</v>
+      </c>
+      <c r="AF6" s="46" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="7" spans="1:32">
+      <c r="A7" s="46">
+        <v>4</v>
+      </c>
+      <c r="B7" s="46"/>
+      <c r="C7" s="46"/>
+      <c r="D7" s="46" t="s">
+        <v>56</v>
+      </c>
+      <c r="E7" s="47" t="s">
+        <v>33</v>
+      </c>
+      <c r="F7" s="47" t="s">
+        <v>33</v>
+      </c>
+      <c r="G7" s="48">
+        <v>1</v>
+      </c>
+      <c r="H7" s="47">
+        <v>609</v>
+      </c>
+      <c r="I7" s="49">
+        <v>609</v>
+      </c>
+      <c r="J7" s="46">
+        <v>0</v>
+      </c>
+      <c r="K7" s="46">
+        <v>0</v>
+      </c>
+      <c r="L7" s="46">
+        <v>0</v>
+      </c>
+      <c r="M7" s="50">
+        <v>609</v>
+      </c>
+      <c r="N7" s="8">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="O7" s="8">
+        <f t="shared" si="1"/>
+        <v>609</v>
+      </c>
+      <c r="P7" s="8">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="Q7" s="8">
+        <f t="shared" si="3"/>
+        <v>609</v>
+      </c>
+      <c r="R7" s="8">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="S7" s="26">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="T7" s="26">
+        <v>0</v>
+      </c>
+      <c r="U7" s="8">
+        <f>(I7-S7)</f>
+        <v>609</v>
+      </c>
+      <c r="V7" s="24">
+        <v>75052200</v>
+      </c>
+      <c r="W7" s="18">
+        <v>0.05</v>
+      </c>
+      <c r="X7" s="24">
+        <f>IF($C$3=1,ROUND(((U7*W7)/2),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="Y7" s="24">
+        <f>IF($C$3=1,ROUND(((U7*W7)/2),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="Z7" s="24">
+        <f>IF($C$3=2,ROUND(((U7*W7)),2),0)</f>
+        <v>30.45</v>
+      </c>
+      <c r="AA7" s="24">
+        <v>0</v>
+      </c>
+      <c r="AB7" s="24">
+        <f>X7+Y7+Z7</f>
+        <v>30.45</v>
+      </c>
+      <c r="AC7" s="24">
+        <f>U7+AB7</f>
+        <v>639.45000000000005</v>
+      </c>
+      <c r="AD7" s="52" t="s">
+        <v>59</v>
+      </c>
+      <c r="AE7" s="46">
+        <v>5050121000</v>
+      </c>
+      <c r="AF7" s="46" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="8" spans="1:32">
+      <c r="A8" s="9">
+        <v>3</v>
+      </c>
+      <c r="B8" s="27" t="s">
+        <v>52</v>
+      </c>
+      <c r="C8" s="27" t="s">
+        <v>52</v>
+      </c>
+      <c r="D8" s="27"/>
+      <c r="E8" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="F8" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="G8" s="24">
+        <v>3</v>
+      </c>
+      <c r="H8" s="9">
+        <v>675</v>
+      </c>
+      <c r="I8" s="8">
+        <v>2025</v>
+      </c>
+      <c r="J8" s="25">
+        <v>0</v>
+      </c>
+      <c r="K8" s="25">
+        <v>0</v>
+      </c>
+      <c r="L8" s="25">
+        <v>0</v>
+      </c>
+      <c r="M8" s="8">
+        <v>2025</v>
+      </c>
+      <c r="N8" s="8">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="O8" s="8">
+        <f t="shared" si="1"/>
+        <v>2025</v>
+      </c>
+      <c r="P8" s="8">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="Q8" s="8">
+        <f t="shared" si="3"/>
+        <v>2025</v>
+      </c>
+      <c r="R8" s="8">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="S8" s="26">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="T8" s="26">
+        <v>0</v>
+      </c>
+      <c r="U8" s="8">
+        <f>(I8-S8)</f>
+        <v>2025</v>
+      </c>
+      <c r="V8" s="24">
+        <v>88363222</v>
+      </c>
+      <c r="W8" s="18">
+        <v>0.18</v>
+      </c>
+      <c r="X8" s="24">
+        <f>IF($C$3=1,ROUND(((U8*W8)/2),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="Y8" s="24">
+        <f>IF($C$3=1,ROUND(((U8*W8)/2),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="Z8" s="24">
+        <f>IF($C$3=2,ROUND(((U8*W8)),2),0)</f>
+        <v>364.5</v>
+      </c>
+      <c r="AA8" s="24">
+        <v>0</v>
+      </c>
+      <c r="AB8" s="24">
+        <f>X8+Y8+Z8</f>
+        <v>364.5</v>
+      </c>
+      <c r="AC8" s="24">
+        <f>U8+AB8</f>
+        <v>2389.5</v>
+      </c>
+      <c r="AD8" s="53" t="s">
+        <v>57</v>
+      </c>
+      <c r="AE8" s="46" t="s">
+        <v>54</v>
+      </c>
+      <c r="AF8" s="46" t="s">
+        <v>61</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:AC1"/>
+    <mergeCell ref="A3:B3"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:AC6"/>
@@ -9873,37 +10601,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="18">
-      <c r="A1" s="83" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="83"/>
-      <c r="C1" s="83"/>
-      <c r="D1" s="83"/>
-      <c r="E1" s="83"/>
-      <c r="F1" s="83"/>
-      <c r="G1" s="83"/>
-      <c r="H1" s="83"/>
-      <c r="I1" s="83"/>
-      <c r="J1" s="83"/>
-      <c r="K1" s="83"/>
-      <c r="L1" s="83"/>
-      <c r="M1" s="83"/>
-      <c r="N1" s="83"/>
-      <c r="O1" s="83"/>
-      <c r="P1" s="83"/>
-      <c r="Q1" s="83"/>
-      <c r="R1" s="83"/>
-      <c r="S1" s="83"/>
-      <c r="T1" s="83"/>
-      <c r="U1" s="83"/>
-      <c r="V1" s="83"/>
-      <c r="W1" s="83"/>
-      <c r="X1" s="83"/>
-      <c r="Y1" s="83"/>
-      <c r="Z1" s="83"/>
-      <c r="AA1" s="83"/>
-      <c r="AB1" s="83"/>
-      <c r="AC1" s="83"/>
+      <c r="A1" s="88" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="88"/>
+      <c r="C1" s="88"/>
+      <c r="D1" s="88"/>
+      <c r="E1" s="88"/>
+      <c r="F1" s="88"/>
+      <c r="G1" s="88"/>
+      <c r="H1" s="88"/>
+      <c r="I1" s="88"/>
+      <c r="J1" s="88"/>
+      <c r="K1" s="88"/>
+      <c r="L1" s="88"/>
+      <c r="M1" s="88"/>
+      <c r="N1" s="88"/>
+      <c r="O1" s="88"/>
+      <c r="P1" s="88"/>
+      <c r="Q1" s="88"/>
+      <c r="R1" s="88"/>
+      <c r="S1" s="88"/>
+      <c r="T1" s="88"/>
+      <c r="U1" s="88"/>
+      <c r="V1" s="88"/>
+      <c r="W1" s="88"/>
+      <c r="X1" s="88"/>
+      <c r="Y1" s="88"/>
+      <c r="Z1" s="88"/>
+      <c r="AA1" s="88"/>
+      <c r="AB1" s="88"/>
+      <c r="AC1" s="88"/>
     </row>
     <row r="2" spans="1:29" ht="18">
       <c r="A2" s="23" t="s">
@@ -9941,10 +10669,10 @@
       <c r="AC2" s="28"/>
     </row>
     <row r="3" spans="1:29">
-      <c r="A3" s="84" t="s">
+      <c r="A3" s="89" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="84"/>
+      <c r="B3" s="89"/>
       <c r="C3" s="29"/>
       <c r="D3" s="3">
         <v>4</v>
@@ -10227,37 +10955,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="18">
-      <c r="A1" s="83" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="83"/>
-      <c r="C1" s="83"/>
-      <c r="D1" s="83"/>
-      <c r="E1" s="83"/>
-      <c r="F1" s="83"/>
-      <c r="G1" s="83"/>
-      <c r="H1" s="83"/>
-      <c r="I1" s="83"/>
-      <c r="J1" s="83"/>
-      <c r="K1" s="83"/>
-      <c r="L1" s="83"/>
-      <c r="M1" s="83"/>
-      <c r="N1" s="83"/>
-      <c r="O1" s="83"/>
-      <c r="P1" s="83"/>
-      <c r="Q1" s="83"/>
-      <c r="R1" s="83"/>
-      <c r="S1" s="83"/>
-      <c r="T1" s="83"/>
-      <c r="U1" s="83"/>
-      <c r="V1" s="83"/>
-      <c r="W1" s="83"/>
-      <c r="X1" s="83"/>
-      <c r="Y1" s="83"/>
-      <c r="Z1" s="83"/>
-      <c r="AA1" s="83"/>
-      <c r="AB1" s="83"/>
-      <c r="AC1" s="83"/>
+      <c r="A1" s="88" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="88"/>
+      <c r="C1" s="88"/>
+      <c r="D1" s="88"/>
+      <c r="E1" s="88"/>
+      <c r="F1" s="88"/>
+      <c r="G1" s="88"/>
+      <c r="H1" s="88"/>
+      <c r="I1" s="88"/>
+      <c r="J1" s="88"/>
+      <c r="K1" s="88"/>
+      <c r="L1" s="88"/>
+      <c r="M1" s="88"/>
+      <c r="N1" s="88"/>
+      <c r="O1" s="88"/>
+      <c r="P1" s="88"/>
+      <c r="Q1" s="88"/>
+      <c r="R1" s="88"/>
+      <c r="S1" s="88"/>
+      <c r="T1" s="88"/>
+      <c r="U1" s="88"/>
+      <c r="V1" s="88"/>
+      <c r="W1" s="88"/>
+      <c r="X1" s="88"/>
+      <c r="Y1" s="88"/>
+      <c r="Z1" s="88"/>
+      <c r="AA1" s="88"/>
+      <c r="AB1" s="88"/>
+      <c r="AC1" s="88"/>
     </row>
     <row r="2" spans="1:29" ht="18">
       <c r="A2" s="23" t="s">
@@ -10295,10 +11023,10 @@
       <c r="AC2" s="28"/>
     </row>
     <row r="3" spans="1:29">
-      <c r="A3" s="84" t="s">
+      <c r="A3" s="89" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="84"/>
+      <c r="B3" s="89"/>
       <c r="C3" s="29"/>
       <c r="D3" s="3">
         <v>3</v>
@@ -10580,37 +11308,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="18">
-      <c r="A1" s="83" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="83"/>
-      <c r="C1" s="83"/>
-      <c r="D1" s="83"/>
-      <c r="E1" s="83"/>
-      <c r="F1" s="83"/>
-      <c r="G1" s="83"/>
-      <c r="H1" s="83"/>
-      <c r="I1" s="83"/>
-      <c r="J1" s="83"/>
-      <c r="K1" s="83"/>
-      <c r="L1" s="83"/>
-      <c r="M1" s="83"/>
-      <c r="N1" s="83"/>
-      <c r="O1" s="83"/>
-      <c r="P1" s="83"/>
-      <c r="Q1" s="83"/>
-      <c r="R1" s="83"/>
-      <c r="S1" s="83"/>
-      <c r="T1" s="83"/>
-      <c r="U1" s="83"/>
-      <c r="V1" s="83"/>
-      <c r="W1" s="83"/>
-      <c r="X1" s="83"/>
-      <c r="Y1" s="83"/>
-      <c r="Z1" s="83"/>
-      <c r="AA1" s="83"/>
-      <c r="AB1" s="83"/>
-      <c r="AC1" s="83"/>
+      <c r="A1" s="88" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="88"/>
+      <c r="C1" s="88"/>
+      <c r="D1" s="88"/>
+      <c r="E1" s="88"/>
+      <c r="F1" s="88"/>
+      <c r="G1" s="88"/>
+      <c r="H1" s="88"/>
+      <c r="I1" s="88"/>
+      <c r="J1" s="88"/>
+      <c r="K1" s="88"/>
+      <c r="L1" s="88"/>
+      <c r="M1" s="88"/>
+      <c r="N1" s="88"/>
+      <c r="O1" s="88"/>
+      <c r="P1" s="88"/>
+      <c r="Q1" s="88"/>
+      <c r="R1" s="88"/>
+      <c r="S1" s="88"/>
+      <c r="T1" s="88"/>
+      <c r="U1" s="88"/>
+      <c r="V1" s="88"/>
+      <c r="W1" s="88"/>
+      <c r="X1" s="88"/>
+      <c r="Y1" s="88"/>
+      <c r="Z1" s="88"/>
+      <c r="AA1" s="88"/>
+      <c r="AB1" s="88"/>
+      <c r="AC1" s="88"/>
     </row>
     <row r="2" spans="1:29" ht="18">
       <c r="A2" s="23" t="s">
@@ -10648,10 +11376,10 @@
       <c r="AC2" s="28"/>
     </row>
     <row r="3" spans="1:29">
-      <c r="A3" s="84" t="s">
+      <c r="A3" s="89" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="84"/>
+      <c r="B3" s="89"/>
       <c r="C3" s="29"/>
       <c r="D3" s="3">
         <v>5</v>
@@ -10935,37 +11663,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="18">
-      <c r="A1" s="83" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="83"/>
-      <c r="C1" s="83"/>
-      <c r="D1" s="83"/>
-      <c r="E1" s="83"/>
-      <c r="F1" s="83"/>
-      <c r="G1" s="83"/>
-      <c r="H1" s="83"/>
-      <c r="I1" s="83"/>
-      <c r="J1" s="83"/>
-      <c r="K1" s="83"/>
-      <c r="L1" s="83"/>
-      <c r="M1" s="83"/>
-      <c r="N1" s="83"/>
-      <c r="O1" s="83"/>
-      <c r="P1" s="83"/>
-      <c r="Q1" s="83"/>
-      <c r="R1" s="83"/>
-      <c r="S1" s="83"/>
-      <c r="T1" s="83"/>
-      <c r="U1" s="83"/>
-      <c r="V1" s="83"/>
-      <c r="W1" s="83"/>
-      <c r="X1" s="83"/>
-      <c r="Y1" s="83"/>
-      <c r="Z1" s="83"/>
-      <c r="AA1" s="83"/>
-      <c r="AB1" s="83"/>
-      <c r="AC1" s="83"/>
+      <c r="A1" s="88" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="88"/>
+      <c r="C1" s="88"/>
+      <c r="D1" s="88"/>
+      <c r="E1" s="88"/>
+      <c r="F1" s="88"/>
+      <c r="G1" s="88"/>
+      <c r="H1" s="88"/>
+      <c r="I1" s="88"/>
+      <c r="J1" s="88"/>
+      <c r="K1" s="88"/>
+      <c r="L1" s="88"/>
+      <c r="M1" s="88"/>
+      <c r="N1" s="88"/>
+      <c r="O1" s="88"/>
+      <c r="P1" s="88"/>
+      <c r="Q1" s="88"/>
+      <c r="R1" s="88"/>
+      <c r="S1" s="88"/>
+      <c r="T1" s="88"/>
+      <c r="U1" s="88"/>
+      <c r="V1" s="88"/>
+      <c r="W1" s="88"/>
+      <c r="X1" s="88"/>
+      <c r="Y1" s="88"/>
+      <c r="Z1" s="88"/>
+      <c r="AA1" s="88"/>
+      <c r="AB1" s="88"/>
+      <c r="AC1" s="88"/>
     </row>
     <row r="2" spans="1:29" ht="18">
       <c r="A2" s="23" t="s">
@@ -11003,10 +11731,10 @@
       <c r="AC2" s="32"/>
     </row>
     <row r="3" spans="1:29">
-      <c r="A3" s="84" t="s">
+      <c r="A3" s="89" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="84"/>
+      <c r="B3" s="89"/>
       <c r="C3" s="33"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -11288,37 +12016,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="18">
-      <c r="A1" s="83" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="83"/>
-      <c r="C1" s="83"/>
-      <c r="D1" s="83"/>
-      <c r="E1" s="83"/>
-      <c r="F1" s="83"/>
-      <c r="G1" s="83"/>
-      <c r="H1" s="83"/>
-      <c r="I1" s="83"/>
-      <c r="J1" s="83"/>
-      <c r="K1" s="83"/>
-      <c r="L1" s="83"/>
-      <c r="M1" s="83"/>
-      <c r="N1" s="83"/>
-      <c r="O1" s="83"/>
-      <c r="P1" s="83"/>
-      <c r="Q1" s="83"/>
-      <c r="R1" s="83"/>
-      <c r="S1" s="83"/>
-      <c r="T1" s="83"/>
-      <c r="U1" s="83"/>
-      <c r="V1" s="83"/>
-      <c r="W1" s="83"/>
-      <c r="X1" s="83"/>
-      <c r="Y1" s="83"/>
-      <c r="Z1" s="83"/>
-      <c r="AA1" s="83"/>
-      <c r="AB1" s="83"/>
-      <c r="AC1" s="83"/>
+      <c r="A1" s="88" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="88"/>
+      <c r="C1" s="88"/>
+      <c r="D1" s="88"/>
+      <c r="E1" s="88"/>
+      <c r="F1" s="88"/>
+      <c r="G1" s="88"/>
+      <c r="H1" s="88"/>
+      <c r="I1" s="88"/>
+      <c r="J1" s="88"/>
+      <c r="K1" s="88"/>
+      <c r="L1" s="88"/>
+      <c r="M1" s="88"/>
+      <c r="N1" s="88"/>
+      <c r="O1" s="88"/>
+      <c r="P1" s="88"/>
+      <c r="Q1" s="88"/>
+      <c r="R1" s="88"/>
+      <c r="S1" s="88"/>
+      <c r="T1" s="88"/>
+      <c r="U1" s="88"/>
+      <c r="V1" s="88"/>
+      <c r="W1" s="88"/>
+      <c r="X1" s="88"/>
+      <c r="Y1" s="88"/>
+      <c r="Z1" s="88"/>
+      <c r="AA1" s="88"/>
+      <c r="AB1" s="88"/>
+      <c r="AC1" s="88"/>
     </row>
     <row r="2" spans="1:29" ht="18">
       <c r="A2" s="23" t="s">
@@ -11356,10 +12084,10 @@
       <c r="AC2" s="34"/>
     </row>
     <row r="3" spans="1:29">
-      <c r="A3" s="84" t="s">
+      <c r="A3" s="89" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="84"/>
+      <c r="B3" s="89"/>
       <c r="C3" s="35"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -11619,66 +12347,67 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AC6"/>
+  <dimension ref="A1:AD6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="20.5703125" customWidth="1"/>
-    <col min="4" max="4" width="29.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="19.28515625" customWidth="1"/>
-    <col min="6" max="6" width="16.28515625" customWidth="1"/>
-    <col min="7" max="7" width="24.42578125" customWidth="1"/>
-    <col min="8" max="8" width="20.28515625" customWidth="1"/>
-    <col min="9" max="9" width="20" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="13.7109375" customWidth="1"/>
-    <col min="18" max="18" width="13" customWidth="1"/>
-    <col min="19" max="19" width="14.42578125" customWidth="1"/>
-    <col min="20" max="20" width="18.42578125" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="20.5703125" customWidth="1"/>
+    <col min="5" max="5" width="29.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.28515625" customWidth="1"/>
+    <col min="7" max="7" width="16.28515625" customWidth="1"/>
+    <col min="8" max="8" width="24.42578125" customWidth="1"/>
+    <col min="9" max="9" width="20.28515625" customWidth="1"/>
+    <col min="10" max="10" width="20" customWidth="1"/>
+    <col min="14" max="14" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="13.7109375" customWidth="1"/>
+    <col min="19" max="19" width="13" customWidth="1"/>
+    <col min="20" max="20" width="14.42578125" customWidth="1"/>
+    <col min="21" max="21" width="18.42578125" customWidth="1"/>
+    <col min="22" max="22" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="10.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:29" ht="18">
-      <c r="A1" s="83" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="83"/>
-      <c r="C1" s="83"/>
-      <c r="D1" s="83"/>
-      <c r="E1" s="83"/>
-      <c r="F1" s="83"/>
-      <c r="G1" s="83"/>
-      <c r="H1" s="83"/>
-      <c r="I1" s="83"/>
-      <c r="J1" s="83"/>
-      <c r="K1" s="83"/>
-      <c r="L1" s="83"/>
-      <c r="M1" s="83"/>
-      <c r="N1" s="83"/>
-      <c r="O1" s="83"/>
-      <c r="P1" s="83"/>
-      <c r="Q1" s="83"/>
-      <c r="R1" s="83"/>
-      <c r="S1" s="83"/>
-      <c r="T1" s="83"/>
-      <c r="U1" s="83"/>
-      <c r="V1" s="83"/>
-      <c r="W1" s="83"/>
-      <c r="X1" s="83"/>
-      <c r="Y1" s="83"/>
-      <c r="Z1" s="83"/>
-      <c r="AA1" s="83"/>
-      <c r="AB1" s="83"/>
-      <c r="AC1" s="83"/>
-    </row>
-    <row r="2" spans="1:29" ht="18">
+    <row r="1" spans="1:30" ht="18">
+      <c r="A1" s="88" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="88"/>
+      <c r="C1" s="88"/>
+      <c r="D1" s="88"/>
+      <c r="E1" s="88"/>
+      <c r="F1" s="88"/>
+      <c r="G1" s="88"/>
+      <c r="H1" s="88"/>
+      <c r="I1" s="88"/>
+      <c r="J1" s="88"/>
+      <c r="K1" s="88"/>
+      <c r="L1" s="88"/>
+      <c r="M1" s="88"/>
+      <c r="N1" s="88"/>
+      <c r="O1" s="88"/>
+      <c r="P1" s="88"/>
+      <c r="Q1" s="88"/>
+      <c r="R1" s="88"/>
+      <c r="S1" s="88"/>
+      <c r="T1" s="88"/>
+      <c r="U1" s="88"/>
+      <c r="V1" s="88"/>
+      <c r="W1" s="88"/>
+      <c r="X1" s="88"/>
+      <c r="Y1" s="88"/>
+      <c r="Z1" s="88"/>
+      <c r="AA1" s="88"/>
+      <c r="AB1" s="88"/>
+      <c r="AC1" s="88"/>
+      <c r="AD1" s="88"/>
+    </row>
+    <row r="2" spans="1:30" ht="18">
       <c r="A2" s="23" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="23" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="36"/>
+      <c r="C2" s="23"/>
       <c r="D2" s="36"/>
       <c r="E2" s="36"/>
       <c r="F2" s="36"/>
@@ -11705,41 +12434,42 @@
       <c r="AA2" s="36"/>
       <c r="AB2" s="36"/>
       <c r="AC2" s="36"/>
-    </row>
-    <row r="3" spans="1:29">
-      <c r="A3" s="84" t="s">
+      <c r="AD2" s="36"/>
+    </row>
+    <row r="3" spans="1:30">
+      <c r="A3" s="89" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="84"/>
-      <c r="C3" s="37"/>
-      <c r="D3" s="3">
+      <c r="B3" s="89"/>
+      <c r="C3" s="83"/>
+      <c r="D3" s="37"/>
+      <c r="E3" s="3">
         <v>2</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="F3" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F3" s="5"/>
       <c r="G3" s="5"/>
       <c r="H3" s="5"/>
-      <c r="I3" s="6"/>
-      <c r="J3" s="7" t="s">
+      <c r="I3" s="5"/>
+      <c r="J3" s="6"/>
+      <c r="K3" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="K3" s="7" t="s">
+      <c r="L3" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="L3" s="7"/>
-      <c r="M3" s="7" t="s">
+      <c r="M3" s="7"/>
+      <c r="N3" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="N3" s="7">
+      <c r="O3" s="7">
         <v>1</v>
       </c>
-      <c r="O3" s="7"/>
       <c r="P3" s="7"/>
       <c r="Q3" s="7"/>
       <c r="R3" s="7"/>
-      <c r="S3" s="6"/>
+      <c r="S3" s="7"/>
       <c r="T3" s="6"/>
       <c r="U3" s="6"/>
       <c r="V3" s="6"/>
@@ -11750,8 +12480,9 @@
       <c r="AA3" s="6"/>
       <c r="AB3" s="6"/>
       <c r="AC3" s="6"/>
-    </row>
-    <row r="4" spans="1:29" ht="42.75">
+      <c r="AD3" s="6"/>
+    </row>
+    <row r="4" spans="1:30" ht="42.75">
       <c r="A4" s="10" t="s">
         <v>8</v>
       </c>
@@ -11759,202 +12490,206 @@
         <v>36</v>
       </c>
       <c r="C4" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="D4" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="D4" s="11" t="s">
+      <c r="E4" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="E4" s="10" t="s">
+      <c r="F4" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="F4" s="10" t="s">
+      <c r="G4" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="G4" s="12" t="s">
+      <c r="H4" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="H4" s="10" t="s">
+      <c r="I4" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="I4" s="10" t="s">
+      <c r="J4" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="J4" s="13" t="s">
+      <c r="K4" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="K4" s="13" t="s">
+      <c r="L4" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="L4" s="13" t="s">
+      <c r="M4" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="M4" s="14" t="s">
+      <c r="N4" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="N4" s="14" t="s">
+      <c r="O4" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="O4" s="14" t="s">
+      <c r="P4" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="P4" s="14" t="s">
+      <c r="Q4" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="Q4" s="15" t="s">
+      <c r="R4" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="R4" s="14" t="s">
+      <c r="S4" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="S4" s="13" t="s">
+      <c r="T4" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="T4" s="13" t="s">
+      <c r="U4" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="U4" s="10" t="s">
+      <c r="V4" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="V4" s="10" t="s">
+      <c r="W4" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="W4" s="16" t="s">
+      <c r="X4" s="16" t="s">
         <v>27</v>
       </c>
-      <c r="X4" s="16" t="s">
+      <c r="Y4" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="Y4" s="16" t="s">
+      <c r="Z4" s="16" t="s">
         <v>29</v>
       </c>
-      <c r="Z4" s="16" t="s">
+      <c r="AA4" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="AA4" s="16" t="s">
+      <c r="AB4" s="16" t="s">
         <v>37</v>
       </c>
-      <c r="AB4" s="16" t="s">
+      <c r="AC4" s="16" t="s">
         <v>31</v>
       </c>
-      <c r="AC4" s="17" t="s">
+      <c r="AD4" s="17" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="5" spans="1:29">
+    <row r="5" spans="1:30">
       <c r="A5" s="9">
         <v>1</v>
       </c>
       <c r="B5" s="27" t="s">
         <v>44</v>
       </c>
-      <c r="C5" s="9">
-        <v>0</v>
-      </c>
-      <c r="D5" s="27" t="s">
+      <c r="C5" s="27"/>
+      <c r="D5" s="9">
+        <v>0</v>
+      </c>
+      <c r="E5" s="27" t="s">
         <v>44</v>
-      </c>
-      <c r="E5" s="9" t="s">
-        <v>33</v>
       </c>
       <c r="F5" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="G5" s="24">
+      <c r="G5" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="H5" s="24">
         <v>2</v>
       </c>
-      <c r="H5" s="9">
+      <c r="I5" s="9">
         <v>250.25</v>
       </c>
-      <c r="I5" s="8">
+      <c r="J5" s="8">
         <v>500.5</v>
       </c>
-      <c r="J5" s="25">
+      <c r="K5" s="25">
         <v>2.21</v>
       </c>
-      <c r="K5" s="25">
+      <c r="L5" s="25">
         <v>1.79</v>
       </c>
-      <c r="L5" s="25">
+      <c r="M5" s="25">
         <v>2.5</v>
       </c>
-      <c r="M5" s="8">
+      <c r="N5" s="8">
         <v>500.5</v>
       </c>
-      <c r="N5" s="8">
-        <f>ROUND(J5*M5%,2)</f>
+      <c r="O5" s="8">
+        <f>ROUND(K5*N5%,2)</f>
         <v>11.06</v>
       </c>
-      <c r="O5" s="8">
-        <f>I5-N5</f>
+      <c r="P5" s="8">
+        <f>J5-O5</f>
         <v>489.44</v>
       </c>
-      <c r="P5" s="8">
-        <f>ROUND(K5*O5%,2)</f>
+      <c r="Q5" s="8">
+        <f>ROUND(L5*P5%,2)</f>
         <v>8.76</v>
       </c>
-      <c r="Q5" s="8">
-        <f>O5-P5</f>
+      <c r="R5" s="8">
+        <f>P5-Q5</f>
         <v>480.68</v>
       </c>
-      <c r="R5" s="8">
-        <f>ROUND(L5*Q5%,2)</f>
+      <c r="S5" s="8">
+        <f>ROUND(M5*R5%,2)</f>
         <v>12.02</v>
       </c>
-      <c r="S5" s="26">
-        <f>N5+P5+R5</f>
+      <c r="T5" s="26">
+        <f>O5+Q5+S5</f>
         <v>31.84</v>
       </c>
-      <c r="T5" s="26">
-        <v>0</v>
-      </c>
-      <c r="U5" s="8">
-        <f>(I5-S5)</f>
+      <c r="U5" s="26">
+        <v>0</v>
+      </c>
+      <c r="V5" s="8">
+        <f>(J5-T5)</f>
         <v>468.66</v>
       </c>
-      <c r="V5" s="24">
+      <c r="W5" s="24">
         <v>88363222</v>
       </c>
-      <c r="W5" s="18">
+      <c r="X5" s="18">
         <v>0.18</v>
       </c>
-      <c r="X5" s="24">
-        <f>IF($D$3=1,ROUND(((U5*W5)/2),2),0)</f>
-        <v>0</v>
-      </c>
       <c r="Y5" s="24">
-        <f>IF($D$3=1,ROUND(((U5*W5)/2),2),0)</f>
-        <v>0</v>
-      </c>
-      <c r="Z5" s="8">
-        <f>IF($D$3=2,ROUND(((U5*W5)),2),0)</f>
+        <f>IF($E$3=1,ROUND(((V5*X5)/2),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="Z5" s="24">
+        <f>IF($E$3=1,ROUND(((V5*X5)/2),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="AA5" s="8">
+        <f>IF($E$3=2,ROUND(((V5*X5)),2),0)</f>
         <v>84.36</v>
       </c>
-      <c r="AA5" s="24">
-        <v>0</v>
-      </c>
       <c r="AB5" s="24">
-        <f>X5+Y5+Z5</f>
+        <v>0</v>
+      </c>
+      <c r="AC5" s="24">
+        <f>Y5+Z5+AA5</f>
         <v>84.36</v>
       </c>
-      <c r="AC5" s="24">
-        <f>U5+AB5</f>
+      <c r="AD5" s="24">
+        <f>V5+AC5</f>
         <v>553.02</v>
       </c>
     </row>
-    <row r="6" spans="1:29">
+    <row r="6" spans="1:30">
       <c r="A6" s="19"/>
       <c r="B6" s="19"/>
       <c r="C6" s="19"/>
       <c r="D6" s="19"/>
       <c r="E6" s="19"/>
       <c r="F6" s="19"/>
-      <c r="G6" s="20"/>
-      <c r="H6" s="21"/>
+      <c r="G6" s="19"/>
+      <c r="H6" s="20"/>
       <c r="I6" s="21"/>
-      <c r="J6" s="22"/>
+      <c r="J6" s="21"/>
       <c r="K6" s="22"/>
       <c r="L6" s="22"/>
-      <c r="M6" s="21"/>
+      <c r="M6" s="22"/>
       <c r="N6" s="21"/>
       <c r="O6" s="21"/>
       <c r="P6" s="21"/>
@@ -11964,17 +12699,18 @@
       <c r="T6" s="21"/>
       <c r="U6" s="21"/>
       <c r="V6" s="21"/>
-      <c r="W6" s="22"/>
-      <c r="X6" s="21"/>
+      <c r="W6" s="21"/>
+      <c r="X6" s="22"/>
       <c r="Y6" s="21"/>
       <c r="Z6" s="21"/>
       <c r="AA6" s="21"/>
       <c r="AB6" s="21"/>
       <c r="AC6" s="21"/>
+      <c r="AD6" s="21"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:AC1"/>
+    <mergeCell ref="A1:AD1"/>
     <mergeCell ref="A3:B3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -12007,37 +12743,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:31" ht="18">
-      <c r="A1" s="83" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="83"/>
-      <c r="C1" s="83"/>
-      <c r="D1" s="83"/>
-      <c r="E1" s="83"/>
-      <c r="F1" s="83"/>
-      <c r="G1" s="83"/>
-      <c r="H1" s="83"/>
-      <c r="I1" s="83"/>
-      <c r="J1" s="83"/>
-      <c r="K1" s="83"/>
-      <c r="L1" s="83"/>
-      <c r="M1" s="83"/>
-      <c r="N1" s="83"/>
-      <c r="O1" s="83"/>
-      <c r="P1" s="83"/>
-      <c r="Q1" s="83"/>
-      <c r="R1" s="83"/>
-      <c r="S1" s="83"/>
-      <c r="T1" s="83"/>
-      <c r="U1" s="83"/>
-      <c r="V1" s="83"/>
-      <c r="W1" s="83"/>
-      <c r="X1" s="83"/>
-      <c r="Y1" s="83"/>
-      <c r="Z1" s="83"/>
-      <c r="AA1" s="83"/>
-      <c r="AB1" s="83"/>
-      <c r="AC1" s="83"/>
+      <c r="A1" s="88" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="88"/>
+      <c r="C1" s="88"/>
+      <c r="D1" s="88"/>
+      <c r="E1" s="88"/>
+      <c r="F1" s="88"/>
+      <c r="G1" s="88"/>
+      <c r="H1" s="88"/>
+      <c r="I1" s="88"/>
+      <c r="J1" s="88"/>
+      <c r="K1" s="88"/>
+      <c r="L1" s="88"/>
+      <c r="M1" s="88"/>
+      <c r="N1" s="88"/>
+      <c r="O1" s="88"/>
+      <c r="P1" s="88"/>
+      <c r="Q1" s="88"/>
+      <c r="R1" s="88"/>
+      <c r="S1" s="88"/>
+      <c r="T1" s="88"/>
+      <c r="U1" s="88"/>
+      <c r="V1" s="88"/>
+      <c r="W1" s="88"/>
+      <c r="X1" s="88"/>
+      <c r="Y1" s="88"/>
+      <c r="Z1" s="88"/>
+      <c r="AA1" s="88"/>
+      <c r="AB1" s="88"/>
+      <c r="AC1" s="88"/>
     </row>
     <row r="2" spans="1:31" ht="16.5" customHeight="1">
       <c r="A2" s="23" t="s">
@@ -12075,10 +12811,10 @@
       <c r="AC2" s="41"/>
     </row>
     <row r="3" spans="1:31">
-      <c r="A3" s="84" t="s">
+      <c r="A3" s="89" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="84"/>
+      <c r="B3" s="89"/>
       <c r="D3">
         <v>2</v>
       </c>

</xml_diff>

<commit_message>
Updated Fixes of Purchase Bills
Updated Fixes of Purchase Bills
</commit_message>
<xml_diff>
--- a/testdata/DBfin.xlsx
+++ b/testdata/DBfin.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4507"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="2520" windowWidth="15240" windowHeight="6540" tabRatio="849" firstSheet="20" activeTab="25"/>
+    <workbookView xWindow="0" yWindow="2520" windowWidth="15240" windowHeight="6540" tabRatio="849" firstSheet="21" activeTab="26"/>
   </bookViews>
   <sheets>
     <sheet name="PurchaseBillsLocal" sheetId="1" r:id="rId1"/>
@@ -33,13 +33,14 @@
     <sheet name="PurchaseBills_Banks" sheetId="23" r:id="rId24"/>
     <sheet name="PurchaseBills_Import" sheetId="24" r:id="rId25"/>
     <sheet name="PurchaseBills_IGST_Validation_2" sheetId="26" r:id="rId26"/>
+    <sheet name="Purchase_Bills_Allow_IGST" sheetId="27" r:id="rId27"/>
   </sheets>
   <calcPr calcId="125725"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1425" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1508" uniqueCount="114">
   <si>
     <t>Scenario  : Local Sales - Stock UOM and Sales UOM (Similar)   DOC NO :  SORD-2425-00089</t>
   </si>
@@ -578,7 +579,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="90">
+  <cellXfs count="92">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -786,6 +787,12 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -1118,68 +1125,68 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:59" ht="18">
-      <c r="A1" s="88" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="88"/>
-      <c r="C1" s="88"/>
-      <c r="D1" s="88"/>
-      <c r="E1" s="88"/>
-      <c r="F1" s="88"/>
-      <c r="G1" s="88"/>
-      <c r="H1" s="88"/>
-      <c r="I1" s="88"/>
-      <c r="J1" s="88"/>
-      <c r="K1" s="88"/>
-      <c r="L1" s="88"/>
-      <c r="M1" s="88"/>
-      <c r="N1" s="88"/>
-      <c r="O1" s="88"/>
-      <c r="P1" s="88"/>
-      <c r="Q1" s="88"/>
-      <c r="R1" s="88"/>
-      <c r="S1" s="88"/>
-      <c r="T1" s="88"/>
-      <c r="U1" s="88"/>
-      <c r="V1" s="88"/>
-      <c r="W1" s="88"/>
-      <c r="X1" s="88"/>
-      <c r="Y1" s="88"/>
-      <c r="Z1" s="88"/>
-      <c r="AA1" s="88"/>
-      <c r="AB1" s="88"/>
-      <c r="AC1" s="88"/>
-      <c r="AD1" s="88" t="s">
-        <v>0</v>
-      </c>
-      <c r="AE1" s="88"/>
-      <c r="AF1" s="88"/>
-      <c r="AG1" s="88"/>
-      <c r="AH1" s="88"/>
-      <c r="AI1" s="88"/>
-      <c r="AJ1" s="88"/>
-      <c r="AK1" s="88"/>
-      <c r="AL1" s="88"/>
-      <c r="AM1" s="88"/>
-      <c r="AN1" s="88"/>
-      <c r="AO1" s="88"/>
-      <c r="AP1" s="88"/>
-      <c r="AQ1" s="88"/>
-      <c r="AR1" s="88"/>
-      <c r="AS1" s="88"/>
-      <c r="AT1" s="88"/>
-      <c r="AU1" s="88"/>
-      <c r="AV1" s="88"/>
-      <c r="AW1" s="88"/>
-      <c r="AX1" s="88"/>
-      <c r="AY1" s="88"/>
-      <c r="AZ1" s="88"/>
-      <c r="BA1" s="88"/>
-      <c r="BB1" s="88"/>
-      <c r="BC1" s="88"/>
-      <c r="BD1" s="88"/>
-      <c r="BE1" s="88"/>
-      <c r="BF1" s="88"/>
+      <c r="A1" s="90" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="90"/>
+      <c r="C1" s="90"/>
+      <c r="D1" s="90"/>
+      <c r="E1" s="90"/>
+      <c r="F1" s="90"/>
+      <c r="G1" s="90"/>
+      <c r="H1" s="90"/>
+      <c r="I1" s="90"/>
+      <c r="J1" s="90"/>
+      <c r="K1" s="90"/>
+      <c r="L1" s="90"/>
+      <c r="M1" s="90"/>
+      <c r="N1" s="90"/>
+      <c r="O1" s="90"/>
+      <c r="P1" s="90"/>
+      <c r="Q1" s="90"/>
+      <c r="R1" s="90"/>
+      <c r="S1" s="90"/>
+      <c r="T1" s="90"/>
+      <c r="U1" s="90"/>
+      <c r="V1" s="90"/>
+      <c r="W1" s="90"/>
+      <c r="X1" s="90"/>
+      <c r="Y1" s="90"/>
+      <c r="Z1" s="90"/>
+      <c r="AA1" s="90"/>
+      <c r="AB1" s="90"/>
+      <c r="AC1" s="90"/>
+      <c r="AD1" s="90" t="s">
+        <v>0</v>
+      </c>
+      <c r="AE1" s="90"/>
+      <c r="AF1" s="90"/>
+      <c r="AG1" s="90"/>
+      <c r="AH1" s="90"/>
+      <c r="AI1" s="90"/>
+      <c r="AJ1" s="90"/>
+      <c r="AK1" s="90"/>
+      <c r="AL1" s="90"/>
+      <c r="AM1" s="90"/>
+      <c r="AN1" s="90"/>
+      <c r="AO1" s="90"/>
+      <c r="AP1" s="90"/>
+      <c r="AQ1" s="90"/>
+      <c r="AR1" s="90"/>
+      <c r="AS1" s="90"/>
+      <c r="AT1" s="90"/>
+      <c r="AU1" s="90"/>
+      <c r="AV1" s="90"/>
+      <c r="AW1" s="90"/>
+      <c r="AX1" s="90"/>
+      <c r="AY1" s="90"/>
+      <c r="AZ1" s="90"/>
+      <c r="BA1" s="90"/>
+      <c r="BB1" s="90"/>
+      <c r="BC1" s="90"/>
+      <c r="BD1" s="90"/>
+      <c r="BE1" s="90"/>
+      <c r="BF1" s="90"/>
     </row>
     <row r="2" spans="1:59" ht="18">
       <c r="A2" s="23" t="s">
@@ -1250,10 +1257,10 @@
       <c r="BF2" s="38"/>
     </row>
     <row r="3" spans="1:59">
-      <c r="A3" s="89" t="s">
+      <c r="A3" s="91" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="89"/>
+      <c r="B3" s="91"/>
       <c r="C3" s="2"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -1293,10 +1300,10 @@
       <c r="AA3" s="6"/>
       <c r="AB3" s="6"/>
       <c r="AC3" s="6"/>
-      <c r="AD3" s="89" t="s">
+      <c r="AD3" s="91" t="s">
         <v>3</v>
       </c>
-      <c r="AE3" s="89"/>
+      <c r="AE3" s="91"/>
       <c r="AF3" s="39"/>
       <c r="AG3" s="3">
         <v>1</v>
@@ -1774,38 +1781,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:33" ht="18">
-      <c r="A1" s="88" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="88"/>
-      <c r="C1" s="88"/>
-      <c r="D1" s="88"/>
-      <c r="E1" s="88"/>
-      <c r="F1" s="88"/>
-      <c r="G1" s="88"/>
-      <c r="H1" s="88"/>
-      <c r="I1" s="88"/>
-      <c r="J1" s="88"/>
-      <c r="K1" s="88"/>
-      <c r="L1" s="88"/>
-      <c r="M1" s="88"/>
-      <c r="N1" s="88"/>
-      <c r="O1" s="88"/>
-      <c r="P1" s="88"/>
-      <c r="Q1" s="88"/>
-      <c r="R1" s="88"/>
-      <c r="S1" s="88"/>
-      <c r="T1" s="88"/>
-      <c r="U1" s="88"/>
-      <c r="V1" s="88"/>
-      <c r="W1" s="88"/>
-      <c r="X1" s="88"/>
-      <c r="Y1" s="88"/>
-      <c r="Z1" s="88"/>
-      <c r="AA1" s="88"/>
-      <c r="AB1" s="88"/>
-      <c r="AC1" s="88"/>
-      <c r="AD1" s="88"/>
+      <c r="A1" s="90" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="90"/>
+      <c r="C1" s="90"/>
+      <c r="D1" s="90"/>
+      <c r="E1" s="90"/>
+      <c r="F1" s="90"/>
+      <c r="G1" s="90"/>
+      <c r="H1" s="90"/>
+      <c r="I1" s="90"/>
+      <c r="J1" s="90"/>
+      <c r="K1" s="90"/>
+      <c r="L1" s="90"/>
+      <c r="M1" s="90"/>
+      <c r="N1" s="90"/>
+      <c r="O1" s="90"/>
+      <c r="P1" s="90"/>
+      <c r="Q1" s="90"/>
+      <c r="R1" s="90"/>
+      <c r="S1" s="90"/>
+      <c r="T1" s="90"/>
+      <c r="U1" s="90"/>
+      <c r="V1" s="90"/>
+      <c r="W1" s="90"/>
+      <c r="X1" s="90"/>
+      <c r="Y1" s="90"/>
+      <c r="Z1" s="90"/>
+      <c r="AA1" s="90"/>
+      <c r="AB1" s="90"/>
+      <c r="AC1" s="90"/>
+      <c r="AD1" s="90"/>
     </row>
     <row r="2" spans="1:33" ht="18">
       <c r="A2" s="23" t="s">
@@ -1844,10 +1851,10 @@
       <c r="AD2" s="43"/>
     </row>
     <row r="3" spans="1:33" ht="15.75" thickBot="1">
-      <c r="A3" s="89" t="s">
+      <c r="A3" s="91" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="89"/>
+      <c r="B3" s="91"/>
       <c r="C3" s="44"/>
       <c r="D3" s="3">
         <v>2</v>
@@ -2461,37 +2468,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:31" ht="18">
-      <c r="A1" s="88" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="88"/>
-      <c r="C1" s="88"/>
-      <c r="D1" s="88"/>
-      <c r="E1" s="88"/>
-      <c r="F1" s="88"/>
-      <c r="G1" s="88"/>
-      <c r="H1" s="88"/>
-      <c r="I1" s="88"/>
-      <c r="J1" s="88"/>
-      <c r="K1" s="88"/>
-      <c r="L1" s="88"/>
-      <c r="M1" s="88"/>
-      <c r="N1" s="88"/>
-      <c r="O1" s="88"/>
-      <c r="P1" s="88"/>
-      <c r="Q1" s="88"/>
-      <c r="R1" s="88"/>
-      <c r="S1" s="88"/>
-      <c r="T1" s="88"/>
-      <c r="U1" s="88"/>
-      <c r="V1" s="88"/>
-      <c r="W1" s="88"/>
-      <c r="X1" s="88"/>
-      <c r="Y1" s="88"/>
-      <c r="Z1" s="88"/>
-      <c r="AA1" s="88"/>
-      <c r="AB1" s="88"/>
-      <c r="AC1" s="88"/>
+      <c r="A1" s="90" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="90"/>
+      <c r="C1" s="90"/>
+      <c r="D1" s="90"/>
+      <c r="E1" s="90"/>
+      <c r="F1" s="90"/>
+      <c r="G1" s="90"/>
+      <c r="H1" s="90"/>
+      <c r="I1" s="90"/>
+      <c r="J1" s="90"/>
+      <c r="K1" s="90"/>
+      <c r="L1" s="90"/>
+      <c r="M1" s="90"/>
+      <c r="N1" s="90"/>
+      <c r="O1" s="90"/>
+      <c r="P1" s="90"/>
+      <c r="Q1" s="90"/>
+      <c r="R1" s="90"/>
+      <c r="S1" s="90"/>
+      <c r="T1" s="90"/>
+      <c r="U1" s="90"/>
+      <c r="V1" s="90"/>
+      <c r="W1" s="90"/>
+      <c r="X1" s="90"/>
+      <c r="Y1" s="90"/>
+      <c r="Z1" s="90"/>
+      <c r="AA1" s="90"/>
+      <c r="AB1" s="90"/>
+      <c r="AC1" s="90"/>
     </row>
     <row r="2" spans="1:31" ht="16.5" customHeight="1">
       <c r="A2" s="23" t="s">
@@ -2529,10 +2536,10 @@
       <c r="AC2" s="54"/>
     </row>
     <row r="3" spans="1:31">
-      <c r="A3" s="89" t="s">
+      <c r="A3" s="91" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="89"/>
+      <c r="B3" s="91"/>
       <c r="D3">
         <v>2</v>
       </c>
@@ -3023,37 +3030,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="18">
-      <c r="A1" s="88" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="88"/>
-      <c r="C1" s="88"/>
-      <c r="D1" s="88"/>
-      <c r="E1" s="88"/>
-      <c r="F1" s="88"/>
-      <c r="G1" s="88"/>
-      <c r="H1" s="88"/>
-      <c r="I1" s="88"/>
-      <c r="J1" s="88"/>
-      <c r="K1" s="88"/>
-      <c r="L1" s="88"/>
-      <c r="M1" s="88"/>
-      <c r="N1" s="88"/>
-      <c r="O1" s="88"/>
-      <c r="P1" s="88"/>
-      <c r="Q1" s="88"/>
-      <c r="R1" s="88"/>
-      <c r="S1" s="88"/>
-      <c r="T1" s="88"/>
-      <c r="U1" s="88"/>
-      <c r="V1" s="88"/>
-      <c r="W1" s="88"/>
-      <c r="X1" s="88"/>
-      <c r="Y1" s="88"/>
-      <c r="Z1" s="88"/>
-      <c r="AA1" s="88"/>
-      <c r="AB1" s="88"/>
-      <c r="AC1" s="88"/>
+      <c r="A1" s="90" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="90"/>
+      <c r="C1" s="90"/>
+      <c r="D1" s="90"/>
+      <c r="E1" s="90"/>
+      <c r="F1" s="90"/>
+      <c r="G1" s="90"/>
+      <c r="H1" s="90"/>
+      <c r="I1" s="90"/>
+      <c r="J1" s="90"/>
+      <c r="K1" s="90"/>
+      <c r="L1" s="90"/>
+      <c r="M1" s="90"/>
+      <c r="N1" s="90"/>
+      <c r="O1" s="90"/>
+      <c r="P1" s="90"/>
+      <c r="Q1" s="90"/>
+      <c r="R1" s="90"/>
+      <c r="S1" s="90"/>
+      <c r="T1" s="90"/>
+      <c r="U1" s="90"/>
+      <c r="V1" s="90"/>
+      <c r="W1" s="90"/>
+      <c r="X1" s="90"/>
+      <c r="Y1" s="90"/>
+      <c r="Z1" s="90"/>
+      <c r="AA1" s="90"/>
+      <c r="AB1" s="90"/>
+      <c r="AC1" s="90"/>
     </row>
     <row r="2" spans="1:29" ht="18">
       <c r="A2" s="23" t="s">
@@ -3091,10 +3098,10 @@
       <c r="AC2" s="56"/>
     </row>
     <row r="3" spans="1:29">
-      <c r="A3" s="89" t="s">
+      <c r="A3" s="91" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="89"/>
+      <c r="B3" s="91"/>
       <c r="C3" s="57"/>
       <c r="D3" s="3">
         <v>2</v>
@@ -3375,37 +3382,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="18">
-      <c r="A1" s="88" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="88"/>
-      <c r="C1" s="88"/>
-      <c r="D1" s="88"/>
-      <c r="E1" s="88"/>
-      <c r="F1" s="88"/>
-      <c r="G1" s="88"/>
-      <c r="H1" s="88"/>
-      <c r="I1" s="88"/>
-      <c r="J1" s="88"/>
-      <c r="K1" s="88"/>
-      <c r="L1" s="88"/>
-      <c r="M1" s="88"/>
-      <c r="N1" s="88"/>
-      <c r="O1" s="88"/>
-      <c r="P1" s="88"/>
-      <c r="Q1" s="88"/>
-      <c r="R1" s="88"/>
-      <c r="S1" s="88"/>
-      <c r="T1" s="88"/>
-      <c r="U1" s="88"/>
-      <c r="V1" s="88"/>
-      <c r="W1" s="88"/>
-      <c r="X1" s="88"/>
-      <c r="Y1" s="88"/>
-      <c r="Z1" s="88"/>
-      <c r="AA1" s="88"/>
-      <c r="AB1" s="88"/>
-      <c r="AC1" s="88"/>
+      <c r="A1" s="90" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="90"/>
+      <c r="C1" s="90"/>
+      <c r="D1" s="90"/>
+      <c r="E1" s="90"/>
+      <c r="F1" s="90"/>
+      <c r="G1" s="90"/>
+      <c r="H1" s="90"/>
+      <c r="I1" s="90"/>
+      <c r="J1" s="90"/>
+      <c r="K1" s="90"/>
+      <c r="L1" s="90"/>
+      <c r="M1" s="90"/>
+      <c r="N1" s="90"/>
+      <c r="O1" s="90"/>
+      <c r="P1" s="90"/>
+      <c r="Q1" s="90"/>
+      <c r="R1" s="90"/>
+      <c r="S1" s="90"/>
+      <c r="T1" s="90"/>
+      <c r="U1" s="90"/>
+      <c r="V1" s="90"/>
+      <c r="W1" s="90"/>
+      <c r="X1" s="90"/>
+      <c r="Y1" s="90"/>
+      <c r="Z1" s="90"/>
+      <c r="AA1" s="90"/>
+      <c r="AB1" s="90"/>
+      <c r="AC1" s="90"/>
     </row>
     <row r="2" spans="1:29" ht="18">
       <c r="A2" s="23" t="s">
@@ -3443,10 +3450,10 @@
       <c r="AC2" s="58"/>
     </row>
     <row r="3" spans="1:29">
-      <c r="A3" s="89" t="s">
+      <c r="A3" s="91" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="89"/>
+      <c r="B3" s="91"/>
       <c r="C3" s="59"/>
       <c r="D3" s="3">
         <v>4</v>
@@ -3729,38 +3736,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:33" ht="18">
-      <c r="A1" s="88" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="88"/>
-      <c r="C1" s="88"/>
-      <c r="D1" s="88"/>
-      <c r="E1" s="88"/>
-      <c r="F1" s="88"/>
-      <c r="G1" s="88"/>
-      <c r="H1" s="88"/>
-      <c r="I1" s="88"/>
-      <c r="J1" s="88"/>
-      <c r="K1" s="88"/>
-      <c r="L1" s="88"/>
-      <c r="M1" s="88"/>
-      <c r="N1" s="88"/>
-      <c r="O1" s="88"/>
-      <c r="P1" s="88"/>
-      <c r="Q1" s="88"/>
-      <c r="R1" s="88"/>
-      <c r="S1" s="88"/>
-      <c r="T1" s="88"/>
-      <c r="U1" s="88"/>
-      <c r="V1" s="88"/>
-      <c r="W1" s="88"/>
-      <c r="X1" s="88"/>
-      <c r="Y1" s="88"/>
-      <c r="Z1" s="88"/>
-      <c r="AA1" s="88"/>
-      <c r="AB1" s="88"/>
-      <c r="AC1" s="88"/>
-      <c r="AD1" s="88"/>
+      <c r="A1" s="90" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="90"/>
+      <c r="C1" s="90"/>
+      <c r="D1" s="90"/>
+      <c r="E1" s="90"/>
+      <c r="F1" s="90"/>
+      <c r="G1" s="90"/>
+      <c r="H1" s="90"/>
+      <c r="I1" s="90"/>
+      <c r="J1" s="90"/>
+      <c r="K1" s="90"/>
+      <c r="L1" s="90"/>
+      <c r="M1" s="90"/>
+      <c r="N1" s="90"/>
+      <c r="O1" s="90"/>
+      <c r="P1" s="90"/>
+      <c r="Q1" s="90"/>
+      <c r="R1" s="90"/>
+      <c r="S1" s="90"/>
+      <c r="T1" s="90"/>
+      <c r="U1" s="90"/>
+      <c r="V1" s="90"/>
+      <c r="W1" s="90"/>
+      <c r="X1" s="90"/>
+      <c r="Y1" s="90"/>
+      <c r="Z1" s="90"/>
+      <c r="AA1" s="90"/>
+      <c r="AB1" s="90"/>
+      <c r="AC1" s="90"/>
+      <c r="AD1" s="90"/>
     </row>
     <row r="2" spans="1:33" ht="18">
       <c r="A2" s="23" t="s">
@@ -3799,10 +3806,10 @@
       <c r="AD2" s="60"/>
     </row>
     <row r="3" spans="1:33" ht="15.75" thickBot="1">
-      <c r="A3" s="89" t="s">
+      <c r="A3" s="91" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="89"/>
+      <c r="B3" s="91"/>
       <c r="C3" s="61"/>
       <c r="D3" s="3">
         <v>2</v>
@@ -4415,37 +4422,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="18">
-      <c r="A1" s="88" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="88"/>
-      <c r="C1" s="88"/>
-      <c r="D1" s="88"/>
-      <c r="E1" s="88"/>
-      <c r="F1" s="88"/>
-      <c r="G1" s="88"/>
-      <c r="H1" s="88"/>
-      <c r="I1" s="88"/>
-      <c r="J1" s="88"/>
-      <c r="K1" s="88"/>
-      <c r="L1" s="88"/>
-      <c r="M1" s="88"/>
-      <c r="N1" s="88"/>
-      <c r="O1" s="88"/>
-      <c r="P1" s="88"/>
-      <c r="Q1" s="88"/>
-      <c r="R1" s="88"/>
-      <c r="S1" s="88"/>
-      <c r="T1" s="88"/>
-      <c r="U1" s="88"/>
-      <c r="V1" s="88"/>
-      <c r="W1" s="88"/>
-      <c r="X1" s="88"/>
-      <c r="Y1" s="88"/>
-      <c r="Z1" s="88"/>
-      <c r="AA1" s="88"/>
-      <c r="AB1" s="88"/>
-      <c r="AC1" s="88"/>
+      <c r="A1" s="90" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="90"/>
+      <c r="C1" s="90"/>
+      <c r="D1" s="90"/>
+      <c r="E1" s="90"/>
+      <c r="F1" s="90"/>
+      <c r="G1" s="90"/>
+      <c r="H1" s="90"/>
+      <c r="I1" s="90"/>
+      <c r="J1" s="90"/>
+      <c r="K1" s="90"/>
+      <c r="L1" s="90"/>
+      <c r="M1" s="90"/>
+      <c r="N1" s="90"/>
+      <c r="O1" s="90"/>
+      <c r="P1" s="90"/>
+      <c r="Q1" s="90"/>
+      <c r="R1" s="90"/>
+      <c r="S1" s="90"/>
+      <c r="T1" s="90"/>
+      <c r="U1" s="90"/>
+      <c r="V1" s="90"/>
+      <c r="W1" s="90"/>
+      <c r="X1" s="90"/>
+      <c r="Y1" s="90"/>
+      <c r="Z1" s="90"/>
+      <c r="AA1" s="90"/>
+      <c r="AB1" s="90"/>
+      <c r="AC1" s="90"/>
     </row>
     <row r="2" spans="1:29" ht="18">
       <c r="A2" s="23" t="s">
@@ -4483,10 +4490,10 @@
       <c r="AC2" s="62"/>
     </row>
     <row r="3" spans="1:29">
-      <c r="A3" s="89" t="s">
+      <c r="A3" s="91" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="89"/>
+      <c r="B3" s="91"/>
       <c r="C3" s="63"/>
       <c r="D3" s="3">
         <v>4</v>
@@ -4775,68 +4782,68 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:59" ht="18">
-      <c r="A1" s="88" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="88"/>
-      <c r="C1" s="88"/>
-      <c r="D1" s="88"/>
-      <c r="E1" s="88"/>
-      <c r="F1" s="88"/>
-      <c r="G1" s="88"/>
-      <c r="H1" s="88"/>
-      <c r="I1" s="88"/>
-      <c r="J1" s="88"/>
-      <c r="K1" s="88"/>
-      <c r="L1" s="88"/>
-      <c r="M1" s="88"/>
-      <c r="N1" s="88"/>
-      <c r="O1" s="88"/>
-      <c r="P1" s="88"/>
-      <c r="Q1" s="88"/>
-      <c r="R1" s="88"/>
-      <c r="S1" s="88"/>
-      <c r="T1" s="88"/>
-      <c r="U1" s="88"/>
-      <c r="V1" s="88"/>
-      <c r="W1" s="88"/>
-      <c r="X1" s="88"/>
-      <c r="Y1" s="88"/>
-      <c r="Z1" s="88"/>
-      <c r="AA1" s="88"/>
-      <c r="AB1" s="88"/>
-      <c r="AC1" s="88"/>
-      <c r="AD1" s="88" t="s">
-        <v>0</v>
-      </c>
-      <c r="AE1" s="88"/>
-      <c r="AF1" s="88"/>
-      <c r="AG1" s="88"/>
-      <c r="AH1" s="88"/>
-      <c r="AI1" s="88"/>
-      <c r="AJ1" s="88"/>
-      <c r="AK1" s="88"/>
-      <c r="AL1" s="88"/>
-      <c r="AM1" s="88"/>
-      <c r="AN1" s="88"/>
-      <c r="AO1" s="88"/>
-      <c r="AP1" s="88"/>
-      <c r="AQ1" s="88"/>
-      <c r="AR1" s="88"/>
-      <c r="AS1" s="88"/>
-      <c r="AT1" s="88"/>
-      <c r="AU1" s="88"/>
-      <c r="AV1" s="88"/>
-      <c r="AW1" s="88"/>
-      <c r="AX1" s="88"/>
-      <c r="AY1" s="88"/>
-      <c r="AZ1" s="88"/>
-      <c r="BA1" s="88"/>
-      <c r="BB1" s="88"/>
-      <c r="BC1" s="88"/>
-      <c r="BD1" s="88"/>
-      <c r="BE1" s="88"/>
-      <c r="BF1" s="88"/>
+      <c r="A1" s="90" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="90"/>
+      <c r="C1" s="90"/>
+      <c r="D1" s="90"/>
+      <c r="E1" s="90"/>
+      <c r="F1" s="90"/>
+      <c r="G1" s="90"/>
+      <c r="H1" s="90"/>
+      <c r="I1" s="90"/>
+      <c r="J1" s="90"/>
+      <c r="K1" s="90"/>
+      <c r="L1" s="90"/>
+      <c r="M1" s="90"/>
+      <c r="N1" s="90"/>
+      <c r="O1" s="90"/>
+      <c r="P1" s="90"/>
+      <c r="Q1" s="90"/>
+      <c r="R1" s="90"/>
+      <c r="S1" s="90"/>
+      <c r="T1" s="90"/>
+      <c r="U1" s="90"/>
+      <c r="V1" s="90"/>
+      <c r="W1" s="90"/>
+      <c r="X1" s="90"/>
+      <c r="Y1" s="90"/>
+      <c r="Z1" s="90"/>
+      <c r="AA1" s="90"/>
+      <c r="AB1" s="90"/>
+      <c r="AC1" s="90"/>
+      <c r="AD1" s="90" t="s">
+        <v>0</v>
+      </c>
+      <c r="AE1" s="90"/>
+      <c r="AF1" s="90"/>
+      <c r="AG1" s="90"/>
+      <c r="AH1" s="90"/>
+      <c r="AI1" s="90"/>
+      <c r="AJ1" s="90"/>
+      <c r="AK1" s="90"/>
+      <c r="AL1" s="90"/>
+      <c r="AM1" s="90"/>
+      <c r="AN1" s="90"/>
+      <c r="AO1" s="90"/>
+      <c r="AP1" s="90"/>
+      <c r="AQ1" s="90"/>
+      <c r="AR1" s="90"/>
+      <c r="AS1" s="90"/>
+      <c r="AT1" s="90"/>
+      <c r="AU1" s="90"/>
+      <c r="AV1" s="90"/>
+      <c r="AW1" s="90"/>
+      <c r="AX1" s="90"/>
+      <c r="AY1" s="90"/>
+      <c r="AZ1" s="90"/>
+      <c r="BA1" s="90"/>
+      <c r="BB1" s="90"/>
+      <c r="BC1" s="90"/>
+      <c r="BD1" s="90"/>
+      <c r="BE1" s="90"/>
+      <c r="BF1" s="90"/>
     </row>
     <row r="2" spans="1:59" ht="18">
       <c r="A2" s="23" t="s">
@@ -4907,10 +4914,10 @@
       <c r="BF2" s="64"/>
     </row>
     <row r="3" spans="1:59">
-      <c r="A3" s="89" t="s">
+      <c r="A3" s="91" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="89"/>
+      <c r="B3" s="91"/>
       <c r="C3" s="65"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -4950,10 +4957,10 @@
       <c r="AA3" s="6"/>
       <c r="AB3" s="6"/>
       <c r="AC3" s="6"/>
-      <c r="AD3" s="89" t="s">
+      <c r="AD3" s="91" t="s">
         <v>3</v>
       </c>
-      <c r="AE3" s="89"/>
+      <c r="AE3" s="91"/>
       <c r="AF3" s="65"/>
       <c r="AG3" s="3">
         <v>2</v>
@@ -5435,68 +5442,68 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:59" ht="18">
-      <c r="A1" s="88" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="88"/>
-      <c r="C1" s="88"/>
-      <c r="D1" s="88"/>
-      <c r="E1" s="88"/>
-      <c r="F1" s="88"/>
-      <c r="G1" s="88"/>
-      <c r="H1" s="88"/>
-      <c r="I1" s="88"/>
-      <c r="J1" s="88"/>
-      <c r="K1" s="88"/>
-      <c r="L1" s="88"/>
-      <c r="M1" s="88"/>
-      <c r="N1" s="88"/>
-      <c r="O1" s="88"/>
-      <c r="P1" s="88"/>
-      <c r="Q1" s="88"/>
-      <c r="R1" s="88"/>
-      <c r="S1" s="88"/>
-      <c r="T1" s="88"/>
-      <c r="U1" s="88"/>
-      <c r="V1" s="88"/>
-      <c r="W1" s="88"/>
-      <c r="X1" s="88"/>
-      <c r="Y1" s="88"/>
-      <c r="Z1" s="88"/>
-      <c r="AA1" s="88"/>
-      <c r="AB1" s="88"/>
-      <c r="AC1" s="88"/>
-      <c r="AD1" s="88" t="s">
-        <v>0</v>
-      </c>
-      <c r="AE1" s="88"/>
-      <c r="AF1" s="88"/>
-      <c r="AG1" s="88"/>
-      <c r="AH1" s="88"/>
-      <c r="AI1" s="88"/>
-      <c r="AJ1" s="88"/>
-      <c r="AK1" s="88"/>
-      <c r="AL1" s="88"/>
-      <c r="AM1" s="88"/>
-      <c r="AN1" s="88"/>
-      <c r="AO1" s="88"/>
-      <c r="AP1" s="88"/>
-      <c r="AQ1" s="88"/>
-      <c r="AR1" s="88"/>
-      <c r="AS1" s="88"/>
-      <c r="AT1" s="88"/>
-      <c r="AU1" s="88"/>
-      <c r="AV1" s="88"/>
-      <c r="AW1" s="88"/>
-      <c r="AX1" s="88"/>
-      <c r="AY1" s="88"/>
-      <c r="AZ1" s="88"/>
-      <c r="BA1" s="88"/>
-      <c r="BB1" s="88"/>
-      <c r="BC1" s="88"/>
-      <c r="BD1" s="88"/>
-      <c r="BE1" s="88"/>
-      <c r="BF1" s="88"/>
+      <c r="A1" s="90" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="90"/>
+      <c r="C1" s="90"/>
+      <c r="D1" s="90"/>
+      <c r="E1" s="90"/>
+      <c r="F1" s="90"/>
+      <c r="G1" s="90"/>
+      <c r="H1" s="90"/>
+      <c r="I1" s="90"/>
+      <c r="J1" s="90"/>
+      <c r="K1" s="90"/>
+      <c r="L1" s="90"/>
+      <c r="M1" s="90"/>
+      <c r="N1" s="90"/>
+      <c r="O1" s="90"/>
+      <c r="P1" s="90"/>
+      <c r="Q1" s="90"/>
+      <c r="R1" s="90"/>
+      <c r="S1" s="90"/>
+      <c r="T1" s="90"/>
+      <c r="U1" s="90"/>
+      <c r="V1" s="90"/>
+      <c r="W1" s="90"/>
+      <c r="X1" s="90"/>
+      <c r="Y1" s="90"/>
+      <c r="Z1" s="90"/>
+      <c r="AA1" s="90"/>
+      <c r="AB1" s="90"/>
+      <c r="AC1" s="90"/>
+      <c r="AD1" s="90" t="s">
+        <v>0</v>
+      </c>
+      <c r="AE1" s="90"/>
+      <c r="AF1" s="90"/>
+      <c r="AG1" s="90"/>
+      <c r="AH1" s="90"/>
+      <c r="AI1" s="90"/>
+      <c r="AJ1" s="90"/>
+      <c r="AK1" s="90"/>
+      <c r="AL1" s="90"/>
+      <c r="AM1" s="90"/>
+      <c r="AN1" s="90"/>
+      <c r="AO1" s="90"/>
+      <c r="AP1" s="90"/>
+      <c r="AQ1" s="90"/>
+      <c r="AR1" s="90"/>
+      <c r="AS1" s="90"/>
+      <c r="AT1" s="90"/>
+      <c r="AU1" s="90"/>
+      <c r="AV1" s="90"/>
+      <c r="AW1" s="90"/>
+      <c r="AX1" s="90"/>
+      <c r="AY1" s="90"/>
+      <c r="AZ1" s="90"/>
+      <c r="BA1" s="90"/>
+      <c r="BB1" s="90"/>
+      <c r="BC1" s="90"/>
+      <c r="BD1" s="90"/>
+      <c r="BE1" s="90"/>
+      <c r="BF1" s="90"/>
     </row>
     <row r="2" spans="1:59" ht="18">
       <c r="A2" s="23" t="s">
@@ -5567,10 +5574,10 @@
       <c r="BF2" s="67"/>
     </row>
     <row r="3" spans="1:59">
-      <c r="A3" s="89" t="s">
+      <c r="A3" s="91" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="89"/>
+      <c r="B3" s="91"/>
       <c r="C3" s="68"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -5610,10 +5617,10 @@
       <c r="AA3" s="6"/>
       <c r="AB3" s="6"/>
       <c r="AC3" s="6"/>
-      <c r="AD3" s="89" t="s">
+      <c r="AD3" s="91" t="s">
         <v>3</v>
       </c>
-      <c r="AE3" s="89"/>
+      <c r="AE3" s="91"/>
       <c r="AF3" s="68"/>
       <c r="AG3" s="3">
         <v>2</v>
@@ -6088,38 +6095,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:33" ht="18">
-      <c r="A1" s="88" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="88"/>
-      <c r="C1" s="88"/>
-      <c r="D1" s="88"/>
-      <c r="E1" s="88"/>
-      <c r="F1" s="88"/>
-      <c r="G1" s="88"/>
-      <c r="H1" s="88"/>
-      <c r="I1" s="88"/>
-      <c r="J1" s="88"/>
-      <c r="K1" s="88"/>
-      <c r="L1" s="88"/>
-      <c r="M1" s="88"/>
-      <c r="N1" s="88"/>
-      <c r="O1" s="88"/>
-      <c r="P1" s="88"/>
-      <c r="Q1" s="88"/>
-      <c r="R1" s="88"/>
-      <c r="S1" s="88"/>
-      <c r="T1" s="88"/>
-      <c r="U1" s="88"/>
-      <c r="V1" s="88"/>
-      <c r="W1" s="88"/>
-      <c r="X1" s="88"/>
-      <c r="Y1" s="88"/>
-      <c r="Z1" s="88"/>
-      <c r="AA1" s="88"/>
-      <c r="AB1" s="88"/>
-      <c r="AC1" s="88"/>
-      <c r="AD1" s="88"/>
+      <c r="A1" s="90" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="90"/>
+      <c r="C1" s="90"/>
+      <c r="D1" s="90"/>
+      <c r="E1" s="90"/>
+      <c r="F1" s="90"/>
+      <c r="G1" s="90"/>
+      <c r="H1" s="90"/>
+      <c r="I1" s="90"/>
+      <c r="J1" s="90"/>
+      <c r="K1" s="90"/>
+      <c r="L1" s="90"/>
+      <c r="M1" s="90"/>
+      <c r="N1" s="90"/>
+      <c r="O1" s="90"/>
+      <c r="P1" s="90"/>
+      <c r="Q1" s="90"/>
+      <c r="R1" s="90"/>
+      <c r="S1" s="90"/>
+      <c r="T1" s="90"/>
+      <c r="U1" s="90"/>
+      <c r="V1" s="90"/>
+      <c r="W1" s="90"/>
+      <c r="X1" s="90"/>
+      <c r="Y1" s="90"/>
+      <c r="Z1" s="90"/>
+      <c r="AA1" s="90"/>
+      <c r="AB1" s="90"/>
+      <c r="AC1" s="90"/>
+      <c r="AD1" s="90"/>
     </row>
     <row r="2" spans="1:33" ht="18">
       <c r="A2" s="23" t="s">
@@ -6158,10 +6165,10 @@
       <c r="AD2" s="70"/>
     </row>
     <row r="3" spans="1:33" ht="15.75" thickBot="1">
-      <c r="A3" s="89" t="s">
+      <c r="A3" s="91" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="89"/>
+      <c r="B3" s="91"/>
       <c r="C3" s="71"/>
       <c r="D3" s="3">
         <v>3</v>
@@ -7011,68 +7018,68 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:58" ht="18">
-      <c r="A1" s="88" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="88"/>
-      <c r="C1" s="88"/>
-      <c r="D1" s="88"/>
-      <c r="E1" s="88"/>
-      <c r="F1" s="88"/>
-      <c r="G1" s="88"/>
-      <c r="H1" s="88"/>
-      <c r="I1" s="88"/>
-      <c r="J1" s="88"/>
-      <c r="K1" s="88"/>
-      <c r="L1" s="88"/>
-      <c r="M1" s="88"/>
-      <c r="N1" s="88"/>
-      <c r="O1" s="88"/>
-      <c r="P1" s="88"/>
-      <c r="Q1" s="88"/>
-      <c r="R1" s="88"/>
-      <c r="S1" s="88"/>
-      <c r="T1" s="88"/>
-      <c r="U1" s="88"/>
-      <c r="V1" s="88"/>
-      <c r="W1" s="88"/>
-      <c r="X1" s="88"/>
-      <c r="Y1" s="88"/>
-      <c r="Z1" s="88"/>
-      <c r="AA1" s="88"/>
-      <c r="AB1" s="88"/>
-      <c r="AC1" s="88"/>
-      <c r="AD1" s="88" t="s">
-        <v>0</v>
-      </c>
-      <c r="AE1" s="88"/>
-      <c r="AF1" s="88"/>
-      <c r="AG1" s="88"/>
-      <c r="AH1" s="88"/>
-      <c r="AI1" s="88"/>
-      <c r="AJ1" s="88"/>
-      <c r="AK1" s="88"/>
-      <c r="AL1" s="88"/>
-      <c r="AM1" s="88"/>
-      <c r="AN1" s="88"/>
-      <c r="AO1" s="88"/>
-      <c r="AP1" s="88"/>
-      <c r="AQ1" s="88"/>
-      <c r="AR1" s="88"/>
-      <c r="AS1" s="88"/>
-      <c r="AT1" s="88"/>
-      <c r="AU1" s="88"/>
-      <c r="AV1" s="88"/>
-      <c r="AW1" s="88"/>
-      <c r="AX1" s="88"/>
-      <c r="AY1" s="88"/>
-      <c r="AZ1" s="88"/>
-      <c r="BA1" s="88"/>
-      <c r="BB1" s="88"/>
-      <c r="BC1" s="88"/>
-      <c r="BD1" s="88"/>
-      <c r="BE1" s="88"/>
-      <c r="BF1" s="88"/>
+      <c r="A1" s="90" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="90"/>
+      <c r="C1" s="90"/>
+      <c r="D1" s="90"/>
+      <c r="E1" s="90"/>
+      <c r="F1" s="90"/>
+      <c r="G1" s="90"/>
+      <c r="H1" s="90"/>
+      <c r="I1" s="90"/>
+      <c r="J1" s="90"/>
+      <c r="K1" s="90"/>
+      <c r="L1" s="90"/>
+      <c r="M1" s="90"/>
+      <c r="N1" s="90"/>
+      <c r="O1" s="90"/>
+      <c r="P1" s="90"/>
+      <c r="Q1" s="90"/>
+      <c r="R1" s="90"/>
+      <c r="S1" s="90"/>
+      <c r="T1" s="90"/>
+      <c r="U1" s="90"/>
+      <c r="V1" s="90"/>
+      <c r="W1" s="90"/>
+      <c r="X1" s="90"/>
+      <c r="Y1" s="90"/>
+      <c r="Z1" s="90"/>
+      <c r="AA1" s="90"/>
+      <c r="AB1" s="90"/>
+      <c r="AC1" s="90"/>
+      <c r="AD1" s="90" t="s">
+        <v>0</v>
+      </c>
+      <c r="AE1" s="90"/>
+      <c r="AF1" s="90"/>
+      <c r="AG1" s="90"/>
+      <c r="AH1" s="90"/>
+      <c r="AI1" s="90"/>
+      <c r="AJ1" s="90"/>
+      <c r="AK1" s="90"/>
+      <c r="AL1" s="90"/>
+      <c r="AM1" s="90"/>
+      <c r="AN1" s="90"/>
+      <c r="AO1" s="90"/>
+      <c r="AP1" s="90"/>
+      <c r="AQ1" s="90"/>
+      <c r="AR1" s="90"/>
+      <c r="AS1" s="90"/>
+      <c r="AT1" s="90"/>
+      <c r="AU1" s="90"/>
+      <c r="AV1" s="90"/>
+      <c r="AW1" s="90"/>
+      <c r="AX1" s="90"/>
+      <c r="AY1" s="90"/>
+      <c r="AZ1" s="90"/>
+      <c r="BA1" s="90"/>
+      <c r="BB1" s="90"/>
+      <c r="BC1" s="90"/>
+      <c r="BD1" s="90"/>
+      <c r="BE1" s="90"/>
+      <c r="BF1" s="90"/>
     </row>
     <row r="2" spans="1:58" ht="18">
       <c r="A2" s="23" t="s">
@@ -7143,10 +7150,10 @@
       <c r="BF2" s="36"/>
     </row>
     <row r="3" spans="1:58">
-      <c r="A3" s="89" t="s">
+      <c r="A3" s="91" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="89"/>
+      <c r="B3" s="91"/>
       <c r="C3" s="29"/>
       <c r="D3" s="3">
         <v>2</v>
@@ -7186,10 +7193,10 @@
       <c r="AA3" s="6"/>
       <c r="AB3" s="6"/>
       <c r="AC3" s="6"/>
-      <c r="AD3" s="89" t="s">
+      <c r="AD3" s="91" t="s">
         <v>3</v>
       </c>
-      <c r="AE3" s="89"/>
+      <c r="AE3" s="91"/>
       <c r="AF3" s="37"/>
       <c r="AG3" s="3">
         <v>2</v>
@@ -7665,37 +7672,37 @@
       <c r="A1" s="84" t="s">
         <v>112</v>
       </c>
-      <c r="B1" s="88" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="88"/>
-      <c r="D1" s="88"/>
-      <c r="E1" s="88"/>
-      <c r="F1" s="88"/>
-      <c r="G1" s="88"/>
-      <c r="H1" s="88"/>
-      <c r="I1" s="88"/>
-      <c r="J1" s="88"/>
-      <c r="K1" s="88"/>
-      <c r="L1" s="88"/>
-      <c r="M1" s="88"/>
-      <c r="N1" s="88"/>
-      <c r="O1" s="88"/>
-      <c r="P1" s="88"/>
-      <c r="Q1" s="88"/>
-      <c r="R1" s="88"/>
-      <c r="S1" s="88"/>
-      <c r="T1" s="88"/>
-      <c r="U1" s="88"/>
-      <c r="V1" s="88"/>
-      <c r="W1" s="88"/>
-      <c r="X1" s="88"/>
-      <c r="Y1" s="88"/>
-      <c r="Z1" s="88"/>
-      <c r="AA1" s="88"/>
-      <c r="AB1" s="88"/>
-      <c r="AC1" s="88"/>
-      <c r="AD1" s="88"/>
+      <c r="B1" s="90" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="90"/>
+      <c r="D1" s="90"/>
+      <c r="E1" s="90"/>
+      <c r="F1" s="90"/>
+      <c r="G1" s="90"/>
+      <c r="H1" s="90"/>
+      <c r="I1" s="90"/>
+      <c r="J1" s="90"/>
+      <c r="K1" s="90"/>
+      <c r="L1" s="90"/>
+      <c r="M1" s="90"/>
+      <c r="N1" s="90"/>
+      <c r="O1" s="90"/>
+      <c r="P1" s="90"/>
+      <c r="Q1" s="90"/>
+      <c r="R1" s="90"/>
+      <c r="S1" s="90"/>
+      <c r="T1" s="90"/>
+      <c r="U1" s="90"/>
+      <c r="V1" s="90"/>
+      <c r="W1" s="90"/>
+      <c r="X1" s="90"/>
+      <c r="Y1" s="90"/>
+      <c r="Z1" s="90"/>
+      <c r="AA1" s="90"/>
+      <c r="AB1" s="90"/>
+      <c r="AC1" s="90"/>
+      <c r="AD1" s="90"/>
     </row>
     <row r="2" spans="1:33" ht="18">
       <c r="A2" s="85"/>
@@ -7735,10 +7742,10 @@
     </row>
     <row r="3" spans="1:33" ht="15.75" thickBot="1">
       <c r="A3" s="85"/>
-      <c r="B3" s="89" t="s">
+      <c r="B3" s="91" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="89"/>
+      <c r="C3" s="91"/>
       <c r="D3" s="3">
         <v>2</v>
       </c>
@@ -9049,36 +9056,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:31" ht="18">
-      <c r="A1" s="88" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="88"/>
-      <c r="C1" s="88"/>
-      <c r="D1" s="88"/>
-      <c r="E1" s="88"/>
-      <c r="F1" s="88"/>
-      <c r="G1" s="88"/>
-      <c r="H1" s="88"/>
-      <c r="I1" s="88"/>
-      <c r="J1" s="88"/>
-      <c r="K1" s="88"/>
-      <c r="L1" s="88"/>
-      <c r="M1" s="88"/>
-      <c r="N1" s="88"/>
-      <c r="O1" s="88"/>
-      <c r="P1" s="88"/>
-      <c r="Q1" s="88"/>
-      <c r="R1" s="88"/>
-      <c r="S1" s="88"/>
-      <c r="T1" s="88"/>
-      <c r="U1" s="88"/>
-      <c r="V1" s="88"/>
-      <c r="W1" s="88"/>
-      <c r="X1" s="88"/>
-      <c r="Y1" s="88"/>
-      <c r="Z1" s="88"/>
-      <c r="AA1" s="88"/>
-      <c r="AB1" s="88"/>
+      <c r="A1" s="90" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="90"/>
+      <c r="C1" s="90"/>
+      <c r="D1" s="90"/>
+      <c r="E1" s="90"/>
+      <c r="F1" s="90"/>
+      <c r="G1" s="90"/>
+      <c r="H1" s="90"/>
+      <c r="I1" s="90"/>
+      <c r="J1" s="90"/>
+      <c r="K1" s="90"/>
+      <c r="L1" s="90"/>
+      <c r="M1" s="90"/>
+      <c r="N1" s="90"/>
+      <c r="O1" s="90"/>
+      <c r="P1" s="90"/>
+      <c r="Q1" s="90"/>
+      <c r="R1" s="90"/>
+      <c r="S1" s="90"/>
+      <c r="T1" s="90"/>
+      <c r="U1" s="90"/>
+      <c r="V1" s="90"/>
+      <c r="W1" s="90"/>
+      <c r="X1" s="90"/>
+      <c r="Y1" s="90"/>
+      <c r="Z1" s="90"/>
+      <c r="AA1" s="90"/>
+      <c r="AB1" s="90"/>
     </row>
     <row r="2" spans="1:31" ht="18">
       <c r="A2" s="23" t="s">
@@ -9115,10 +9122,10 @@
       <c r="AB2" s="80"/>
     </row>
     <row r="3" spans="1:31" ht="15.75" thickBot="1">
-      <c r="A3" s="89" t="s">
+      <c r="A3" s="91" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="89"/>
+      <c r="B3" s="91"/>
       <c r="C3" s="81"/>
       <c r="D3" s="3">
         <v>2</v>
@@ -9931,37 +9938,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:32" ht="18">
-      <c r="A1" s="88" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="88"/>
-      <c r="C1" s="88"/>
-      <c r="D1" s="88"/>
-      <c r="E1" s="88"/>
-      <c r="F1" s="88"/>
-      <c r="G1" s="88"/>
-      <c r="H1" s="88"/>
-      <c r="I1" s="88"/>
-      <c r="J1" s="88"/>
-      <c r="K1" s="88"/>
-      <c r="L1" s="88"/>
-      <c r="M1" s="88"/>
-      <c r="N1" s="88"/>
-      <c r="O1" s="88"/>
-      <c r="P1" s="88"/>
-      <c r="Q1" s="88"/>
-      <c r="R1" s="88"/>
-      <c r="S1" s="88"/>
-      <c r="T1" s="88"/>
-      <c r="U1" s="88"/>
-      <c r="V1" s="88"/>
-      <c r="W1" s="88"/>
-      <c r="X1" s="88"/>
-      <c r="Y1" s="88"/>
-      <c r="Z1" s="88"/>
-      <c r="AA1" s="88"/>
-      <c r="AB1" s="88"/>
-      <c r="AC1" s="88"/>
+      <c r="A1" s="90" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="90"/>
+      <c r="C1" s="90"/>
+      <c r="D1" s="90"/>
+      <c r="E1" s="90"/>
+      <c r="F1" s="90"/>
+      <c r="G1" s="90"/>
+      <c r="H1" s="90"/>
+      <c r="I1" s="90"/>
+      <c r="J1" s="90"/>
+      <c r="K1" s="90"/>
+      <c r="L1" s="90"/>
+      <c r="M1" s="90"/>
+      <c r="N1" s="90"/>
+      <c r="O1" s="90"/>
+      <c r="P1" s="90"/>
+      <c r="Q1" s="90"/>
+      <c r="R1" s="90"/>
+      <c r="S1" s="90"/>
+      <c r="T1" s="90"/>
+      <c r="U1" s="90"/>
+      <c r="V1" s="90"/>
+      <c r="W1" s="90"/>
+      <c r="X1" s="90"/>
+      <c r="Y1" s="90"/>
+      <c r="Z1" s="90"/>
+      <c r="AA1" s="90"/>
+      <c r="AB1" s="90"/>
+      <c r="AC1" s="90"/>
     </row>
     <row r="2" spans="1:32" ht="18">
       <c r="A2" s="23" t="s">
@@ -9999,10 +10006,10 @@
       <c r="AC2" s="87"/>
     </row>
     <row r="3" spans="1:32" ht="15.75" thickBot="1">
-      <c r="A3" s="89" t="s">
+      <c r="A3" s="91" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="89"/>
+      <c r="B3" s="91"/>
       <c r="C3" s="3">
         <v>2</v>
       </c>
@@ -10574,6 +10581,666 @@
   <mergeCells count="2">
     <mergeCell ref="A1:AC1"/>
     <mergeCell ref="A3:B3"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:BG6"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="3" max="3" width="20.5703125" customWidth="1"/>
+    <col min="5" max="5" width="29.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.28515625" customWidth="1"/>
+    <col min="7" max="7" width="16.28515625" customWidth="1"/>
+    <col min="8" max="8" width="24.42578125" customWidth="1"/>
+    <col min="9" max="9" width="20.28515625" customWidth="1"/>
+    <col min="10" max="10" width="20" customWidth="1"/>
+    <col min="14" max="14" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="13.7109375" customWidth="1"/>
+    <col min="19" max="19" width="13" customWidth="1"/>
+    <col min="20" max="20" width="14.42578125" customWidth="1"/>
+    <col min="21" max="21" width="18.42578125" customWidth="1"/>
+    <col min="22" max="22" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="17" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="11" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="20.42578125" customWidth="1"/>
+    <col min="43" max="43" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="52" max="52" width="10.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:59" ht="18">
+      <c r="B1" s="90" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="90"/>
+      <c r="D1" s="90"/>
+      <c r="E1" s="90"/>
+      <c r="F1" s="90"/>
+      <c r="G1" s="90"/>
+      <c r="H1" s="90"/>
+      <c r="I1" s="90"/>
+      <c r="J1" s="90"/>
+      <c r="K1" s="90"/>
+      <c r="L1" s="90"/>
+      <c r="M1" s="90"/>
+      <c r="N1" s="90"/>
+      <c r="O1" s="90"/>
+      <c r="P1" s="90"/>
+      <c r="Q1" s="90"/>
+      <c r="R1" s="90"/>
+      <c r="S1" s="90"/>
+      <c r="T1" s="90"/>
+      <c r="U1" s="90"/>
+      <c r="V1" s="90"/>
+      <c r="W1" s="90"/>
+      <c r="X1" s="90"/>
+      <c r="Y1" s="90"/>
+      <c r="Z1" s="90"/>
+      <c r="AA1" s="90"/>
+      <c r="AB1" s="90"/>
+      <c r="AC1" s="90"/>
+      <c r="AD1" s="90"/>
+      <c r="AE1" s="90" t="s">
+        <v>0</v>
+      </c>
+      <c r="AF1" s="90"/>
+      <c r="AG1" s="90"/>
+      <c r="AH1" s="90"/>
+      <c r="AI1" s="90"/>
+      <c r="AJ1" s="90"/>
+      <c r="AK1" s="90"/>
+      <c r="AL1" s="90"/>
+      <c r="AM1" s="90"/>
+      <c r="AN1" s="90"/>
+      <c r="AO1" s="90"/>
+      <c r="AP1" s="90"/>
+      <c r="AQ1" s="90"/>
+      <c r="AR1" s="90"/>
+      <c r="AS1" s="90"/>
+      <c r="AT1" s="90"/>
+      <c r="AU1" s="90"/>
+      <c r="AV1" s="90"/>
+      <c r="AW1" s="90"/>
+      <c r="AX1" s="90"/>
+      <c r="AY1" s="90"/>
+      <c r="AZ1" s="90"/>
+      <c r="BA1" s="90"/>
+      <c r="BB1" s="90"/>
+      <c r="BC1" s="90"/>
+      <c r="BD1" s="90"/>
+      <c r="BE1" s="90"/>
+      <c r="BF1" s="90"/>
+      <c r="BG1" s="90"/>
+    </row>
+    <row r="2" spans="1:59" ht="18">
+      <c r="B2" s="23" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="23" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" s="88"/>
+      <c r="E2" s="88"/>
+      <c r="F2" s="88"/>
+      <c r="G2" s="88"/>
+      <c r="H2" s="88"/>
+      <c r="I2" s="88"/>
+      <c r="J2" s="88"/>
+      <c r="K2" s="88"/>
+      <c r="L2" s="88"/>
+      <c r="M2" s="88"/>
+      <c r="N2" s="88"/>
+      <c r="O2" s="88"/>
+      <c r="P2" s="88"/>
+      <c r="Q2" s="88"/>
+      <c r="R2" s="88"/>
+      <c r="S2" s="88"/>
+      <c r="T2" s="88"/>
+      <c r="U2" s="88"/>
+      <c r="V2" s="88"/>
+      <c r="W2" s="88"/>
+      <c r="X2" s="88"/>
+      <c r="Y2" s="88"/>
+      <c r="Z2" s="88"/>
+      <c r="AA2" s="88"/>
+      <c r="AB2" s="88"/>
+      <c r="AC2" s="88"/>
+      <c r="AD2" s="88"/>
+      <c r="AE2" s="23" t="s">
+        <v>1</v>
+      </c>
+      <c r="AF2" s="23" t="s">
+        <v>2</v>
+      </c>
+      <c r="AG2" s="88"/>
+      <c r="AH2" s="88"/>
+      <c r="AI2" s="88"/>
+      <c r="AJ2" s="88"/>
+      <c r="AK2" s="88"/>
+      <c r="AL2" s="88"/>
+      <c r="AM2" s="88"/>
+      <c r="AN2" s="88"/>
+      <c r="AO2" s="88"/>
+      <c r="AP2" s="88"/>
+      <c r="AQ2" s="88"/>
+      <c r="AR2" s="88"/>
+      <c r="AS2" s="88"/>
+      <c r="AT2" s="88"/>
+      <c r="AU2" s="88"/>
+      <c r="AV2" s="88"/>
+      <c r="AW2" s="88"/>
+      <c r="AX2" s="88"/>
+      <c r="AY2" s="88"/>
+      <c r="AZ2" s="88"/>
+      <c r="BA2" s="88"/>
+      <c r="BB2" s="88"/>
+      <c r="BC2" s="88"/>
+      <c r="BD2" s="88"/>
+      <c r="BE2" s="88"/>
+      <c r="BF2" s="88"/>
+      <c r="BG2" s="88"/>
+    </row>
+    <row r="3" spans="1:59">
+      <c r="B3" s="91" t="s">
+        <v>3</v>
+      </c>
+      <c r="C3" s="91"/>
+      <c r="D3" s="89"/>
+      <c r="E3" s="3">
+        <v>2</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="G3" s="5"/>
+      <c r="H3" s="5"/>
+      <c r="I3" s="5"/>
+      <c r="J3" s="6"/>
+      <c r="K3" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="L3" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="M3" s="7"/>
+      <c r="N3" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="O3" s="7">
+        <v>1</v>
+      </c>
+      <c r="P3" s="7"/>
+      <c r="Q3" s="7"/>
+      <c r="R3" s="7"/>
+      <c r="S3" s="7"/>
+      <c r="T3" s="6"/>
+      <c r="U3" s="6"/>
+      <c r="V3" s="6"/>
+      <c r="W3" s="6"/>
+      <c r="X3" s="6"/>
+      <c r="Y3" s="6"/>
+      <c r="Z3" s="6"/>
+      <c r="AA3" s="6"/>
+      <c r="AB3" s="6"/>
+      <c r="AC3" s="6"/>
+      <c r="AD3" s="6"/>
+      <c r="AE3" s="91" t="s">
+        <v>3</v>
+      </c>
+      <c r="AF3" s="91"/>
+      <c r="AG3" s="89"/>
+      <c r="AH3" s="3">
+        <v>2</v>
+      </c>
+      <c r="AI3" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="AJ3" s="5"/>
+      <c r="AK3" s="5"/>
+      <c r="AL3" s="5"/>
+      <c r="AM3" s="6"/>
+      <c r="AN3" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="AO3" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="AP3" s="7"/>
+      <c r="AQ3" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="AR3" s="7">
+        <v>1</v>
+      </c>
+      <c r="AS3" s="7"/>
+      <c r="AT3" s="7"/>
+      <c r="AU3" s="7"/>
+      <c r="AV3" s="7"/>
+      <c r="AW3" s="6"/>
+      <c r="AX3" s="6"/>
+      <c r="AY3" s="6"/>
+      <c r="AZ3" s="6"/>
+      <c r="BA3" s="6"/>
+      <c r="BB3" s="6"/>
+      <c r="BC3" s="6"/>
+      <c r="BD3" s="6"/>
+      <c r="BE3" s="6"/>
+      <c r="BF3" s="6"/>
+      <c r="BG3" s="6"/>
+    </row>
+    <row r="4" spans="1:59" ht="42.75">
+      <c r="A4" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="D4" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="E4" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="F4" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="G4" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="H4" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="I4" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="J4" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="K4" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="L4" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="M4" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="N4" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="O4" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="P4" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="Q4" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="R4" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="S4" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="T4" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="U4" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="V4" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="W4" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="X4" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y4" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z4" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="AA4" s="16" t="s">
+        <v>30</v>
+      </c>
+      <c r="AB4" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="AC4" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="AD4" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="AE4" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="AF4" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="AG4" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="AH4" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="AI4" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="AJ4" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="AK4" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="AL4" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="AM4" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="AN4" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="AO4" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="AP4" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="AQ4" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="AR4" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="AS4" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="AT4" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="AU4" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="AV4" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="AW4" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="AX4" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="AY4" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="AZ4" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="BA4" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="BB4" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="BC4" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="BD4" s="16" t="s">
+        <v>30</v>
+      </c>
+      <c r="BE4" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="BF4" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="BG4" s="17" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="5" spans="1:59">
+      <c r="A5" s="9">
+        <v>1</v>
+      </c>
+      <c r="B5" s="9">
+        <v>1</v>
+      </c>
+      <c r="C5" s="27" t="s">
+        <v>41</v>
+      </c>
+      <c r="D5" s="9">
+        <v>0</v>
+      </c>
+      <c r="E5" s="27" t="s">
+        <v>42</v>
+      </c>
+      <c r="F5" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="G5" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="H5" s="24">
+        <v>1</v>
+      </c>
+      <c r="I5" s="9">
+        <v>2255</v>
+      </c>
+      <c r="J5" s="8">
+        <v>2255</v>
+      </c>
+      <c r="K5" s="25"/>
+      <c r="L5" s="25"/>
+      <c r="M5" s="25"/>
+      <c r="N5" s="8">
+        <v>2255</v>
+      </c>
+      <c r="O5" s="8">
+        <v>0</v>
+      </c>
+      <c r="P5" s="8">
+        <v>2255</v>
+      </c>
+      <c r="Q5" s="8">
+        <v>0</v>
+      </c>
+      <c r="R5" s="8">
+        <v>2255</v>
+      </c>
+      <c r="S5" s="8">
+        <v>0</v>
+      </c>
+      <c r="T5" s="26">
+        <v>0</v>
+      </c>
+      <c r="U5" s="26">
+        <v>0</v>
+      </c>
+      <c r="V5" s="8">
+        <f>(J5-T5)</f>
+        <v>2255</v>
+      </c>
+      <c r="W5" s="24">
+        <v>88363222</v>
+      </c>
+      <c r="X5" s="18">
+        <v>0.18</v>
+      </c>
+      <c r="Y5" s="24">
+        <f>IF($E$3=1,ROUND(((V5*X5)/2),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="Z5" s="24">
+        <f>IF($E$3=1,ROUND(((V5*X5)/2),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="AA5" s="24">
+        <f>IF($E$3=2,ROUND(((V5*X5)),2),0)</f>
+        <v>405.9</v>
+      </c>
+      <c r="AB5" s="24">
+        <v>0</v>
+      </c>
+      <c r="AC5" s="24">
+        <f>Y5+Z5+AA5</f>
+        <v>405.9</v>
+      </c>
+      <c r="AD5" s="24">
+        <f>V5+AC5</f>
+        <v>2660.9</v>
+      </c>
+      <c r="AE5" s="9">
+        <v>1</v>
+      </c>
+      <c r="AF5" s="27" t="s">
+        <v>44</v>
+      </c>
+      <c r="AG5" s="9">
+        <v>0</v>
+      </c>
+      <c r="AH5" s="27" t="s">
+        <v>44</v>
+      </c>
+      <c r="AI5" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="AJ5" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="AK5" s="24">
+        <v>2</v>
+      </c>
+      <c r="AL5" s="9">
+        <v>250.25</v>
+      </c>
+      <c r="AM5" s="8">
+        <v>500.5</v>
+      </c>
+      <c r="AN5" s="25">
+        <v>2.21</v>
+      </c>
+      <c r="AO5" s="25">
+        <v>1.79</v>
+      </c>
+      <c r="AP5" s="25">
+        <v>2.5</v>
+      </c>
+      <c r="AQ5" s="8">
+        <v>500.5</v>
+      </c>
+      <c r="AR5" s="8">
+        <f>ROUND(AN5*AQ5%,2)</f>
+        <v>11.06</v>
+      </c>
+      <c r="AS5" s="8">
+        <f>AM5-AR5</f>
+        <v>489.44</v>
+      </c>
+      <c r="AT5" s="8">
+        <f>ROUND(AO5*AS5%,2)</f>
+        <v>8.76</v>
+      </c>
+      <c r="AU5" s="8">
+        <f>AS5-AT5</f>
+        <v>480.68</v>
+      </c>
+      <c r="AV5" s="8">
+        <f>ROUND(AP5*AU5%,2)</f>
+        <v>12.02</v>
+      </c>
+      <c r="AW5" s="26">
+        <f>AR5+AT5+AV5</f>
+        <v>31.84</v>
+      </c>
+      <c r="AX5" s="26">
+        <v>0</v>
+      </c>
+      <c r="AY5" s="8">
+        <f>(AM5-AW5)</f>
+        <v>468.66</v>
+      </c>
+      <c r="AZ5" s="24">
+        <v>88363222</v>
+      </c>
+      <c r="BA5" s="18">
+        <v>0.18</v>
+      </c>
+      <c r="BB5" s="24">
+        <f>IF($AH$3=1,ROUND(((AY5*BA5)/2),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="BC5" s="24">
+        <f>IF($AH$3=1,ROUND(((AY5*BA5)/2),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="BD5" s="40">
+        <f>IF($AH$3=2,ROUND(((AY5*BA5)),2),0)</f>
+        <v>84.36</v>
+      </c>
+      <c r="BE5" s="24">
+        <f>IF($AH$3=4,ROUND(((AY5*BA5)),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="BF5" s="40">
+        <f>BB5+BC5+BD5</f>
+        <v>84.36</v>
+      </c>
+      <c r="BG5" s="24">
+        <f>AY5+BF5</f>
+        <v>553.02</v>
+      </c>
+    </row>
+    <row r="6" spans="1:59">
+      <c r="B6" s="19"/>
+      <c r="C6" s="19"/>
+      <c r="D6" s="19"/>
+      <c r="E6" s="19"/>
+      <c r="F6" s="19"/>
+      <c r="G6" s="19"/>
+      <c r="H6" s="20"/>
+      <c r="I6" s="21"/>
+      <c r="J6" s="21"/>
+      <c r="K6" s="22"/>
+      <c r="L6" s="22"/>
+      <c r="M6" s="22"/>
+      <c r="N6" s="21"/>
+      <c r="O6" s="21"/>
+      <c r="P6" s="21"/>
+      <c r="Q6" s="21"/>
+      <c r="R6" s="21"/>
+      <c r="S6" s="21"/>
+      <c r="T6" s="21"/>
+      <c r="U6" s="21"/>
+      <c r="V6" s="21"/>
+      <c r="W6" s="21"/>
+      <c r="X6" s="22"/>
+      <c r="Y6" s="21"/>
+      <c r="Z6" s="21"/>
+      <c r="AA6" s="21"/>
+      <c r="AB6" s="21"/>
+      <c r="AC6" s="21"/>
+      <c r="AD6" s="21"/>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="B1:AD1"/>
+    <mergeCell ref="AE1:BG1"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="AE3:AF3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -10601,37 +11268,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="18">
-      <c r="A1" s="88" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="88"/>
-      <c r="C1" s="88"/>
-      <c r="D1" s="88"/>
-      <c r="E1" s="88"/>
-      <c r="F1" s="88"/>
-      <c r="G1" s="88"/>
-      <c r="H1" s="88"/>
-      <c r="I1" s="88"/>
-      <c r="J1" s="88"/>
-      <c r="K1" s="88"/>
-      <c r="L1" s="88"/>
-      <c r="M1" s="88"/>
-      <c r="N1" s="88"/>
-      <c r="O1" s="88"/>
-      <c r="P1" s="88"/>
-      <c r="Q1" s="88"/>
-      <c r="R1" s="88"/>
-      <c r="S1" s="88"/>
-      <c r="T1" s="88"/>
-      <c r="U1" s="88"/>
-      <c r="V1" s="88"/>
-      <c r="W1" s="88"/>
-      <c r="X1" s="88"/>
-      <c r="Y1" s="88"/>
-      <c r="Z1" s="88"/>
-      <c r="AA1" s="88"/>
-      <c r="AB1" s="88"/>
-      <c r="AC1" s="88"/>
+      <c r="A1" s="90" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="90"/>
+      <c r="C1" s="90"/>
+      <c r="D1" s="90"/>
+      <c r="E1" s="90"/>
+      <c r="F1" s="90"/>
+      <c r="G1" s="90"/>
+      <c r="H1" s="90"/>
+      <c r="I1" s="90"/>
+      <c r="J1" s="90"/>
+      <c r="K1" s="90"/>
+      <c r="L1" s="90"/>
+      <c r="M1" s="90"/>
+      <c r="N1" s="90"/>
+      <c r="O1" s="90"/>
+      <c r="P1" s="90"/>
+      <c r="Q1" s="90"/>
+      <c r="R1" s="90"/>
+      <c r="S1" s="90"/>
+      <c r="T1" s="90"/>
+      <c r="U1" s="90"/>
+      <c r="V1" s="90"/>
+      <c r="W1" s="90"/>
+      <c r="X1" s="90"/>
+      <c r="Y1" s="90"/>
+      <c r="Z1" s="90"/>
+      <c r="AA1" s="90"/>
+      <c r="AB1" s="90"/>
+      <c r="AC1" s="90"/>
     </row>
     <row r="2" spans="1:29" ht="18">
       <c r="A2" s="23" t="s">
@@ -10669,10 +11336,10 @@
       <c r="AC2" s="28"/>
     </row>
     <row r="3" spans="1:29">
-      <c r="A3" s="89" t="s">
+      <c r="A3" s="91" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="89"/>
+      <c r="B3" s="91"/>
       <c r="C3" s="29"/>
       <c r="D3" s="3">
         <v>4</v>
@@ -10955,37 +11622,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="18">
-      <c r="A1" s="88" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="88"/>
-      <c r="C1" s="88"/>
-      <c r="D1" s="88"/>
-      <c r="E1" s="88"/>
-      <c r="F1" s="88"/>
-      <c r="G1" s="88"/>
-      <c r="H1" s="88"/>
-      <c r="I1" s="88"/>
-      <c r="J1" s="88"/>
-      <c r="K1" s="88"/>
-      <c r="L1" s="88"/>
-      <c r="M1" s="88"/>
-      <c r="N1" s="88"/>
-      <c r="O1" s="88"/>
-      <c r="P1" s="88"/>
-      <c r="Q1" s="88"/>
-      <c r="R1" s="88"/>
-      <c r="S1" s="88"/>
-      <c r="T1" s="88"/>
-      <c r="U1" s="88"/>
-      <c r="V1" s="88"/>
-      <c r="W1" s="88"/>
-      <c r="X1" s="88"/>
-      <c r="Y1" s="88"/>
-      <c r="Z1" s="88"/>
-      <c r="AA1" s="88"/>
-      <c r="AB1" s="88"/>
-      <c r="AC1" s="88"/>
+      <c r="A1" s="90" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="90"/>
+      <c r="C1" s="90"/>
+      <c r="D1" s="90"/>
+      <c r="E1" s="90"/>
+      <c r="F1" s="90"/>
+      <c r="G1" s="90"/>
+      <c r="H1" s="90"/>
+      <c r="I1" s="90"/>
+      <c r="J1" s="90"/>
+      <c r="K1" s="90"/>
+      <c r="L1" s="90"/>
+      <c r="M1" s="90"/>
+      <c r="N1" s="90"/>
+      <c r="O1" s="90"/>
+      <c r="P1" s="90"/>
+      <c r="Q1" s="90"/>
+      <c r="R1" s="90"/>
+      <c r="S1" s="90"/>
+      <c r="T1" s="90"/>
+      <c r="U1" s="90"/>
+      <c r="V1" s="90"/>
+      <c r="W1" s="90"/>
+      <c r="X1" s="90"/>
+      <c r="Y1" s="90"/>
+      <c r="Z1" s="90"/>
+      <c r="AA1" s="90"/>
+      <c r="AB1" s="90"/>
+      <c r="AC1" s="90"/>
     </row>
     <row r="2" spans="1:29" ht="18">
       <c r="A2" s="23" t="s">
@@ -11023,10 +11690,10 @@
       <c r="AC2" s="28"/>
     </row>
     <row r="3" spans="1:29">
-      <c r="A3" s="89" t="s">
+      <c r="A3" s="91" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="89"/>
+      <c r="B3" s="91"/>
       <c r="C3" s="29"/>
       <c r="D3" s="3">
         <v>3</v>
@@ -11308,37 +11975,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="18">
-      <c r="A1" s="88" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="88"/>
-      <c r="C1" s="88"/>
-      <c r="D1" s="88"/>
-      <c r="E1" s="88"/>
-      <c r="F1" s="88"/>
-      <c r="G1" s="88"/>
-      <c r="H1" s="88"/>
-      <c r="I1" s="88"/>
-      <c r="J1" s="88"/>
-      <c r="K1" s="88"/>
-      <c r="L1" s="88"/>
-      <c r="M1" s="88"/>
-      <c r="N1" s="88"/>
-      <c r="O1" s="88"/>
-      <c r="P1" s="88"/>
-      <c r="Q1" s="88"/>
-      <c r="R1" s="88"/>
-      <c r="S1" s="88"/>
-      <c r="T1" s="88"/>
-      <c r="U1" s="88"/>
-      <c r="V1" s="88"/>
-      <c r="W1" s="88"/>
-      <c r="X1" s="88"/>
-      <c r="Y1" s="88"/>
-      <c r="Z1" s="88"/>
-      <c r="AA1" s="88"/>
-      <c r="AB1" s="88"/>
-      <c r="AC1" s="88"/>
+      <c r="A1" s="90" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="90"/>
+      <c r="C1" s="90"/>
+      <c r="D1" s="90"/>
+      <c r="E1" s="90"/>
+      <c r="F1" s="90"/>
+      <c r="G1" s="90"/>
+      <c r="H1" s="90"/>
+      <c r="I1" s="90"/>
+      <c r="J1" s="90"/>
+      <c r="K1" s="90"/>
+      <c r="L1" s="90"/>
+      <c r="M1" s="90"/>
+      <c r="N1" s="90"/>
+      <c r="O1" s="90"/>
+      <c r="P1" s="90"/>
+      <c r="Q1" s="90"/>
+      <c r="R1" s="90"/>
+      <c r="S1" s="90"/>
+      <c r="T1" s="90"/>
+      <c r="U1" s="90"/>
+      <c r="V1" s="90"/>
+      <c r="W1" s="90"/>
+      <c r="X1" s="90"/>
+      <c r="Y1" s="90"/>
+      <c r="Z1" s="90"/>
+      <c r="AA1" s="90"/>
+      <c r="AB1" s="90"/>
+      <c r="AC1" s="90"/>
     </row>
     <row r="2" spans="1:29" ht="18">
       <c r="A2" s="23" t="s">
@@ -11376,10 +12043,10 @@
       <c r="AC2" s="28"/>
     </row>
     <row r="3" spans="1:29">
-      <c r="A3" s="89" t="s">
+      <c r="A3" s="91" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="89"/>
+      <c r="B3" s="91"/>
       <c r="C3" s="29"/>
       <c r="D3" s="3">
         <v>5</v>
@@ -11663,37 +12330,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="18">
-      <c r="A1" s="88" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="88"/>
-      <c r="C1" s="88"/>
-      <c r="D1" s="88"/>
-      <c r="E1" s="88"/>
-      <c r="F1" s="88"/>
-      <c r="G1" s="88"/>
-      <c r="H1" s="88"/>
-      <c r="I1" s="88"/>
-      <c r="J1" s="88"/>
-      <c r="K1" s="88"/>
-      <c r="L1" s="88"/>
-      <c r="M1" s="88"/>
-      <c r="N1" s="88"/>
-      <c r="O1" s="88"/>
-      <c r="P1" s="88"/>
-      <c r="Q1" s="88"/>
-      <c r="R1" s="88"/>
-      <c r="S1" s="88"/>
-      <c r="T1" s="88"/>
-      <c r="U1" s="88"/>
-      <c r="V1" s="88"/>
-      <c r="W1" s="88"/>
-      <c r="X1" s="88"/>
-      <c r="Y1" s="88"/>
-      <c r="Z1" s="88"/>
-      <c r="AA1" s="88"/>
-      <c r="AB1" s="88"/>
-      <c r="AC1" s="88"/>
+      <c r="A1" s="90" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="90"/>
+      <c r="C1" s="90"/>
+      <c r="D1" s="90"/>
+      <c r="E1" s="90"/>
+      <c r="F1" s="90"/>
+      <c r="G1" s="90"/>
+      <c r="H1" s="90"/>
+      <c r="I1" s="90"/>
+      <c r="J1" s="90"/>
+      <c r="K1" s="90"/>
+      <c r="L1" s="90"/>
+      <c r="M1" s="90"/>
+      <c r="N1" s="90"/>
+      <c r="O1" s="90"/>
+      <c r="P1" s="90"/>
+      <c r="Q1" s="90"/>
+      <c r="R1" s="90"/>
+      <c r="S1" s="90"/>
+      <c r="T1" s="90"/>
+      <c r="U1" s="90"/>
+      <c r="V1" s="90"/>
+      <c r="W1" s="90"/>
+      <c r="X1" s="90"/>
+      <c r="Y1" s="90"/>
+      <c r="Z1" s="90"/>
+      <c r="AA1" s="90"/>
+      <c r="AB1" s="90"/>
+      <c r="AC1" s="90"/>
     </row>
     <row r="2" spans="1:29" ht="18">
       <c r="A2" s="23" t="s">
@@ -11731,10 +12398,10 @@
       <c r="AC2" s="32"/>
     </row>
     <row r="3" spans="1:29">
-      <c r="A3" s="89" t="s">
+      <c r="A3" s="91" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="89"/>
+      <c r="B3" s="91"/>
       <c r="C3" s="33"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -12016,37 +12683,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="18">
-      <c r="A1" s="88" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="88"/>
-      <c r="C1" s="88"/>
-      <c r="D1" s="88"/>
-      <c r="E1" s="88"/>
-      <c r="F1" s="88"/>
-      <c r="G1" s="88"/>
-      <c r="H1" s="88"/>
-      <c r="I1" s="88"/>
-      <c r="J1" s="88"/>
-      <c r="K1" s="88"/>
-      <c r="L1" s="88"/>
-      <c r="M1" s="88"/>
-      <c r="N1" s="88"/>
-      <c r="O1" s="88"/>
-      <c r="P1" s="88"/>
-      <c r="Q1" s="88"/>
-      <c r="R1" s="88"/>
-      <c r="S1" s="88"/>
-      <c r="T1" s="88"/>
-      <c r="U1" s="88"/>
-      <c r="V1" s="88"/>
-      <c r="W1" s="88"/>
-      <c r="X1" s="88"/>
-      <c r="Y1" s="88"/>
-      <c r="Z1" s="88"/>
-      <c r="AA1" s="88"/>
-      <c r="AB1" s="88"/>
-      <c r="AC1" s="88"/>
+      <c r="A1" s="90" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="90"/>
+      <c r="C1" s="90"/>
+      <c r="D1" s="90"/>
+      <c r="E1" s="90"/>
+      <c r="F1" s="90"/>
+      <c r="G1" s="90"/>
+      <c r="H1" s="90"/>
+      <c r="I1" s="90"/>
+      <c r="J1" s="90"/>
+      <c r="K1" s="90"/>
+      <c r="L1" s="90"/>
+      <c r="M1" s="90"/>
+      <c r="N1" s="90"/>
+      <c r="O1" s="90"/>
+      <c r="P1" s="90"/>
+      <c r="Q1" s="90"/>
+      <c r="R1" s="90"/>
+      <c r="S1" s="90"/>
+      <c r="T1" s="90"/>
+      <c r="U1" s="90"/>
+      <c r="V1" s="90"/>
+      <c r="W1" s="90"/>
+      <c r="X1" s="90"/>
+      <c r="Y1" s="90"/>
+      <c r="Z1" s="90"/>
+      <c r="AA1" s="90"/>
+      <c r="AB1" s="90"/>
+      <c r="AC1" s="90"/>
     </row>
     <row r="2" spans="1:29" ht="18">
       <c r="A2" s="23" t="s">
@@ -12084,10 +12751,10 @@
       <c r="AC2" s="34"/>
     </row>
     <row r="3" spans="1:29">
-      <c r="A3" s="89" t="s">
+      <c r="A3" s="91" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="89"/>
+      <c r="B3" s="91"/>
       <c r="C3" s="35"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -12367,38 +13034,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:30" ht="18">
-      <c r="A1" s="88" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="88"/>
-      <c r="C1" s="88"/>
-      <c r="D1" s="88"/>
-      <c r="E1" s="88"/>
-      <c r="F1" s="88"/>
-      <c r="G1" s="88"/>
-      <c r="H1" s="88"/>
-      <c r="I1" s="88"/>
-      <c r="J1" s="88"/>
-      <c r="K1" s="88"/>
-      <c r="L1" s="88"/>
-      <c r="M1" s="88"/>
-      <c r="N1" s="88"/>
-      <c r="O1" s="88"/>
-      <c r="P1" s="88"/>
-      <c r="Q1" s="88"/>
-      <c r="R1" s="88"/>
-      <c r="S1" s="88"/>
-      <c r="T1" s="88"/>
-      <c r="U1" s="88"/>
-      <c r="V1" s="88"/>
-      <c r="W1" s="88"/>
-      <c r="X1" s="88"/>
-      <c r="Y1" s="88"/>
-      <c r="Z1" s="88"/>
-      <c r="AA1" s="88"/>
-      <c r="AB1" s="88"/>
-      <c r="AC1" s="88"/>
-      <c r="AD1" s="88"/>
+      <c r="A1" s="90" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="90"/>
+      <c r="C1" s="90"/>
+      <c r="D1" s="90"/>
+      <c r="E1" s="90"/>
+      <c r="F1" s="90"/>
+      <c r="G1" s="90"/>
+      <c r="H1" s="90"/>
+      <c r="I1" s="90"/>
+      <c r="J1" s="90"/>
+      <c r="K1" s="90"/>
+      <c r="L1" s="90"/>
+      <c r="M1" s="90"/>
+      <c r="N1" s="90"/>
+      <c r="O1" s="90"/>
+      <c r="P1" s="90"/>
+      <c r="Q1" s="90"/>
+      <c r="R1" s="90"/>
+      <c r="S1" s="90"/>
+      <c r="T1" s="90"/>
+      <c r="U1" s="90"/>
+      <c r="V1" s="90"/>
+      <c r="W1" s="90"/>
+      <c r="X1" s="90"/>
+      <c r="Y1" s="90"/>
+      <c r="Z1" s="90"/>
+      <c r="AA1" s="90"/>
+      <c r="AB1" s="90"/>
+      <c r="AC1" s="90"/>
+      <c r="AD1" s="90"/>
     </row>
     <row r="2" spans="1:30" ht="18">
       <c r="A2" s="23" t="s">
@@ -12437,10 +13104,10 @@
       <c r="AD2" s="36"/>
     </row>
     <row r="3" spans="1:30">
-      <c r="A3" s="89" t="s">
+      <c r="A3" s="91" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="89"/>
+      <c r="B3" s="91"/>
       <c r="C3" s="83"/>
       <c r="D3" s="37"/>
       <c r="E3" s="3">
@@ -12743,37 +13410,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:31" ht="18">
-      <c r="A1" s="88" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="88"/>
-      <c r="C1" s="88"/>
-      <c r="D1" s="88"/>
-      <c r="E1" s="88"/>
-      <c r="F1" s="88"/>
-      <c r="G1" s="88"/>
-      <c r="H1" s="88"/>
-      <c r="I1" s="88"/>
-      <c r="J1" s="88"/>
-      <c r="K1" s="88"/>
-      <c r="L1" s="88"/>
-      <c r="M1" s="88"/>
-      <c r="N1" s="88"/>
-      <c r="O1" s="88"/>
-      <c r="P1" s="88"/>
-      <c r="Q1" s="88"/>
-      <c r="R1" s="88"/>
-      <c r="S1" s="88"/>
-      <c r="T1" s="88"/>
-      <c r="U1" s="88"/>
-      <c r="V1" s="88"/>
-      <c r="W1" s="88"/>
-      <c r="X1" s="88"/>
-      <c r="Y1" s="88"/>
-      <c r="Z1" s="88"/>
-      <c r="AA1" s="88"/>
-      <c r="AB1" s="88"/>
-      <c r="AC1" s="88"/>
+      <c r="A1" s="90" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="90"/>
+      <c r="C1" s="90"/>
+      <c r="D1" s="90"/>
+      <c r="E1" s="90"/>
+      <c r="F1" s="90"/>
+      <c r="G1" s="90"/>
+      <c r="H1" s="90"/>
+      <c r="I1" s="90"/>
+      <c r="J1" s="90"/>
+      <c r="K1" s="90"/>
+      <c r="L1" s="90"/>
+      <c r="M1" s="90"/>
+      <c r="N1" s="90"/>
+      <c r="O1" s="90"/>
+      <c r="P1" s="90"/>
+      <c r="Q1" s="90"/>
+      <c r="R1" s="90"/>
+      <c r="S1" s="90"/>
+      <c r="T1" s="90"/>
+      <c r="U1" s="90"/>
+      <c r="V1" s="90"/>
+      <c r="W1" s="90"/>
+      <c r="X1" s="90"/>
+      <c r="Y1" s="90"/>
+      <c r="Z1" s="90"/>
+      <c r="AA1" s="90"/>
+      <c r="AB1" s="90"/>
+      <c r="AC1" s="90"/>
     </row>
     <row r="2" spans="1:31" ht="16.5" customHeight="1">
       <c r="A2" s="23" t="s">
@@ -12811,10 +13478,10 @@
       <c r="AC2" s="41"/>
     </row>
     <row r="3" spans="1:31">
-      <c r="A3" s="89" t="s">
+      <c r="A3" s="91" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="89"/>
+      <c r="B3" s="91"/>
       <c r="D3">
         <v>2</v>
       </c>

</xml_diff>

<commit_message>
Purchase Bills Function Failure Fixes
Purchase Bills Function Failure Fixes
</commit_message>
<xml_diff>
--- a/testdata/DBfin.xlsx
+++ b/testdata/DBfin.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4507"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="2520" windowWidth="15240" windowHeight="6540" tabRatio="849" firstSheet="21" activeTab="26"/>
+    <workbookView xWindow="0" yWindow="2520" windowWidth="15240" windowHeight="6540" tabRatio="849" firstSheet="22" activeTab="27"/>
   </bookViews>
   <sheets>
     <sheet name="PurchaseBillsLocal" sheetId="1" r:id="rId1"/>
@@ -34,13 +34,14 @@
     <sheet name="PurchaseBills_Import" sheetId="24" r:id="rId25"/>
     <sheet name="PurchaseBills_IGST_Validation_2" sheetId="26" r:id="rId26"/>
     <sheet name="Purchase_Bills_Allow_IGST" sheetId="27" r:id="rId27"/>
+    <sheet name="purchaseBills_GRN_igst" sheetId="28" r:id="rId28"/>
   </sheets>
   <calcPr calcId="125725"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1508" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1566" uniqueCount="115">
   <si>
     <t>Scenario  : Local Sales - Stock UOM and Sales UOM (Similar)   DOC NO :  SORD-2425-00089</t>
   </si>
@@ -384,15 +385,19 @@
   <si>
     <t>null</t>
   </si>
+  <si>
+    <t>Null</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="0.000"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
+    <numFmt numFmtId="167" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="11">
     <font>
@@ -579,7 +584,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="92">
+  <cellXfs count="94">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -797,9 +802,13 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="167" fontId="3" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Comma" xfId="2" builtinId="3"/>
@@ -1125,68 +1134,68 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:59" ht="18">
-      <c r="A1" s="90" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="90"/>
-      <c r="C1" s="90"/>
-      <c r="D1" s="90"/>
-      <c r="E1" s="90"/>
-      <c r="F1" s="90"/>
-      <c r="G1" s="90"/>
-      <c r="H1" s="90"/>
-      <c r="I1" s="90"/>
-      <c r="J1" s="90"/>
-      <c r="K1" s="90"/>
-      <c r="L1" s="90"/>
-      <c r="M1" s="90"/>
-      <c r="N1" s="90"/>
-      <c r="O1" s="90"/>
-      <c r="P1" s="90"/>
-      <c r="Q1" s="90"/>
-      <c r="R1" s="90"/>
-      <c r="S1" s="90"/>
-      <c r="T1" s="90"/>
-      <c r="U1" s="90"/>
-      <c r="V1" s="90"/>
-      <c r="W1" s="90"/>
-      <c r="X1" s="90"/>
-      <c r="Y1" s="90"/>
-      <c r="Z1" s="90"/>
-      <c r="AA1" s="90"/>
-      <c r="AB1" s="90"/>
-      <c r="AC1" s="90"/>
-      <c r="AD1" s="90" t="s">
-        <v>0</v>
-      </c>
-      <c r="AE1" s="90"/>
-      <c r="AF1" s="90"/>
-      <c r="AG1" s="90"/>
-      <c r="AH1" s="90"/>
-      <c r="AI1" s="90"/>
-      <c r="AJ1" s="90"/>
-      <c r="AK1" s="90"/>
-      <c r="AL1" s="90"/>
-      <c r="AM1" s="90"/>
-      <c r="AN1" s="90"/>
-      <c r="AO1" s="90"/>
-      <c r="AP1" s="90"/>
-      <c r="AQ1" s="90"/>
-      <c r="AR1" s="90"/>
-      <c r="AS1" s="90"/>
-      <c r="AT1" s="90"/>
-      <c r="AU1" s="90"/>
-      <c r="AV1" s="90"/>
-      <c r="AW1" s="90"/>
-      <c r="AX1" s="90"/>
-      <c r="AY1" s="90"/>
-      <c r="AZ1" s="90"/>
-      <c r="BA1" s="90"/>
-      <c r="BB1" s="90"/>
-      <c r="BC1" s="90"/>
-      <c r="BD1" s="90"/>
-      <c r="BE1" s="90"/>
-      <c r="BF1" s="90"/>
+      <c r="A1" s="91" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="91"/>
+      <c r="C1" s="91"/>
+      <c r="D1" s="91"/>
+      <c r="E1" s="91"/>
+      <c r="F1" s="91"/>
+      <c r="G1" s="91"/>
+      <c r="H1" s="91"/>
+      <c r="I1" s="91"/>
+      <c r="J1" s="91"/>
+      <c r="K1" s="91"/>
+      <c r="L1" s="91"/>
+      <c r="M1" s="91"/>
+      <c r="N1" s="91"/>
+      <c r="O1" s="91"/>
+      <c r="P1" s="91"/>
+      <c r="Q1" s="91"/>
+      <c r="R1" s="91"/>
+      <c r="S1" s="91"/>
+      <c r="T1" s="91"/>
+      <c r="U1" s="91"/>
+      <c r="V1" s="91"/>
+      <c r="W1" s="91"/>
+      <c r="X1" s="91"/>
+      <c r="Y1" s="91"/>
+      <c r="Z1" s="91"/>
+      <c r="AA1" s="91"/>
+      <c r="AB1" s="91"/>
+      <c r="AC1" s="91"/>
+      <c r="AD1" s="91" t="s">
+        <v>0</v>
+      </c>
+      <c r="AE1" s="91"/>
+      <c r="AF1" s="91"/>
+      <c r="AG1" s="91"/>
+      <c r="AH1" s="91"/>
+      <c r="AI1" s="91"/>
+      <c r="AJ1" s="91"/>
+      <c r="AK1" s="91"/>
+      <c r="AL1" s="91"/>
+      <c r="AM1" s="91"/>
+      <c r="AN1" s="91"/>
+      <c r="AO1" s="91"/>
+      <c r="AP1" s="91"/>
+      <c r="AQ1" s="91"/>
+      <c r="AR1" s="91"/>
+      <c r="AS1" s="91"/>
+      <c r="AT1" s="91"/>
+      <c r="AU1" s="91"/>
+      <c r="AV1" s="91"/>
+      <c r="AW1" s="91"/>
+      <c r="AX1" s="91"/>
+      <c r="AY1" s="91"/>
+      <c r="AZ1" s="91"/>
+      <c r="BA1" s="91"/>
+      <c r="BB1" s="91"/>
+      <c r="BC1" s="91"/>
+      <c r="BD1" s="91"/>
+      <c r="BE1" s="91"/>
+      <c r="BF1" s="91"/>
     </row>
     <row r="2" spans="1:59" ht="18">
       <c r="A2" s="23" t="s">
@@ -1257,10 +1266,10 @@
       <c r="BF2" s="38"/>
     </row>
     <row r="3" spans="1:59">
-      <c r="A3" s="91" t="s">
+      <c r="A3" s="92" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="91"/>
+      <c r="B3" s="92"/>
       <c r="C3" s="2"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -1300,10 +1309,10 @@
       <c r="AA3" s="6"/>
       <c r="AB3" s="6"/>
       <c r="AC3" s="6"/>
-      <c r="AD3" s="91" t="s">
+      <c r="AD3" s="92" t="s">
         <v>3</v>
       </c>
-      <c r="AE3" s="91"/>
+      <c r="AE3" s="92"/>
       <c r="AF3" s="39"/>
       <c r="AG3" s="3">
         <v>1</v>
@@ -1781,38 +1790,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:33" ht="18">
-      <c r="A1" s="90" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="90"/>
-      <c r="C1" s="90"/>
-      <c r="D1" s="90"/>
-      <c r="E1" s="90"/>
-      <c r="F1" s="90"/>
-      <c r="G1" s="90"/>
-      <c r="H1" s="90"/>
-      <c r="I1" s="90"/>
-      <c r="J1" s="90"/>
-      <c r="K1" s="90"/>
-      <c r="L1" s="90"/>
-      <c r="M1" s="90"/>
-      <c r="N1" s="90"/>
-      <c r="O1" s="90"/>
-      <c r="P1" s="90"/>
-      <c r="Q1" s="90"/>
-      <c r="R1" s="90"/>
-      <c r="S1" s="90"/>
-      <c r="T1" s="90"/>
-      <c r="U1" s="90"/>
-      <c r="V1" s="90"/>
-      <c r="W1" s="90"/>
-      <c r="X1" s="90"/>
-      <c r="Y1" s="90"/>
-      <c r="Z1" s="90"/>
-      <c r="AA1" s="90"/>
-      <c r="AB1" s="90"/>
-      <c r="AC1" s="90"/>
-      <c r="AD1" s="90"/>
+      <c r="A1" s="91" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="91"/>
+      <c r="C1" s="91"/>
+      <c r="D1" s="91"/>
+      <c r="E1" s="91"/>
+      <c r="F1" s="91"/>
+      <c r="G1" s="91"/>
+      <c r="H1" s="91"/>
+      <c r="I1" s="91"/>
+      <c r="J1" s="91"/>
+      <c r="K1" s="91"/>
+      <c r="L1" s="91"/>
+      <c r="M1" s="91"/>
+      <c r="N1" s="91"/>
+      <c r="O1" s="91"/>
+      <c r="P1" s="91"/>
+      <c r="Q1" s="91"/>
+      <c r="R1" s="91"/>
+      <c r="S1" s="91"/>
+      <c r="T1" s="91"/>
+      <c r="U1" s="91"/>
+      <c r="V1" s="91"/>
+      <c r="W1" s="91"/>
+      <c r="X1" s="91"/>
+      <c r="Y1" s="91"/>
+      <c r="Z1" s="91"/>
+      <c r="AA1" s="91"/>
+      <c r="AB1" s="91"/>
+      <c r="AC1" s="91"/>
+      <c r="AD1" s="91"/>
     </row>
     <row r="2" spans="1:33" ht="18">
       <c r="A2" s="23" t="s">
@@ -1851,10 +1860,10 @@
       <c r="AD2" s="43"/>
     </row>
     <row r="3" spans="1:33" ht="15.75" thickBot="1">
-      <c r="A3" s="91" t="s">
+      <c r="A3" s="92" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="91"/>
+      <c r="B3" s="92"/>
       <c r="C3" s="44"/>
       <c r="D3" s="3">
         <v>2</v>
@@ -2468,37 +2477,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:31" ht="18">
-      <c r="A1" s="90" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="90"/>
-      <c r="C1" s="90"/>
-      <c r="D1" s="90"/>
-      <c r="E1" s="90"/>
-      <c r="F1" s="90"/>
-      <c r="G1" s="90"/>
-      <c r="H1" s="90"/>
-      <c r="I1" s="90"/>
-      <c r="J1" s="90"/>
-      <c r="K1" s="90"/>
-      <c r="L1" s="90"/>
-      <c r="M1" s="90"/>
-      <c r="N1" s="90"/>
-      <c r="O1" s="90"/>
-      <c r="P1" s="90"/>
-      <c r="Q1" s="90"/>
-      <c r="R1" s="90"/>
-      <c r="S1" s="90"/>
-      <c r="T1" s="90"/>
-      <c r="U1" s="90"/>
-      <c r="V1" s="90"/>
-      <c r="W1" s="90"/>
-      <c r="X1" s="90"/>
-      <c r="Y1" s="90"/>
-      <c r="Z1" s="90"/>
-      <c r="AA1" s="90"/>
-      <c r="AB1" s="90"/>
-      <c r="AC1" s="90"/>
+      <c r="A1" s="91" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="91"/>
+      <c r="C1" s="91"/>
+      <c r="D1" s="91"/>
+      <c r="E1" s="91"/>
+      <c r="F1" s="91"/>
+      <c r="G1" s="91"/>
+      <c r="H1" s="91"/>
+      <c r="I1" s="91"/>
+      <c r="J1" s="91"/>
+      <c r="K1" s="91"/>
+      <c r="L1" s="91"/>
+      <c r="M1" s="91"/>
+      <c r="N1" s="91"/>
+      <c r="O1" s="91"/>
+      <c r="P1" s="91"/>
+      <c r="Q1" s="91"/>
+      <c r="R1" s="91"/>
+      <c r="S1" s="91"/>
+      <c r="T1" s="91"/>
+      <c r="U1" s="91"/>
+      <c r="V1" s="91"/>
+      <c r="W1" s="91"/>
+      <c r="X1" s="91"/>
+      <c r="Y1" s="91"/>
+      <c r="Z1" s="91"/>
+      <c r="AA1" s="91"/>
+      <c r="AB1" s="91"/>
+      <c r="AC1" s="91"/>
     </row>
     <row r="2" spans="1:31" ht="16.5" customHeight="1">
       <c r="A2" s="23" t="s">
@@ -2536,10 +2545,10 @@
       <c r="AC2" s="54"/>
     </row>
     <row r="3" spans="1:31">
-      <c r="A3" s="91" t="s">
+      <c r="A3" s="92" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="91"/>
+      <c r="B3" s="92"/>
       <c r="D3">
         <v>2</v>
       </c>
@@ -3030,37 +3039,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="18">
-      <c r="A1" s="90" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="90"/>
-      <c r="C1" s="90"/>
-      <c r="D1" s="90"/>
-      <c r="E1" s="90"/>
-      <c r="F1" s="90"/>
-      <c r="G1" s="90"/>
-      <c r="H1" s="90"/>
-      <c r="I1" s="90"/>
-      <c r="J1" s="90"/>
-      <c r="K1" s="90"/>
-      <c r="L1" s="90"/>
-      <c r="M1" s="90"/>
-      <c r="N1" s="90"/>
-      <c r="O1" s="90"/>
-      <c r="P1" s="90"/>
-      <c r="Q1" s="90"/>
-      <c r="R1" s="90"/>
-      <c r="S1" s="90"/>
-      <c r="T1" s="90"/>
-      <c r="U1" s="90"/>
-      <c r="V1" s="90"/>
-      <c r="W1" s="90"/>
-      <c r="X1" s="90"/>
-      <c r="Y1" s="90"/>
-      <c r="Z1" s="90"/>
-      <c r="AA1" s="90"/>
-      <c r="AB1" s="90"/>
-      <c r="AC1" s="90"/>
+      <c r="A1" s="91" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="91"/>
+      <c r="C1" s="91"/>
+      <c r="D1" s="91"/>
+      <c r="E1" s="91"/>
+      <c r="F1" s="91"/>
+      <c r="G1" s="91"/>
+      <c r="H1" s="91"/>
+      <c r="I1" s="91"/>
+      <c r="J1" s="91"/>
+      <c r="K1" s="91"/>
+      <c r="L1" s="91"/>
+      <c r="M1" s="91"/>
+      <c r="N1" s="91"/>
+      <c r="O1" s="91"/>
+      <c r="P1" s="91"/>
+      <c r="Q1" s="91"/>
+      <c r="R1" s="91"/>
+      <c r="S1" s="91"/>
+      <c r="T1" s="91"/>
+      <c r="U1" s="91"/>
+      <c r="V1" s="91"/>
+      <c r="W1" s="91"/>
+      <c r="X1" s="91"/>
+      <c r="Y1" s="91"/>
+      <c r="Z1" s="91"/>
+      <c r="AA1" s="91"/>
+      <c r="AB1" s="91"/>
+      <c r="AC1" s="91"/>
     </row>
     <row r="2" spans="1:29" ht="18">
       <c r="A2" s="23" t="s">
@@ -3098,10 +3107,10 @@
       <c r="AC2" s="56"/>
     </row>
     <row r="3" spans="1:29">
-      <c r="A3" s="91" t="s">
+      <c r="A3" s="92" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="91"/>
+      <c r="B3" s="92"/>
       <c r="C3" s="57"/>
       <c r="D3" s="3">
         <v>2</v>
@@ -3382,37 +3391,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="18">
-      <c r="A1" s="90" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="90"/>
-      <c r="C1" s="90"/>
-      <c r="D1" s="90"/>
-      <c r="E1" s="90"/>
-      <c r="F1" s="90"/>
-      <c r="G1" s="90"/>
-      <c r="H1" s="90"/>
-      <c r="I1" s="90"/>
-      <c r="J1" s="90"/>
-      <c r="K1" s="90"/>
-      <c r="L1" s="90"/>
-      <c r="M1" s="90"/>
-      <c r="N1" s="90"/>
-      <c r="O1" s="90"/>
-      <c r="P1" s="90"/>
-      <c r="Q1" s="90"/>
-      <c r="R1" s="90"/>
-      <c r="S1" s="90"/>
-      <c r="T1" s="90"/>
-      <c r="U1" s="90"/>
-      <c r="V1" s="90"/>
-      <c r="W1" s="90"/>
-      <c r="X1" s="90"/>
-      <c r="Y1" s="90"/>
-      <c r="Z1" s="90"/>
-      <c r="AA1" s="90"/>
-      <c r="AB1" s="90"/>
-      <c r="AC1" s="90"/>
+      <c r="A1" s="91" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="91"/>
+      <c r="C1" s="91"/>
+      <c r="D1" s="91"/>
+      <c r="E1" s="91"/>
+      <c r="F1" s="91"/>
+      <c r="G1" s="91"/>
+      <c r="H1" s="91"/>
+      <c r="I1" s="91"/>
+      <c r="J1" s="91"/>
+      <c r="K1" s="91"/>
+      <c r="L1" s="91"/>
+      <c r="M1" s="91"/>
+      <c r="N1" s="91"/>
+      <c r="O1" s="91"/>
+      <c r="P1" s="91"/>
+      <c r="Q1" s="91"/>
+      <c r="R1" s="91"/>
+      <c r="S1" s="91"/>
+      <c r="T1" s="91"/>
+      <c r="U1" s="91"/>
+      <c r="V1" s="91"/>
+      <c r="W1" s="91"/>
+      <c r="X1" s="91"/>
+      <c r="Y1" s="91"/>
+      <c r="Z1" s="91"/>
+      <c r="AA1" s="91"/>
+      <c r="AB1" s="91"/>
+      <c r="AC1" s="91"/>
     </row>
     <row r="2" spans="1:29" ht="18">
       <c r="A2" s="23" t="s">
@@ -3450,10 +3459,10 @@
       <c r="AC2" s="58"/>
     </row>
     <row r="3" spans="1:29">
-      <c r="A3" s="91" t="s">
+      <c r="A3" s="92" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="91"/>
+      <c r="B3" s="92"/>
       <c r="C3" s="59"/>
       <c r="D3" s="3">
         <v>4</v>
@@ -3736,38 +3745,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:33" ht="18">
-      <c r="A1" s="90" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="90"/>
-      <c r="C1" s="90"/>
-      <c r="D1" s="90"/>
-      <c r="E1" s="90"/>
-      <c r="F1" s="90"/>
-      <c r="G1" s="90"/>
-      <c r="H1" s="90"/>
-      <c r="I1" s="90"/>
-      <c r="J1" s="90"/>
-      <c r="K1" s="90"/>
-      <c r="L1" s="90"/>
-      <c r="M1" s="90"/>
-      <c r="N1" s="90"/>
-      <c r="O1" s="90"/>
-      <c r="P1" s="90"/>
-      <c r="Q1" s="90"/>
-      <c r="R1" s="90"/>
-      <c r="S1" s="90"/>
-      <c r="T1" s="90"/>
-      <c r="U1" s="90"/>
-      <c r="V1" s="90"/>
-      <c r="W1" s="90"/>
-      <c r="X1" s="90"/>
-      <c r="Y1" s="90"/>
-      <c r="Z1" s="90"/>
-      <c r="AA1" s="90"/>
-      <c r="AB1" s="90"/>
-      <c r="AC1" s="90"/>
-      <c r="AD1" s="90"/>
+      <c r="A1" s="91" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="91"/>
+      <c r="C1" s="91"/>
+      <c r="D1" s="91"/>
+      <c r="E1" s="91"/>
+      <c r="F1" s="91"/>
+      <c r="G1" s="91"/>
+      <c r="H1" s="91"/>
+      <c r="I1" s="91"/>
+      <c r="J1" s="91"/>
+      <c r="K1" s="91"/>
+      <c r="L1" s="91"/>
+      <c r="M1" s="91"/>
+      <c r="N1" s="91"/>
+      <c r="O1" s="91"/>
+      <c r="P1" s="91"/>
+      <c r="Q1" s="91"/>
+      <c r="R1" s="91"/>
+      <c r="S1" s="91"/>
+      <c r="T1" s="91"/>
+      <c r="U1" s="91"/>
+      <c r="V1" s="91"/>
+      <c r="W1" s="91"/>
+      <c r="X1" s="91"/>
+      <c r="Y1" s="91"/>
+      <c r="Z1" s="91"/>
+      <c r="AA1" s="91"/>
+      <c r="AB1" s="91"/>
+      <c r="AC1" s="91"/>
+      <c r="AD1" s="91"/>
     </row>
     <row r="2" spans="1:33" ht="18">
       <c r="A2" s="23" t="s">
@@ -3806,10 +3815,10 @@
       <c r="AD2" s="60"/>
     </row>
     <row r="3" spans="1:33" ht="15.75" thickBot="1">
-      <c r="A3" s="91" t="s">
+      <c r="A3" s="92" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="91"/>
+      <c r="B3" s="92"/>
       <c r="C3" s="61"/>
       <c r="D3" s="3">
         <v>2</v>
@@ -4422,37 +4431,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="18">
-      <c r="A1" s="90" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="90"/>
-      <c r="C1" s="90"/>
-      <c r="D1" s="90"/>
-      <c r="E1" s="90"/>
-      <c r="F1" s="90"/>
-      <c r="G1" s="90"/>
-      <c r="H1" s="90"/>
-      <c r="I1" s="90"/>
-      <c r="J1" s="90"/>
-      <c r="K1" s="90"/>
-      <c r="L1" s="90"/>
-      <c r="M1" s="90"/>
-      <c r="N1" s="90"/>
-      <c r="O1" s="90"/>
-      <c r="P1" s="90"/>
-      <c r="Q1" s="90"/>
-      <c r="R1" s="90"/>
-      <c r="S1" s="90"/>
-      <c r="T1" s="90"/>
-      <c r="U1" s="90"/>
-      <c r="V1" s="90"/>
-      <c r="W1" s="90"/>
-      <c r="X1" s="90"/>
-      <c r="Y1" s="90"/>
-      <c r="Z1" s="90"/>
-      <c r="AA1" s="90"/>
-      <c r="AB1" s="90"/>
-      <c r="AC1" s="90"/>
+      <c r="A1" s="91" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="91"/>
+      <c r="C1" s="91"/>
+      <c r="D1" s="91"/>
+      <c r="E1" s="91"/>
+      <c r="F1" s="91"/>
+      <c r="G1" s="91"/>
+      <c r="H1" s="91"/>
+      <c r="I1" s="91"/>
+      <c r="J1" s="91"/>
+      <c r="K1" s="91"/>
+      <c r="L1" s="91"/>
+      <c r="M1" s="91"/>
+      <c r="N1" s="91"/>
+      <c r="O1" s="91"/>
+      <c r="P1" s="91"/>
+      <c r="Q1" s="91"/>
+      <c r="R1" s="91"/>
+      <c r="S1" s="91"/>
+      <c r="T1" s="91"/>
+      <c r="U1" s="91"/>
+      <c r="V1" s="91"/>
+      <c r="W1" s="91"/>
+      <c r="X1" s="91"/>
+      <c r="Y1" s="91"/>
+      <c r="Z1" s="91"/>
+      <c r="AA1" s="91"/>
+      <c r="AB1" s="91"/>
+      <c r="AC1" s="91"/>
     </row>
     <row r="2" spans="1:29" ht="18">
       <c r="A2" s="23" t="s">
@@ -4490,10 +4499,10 @@
       <c r="AC2" s="62"/>
     </row>
     <row r="3" spans="1:29">
-      <c r="A3" s="91" t="s">
+      <c r="A3" s="92" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="91"/>
+      <c r="B3" s="92"/>
       <c r="C3" s="63"/>
       <c r="D3" s="3">
         <v>4</v>
@@ -4782,68 +4791,68 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:59" ht="18">
-      <c r="A1" s="90" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="90"/>
-      <c r="C1" s="90"/>
-      <c r="D1" s="90"/>
-      <c r="E1" s="90"/>
-      <c r="F1" s="90"/>
-      <c r="G1" s="90"/>
-      <c r="H1" s="90"/>
-      <c r="I1" s="90"/>
-      <c r="J1" s="90"/>
-      <c r="K1" s="90"/>
-      <c r="L1" s="90"/>
-      <c r="M1" s="90"/>
-      <c r="N1" s="90"/>
-      <c r="O1" s="90"/>
-      <c r="P1" s="90"/>
-      <c r="Q1" s="90"/>
-      <c r="R1" s="90"/>
-      <c r="S1" s="90"/>
-      <c r="T1" s="90"/>
-      <c r="U1" s="90"/>
-      <c r="V1" s="90"/>
-      <c r="W1" s="90"/>
-      <c r="X1" s="90"/>
-      <c r="Y1" s="90"/>
-      <c r="Z1" s="90"/>
-      <c r="AA1" s="90"/>
-      <c r="AB1" s="90"/>
-      <c r="AC1" s="90"/>
-      <c r="AD1" s="90" t="s">
-        <v>0</v>
-      </c>
-      <c r="AE1" s="90"/>
-      <c r="AF1" s="90"/>
-      <c r="AG1" s="90"/>
-      <c r="AH1" s="90"/>
-      <c r="AI1" s="90"/>
-      <c r="AJ1" s="90"/>
-      <c r="AK1" s="90"/>
-      <c r="AL1" s="90"/>
-      <c r="AM1" s="90"/>
-      <c r="AN1" s="90"/>
-      <c r="AO1" s="90"/>
-      <c r="AP1" s="90"/>
-      <c r="AQ1" s="90"/>
-      <c r="AR1" s="90"/>
-      <c r="AS1" s="90"/>
-      <c r="AT1" s="90"/>
-      <c r="AU1" s="90"/>
-      <c r="AV1" s="90"/>
-      <c r="AW1" s="90"/>
-      <c r="AX1" s="90"/>
-      <c r="AY1" s="90"/>
-      <c r="AZ1" s="90"/>
-      <c r="BA1" s="90"/>
-      <c r="BB1" s="90"/>
-      <c r="BC1" s="90"/>
-      <c r="BD1" s="90"/>
-      <c r="BE1" s="90"/>
-      <c r="BF1" s="90"/>
+      <c r="A1" s="91" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="91"/>
+      <c r="C1" s="91"/>
+      <c r="D1" s="91"/>
+      <c r="E1" s="91"/>
+      <c r="F1" s="91"/>
+      <c r="G1" s="91"/>
+      <c r="H1" s="91"/>
+      <c r="I1" s="91"/>
+      <c r="J1" s="91"/>
+      <c r="K1" s="91"/>
+      <c r="L1" s="91"/>
+      <c r="M1" s="91"/>
+      <c r="N1" s="91"/>
+      <c r="O1" s="91"/>
+      <c r="P1" s="91"/>
+      <c r="Q1" s="91"/>
+      <c r="R1" s="91"/>
+      <c r="S1" s="91"/>
+      <c r="T1" s="91"/>
+      <c r="U1" s="91"/>
+      <c r="V1" s="91"/>
+      <c r="W1" s="91"/>
+      <c r="X1" s="91"/>
+      <c r="Y1" s="91"/>
+      <c r="Z1" s="91"/>
+      <c r="AA1" s="91"/>
+      <c r="AB1" s="91"/>
+      <c r="AC1" s="91"/>
+      <c r="AD1" s="91" t="s">
+        <v>0</v>
+      </c>
+      <c r="AE1" s="91"/>
+      <c r="AF1" s="91"/>
+      <c r="AG1" s="91"/>
+      <c r="AH1" s="91"/>
+      <c r="AI1" s="91"/>
+      <c r="AJ1" s="91"/>
+      <c r="AK1" s="91"/>
+      <c r="AL1" s="91"/>
+      <c r="AM1" s="91"/>
+      <c r="AN1" s="91"/>
+      <c r="AO1" s="91"/>
+      <c r="AP1" s="91"/>
+      <c r="AQ1" s="91"/>
+      <c r="AR1" s="91"/>
+      <c r="AS1" s="91"/>
+      <c r="AT1" s="91"/>
+      <c r="AU1" s="91"/>
+      <c r="AV1" s="91"/>
+      <c r="AW1" s="91"/>
+      <c r="AX1" s="91"/>
+      <c r="AY1" s="91"/>
+      <c r="AZ1" s="91"/>
+      <c r="BA1" s="91"/>
+      <c r="BB1" s="91"/>
+      <c r="BC1" s="91"/>
+      <c r="BD1" s="91"/>
+      <c r="BE1" s="91"/>
+      <c r="BF1" s="91"/>
     </row>
     <row r="2" spans="1:59" ht="18">
       <c r="A2" s="23" t="s">
@@ -4914,10 +4923,10 @@
       <c r="BF2" s="64"/>
     </row>
     <row r="3" spans="1:59">
-      <c r="A3" s="91" t="s">
+      <c r="A3" s="92" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="91"/>
+      <c r="B3" s="92"/>
       <c r="C3" s="65"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -4957,10 +4966,10 @@
       <c r="AA3" s="6"/>
       <c r="AB3" s="6"/>
       <c r="AC3" s="6"/>
-      <c r="AD3" s="91" t="s">
+      <c r="AD3" s="92" t="s">
         <v>3</v>
       </c>
-      <c r="AE3" s="91"/>
+      <c r="AE3" s="92"/>
       <c r="AF3" s="65"/>
       <c r="AG3" s="3">
         <v>2</v>
@@ -5442,68 +5451,68 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:59" ht="18">
-      <c r="A1" s="90" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="90"/>
-      <c r="C1" s="90"/>
-      <c r="D1" s="90"/>
-      <c r="E1" s="90"/>
-      <c r="F1" s="90"/>
-      <c r="G1" s="90"/>
-      <c r="H1" s="90"/>
-      <c r="I1" s="90"/>
-      <c r="J1" s="90"/>
-      <c r="K1" s="90"/>
-      <c r="L1" s="90"/>
-      <c r="M1" s="90"/>
-      <c r="N1" s="90"/>
-      <c r="O1" s="90"/>
-      <c r="P1" s="90"/>
-      <c r="Q1" s="90"/>
-      <c r="R1" s="90"/>
-      <c r="S1" s="90"/>
-      <c r="T1" s="90"/>
-      <c r="U1" s="90"/>
-      <c r="V1" s="90"/>
-      <c r="W1" s="90"/>
-      <c r="X1" s="90"/>
-      <c r="Y1" s="90"/>
-      <c r="Z1" s="90"/>
-      <c r="AA1" s="90"/>
-      <c r="AB1" s="90"/>
-      <c r="AC1" s="90"/>
-      <c r="AD1" s="90" t="s">
-        <v>0</v>
-      </c>
-      <c r="AE1" s="90"/>
-      <c r="AF1" s="90"/>
-      <c r="AG1" s="90"/>
-      <c r="AH1" s="90"/>
-      <c r="AI1" s="90"/>
-      <c r="AJ1" s="90"/>
-      <c r="AK1" s="90"/>
-      <c r="AL1" s="90"/>
-      <c r="AM1" s="90"/>
-      <c r="AN1" s="90"/>
-      <c r="AO1" s="90"/>
-      <c r="AP1" s="90"/>
-      <c r="AQ1" s="90"/>
-      <c r="AR1" s="90"/>
-      <c r="AS1" s="90"/>
-      <c r="AT1" s="90"/>
-      <c r="AU1" s="90"/>
-      <c r="AV1" s="90"/>
-      <c r="AW1" s="90"/>
-      <c r="AX1" s="90"/>
-      <c r="AY1" s="90"/>
-      <c r="AZ1" s="90"/>
-      <c r="BA1" s="90"/>
-      <c r="BB1" s="90"/>
-      <c r="BC1" s="90"/>
-      <c r="BD1" s="90"/>
-      <c r="BE1" s="90"/>
-      <c r="BF1" s="90"/>
+      <c r="A1" s="91" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="91"/>
+      <c r="C1" s="91"/>
+      <c r="D1" s="91"/>
+      <c r="E1" s="91"/>
+      <c r="F1" s="91"/>
+      <c r="G1" s="91"/>
+      <c r="H1" s="91"/>
+      <c r="I1" s="91"/>
+      <c r="J1" s="91"/>
+      <c r="K1" s="91"/>
+      <c r="L1" s="91"/>
+      <c r="M1" s="91"/>
+      <c r="N1" s="91"/>
+      <c r="O1" s="91"/>
+      <c r="P1" s="91"/>
+      <c r="Q1" s="91"/>
+      <c r="R1" s="91"/>
+      <c r="S1" s="91"/>
+      <c r="T1" s="91"/>
+      <c r="U1" s="91"/>
+      <c r="V1" s="91"/>
+      <c r="W1" s="91"/>
+      <c r="X1" s="91"/>
+      <c r="Y1" s="91"/>
+      <c r="Z1" s="91"/>
+      <c r="AA1" s="91"/>
+      <c r="AB1" s="91"/>
+      <c r="AC1" s="91"/>
+      <c r="AD1" s="91" t="s">
+        <v>0</v>
+      </c>
+      <c r="AE1" s="91"/>
+      <c r="AF1" s="91"/>
+      <c r="AG1" s="91"/>
+      <c r="AH1" s="91"/>
+      <c r="AI1" s="91"/>
+      <c r="AJ1" s="91"/>
+      <c r="AK1" s="91"/>
+      <c r="AL1" s="91"/>
+      <c r="AM1" s="91"/>
+      <c r="AN1" s="91"/>
+      <c r="AO1" s="91"/>
+      <c r="AP1" s="91"/>
+      <c r="AQ1" s="91"/>
+      <c r="AR1" s="91"/>
+      <c r="AS1" s="91"/>
+      <c r="AT1" s="91"/>
+      <c r="AU1" s="91"/>
+      <c r="AV1" s="91"/>
+      <c r="AW1" s="91"/>
+      <c r="AX1" s="91"/>
+      <c r="AY1" s="91"/>
+      <c r="AZ1" s="91"/>
+      <c r="BA1" s="91"/>
+      <c r="BB1" s="91"/>
+      <c r="BC1" s="91"/>
+      <c r="BD1" s="91"/>
+      <c r="BE1" s="91"/>
+      <c r="BF1" s="91"/>
     </row>
     <row r="2" spans="1:59" ht="18">
       <c r="A2" s="23" t="s">
@@ -5574,10 +5583,10 @@
       <c r="BF2" s="67"/>
     </row>
     <row r="3" spans="1:59">
-      <c r="A3" s="91" t="s">
+      <c r="A3" s="92" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="91"/>
+      <c r="B3" s="92"/>
       <c r="C3" s="68"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -5617,10 +5626,10 @@
       <c r="AA3" s="6"/>
       <c r="AB3" s="6"/>
       <c r="AC3" s="6"/>
-      <c r="AD3" s="91" t="s">
+      <c r="AD3" s="92" t="s">
         <v>3</v>
       </c>
-      <c r="AE3" s="91"/>
+      <c r="AE3" s="92"/>
       <c r="AF3" s="68"/>
       <c r="AG3" s="3">
         <v>2</v>
@@ -6095,38 +6104,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:33" ht="18">
-      <c r="A1" s="90" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="90"/>
-      <c r="C1" s="90"/>
-      <c r="D1" s="90"/>
-      <c r="E1" s="90"/>
-      <c r="F1" s="90"/>
-      <c r="G1" s="90"/>
-      <c r="H1" s="90"/>
-      <c r="I1" s="90"/>
-      <c r="J1" s="90"/>
-      <c r="K1" s="90"/>
-      <c r="L1" s="90"/>
-      <c r="M1" s="90"/>
-      <c r="N1" s="90"/>
-      <c r="O1" s="90"/>
-      <c r="P1" s="90"/>
-      <c r="Q1" s="90"/>
-      <c r="R1" s="90"/>
-      <c r="S1" s="90"/>
-      <c r="T1" s="90"/>
-      <c r="U1" s="90"/>
-      <c r="V1" s="90"/>
-      <c r="W1" s="90"/>
-      <c r="X1" s="90"/>
-      <c r="Y1" s="90"/>
-      <c r="Z1" s="90"/>
-      <c r="AA1" s="90"/>
-      <c r="AB1" s="90"/>
-      <c r="AC1" s="90"/>
-      <c r="AD1" s="90"/>
+      <c r="A1" s="91" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="91"/>
+      <c r="C1" s="91"/>
+      <c r="D1" s="91"/>
+      <c r="E1" s="91"/>
+      <c r="F1" s="91"/>
+      <c r="G1" s="91"/>
+      <c r="H1" s="91"/>
+      <c r="I1" s="91"/>
+      <c r="J1" s="91"/>
+      <c r="K1" s="91"/>
+      <c r="L1" s="91"/>
+      <c r="M1" s="91"/>
+      <c r="N1" s="91"/>
+      <c r="O1" s="91"/>
+      <c r="P1" s="91"/>
+      <c r="Q1" s="91"/>
+      <c r="R1" s="91"/>
+      <c r="S1" s="91"/>
+      <c r="T1" s="91"/>
+      <c r="U1" s="91"/>
+      <c r="V1" s="91"/>
+      <c r="W1" s="91"/>
+      <c r="X1" s="91"/>
+      <c r="Y1" s="91"/>
+      <c r="Z1" s="91"/>
+      <c r="AA1" s="91"/>
+      <c r="AB1" s="91"/>
+      <c r="AC1" s="91"/>
+      <c r="AD1" s="91"/>
     </row>
     <row r="2" spans="1:33" ht="18">
       <c r="A2" s="23" t="s">
@@ -6165,10 +6174,10 @@
       <c r="AD2" s="70"/>
     </row>
     <row r="3" spans="1:33" ht="15.75" thickBot="1">
-      <c r="A3" s="91" t="s">
+      <c r="A3" s="92" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="91"/>
+      <c r="B3" s="92"/>
       <c r="C3" s="71"/>
       <c r="D3" s="3">
         <v>3</v>
@@ -7018,68 +7027,68 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:58" ht="18">
-      <c r="A1" s="90" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="90"/>
-      <c r="C1" s="90"/>
-      <c r="D1" s="90"/>
-      <c r="E1" s="90"/>
-      <c r="F1" s="90"/>
-      <c r="G1" s="90"/>
-      <c r="H1" s="90"/>
-      <c r="I1" s="90"/>
-      <c r="J1" s="90"/>
-      <c r="K1" s="90"/>
-      <c r="L1" s="90"/>
-      <c r="M1" s="90"/>
-      <c r="N1" s="90"/>
-      <c r="O1" s="90"/>
-      <c r="P1" s="90"/>
-      <c r="Q1" s="90"/>
-      <c r="R1" s="90"/>
-      <c r="S1" s="90"/>
-      <c r="T1" s="90"/>
-      <c r="U1" s="90"/>
-      <c r="V1" s="90"/>
-      <c r="W1" s="90"/>
-      <c r="X1" s="90"/>
-      <c r="Y1" s="90"/>
-      <c r="Z1" s="90"/>
-      <c r="AA1" s="90"/>
-      <c r="AB1" s="90"/>
-      <c r="AC1" s="90"/>
-      <c r="AD1" s="90" t="s">
-        <v>0</v>
-      </c>
-      <c r="AE1" s="90"/>
-      <c r="AF1" s="90"/>
-      <c r="AG1" s="90"/>
-      <c r="AH1" s="90"/>
-      <c r="AI1" s="90"/>
-      <c r="AJ1" s="90"/>
-      <c r="AK1" s="90"/>
-      <c r="AL1" s="90"/>
-      <c r="AM1" s="90"/>
-      <c r="AN1" s="90"/>
-      <c r="AO1" s="90"/>
-      <c r="AP1" s="90"/>
-      <c r="AQ1" s="90"/>
-      <c r="AR1" s="90"/>
-      <c r="AS1" s="90"/>
-      <c r="AT1" s="90"/>
-      <c r="AU1" s="90"/>
-      <c r="AV1" s="90"/>
-      <c r="AW1" s="90"/>
-      <c r="AX1" s="90"/>
-      <c r="AY1" s="90"/>
-      <c r="AZ1" s="90"/>
-      <c r="BA1" s="90"/>
-      <c r="BB1" s="90"/>
-      <c r="BC1" s="90"/>
-      <c r="BD1" s="90"/>
-      <c r="BE1" s="90"/>
-      <c r="BF1" s="90"/>
+      <c r="A1" s="91" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="91"/>
+      <c r="C1" s="91"/>
+      <c r="D1" s="91"/>
+      <c r="E1" s="91"/>
+      <c r="F1" s="91"/>
+      <c r="G1" s="91"/>
+      <c r="H1" s="91"/>
+      <c r="I1" s="91"/>
+      <c r="J1" s="91"/>
+      <c r="K1" s="91"/>
+      <c r="L1" s="91"/>
+      <c r="M1" s="91"/>
+      <c r="N1" s="91"/>
+      <c r="O1" s="91"/>
+      <c r="P1" s="91"/>
+      <c r="Q1" s="91"/>
+      <c r="R1" s="91"/>
+      <c r="S1" s="91"/>
+      <c r="T1" s="91"/>
+      <c r="U1" s="91"/>
+      <c r="V1" s="91"/>
+      <c r="W1" s="91"/>
+      <c r="X1" s="91"/>
+      <c r="Y1" s="91"/>
+      <c r="Z1" s="91"/>
+      <c r="AA1" s="91"/>
+      <c r="AB1" s="91"/>
+      <c r="AC1" s="91"/>
+      <c r="AD1" s="91" t="s">
+        <v>0</v>
+      </c>
+      <c r="AE1" s="91"/>
+      <c r="AF1" s="91"/>
+      <c r="AG1" s="91"/>
+      <c r="AH1" s="91"/>
+      <c r="AI1" s="91"/>
+      <c r="AJ1" s="91"/>
+      <c r="AK1" s="91"/>
+      <c r="AL1" s="91"/>
+      <c r="AM1" s="91"/>
+      <c r="AN1" s="91"/>
+      <c r="AO1" s="91"/>
+      <c r="AP1" s="91"/>
+      <c r="AQ1" s="91"/>
+      <c r="AR1" s="91"/>
+      <c r="AS1" s="91"/>
+      <c r="AT1" s="91"/>
+      <c r="AU1" s="91"/>
+      <c r="AV1" s="91"/>
+      <c r="AW1" s="91"/>
+      <c r="AX1" s="91"/>
+      <c r="AY1" s="91"/>
+      <c r="AZ1" s="91"/>
+      <c r="BA1" s="91"/>
+      <c r="BB1" s="91"/>
+      <c r="BC1" s="91"/>
+      <c r="BD1" s="91"/>
+      <c r="BE1" s="91"/>
+      <c r="BF1" s="91"/>
     </row>
     <row r="2" spans="1:58" ht="18">
       <c r="A2" s="23" t="s">
@@ -7150,10 +7159,10 @@
       <c r="BF2" s="36"/>
     </row>
     <row r="3" spans="1:58">
-      <c r="A3" s="91" t="s">
+      <c r="A3" s="92" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="91"/>
+      <c r="B3" s="92"/>
       <c r="C3" s="29"/>
       <c r="D3" s="3">
         <v>2</v>
@@ -7193,10 +7202,10 @@
       <c r="AA3" s="6"/>
       <c r="AB3" s="6"/>
       <c r="AC3" s="6"/>
-      <c r="AD3" s="91" t="s">
+      <c r="AD3" s="92" t="s">
         <v>3</v>
       </c>
-      <c r="AE3" s="91"/>
+      <c r="AE3" s="92"/>
       <c r="AF3" s="37"/>
       <c r="AG3" s="3">
         <v>2</v>
@@ -7672,37 +7681,37 @@
       <c r="A1" s="84" t="s">
         <v>112</v>
       </c>
-      <c r="B1" s="90" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="90"/>
-      <c r="D1" s="90"/>
-      <c r="E1" s="90"/>
-      <c r="F1" s="90"/>
-      <c r="G1" s="90"/>
-      <c r="H1" s="90"/>
-      <c r="I1" s="90"/>
-      <c r="J1" s="90"/>
-      <c r="K1" s="90"/>
-      <c r="L1" s="90"/>
-      <c r="M1" s="90"/>
-      <c r="N1" s="90"/>
-      <c r="O1" s="90"/>
-      <c r="P1" s="90"/>
-      <c r="Q1" s="90"/>
-      <c r="R1" s="90"/>
-      <c r="S1" s="90"/>
-      <c r="T1" s="90"/>
-      <c r="U1" s="90"/>
-      <c r="V1" s="90"/>
-      <c r="W1" s="90"/>
-      <c r="X1" s="90"/>
-      <c r="Y1" s="90"/>
-      <c r="Z1" s="90"/>
-      <c r="AA1" s="90"/>
-      <c r="AB1" s="90"/>
-      <c r="AC1" s="90"/>
-      <c r="AD1" s="90"/>
+      <c r="B1" s="91" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="91"/>
+      <c r="D1" s="91"/>
+      <c r="E1" s="91"/>
+      <c r="F1" s="91"/>
+      <c r="G1" s="91"/>
+      <c r="H1" s="91"/>
+      <c r="I1" s="91"/>
+      <c r="J1" s="91"/>
+      <c r="K1" s="91"/>
+      <c r="L1" s="91"/>
+      <c r="M1" s="91"/>
+      <c r="N1" s="91"/>
+      <c r="O1" s="91"/>
+      <c r="P1" s="91"/>
+      <c r="Q1" s="91"/>
+      <c r="R1" s="91"/>
+      <c r="S1" s="91"/>
+      <c r="T1" s="91"/>
+      <c r="U1" s="91"/>
+      <c r="V1" s="91"/>
+      <c r="W1" s="91"/>
+      <c r="X1" s="91"/>
+      <c r="Y1" s="91"/>
+      <c r="Z1" s="91"/>
+      <c r="AA1" s="91"/>
+      <c r="AB1" s="91"/>
+      <c r="AC1" s="91"/>
+      <c r="AD1" s="91"/>
     </row>
     <row r="2" spans="1:33" ht="18">
       <c r="A2" s="85"/>
@@ -7742,10 +7751,10 @@
     </row>
     <row r="3" spans="1:33" ht="15.75" thickBot="1">
       <c r="A3" s="85"/>
-      <c r="B3" s="91" t="s">
+      <c r="B3" s="92" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="91"/>
+      <c r="C3" s="92"/>
       <c r="D3" s="3">
         <v>2</v>
       </c>
@@ -9056,36 +9065,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:31" ht="18">
-      <c r="A1" s="90" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="90"/>
-      <c r="C1" s="90"/>
-      <c r="D1" s="90"/>
-      <c r="E1" s="90"/>
-      <c r="F1" s="90"/>
-      <c r="G1" s="90"/>
-      <c r="H1" s="90"/>
-      <c r="I1" s="90"/>
-      <c r="J1" s="90"/>
-      <c r="K1" s="90"/>
-      <c r="L1" s="90"/>
-      <c r="M1" s="90"/>
-      <c r="N1" s="90"/>
-      <c r="O1" s="90"/>
-      <c r="P1" s="90"/>
-      <c r="Q1" s="90"/>
-      <c r="R1" s="90"/>
-      <c r="S1" s="90"/>
-      <c r="T1" s="90"/>
-      <c r="U1" s="90"/>
-      <c r="V1" s="90"/>
-      <c r="W1" s="90"/>
-      <c r="X1" s="90"/>
-      <c r="Y1" s="90"/>
-      <c r="Z1" s="90"/>
-      <c r="AA1" s="90"/>
-      <c r="AB1" s="90"/>
+      <c r="A1" s="91" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="91"/>
+      <c r="C1" s="91"/>
+      <c r="D1" s="91"/>
+      <c r="E1" s="91"/>
+      <c r="F1" s="91"/>
+      <c r="G1" s="91"/>
+      <c r="H1" s="91"/>
+      <c r="I1" s="91"/>
+      <c r="J1" s="91"/>
+      <c r="K1" s="91"/>
+      <c r="L1" s="91"/>
+      <c r="M1" s="91"/>
+      <c r="N1" s="91"/>
+      <c r="O1" s="91"/>
+      <c r="P1" s="91"/>
+      <c r="Q1" s="91"/>
+      <c r="R1" s="91"/>
+      <c r="S1" s="91"/>
+      <c r="T1" s="91"/>
+      <c r="U1" s="91"/>
+      <c r="V1" s="91"/>
+      <c r="W1" s="91"/>
+      <c r="X1" s="91"/>
+      <c r="Y1" s="91"/>
+      <c r="Z1" s="91"/>
+      <c r="AA1" s="91"/>
+      <c r="AB1" s="91"/>
     </row>
     <row r="2" spans="1:31" ht="18">
       <c r="A2" s="23" t="s">
@@ -9122,10 +9131,10 @@
       <c r="AB2" s="80"/>
     </row>
     <row r="3" spans="1:31" ht="15.75" thickBot="1">
-      <c r="A3" s="91" t="s">
+      <c r="A3" s="92" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="91"/>
+      <c r="B3" s="92"/>
       <c r="C3" s="81"/>
       <c r="D3" s="3">
         <v>2</v>
@@ -9938,37 +9947,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:32" ht="18">
-      <c r="A1" s="90" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="90"/>
-      <c r="C1" s="90"/>
-      <c r="D1" s="90"/>
-      <c r="E1" s="90"/>
-      <c r="F1" s="90"/>
-      <c r="G1" s="90"/>
-      <c r="H1" s="90"/>
-      <c r="I1" s="90"/>
-      <c r="J1" s="90"/>
-      <c r="K1" s="90"/>
-      <c r="L1" s="90"/>
-      <c r="M1" s="90"/>
-      <c r="N1" s="90"/>
-      <c r="O1" s="90"/>
-      <c r="P1" s="90"/>
-      <c r="Q1" s="90"/>
-      <c r="R1" s="90"/>
-      <c r="S1" s="90"/>
-      <c r="T1" s="90"/>
-      <c r="U1" s="90"/>
-      <c r="V1" s="90"/>
-      <c r="W1" s="90"/>
-      <c r="X1" s="90"/>
-      <c r="Y1" s="90"/>
-      <c r="Z1" s="90"/>
-      <c r="AA1" s="90"/>
-      <c r="AB1" s="90"/>
-      <c r="AC1" s="90"/>
+      <c r="A1" s="91" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="91"/>
+      <c r="C1" s="91"/>
+      <c r="D1" s="91"/>
+      <c r="E1" s="91"/>
+      <c r="F1" s="91"/>
+      <c r="G1" s="91"/>
+      <c r="H1" s="91"/>
+      <c r="I1" s="91"/>
+      <c r="J1" s="91"/>
+      <c r="K1" s="91"/>
+      <c r="L1" s="91"/>
+      <c r="M1" s="91"/>
+      <c r="N1" s="91"/>
+      <c r="O1" s="91"/>
+      <c r="P1" s="91"/>
+      <c r="Q1" s="91"/>
+      <c r="R1" s="91"/>
+      <c r="S1" s="91"/>
+      <c r="T1" s="91"/>
+      <c r="U1" s="91"/>
+      <c r="V1" s="91"/>
+      <c r="W1" s="91"/>
+      <c r="X1" s="91"/>
+      <c r="Y1" s="91"/>
+      <c r="Z1" s="91"/>
+      <c r="AA1" s="91"/>
+      <c r="AB1" s="91"/>
+      <c r="AC1" s="91"/>
     </row>
     <row r="2" spans="1:32" ht="18">
       <c r="A2" s="23" t="s">
@@ -10006,10 +10015,10 @@
       <c r="AC2" s="87"/>
     </row>
     <row r="3" spans="1:32" ht="15.75" thickBot="1">
-      <c r="A3" s="91" t="s">
+      <c r="A3" s="92" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="91"/>
+      <c r="B3" s="92"/>
       <c r="C3" s="3">
         <v>2</v>
       </c>
@@ -10614,68 +10623,68 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:59" ht="18">
-      <c r="B1" s="90" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="90"/>
-      <c r="D1" s="90"/>
-      <c r="E1" s="90"/>
-      <c r="F1" s="90"/>
-      <c r="G1" s="90"/>
-      <c r="H1" s="90"/>
-      <c r="I1" s="90"/>
-      <c r="J1" s="90"/>
-      <c r="K1" s="90"/>
-      <c r="L1" s="90"/>
-      <c r="M1" s="90"/>
-      <c r="N1" s="90"/>
-      <c r="O1" s="90"/>
-      <c r="P1" s="90"/>
-      <c r="Q1" s="90"/>
-      <c r="R1" s="90"/>
-      <c r="S1" s="90"/>
-      <c r="T1" s="90"/>
-      <c r="U1" s="90"/>
-      <c r="V1" s="90"/>
-      <c r="W1" s="90"/>
-      <c r="X1" s="90"/>
-      <c r="Y1" s="90"/>
-      <c r="Z1" s="90"/>
-      <c r="AA1" s="90"/>
-      <c r="AB1" s="90"/>
-      <c r="AC1" s="90"/>
-      <c r="AD1" s="90"/>
-      <c r="AE1" s="90" t="s">
-        <v>0</v>
-      </c>
-      <c r="AF1" s="90"/>
-      <c r="AG1" s="90"/>
-      <c r="AH1" s="90"/>
-      <c r="AI1" s="90"/>
-      <c r="AJ1" s="90"/>
-      <c r="AK1" s="90"/>
-      <c r="AL1" s="90"/>
-      <c r="AM1" s="90"/>
-      <c r="AN1" s="90"/>
-      <c r="AO1" s="90"/>
-      <c r="AP1" s="90"/>
-      <c r="AQ1" s="90"/>
-      <c r="AR1" s="90"/>
-      <c r="AS1" s="90"/>
-      <c r="AT1" s="90"/>
-      <c r="AU1" s="90"/>
-      <c r="AV1" s="90"/>
-      <c r="AW1" s="90"/>
-      <c r="AX1" s="90"/>
-      <c r="AY1" s="90"/>
-      <c r="AZ1" s="90"/>
-      <c r="BA1" s="90"/>
-      <c r="BB1" s="90"/>
-      <c r="BC1" s="90"/>
-      <c r="BD1" s="90"/>
-      <c r="BE1" s="90"/>
-      <c r="BF1" s="90"/>
-      <c r="BG1" s="90"/>
+      <c r="B1" s="91" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="91"/>
+      <c r="D1" s="91"/>
+      <c r="E1" s="91"/>
+      <c r="F1" s="91"/>
+      <c r="G1" s="91"/>
+      <c r="H1" s="91"/>
+      <c r="I1" s="91"/>
+      <c r="J1" s="91"/>
+      <c r="K1" s="91"/>
+      <c r="L1" s="91"/>
+      <c r="M1" s="91"/>
+      <c r="N1" s="91"/>
+      <c r="O1" s="91"/>
+      <c r="P1" s="91"/>
+      <c r="Q1" s="91"/>
+      <c r="R1" s="91"/>
+      <c r="S1" s="91"/>
+      <c r="T1" s="91"/>
+      <c r="U1" s="91"/>
+      <c r="V1" s="91"/>
+      <c r="W1" s="91"/>
+      <c r="X1" s="91"/>
+      <c r="Y1" s="91"/>
+      <c r="Z1" s="91"/>
+      <c r="AA1" s="91"/>
+      <c r="AB1" s="91"/>
+      <c r="AC1" s="91"/>
+      <c r="AD1" s="91"/>
+      <c r="AE1" s="91" t="s">
+        <v>0</v>
+      </c>
+      <c r="AF1" s="91"/>
+      <c r="AG1" s="91"/>
+      <c r="AH1" s="91"/>
+      <c r="AI1" s="91"/>
+      <c r="AJ1" s="91"/>
+      <c r="AK1" s="91"/>
+      <c r="AL1" s="91"/>
+      <c r="AM1" s="91"/>
+      <c r="AN1" s="91"/>
+      <c r="AO1" s="91"/>
+      <c r="AP1" s="91"/>
+      <c r="AQ1" s="91"/>
+      <c r="AR1" s="91"/>
+      <c r="AS1" s="91"/>
+      <c r="AT1" s="91"/>
+      <c r="AU1" s="91"/>
+      <c r="AV1" s="91"/>
+      <c r="AW1" s="91"/>
+      <c r="AX1" s="91"/>
+      <c r="AY1" s="91"/>
+      <c r="AZ1" s="91"/>
+      <c r="BA1" s="91"/>
+      <c r="BB1" s="91"/>
+      <c r="BC1" s="91"/>
+      <c r="BD1" s="91"/>
+      <c r="BE1" s="91"/>
+      <c r="BF1" s="91"/>
+      <c r="BG1" s="91"/>
     </row>
     <row r="2" spans="1:59" ht="18">
       <c r="B2" s="23" t="s">
@@ -10746,10 +10755,10 @@
       <c r="BG2" s="88"/>
     </row>
     <row r="3" spans="1:59">
-      <c r="B3" s="91" t="s">
+      <c r="B3" s="92" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="91"/>
+      <c r="C3" s="92"/>
       <c r="D3" s="89"/>
       <c r="E3" s="3">
         <v>2</v>
@@ -10789,10 +10798,10 @@
       <c r="AB3" s="6"/>
       <c r="AC3" s="6"/>
       <c r="AD3" s="6"/>
-      <c r="AE3" s="91" t="s">
+      <c r="AE3" s="92" t="s">
         <v>3</v>
       </c>
-      <c r="AF3" s="91"/>
+      <c r="AF3" s="92"/>
       <c r="AG3" s="89"/>
       <c r="AH3" s="3">
         <v>2</v>
@@ -11246,6 +11255,583 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:AF8"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="3" max="3" width="20.5703125" customWidth="1"/>
+    <col min="4" max="4" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="29.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.28515625" customWidth="1"/>
+    <col min="7" max="7" width="16.28515625" customWidth="1"/>
+    <col min="8" max="8" width="24.42578125" customWidth="1"/>
+    <col min="9" max="9" width="20.28515625" customWidth="1"/>
+    <col min="10" max="10" width="20" customWidth="1"/>
+    <col min="14" max="14" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="13.7109375" customWidth="1"/>
+    <col min="19" max="19" width="13" customWidth="1"/>
+    <col min="20" max="20" width="14.42578125" customWidth="1"/>
+    <col min="21" max="21" width="18.42578125" customWidth="1"/>
+    <col min="22" max="22" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="11.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:32" ht="18">
+      <c r="B1" s="91" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="91"/>
+      <c r="D1" s="91"/>
+      <c r="E1" s="91"/>
+      <c r="F1" s="91"/>
+      <c r="G1" s="91"/>
+      <c r="H1" s="91"/>
+      <c r="I1" s="91"/>
+      <c r="J1" s="91"/>
+      <c r="K1" s="91"/>
+      <c r="L1" s="91"/>
+      <c r="M1" s="91"/>
+      <c r="N1" s="91"/>
+      <c r="O1" s="91"/>
+      <c r="P1" s="91"/>
+      <c r="Q1" s="91"/>
+      <c r="R1" s="91"/>
+      <c r="S1" s="91"/>
+      <c r="T1" s="91"/>
+      <c r="U1" s="91"/>
+      <c r="V1" s="91"/>
+      <c r="W1" s="91"/>
+      <c r="X1" s="91"/>
+      <c r="Y1" s="91"/>
+      <c r="Z1" s="91"/>
+      <c r="AA1" s="91"/>
+      <c r="AB1" s="91"/>
+      <c r="AC1" s="91"/>
+      <c r="AD1" s="91"/>
+    </row>
+    <row r="2" spans="1:32" ht="16.5" customHeight="1">
+      <c r="B2" s="23" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="23" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" s="90"/>
+      <c r="E2" s="90"/>
+      <c r="F2" s="90"/>
+      <c r="G2" s="90"/>
+      <c r="H2" s="90"/>
+      <c r="I2" s="90"/>
+      <c r="J2" s="90"/>
+      <c r="K2" s="90"/>
+      <c r="L2" s="90"/>
+      <c r="M2" s="90"/>
+      <c r="N2" s="90"/>
+      <c r="O2" s="90"/>
+      <c r="P2" s="90"/>
+      <c r="Q2" s="90"/>
+      <c r="R2" s="90"/>
+      <c r="S2" s="90"/>
+      <c r="T2" s="90"/>
+      <c r="U2" s="90"/>
+      <c r="V2" s="90"/>
+      <c r="W2" s="90"/>
+      <c r="X2" s="90"/>
+      <c r="Y2" s="90"/>
+      <c r="Z2" s="90"/>
+      <c r="AA2" s="90"/>
+      <c r="AB2" s="90"/>
+      <c r="AC2" s="90"/>
+      <c r="AD2" s="90"/>
+    </row>
+    <row r="3" spans="1:32">
+      <c r="B3" s="92" t="s">
+        <v>3</v>
+      </c>
+      <c r="C3" s="92"/>
+      <c r="E3">
+        <v>2</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="G3" s="5"/>
+      <c r="H3" s="5"/>
+      <c r="I3" s="5"/>
+      <c r="J3" s="6"/>
+      <c r="K3" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="L3" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="M3" s="7"/>
+      <c r="N3" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="O3" s="7">
+        <v>1</v>
+      </c>
+      <c r="P3" s="7"/>
+      <c r="Q3" s="7"/>
+      <c r="R3" s="7"/>
+      <c r="S3" s="7"/>
+      <c r="T3" s="6"/>
+      <c r="U3" s="6"/>
+      <c r="V3" s="6"/>
+      <c r="W3" s="6"/>
+      <c r="X3" s="6"/>
+      <c r="Y3" s="6"/>
+      <c r="Z3" s="6"/>
+      <c r="AA3" s="6"/>
+      <c r="AB3" s="6"/>
+      <c r="AC3" s="6"/>
+      <c r="AD3" s="6"/>
+    </row>
+    <row r="4" spans="1:32" ht="42.75">
+      <c r="A4" s="10" t="s">
+        <v>114</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="D4" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="E4" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="F4" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="G4" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="H4" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="I4" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="J4" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="K4" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="L4" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="M4" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="N4" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="O4" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="P4" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="Q4" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="R4" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="S4" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="T4" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="U4" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="V4" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="W4" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="X4" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y4" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z4" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="AA4" s="16" t="s">
+        <v>30</v>
+      </c>
+      <c r="AB4" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="AC4" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="AD4" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="AE4" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="AF4" s="10" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="5" spans="1:32">
+      <c r="A5" s="9">
+        <v>1</v>
+      </c>
+      <c r="B5" s="9">
+        <v>1</v>
+      </c>
+      <c r="C5" s="27" t="s">
+        <v>44</v>
+      </c>
+      <c r="D5" s="9">
+        <v>0</v>
+      </c>
+      <c r="E5" s="27" t="s">
+        <v>44</v>
+      </c>
+      <c r="F5" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="G5" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="H5" s="24">
+        <v>2</v>
+      </c>
+      <c r="I5" s="9">
+        <v>250.25</v>
+      </c>
+      <c r="J5" s="8">
+        <v>500.5</v>
+      </c>
+      <c r="K5" s="25">
+        <v>0</v>
+      </c>
+      <c r="L5" s="25">
+        <v>0</v>
+      </c>
+      <c r="M5" s="25">
+        <v>0</v>
+      </c>
+      <c r="N5" s="8">
+        <v>500.5</v>
+      </c>
+      <c r="O5" s="8">
+        <f>ROUND(K5*N5%,2)</f>
+        <v>0</v>
+      </c>
+      <c r="P5" s="8">
+        <f>J5-O5</f>
+        <v>500.5</v>
+      </c>
+      <c r="Q5" s="8">
+        <f>ROUND(L5*P5%,2)</f>
+        <v>0</v>
+      </c>
+      <c r="R5" s="8">
+        <f>P5-Q5</f>
+        <v>500.5</v>
+      </c>
+      <c r="S5" s="8">
+        <f>ROUND(M5*R5%,2)</f>
+        <v>0</v>
+      </c>
+      <c r="T5" s="26">
+        <f>O5+Q5+S5</f>
+        <v>0</v>
+      </c>
+      <c r="U5" s="26">
+        <v>0</v>
+      </c>
+      <c r="V5" s="8">
+        <f>(J5-T5)</f>
+        <v>500.5</v>
+      </c>
+      <c r="W5" s="24">
+        <v>88363222</v>
+      </c>
+      <c r="X5" s="18">
+        <v>0.18</v>
+      </c>
+      <c r="Y5" s="24">
+        <f>IF($E$3=1,ROUND(((V5*X5)/2),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="Z5" s="24">
+        <f>IF($E$3=1,ROUND(((V5*X5)/2),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="AA5" s="93">
+        <f>IF($E$3=2,ROUND(((V5*X5)),2),0)</f>
+        <v>90.09</v>
+      </c>
+      <c r="AB5" s="24">
+        <v>0</v>
+      </c>
+      <c r="AC5" s="24">
+        <f>Y5+Z5+AA5</f>
+        <v>90.09</v>
+      </c>
+      <c r="AD5" s="24">
+        <f>V5+AC5</f>
+        <v>590.59</v>
+      </c>
+      <c r="AE5" s="46" t="s">
+        <v>42</v>
+      </c>
+      <c r="AF5" s="46" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="6" spans="1:32" ht="16.5" customHeight="1">
+      <c r="A6" s="9">
+        <v>2</v>
+      </c>
+      <c r="B6" s="9">
+        <v>2</v>
+      </c>
+      <c r="C6" s="45" t="s">
+        <v>51</v>
+      </c>
+      <c r="D6" s="9">
+        <v>0</v>
+      </c>
+      <c r="E6" s="45" t="s">
+        <v>50</v>
+      </c>
+      <c r="F6" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="G6" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="H6" s="24">
+        <v>1</v>
+      </c>
+      <c r="I6" s="9">
+        <v>3458</v>
+      </c>
+      <c r="J6" s="8">
+        <v>3458</v>
+      </c>
+      <c r="K6" s="25">
+        <v>0</v>
+      </c>
+      <c r="L6" s="25">
+        <v>0</v>
+      </c>
+      <c r="M6" s="25">
+        <v>0</v>
+      </c>
+      <c r="N6" s="8">
+        <v>3458</v>
+      </c>
+      <c r="O6" s="8">
+        <f t="shared" ref="O6:O7" si="0">ROUND(K6*N6%,2)</f>
+        <v>0</v>
+      </c>
+      <c r="P6" s="8">
+        <f t="shared" ref="P6:P7" si="1">J6-O6</f>
+        <v>3458</v>
+      </c>
+      <c r="Q6" s="8">
+        <f t="shared" ref="Q6:Q7" si="2">ROUND(L6*P6%,2)</f>
+        <v>0</v>
+      </c>
+      <c r="R6" s="8">
+        <f t="shared" ref="R6:R7" si="3">P6-Q6</f>
+        <v>3458</v>
+      </c>
+      <c r="S6" s="8">
+        <f t="shared" ref="S6:S7" si="4">ROUND(M6*R6%,2)</f>
+        <v>0</v>
+      </c>
+      <c r="T6" s="26">
+        <f t="shared" ref="T6:T7" si="5">O6+Q6+S6</f>
+        <v>0</v>
+      </c>
+      <c r="U6" s="26">
+        <v>0</v>
+      </c>
+      <c r="V6" s="8">
+        <f>(J6-T6)</f>
+        <v>3458</v>
+      </c>
+      <c r="W6" s="24">
+        <v>88363222</v>
+      </c>
+      <c r="X6" s="18">
+        <v>0.18</v>
+      </c>
+      <c r="Y6" s="24">
+        <f>IF($E$3=1,ROUND(((V6*X6)/2),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="Z6" s="24">
+        <f>IF($E$3=1,ROUND(((V6*X6)/2),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="AA6" s="93">
+        <f t="shared" ref="AA6:AA7" si="6">IF($E$3=2,ROUND(((V6*X6)),2),0)</f>
+        <v>622.44000000000005</v>
+      </c>
+      <c r="AB6" s="24">
+        <v>0</v>
+      </c>
+      <c r="AC6" s="24">
+        <f>Y6+Z6+AA6</f>
+        <v>622.44000000000005</v>
+      </c>
+      <c r="AD6" s="24">
+        <f>V6+AC6</f>
+        <v>4080.44</v>
+      </c>
+      <c r="AE6" s="46" t="s">
+        <v>53</v>
+      </c>
+      <c r="AF6" s="46" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="7" spans="1:32">
+      <c r="A7" s="9">
+        <v>3</v>
+      </c>
+      <c r="B7" s="9">
+        <v>3</v>
+      </c>
+      <c r="C7" s="27" t="s">
+        <v>52</v>
+      </c>
+      <c r="D7" s="9">
+        <v>0</v>
+      </c>
+      <c r="E7" s="27" t="s">
+        <v>52</v>
+      </c>
+      <c r="F7" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="G7" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="H7" s="24">
+        <v>3</v>
+      </c>
+      <c r="I7" s="9">
+        <v>675</v>
+      </c>
+      <c r="J7" s="8">
+        <v>2025</v>
+      </c>
+      <c r="K7" s="25">
+        <v>0</v>
+      </c>
+      <c r="L7" s="25">
+        <v>0</v>
+      </c>
+      <c r="M7" s="25">
+        <v>0</v>
+      </c>
+      <c r="N7" s="8">
+        <v>2025</v>
+      </c>
+      <c r="O7" s="8">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="P7" s="8">
+        <f t="shared" si="1"/>
+        <v>2025</v>
+      </c>
+      <c r="Q7" s="8">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="R7" s="8">
+        <f t="shared" si="3"/>
+        <v>2025</v>
+      </c>
+      <c r="S7" s="8">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="T7" s="26">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="U7" s="26">
+        <v>0</v>
+      </c>
+      <c r="V7" s="8">
+        <f>(J7-T7)</f>
+        <v>2025</v>
+      </c>
+      <c r="W7" s="24">
+        <v>88363222</v>
+      </c>
+      <c r="X7" s="18">
+        <v>0.18</v>
+      </c>
+      <c r="Y7" s="24">
+        <f>IF($E$3=1,ROUND(((V7*X7)/2),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="Z7" s="24">
+        <f>IF($E$3=1,ROUND(((V7*X7)/2),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="AA7" s="93">
+        <f t="shared" si="6"/>
+        <v>364.5</v>
+      </c>
+      <c r="AB7" s="24">
+        <v>0</v>
+      </c>
+      <c r="AC7" s="24">
+        <f>Y7+Z7+AA7</f>
+        <v>364.5</v>
+      </c>
+      <c r="AD7" s="24">
+        <f>V7+AC7</f>
+        <v>2389.5</v>
+      </c>
+      <c r="AE7" s="46" t="s">
+        <v>54</v>
+      </c>
+      <c r="AF7" s="46" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="8" spans="1:32">
+      <c r="AF8" s="46"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B1:AD1"/>
+    <mergeCell ref="B3:C3"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:AC6"/>
@@ -11268,37 +11854,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="18">
-      <c r="A1" s="90" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="90"/>
-      <c r="C1" s="90"/>
-      <c r="D1" s="90"/>
-      <c r="E1" s="90"/>
-      <c r="F1" s="90"/>
-      <c r="G1" s="90"/>
-      <c r="H1" s="90"/>
-      <c r="I1" s="90"/>
-      <c r="J1" s="90"/>
-      <c r="K1" s="90"/>
-      <c r="L1" s="90"/>
-      <c r="M1" s="90"/>
-      <c r="N1" s="90"/>
-      <c r="O1" s="90"/>
-      <c r="P1" s="90"/>
-      <c r="Q1" s="90"/>
-      <c r="R1" s="90"/>
-      <c r="S1" s="90"/>
-      <c r="T1" s="90"/>
-      <c r="U1" s="90"/>
-      <c r="V1" s="90"/>
-      <c r="W1" s="90"/>
-      <c r="X1" s="90"/>
-      <c r="Y1" s="90"/>
-      <c r="Z1" s="90"/>
-      <c r="AA1" s="90"/>
-      <c r="AB1" s="90"/>
-      <c r="AC1" s="90"/>
+      <c r="A1" s="91" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="91"/>
+      <c r="C1" s="91"/>
+      <c r="D1" s="91"/>
+      <c r="E1" s="91"/>
+      <c r="F1" s="91"/>
+      <c r="G1" s="91"/>
+      <c r="H1" s="91"/>
+      <c r="I1" s="91"/>
+      <c r="J1" s="91"/>
+      <c r="K1" s="91"/>
+      <c r="L1" s="91"/>
+      <c r="M1" s="91"/>
+      <c r="N1" s="91"/>
+      <c r="O1" s="91"/>
+      <c r="P1" s="91"/>
+      <c r="Q1" s="91"/>
+      <c r="R1" s="91"/>
+      <c r="S1" s="91"/>
+      <c r="T1" s="91"/>
+      <c r="U1" s="91"/>
+      <c r="V1" s="91"/>
+      <c r="W1" s="91"/>
+      <c r="X1" s="91"/>
+      <c r="Y1" s="91"/>
+      <c r="Z1" s="91"/>
+      <c r="AA1" s="91"/>
+      <c r="AB1" s="91"/>
+      <c r="AC1" s="91"/>
     </row>
     <row r="2" spans="1:29" ht="18">
       <c r="A2" s="23" t="s">
@@ -11336,10 +11922,10 @@
       <c r="AC2" s="28"/>
     </row>
     <row r="3" spans="1:29">
-      <c r="A3" s="91" t="s">
+      <c r="A3" s="92" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="91"/>
+      <c r="B3" s="92"/>
       <c r="C3" s="29"/>
       <c r="D3" s="3">
         <v>4</v>
@@ -11622,37 +12208,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="18">
-      <c r="A1" s="90" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="90"/>
-      <c r="C1" s="90"/>
-      <c r="D1" s="90"/>
-      <c r="E1" s="90"/>
-      <c r="F1" s="90"/>
-      <c r="G1" s="90"/>
-      <c r="H1" s="90"/>
-      <c r="I1" s="90"/>
-      <c r="J1" s="90"/>
-      <c r="K1" s="90"/>
-      <c r="L1" s="90"/>
-      <c r="M1" s="90"/>
-      <c r="N1" s="90"/>
-      <c r="O1" s="90"/>
-      <c r="P1" s="90"/>
-      <c r="Q1" s="90"/>
-      <c r="R1" s="90"/>
-      <c r="S1" s="90"/>
-      <c r="T1" s="90"/>
-      <c r="U1" s="90"/>
-      <c r="V1" s="90"/>
-      <c r="W1" s="90"/>
-      <c r="X1" s="90"/>
-      <c r="Y1" s="90"/>
-      <c r="Z1" s="90"/>
-      <c r="AA1" s="90"/>
-      <c r="AB1" s="90"/>
-      <c r="AC1" s="90"/>
+      <c r="A1" s="91" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="91"/>
+      <c r="C1" s="91"/>
+      <c r="D1" s="91"/>
+      <c r="E1" s="91"/>
+      <c r="F1" s="91"/>
+      <c r="G1" s="91"/>
+      <c r="H1" s="91"/>
+      <c r="I1" s="91"/>
+      <c r="J1" s="91"/>
+      <c r="K1" s="91"/>
+      <c r="L1" s="91"/>
+      <c r="M1" s="91"/>
+      <c r="N1" s="91"/>
+      <c r="O1" s="91"/>
+      <c r="P1" s="91"/>
+      <c r="Q1" s="91"/>
+      <c r="R1" s="91"/>
+      <c r="S1" s="91"/>
+      <c r="T1" s="91"/>
+      <c r="U1" s="91"/>
+      <c r="V1" s="91"/>
+      <c r="W1" s="91"/>
+      <c r="X1" s="91"/>
+      <c r="Y1" s="91"/>
+      <c r="Z1" s="91"/>
+      <c r="AA1" s="91"/>
+      <c r="AB1" s="91"/>
+      <c r="AC1" s="91"/>
     </row>
     <row r="2" spans="1:29" ht="18">
       <c r="A2" s="23" t="s">
@@ -11690,10 +12276,10 @@
       <c r="AC2" s="28"/>
     </row>
     <row r="3" spans="1:29">
-      <c r="A3" s="91" t="s">
+      <c r="A3" s="92" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="91"/>
+      <c r="B3" s="92"/>
       <c r="C3" s="29"/>
       <c r="D3" s="3">
         <v>3</v>
@@ -11975,37 +12561,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="18">
-      <c r="A1" s="90" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="90"/>
-      <c r="C1" s="90"/>
-      <c r="D1" s="90"/>
-      <c r="E1" s="90"/>
-      <c r="F1" s="90"/>
-      <c r="G1" s="90"/>
-      <c r="H1" s="90"/>
-      <c r="I1" s="90"/>
-      <c r="J1" s="90"/>
-      <c r="K1" s="90"/>
-      <c r="L1" s="90"/>
-      <c r="M1" s="90"/>
-      <c r="N1" s="90"/>
-      <c r="O1" s="90"/>
-      <c r="P1" s="90"/>
-      <c r="Q1" s="90"/>
-      <c r="R1" s="90"/>
-      <c r="S1" s="90"/>
-      <c r="T1" s="90"/>
-      <c r="U1" s="90"/>
-      <c r="V1" s="90"/>
-      <c r="W1" s="90"/>
-      <c r="X1" s="90"/>
-      <c r="Y1" s="90"/>
-      <c r="Z1" s="90"/>
-      <c r="AA1" s="90"/>
-      <c r="AB1" s="90"/>
-      <c r="AC1" s="90"/>
+      <c r="A1" s="91" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="91"/>
+      <c r="C1" s="91"/>
+      <c r="D1" s="91"/>
+      <c r="E1" s="91"/>
+      <c r="F1" s="91"/>
+      <c r="G1" s="91"/>
+      <c r="H1" s="91"/>
+      <c r="I1" s="91"/>
+      <c r="J1" s="91"/>
+      <c r="K1" s="91"/>
+      <c r="L1" s="91"/>
+      <c r="M1" s="91"/>
+      <c r="N1" s="91"/>
+      <c r="O1" s="91"/>
+      <c r="P1" s="91"/>
+      <c r="Q1" s="91"/>
+      <c r="R1" s="91"/>
+      <c r="S1" s="91"/>
+      <c r="T1" s="91"/>
+      <c r="U1" s="91"/>
+      <c r="V1" s="91"/>
+      <c r="W1" s="91"/>
+      <c r="X1" s="91"/>
+      <c r="Y1" s="91"/>
+      <c r="Z1" s="91"/>
+      <c r="AA1" s="91"/>
+      <c r="AB1" s="91"/>
+      <c r="AC1" s="91"/>
     </row>
     <row r="2" spans="1:29" ht="18">
       <c r="A2" s="23" t="s">
@@ -12043,10 +12629,10 @@
       <c r="AC2" s="28"/>
     </row>
     <row r="3" spans="1:29">
-      <c r="A3" s="91" t="s">
+      <c r="A3" s="92" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="91"/>
+      <c r="B3" s="92"/>
       <c r="C3" s="29"/>
       <c r="D3" s="3">
         <v>5</v>
@@ -12330,37 +12916,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="18">
-      <c r="A1" s="90" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="90"/>
-      <c r="C1" s="90"/>
-      <c r="D1" s="90"/>
-      <c r="E1" s="90"/>
-      <c r="F1" s="90"/>
-      <c r="G1" s="90"/>
-      <c r="H1" s="90"/>
-      <c r="I1" s="90"/>
-      <c r="J1" s="90"/>
-      <c r="K1" s="90"/>
-      <c r="L1" s="90"/>
-      <c r="M1" s="90"/>
-      <c r="N1" s="90"/>
-      <c r="O1" s="90"/>
-      <c r="P1" s="90"/>
-      <c r="Q1" s="90"/>
-      <c r="R1" s="90"/>
-      <c r="S1" s="90"/>
-      <c r="T1" s="90"/>
-      <c r="U1" s="90"/>
-      <c r="V1" s="90"/>
-      <c r="W1" s="90"/>
-      <c r="X1" s="90"/>
-      <c r="Y1" s="90"/>
-      <c r="Z1" s="90"/>
-      <c r="AA1" s="90"/>
-      <c r="AB1" s="90"/>
-      <c r="AC1" s="90"/>
+      <c r="A1" s="91" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="91"/>
+      <c r="C1" s="91"/>
+      <c r="D1" s="91"/>
+      <c r="E1" s="91"/>
+      <c r="F1" s="91"/>
+      <c r="G1" s="91"/>
+      <c r="H1" s="91"/>
+      <c r="I1" s="91"/>
+      <c r="J1" s="91"/>
+      <c r="K1" s="91"/>
+      <c r="L1" s="91"/>
+      <c r="M1" s="91"/>
+      <c r="N1" s="91"/>
+      <c r="O1" s="91"/>
+      <c r="P1" s="91"/>
+      <c r="Q1" s="91"/>
+      <c r="R1" s="91"/>
+      <c r="S1" s="91"/>
+      <c r="T1" s="91"/>
+      <c r="U1" s="91"/>
+      <c r="V1" s="91"/>
+      <c r="W1" s="91"/>
+      <c r="X1" s="91"/>
+      <c r="Y1" s="91"/>
+      <c r="Z1" s="91"/>
+      <c r="AA1" s="91"/>
+      <c r="AB1" s="91"/>
+      <c r="AC1" s="91"/>
     </row>
     <row r="2" spans="1:29" ht="18">
       <c r="A2" s="23" t="s">
@@ -12398,10 +12984,10 @@
       <c r="AC2" s="32"/>
     </row>
     <row r="3" spans="1:29">
-      <c r="A3" s="91" t="s">
+      <c r="A3" s="92" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="91"/>
+      <c r="B3" s="92"/>
       <c r="C3" s="33"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -12683,37 +13269,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="18">
-      <c r="A1" s="90" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="90"/>
-      <c r="C1" s="90"/>
-      <c r="D1" s="90"/>
-      <c r="E1" s="90"/>
-      <c r="F1" s="90"/>
-      <c r="G1" s="90"/>
-      <c r="H1" s="90"/>
-      <c r="I1" s="90"/>
-      <c r="J1" s="90"/>
-      <c r="K1" s="90"/>
-      <c r="L1" s="90"/>
-      <c r="M1" s="90"/>
-      <c r="N1" s="90"/>
-      <c r="O1" s="90"/>
-      <c r="P1" s="90"/>
-      <c r="Q1" s="90"/>
-      <c r="R1" s="90"/>
-      <c r="S1" s="90"/>
-      <c r="T1" s="90"/>
-      <c r="U1" s="90"/>
-      <c r="V1" s="90"/>
-      <c r="W1" s="90"/>
-      <c r="X1" s="90"/>
-      <c r="Y1" s="90"/>
-      <c r="Z1" s="90"/>
-      <c r="AA1" s="90"/>
-      <c r="AB1" s="90"/>
-      <c r="AC1" s="90"/>
+      <c r="A1" s="91" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="91"/>
+      <c r="C1" s="91"/>
+      <c r="D1" s="91"/>
+      <c r="E1" s="91"/>
+      <c r="F1" s="91"/>
+      <c r="G1" s="91"/>
+      <c r="H1" s="91"/>
+      <c r="I1" s="91"/>
+      <c r="J1" s="91"/>
+      <c r="K1" s="91"/>
+      <c r="L1" s="91"/>
+      <c r="M1" s="91"/>
+      <c r="N1" s="91"/>
+      <c r="O1" s="91"/>
+      <c r="P1" s="91"/>
+      <c r="Q1" s="91"/>
+      <c r="R1" s="91"/>
+      <c r="S1" s="91"/>
+      <c r="T1" s="91"/>
+      <c r="U1" s="91"/>
+      <c r="V1" s="91"/>
+      <c r="W1" s="91"/>
+      <c r="X1" s="91"/>
+      <c r="Y1" s="91"/>
+      <c r="Z1" s="91"/>
+      <c r="AA1" s="91"/>
+      <c r="AB1" s="91"/>
+      <c r="AC1" s="91"/>
     </row>
     <row r="2" spans="1:29" ht="18">
       <c r="A2" s="23" t="s">
@@ -12751,10 +13337,10 @@
       <c r="AC2" s="34"/>
     </row>
     <row r="3" spans="1:29">
-      <c r="A3" s="91" t="s">
+      <c r="A3" s="92" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="91"/>
+      <c r="B3" s="92"/>
       <c r="C3" s="35"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -13034,38 +13620,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:30" ht="18">
-      <c r="A1" s="90" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="90"/>
-      <c r="C1" s="90"/>
-      <c r="D1" s="90"/>
-      <c r="E1" s="90"/>
-      <c r="F1" s="90"/>
-      <c r="G1" s="90"/>
-      <c r="H1" s="90"/>
-      <c r="I1" s="90"/>
-      <c r="J1" s="90"/>
-      <c r="K1" s="90"/>
-      <c r="L1" s="90"/>
-      <c r="M1" s="90"/>
-      <c r="N1" s="90"/>
-      <c r="O1" s="90"/>
-      <c r="P1" s="90"/>
-      <c r="Q1" s="90"/>
-      <c r="R1" s="90"/>
-      <c r="S1" s="90"/>
-      <c r="T1" s="90"/>
-      <c r="U1" s="90"/>
-      <c r="V1" s="90"/>
-      <c r="W1" s="90"/>
-      <c r="X1" s="90"/>
-      <c r="Y1" s="90"/>
-      <c r="Z1" s="90"/>
-      <c r="AA1" s="90"/>
-      <c r="AB1" s="90"/>
-      <c r="AC1" s="90"/>
-      <c r="AD1" s="90"/>
+      <c r="A1" s="91" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="91"/>
+      <c r="C1" s="91"/>
+      <c r="D1" s="91"/>
+      <c r="E1" s="91"/>
+      <c r="F1" s="91"/>
+      <c r="G1" s="91"/>
+      <c r="H1" s="91"/>
+      <c r="I1" s="91"/>
+      <c r="J1" s="91"/>
+      <c r="K1" s="91"/>
+      <c r="L1" s="91"/>
+      <c r="M1" s="91"/>
+      <c r="N1" s="91"/>
+      <c r="O1" s="91"/>
+      <c r="P1" s="91"/>
+      <c r="Q1" s="91"/>
+      <c r="R1" s="91"/>
+      <c r="S1" s="91"/>
+      <c r="T1" s="91"/>
+      <c r="U1" s="91"/>
+      <c r="V1" s="91"/>
+      <c r="W1" s="91"/>
+      <c r="X1" s="91"/>
+      <c r="Y1" s="91"/>
+      <c r="Z1" s="91"/>
+      <c r="AA1" s="91"/>
+      <c r="AB1" s="91"/>
+      <c r="AC1" s="91"/>
+      <c r="AD1" s="91"/>
     </row>
     <row r="2" spans="1:30" ht="18">
       <c r="A2" s="23" t="s">
@@ -13104,10 +13690,10 @@
       <c r="AD2" s="36"/>
     </row>
     <row r="3" spans="1:30">
-      <c r="A3" s="91" t="s">
+      <c r="A3" s="92" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="91"/>
+      <c r="B3" s="92"/>
       <c r="C3" s="83"/>
       <c r="D3" s="37"/>
       <c r="E3" s="3">
@@ -13410,37 +13996,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:31" ht="18">
-      <c r="A1" s="90" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="90"/>
-      <c r="C1" s="90"/>
-      <c r="D1" s="90"/>
-      <c r="E1" s="90"/>
-      <c r="F1" s="90"/>
-      <c r="G1" s="90"/>
-      <c r="H1" s="90"/>
-      <c r="I1" s="90"/>
-      <c r="J1" s="90"/>
-      <c r="K1" s="90"/>
-      <c r="L1" s="90"/>
-      <c r="M1" s="90"/>
-      <c r="N1" s="90"/>
-      <c r="O1" s="90"/>
-      <c r="P1" s="90"/>
-      <c r="Q1" s="90"/>
-      <c r="R1" s="90"/>
-      <c r="S1" s="90"/>
-      <c r="T1" s="90"/>
-      <c r="U1" s="90"/>
-      <c r="V1" s="90"/>
-      <c r="W1" s="90"/>
-      <c r="X1" s="90"/>
-      <c r="Y1" s="90"/>
-      <c r="Z1" s="90"/>
-      <c r="AA1" s="90"/>
-      <c r="AB1" s="90"/>
-      <c r="AC1" s="90"/>
+      <c r="A1" s="91" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="91"/>
+      <c r="C1" s="91"/>
+      <c r="D1" s="91"/>
+      <c r="E1" s="91"/>
+      <c r="F1" s="91"/>
+      <c r="G1" s="91"/>
+      <c r="H1" s="91"/>
+      <c r="I1" s="91"/>
+      <c r="J1" s="91"/>
+      <c r="K1" s="91"/>
+      <c r="L1" s="91"/>
+      <c r="M1" s="91"/>
+      <c r="N1" s="91"/>
+      <c r="O1" s="91"/>
+      <c r="P1" s="91"/>
+      <c r="Q1" s="91"/>
+      <c r="R1" s="91"/>
+      <c r="S1" s="91"/>
+      <c r="T1" s="91"/>
+      <c r="U1" s="91"/>
+      <c r="V1" s="91"/>
+      <c r="W1" s="91"/>
+      <c r="X1" s="91"/>
+      <c r="Y1" s="91"/>
+      <c r="Z1" s="91"/>
+      <c r="AA1" s="91"/>
+      <c r="AB1" s="91"/>
+      <c r="AC1" s="91"/>
     </row>
     <row r="2" spans="1:31" ht="16.5" customHeight="1">
       <c r="A2" s="23" t="s">
@@ -13478,10 +14064,10 @@
       <c r="AC2" s="41"/>
     </row>
     <row r="3" spans="1:31">
-      <c r="A3" s="91" t="s">
+      <c r="A3" s="92" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="91"/>
+      <c r="B3" s="92"/>
       <c r="D3">
         <v>2</v>
       </c>

</xml_diff>

<commit_message>
Failure Fixes of Purchase bills and Standard Price List
Failure Fixes of Purchase bills and Standard Price List
</commit_message>
<xml_diff>
--- a/testdata/DBfin.xlsx
+++ b/testdata/DBfin.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4507"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="2520" windowWidth="15240" windowHeight="6540" tabRatio="849" firstSheet="24" activeTab="28"/>
+    <workbookView xWindow="0" yWindow="2520" windowWidth="15240" windowHeight="6540" tabRatio="849" firstSheet="25" activeTab="28"/>
   </bookViews>
   <sheets>
     <sheet name="PurchaseBillsLocal" sheetId="1" r:id="rId1"/>
@@ -37,6 +37,7 @@
     <sheet name="purchaseBills_GRN_igst" sheetId="28" r:id="rId28"/>
     <sheet name="PurchaseBills_IGST_Validation_3" sheetId="29" r:id="rId29"/>
     <sheet name="Sheet1" sheetId="30" r:id="rId30"/>
+    <sheet name="Sheet2" sheetId="31" r:id="rId31"/>
   </sheets>
   <calcPr calcId="125725"/>
 </workbook>
@@ -12882,6 +12883,15 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:AC6"/>

</xml_diff>

<commit_message>
Failure Fixes of Purchase bills
Failure Fixes of Purchase bills
</commit_message>
<xml_diff>
--- a/testdata/DBfin.xlsx
+++ b/testdata/DBfin.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4507"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="2520" windowWidth="15240" windowHeight="6540" tabRatio="849" firstSheet="25" activeTab="28"/>
+    <workbookView xWindow="0" yWindow="2520" windowWidth="15240" windowHeight="6540" tabRatio="849" firstSheet="26" activeTab="29"/>
   </bookViews>
   <sheets>
     <sheet name="PurchaseBillsLocal" sheetId="1" r:id="rId1"/>
@@ -36,15 +36,17 @@
     <sheet name="Purchase_Bills_Allow_IGST" sheetId="27" r:id="rId27"/>
     <sheet name="purchaseBills_GRN_igst" sheetId="28" r:id="rId28"/>
     <sheet name="PurchaseBills_IGST_Validation_3" sheetId="29" r:id="rId29"/>
-    <sheet name="Sheet1" sheetId="30" r:id="rId30"/>
-    <sheet name="Sheet2" sheetId="31" r:id="rId31"/>
+    <sheet name="PurchaseBills_2_67" sheetId="30" r:id="rId30"/>
+    <sheet name="Purchasebills_IGST_Updated_1" sheetId="31" r:id="rId31"/>
+    <sheet name="Sheet3" sheetId="32" r:id="rId32"/>
+    <sheet name="Sheet1" sheetId="33" r:id="rId33"/>
   </sheets>
   <calcPr calcId="125725"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1635" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1750" uniqueCount="115">
   <si>
     <t>Scenario  : Local Sales - Stock UOM and Sales UOM (Similar)   DOC NO :  SORD-2425-00089</t>
   </si>
@@ -396,11 +398,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="0.000"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
     <numFmt numFmtId="166" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="167" formatCode="_(* #,##0.0_);_(* \(#,##0.0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="11">
     <font>
@@ -587,7 +590,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="96">
+  <cellXfs count="99">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -812,6 +815,13 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="167" fontId="3" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -1143,68 +1153,68 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:59" ht="18">
-      <c r="A1" s="94" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="94"/>
-      <c r="C1" s="94"/>
-      <c r="D1" s="94"/>
-      <c r="E1" s="94"/>
-      <c r="F1" s="94"/>
-      <c r="G1" s="94"/>
-      <c r="H1" s="94"/>
-      <c r="I1" s="94"/>
-      <c r="J1" s="94"/>
-      <c r="K1" s="94"/>
-      <c r="L1" s="94"/>
-      <c r="M1" s="94"/>
-      <c r="N1" s="94"/>
-      <c r="O1" s="94"/>
-      <c r="P1" s="94"/>
-      <c r="Q1" s="94"/>
-      <c r="R1" s="94"/>
-      <c r="S1" s="94"/>
-      <c r="T1" s="94"/>
-      <c r="U1" s="94"/>
-      <c r="V1" s="94"/>
-      <c r="W1" s="94"/>
-      <c r="X1" s="94"/>
-      <c r="Y1" s="94"/>
-      <c r="Z1" s="94"/>
-      <c r="AA1" s="94"/>
-      <c r="AB1" s="94"/>
-      <c r="AC1" s="94"/>
-      <c r="AD1" s="94" t="s">
-        <v>0</v>
-      </c>
-      <c r="AE1" s="94"/>
-      <c r="AF1" s="94"/>
-      <c r="AG1" s="94"/>
-      <c r="AH1" s="94"/>
-      <c r="AI1" s="94"/>
-      <c r="AJ1" s="94"/>
-      <c r="AK1" s="94"/>
-      <c r="AL1" s="94"/>
-      <c r="AM1" s="94"/>
-      <c r="AN1" s="94"/>
-      <c r="AO1" s="94"/>
-      <c r="AP1" s="94"/>
-      <c r="AQ1" s="94"/>
-      <c r="AR1" s="94"/>
-      <c r="AS1" s="94"/>
-      <c r="AT1" s="94"/>
-      <c r="AU1" s="94"/>
-      <c r="AV1" s="94"/>
-      <c r="AW1" s="94"/>
-      <c r="AX1" s="94"/>
-      <c r="AY1" s="94"/>
-      <c r="AZ1" s="94"/>
-      <c r="BA1" s="94"/>
-      <c r="BB1" s="94"/>
-      <c r="BC1" s="94"/>
-      <c r="BD1" s="94"/>
-      <c r="BE1" s="94"/>
-      <c r="BF1" s="94"/>
+      <c r="A1" s="97" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="97"/>
+      <c r="C1" s="97"/>
+      <c r="D1" s="97"/>
+      <c r="E1" s="97"/>
+      <c r="F1" s="97"/>
+      <c r="G1" s="97"/>
+      <c r="H1" s="97"/>
+      <c r="I1" s="97"/>
+      <c r="J1" s="97"/>
+      <c r="K1" s="97"/>
+      <c r="L1" s="97"/>
+      <c r="M1" s="97"/>
+      <c r="N1" s="97"/>
+      <c r="O1" s="97"/>
+      <c r="P1" s="97"/>
+      <c r="Q1" s="97"/>
+      <c r="R1" s="97"/>
+      <c r="S1" s="97"/>
+      <c r="T1" s="97"/>
+      <c r="U1" s="97"/>
+      <c r="V1" s="97"/>
+      <c r="W1" s="97"/>
+      <c r="X1" s="97"/>
+      <c r="Y1" s="97"/>
+      <c r="Z1" s="97"/>
+      <c r="AA1" s="97"/>
+      <c r="AB1" s="97"/>
+      <c r="AC1" s="97"/>
+      <c r="AD1" s="97" t="s">
+        <v>0</v>
+      </c>
+      <c r="AE1" s="97"/>
+      <c r="AF1" s="97"/>
+      <c r="AG1" s="97"/>
+      <c r="AH1" s="97"/>
+      <c r="AI1" s="97"/>
+      <c r="AJ1" s="97"/>
+      <c r="AK1" s="97"/>
+      <c r="AL1" s="97"/>
+      <c r="AM1" s="97"/>
+      <c r="AN1" s="97"/>
+      <c r="AO1" s="97"/>
+      <c r="AP1" s="97"/>
+      <c r="AQ1" s="97"/>
+      <c r="AR1" s="97"/>
+      <c r="AS1" s="97"/>
+      <c r="AT1" s="97"/>
+      <c r="AU1" s="97"/>
+      <c r="AV1" s="97"/>
+      <c r="AW1" s="97"/>
+      <c r="AX1" s="97"/>
+      <c r="AY1" s="97"/>
+      <c r="AZ1" s="97"/>
+      <c r="BA1" s="97"/>
+      <c r="BB1" s="97"/>
+      <c r="BC1" s="97"/>
+      <c r="BD1" s="97"/>
+      <c r="BE1" s="97"/>
+      <c r="BF1" s="97"/>
     </row>
     <row r="2" spans="1:59" ht="18">
       <c r="A2" s="23" t="s">
@@ -1275,10 +1285,10 @@
       <c r="BF2" s="38"/>
     </row>
     <row r="3" spans="1:59">
-      <c r="A3" s="95" t="s">
+      <c r="A3" s="98" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="95"/>
+      <c r="B3" s="98"/>
       <c r="C3" s="2"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -1318,10 +1328,10 @@
       <c r="AA3" s="6"/>
       <c r="AB3" s="6"/>
       <c r="AC3" s="6"/>
-      <c r="AD3" s="95" t="s">
+      <c r="AD3" s="98" t="s">
         <v>3</v>
       </c>
-      <c r="AE3" s="95"/>
+      <c r="AE3" s="98"/>
       <c r="AF3" s="39"/>
       <c r="AG3" s="3">
         <v>1</v>
@@ -1799,38 +1809,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:33" ht="18">
-      <c r="A1" s="94" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="94"/>
-      <c r="C1" s="94"/>
-      <c r="D1" s="94"/>
-      <c r="E1" s="94"/>
-      <c r="F1" s="94"/>
-      <c r="G1" s="94"/>
-      <c r="H1" s="94"/>
-      <c r="I1" s="94"/>
-      <c r="J1" s="94"/>
-      <c r="K1" s="94"/>
-      <c r="L1" s="94"/>
-      <c r="M1" s="94"/>
-      <c r="N1" s="94"/>
-      <c r="O1" s="94"/>
-      <c r="P1" s="94"/>
-      <c r="Q1" s="94"/>
-      <c r="R1" s="94"/>
-      <c r="S1" s="94"/>
-      <c r="T1" s="94"/>
-      <c r="U1" s="94"/>
-      <c r="V1" s="94"/>
-      <c r="W1" s="94"/>
-      <c r="X1" s="94"/>
-      <c r="Y1" s="94"/>
-      <c r="Z1" s="94"/>
-      <c r="AA1" s="94"/>
-      <c r="AB1" s="94"/>
-      <c r="AC1" s="94"/>
-      <c r="AD1" s="94"/>
+      <c r="A1" s="97" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="97"/>
+      <c r="C1" s="97"/>
+      <c r="D1" s="97"/>
+      <c r="E1" s="97"/>
+      <c r="F1" s="97"/>
+      <c r="G1" s="97"/>
+      <c r="H1" s="97"/>
+      <c r="I1" s="97"/>
+      <c r="J1" s="97"/>
+      <c r="K1" s="97"/>
+      <c r="L1" s="97"/>
+      <c r="M1" s="97"/>
+      <c r="N1" s="97"/>
+      <c r="O1" s="97"/>
+      <c r="P1" s="97"/>
+      <c r="Q1" s="97"/>
+      <c r="R1" s="97"/>
+      <c r="S1" s="97"/>
+      <c r="T1" s="97"/>
+      <c r="U1" s="97"/>
+      <c r="V1" s="97"/>
+      <c r="W1" s="97"/>
+      <c r="X1" s="97"/>
+      <c r="Y1" s="97"/>
+      <c r="Z1" s="97"/>
+      <c r="AA1" s="97"/>
+      <c r="AB1" s="97"/>
+      <c r="AC1" s="97"/>
+      <c r="AD1" s="97"/>
     </row>
     <row r="2" spans="1:33" ht="18">
       <c r="A2" s="23" t="s">
@@ -1869,10 +1879,10 @@
       <c r="AD2" s="43"/>
     </row>
     <row r="3" spans="1:33" ht="15.75" thickBot="1">
-      <c r="A3" s="95" t="s">
+      <c r="A3" s="98" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="95"/>
+      <c r="B3" s="98"/>
       <c r="C3" s="44"/>
       <c r="D3" s="3">
         <v>2</v>
@@ -2486,37 +2496,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:31" ht="18">
-      <c r="A1" s="94" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="94"/>
-      <c r="C1" s="94"/>
-      <c r="D1" s="94"/>
-      <c r="E1" s="94"/>
-      <c r="F1" s="94"/>
-      <c r="G1" s="94"/>
-      <c r="H1" s="94"/>
-      <c r="I1" s="94"/>
-      <c r="J1" s="94"/>
-      <c r="K1" s="94"/>
-      <c r="L1" s="94"/>
-      <c r="M1" s="94"/>
-      <c r="N1" s="94"/>
-      <c r="O1" s="94"/>
-      <c r="P1" s="94"/>
-      <c r="Q1" s="94"/>
-      <c r="R1" s="94"/>
-      <c r="S1" s="94"/>
-      <c r="T1" s="94"/>
-      <c r="U1" s="94"/>
-      <c r="V1" s="94"/>
-      <c r="W1" s="94"/>
-      <c r="X1" s="94"/>
-      <c r="Y1" s="94"/>
-      <c r="Z1" s="94"/>
-      <c r="AA1" s="94"/>
-      <c r="AB1" s="94"/>
-      <c r="AC1" s="94"/>
+      <c r="A1" s="97" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="97"/>
+      <c r="C1" s="97"/>
+      <c r="D1" s="97"/>
+      <c r="E1" s="97"/>
+      <c r="F1" s="97"/>
+      <c r="G1" s="97"/>
+      <c r="H1" s="97"/>
+      <c r="I1" s="97"/>
+      <c r="J1" s="97"/>
+      <c r="K1" s="97"/>
+      <c r="L1" s="97"/>
+      <c r="M1" s="97"/>
+      <c r="N1" s="97"/>
+      <c r="O1" s="97"/>
+      <c r="P1" s="97"/>
+      <c r="Q1" s="97"/>
+      <c r="R1" s="97"/>
+      <c r="S1" s="97"/>
+      <c r="T1" s="97"/>
+      <c r="U1" s="97"/>
+      <c r="V1" s="97"/>
+      <c r="W1" s="97"/>
+      <c r="X1" s="97"/>
+      <c r="Y1" s="97"/>
+      <c r="Z1" s="97"/>
+      <c r="AA1" s="97"/>
+      <c r="AB1" s="97"/>
+      <c r="AC1" s="97"/>
     </row>
     <row r="2" spans="1:31" ht="16.5" customHeight="1">
       <c r="A2" s="23" t="s">
@@ -2554,10 +2564,10 @@
       <c r="AC2" s="54"/>
     </row>
     <row r="3" spans="1:31">
-      <c r="A3" s="95" t="s">
+      <c r="A3" s="98" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="95"/>
+      <c r="B3" s="98"/>
       <c r="D3">
         <v>2</v>
       </c>
@@ -3048,37 +3058,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="18">
-      <c r="A1" s="94" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="94"/>
-      <c r="C1" s="94"/>
-      <c r="D1" s="94"/>
-      <c r="E1" s="94"/>
-      <c r="F1" s="94"/>
-      <c r="G1" s="94"/>
-      <c r="H1" s="94"/>
-      <c r="I1" s="94"/>
-      <c r="J1" s="94"/>
-      <c r="K1" s="94"/>
-      <c r="L1" s="94"/>
-      <c r="M1" s="94"/>
-      <c r="N1" s="94"/>
-      <c r="O1" s="94"/>
-      <c r="P1" s="94"/>
-      <c r="Q1" s="94"/>
-      <c r="R1" s="94"/>
-      <c r="S1" s="94"/>
-      <c r="T1" s="94"/>
-      <c r="U1" s="94"/>
-      <c r="V1" s="94"/>
-      <c r="W1" s="94"/>
-      <c r="X1" s="94"/>
-      <c r="Y1" s="94"/>
-      <c r="Z1" s="94"/>
-      <c r="AA1" s="94"/>
-      <c r="AB1" s="94"/>
-      <c r="AC1" s="94"/>
+      <c r="A1" s="97" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="97"/>
+      <c r="C1" s="97"/>
+      <c r="D1" s="97"/>
+      <c r="E1" s="97"/>
+      <c r="F1" s="97"/>
+      <c r="G1" s="97"/>
+      <c r="H1" s="97"/>
+      <c r="I1" s="97"/>
+      <c r="J1" s="97"/>
+      <c r="K1" s="97"/>
+      <c r="L1" s="97"/>
+      <c r="M1" s="97"/>
+      <c r="N1" s="97"/>
+      <c r="O1" s="97"/>
+      <c r="P1" s="97"/>
+      <c r="Q1" s="97"/>
+      <c r="R1" s="97"/>
+      <c r="S1" s="97"/>
+      <c r="T1" s="97"/>
+      <c r="U1" s="97"/>
+      <c r="V1" s="97"/>
+      <c r="W1" s="97"/>
+      <c r="X1" s="97"/>
+      <c r="Y1" s="97"/>
+      <c r="Z1" s="97"/>
+      <c r="AA1" s="97"/>
+      <c r="AB1" s="97"/>
+      <c r="AC1" s="97"/>
     </row>
     <row r="2" spans="1:29" ht="18">
       <c r="A2" s="23" t="s">
@@ -3116,10 +3126,10 @@
       <c r="AC2" s="56"/>
     </row>
     <row r="3" spans="1:29">
-      <c r="A3" s="95" t="s">
+      <c r="A3" s="98" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="95"/>
+      <c r="B3" s="98"/>
       <c r="C3" s="57"/>
       <c r="D3" s="3">
         <v>2</v>
@@ -3400,37 +3410,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="18">
-      <c r="A1" s="94" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="94"/>
-      <c r="C1" s="94"/>
-      <c r="D1" s="94"/>
-      <c r="E1" s="94"/>
-      <c r="F1" s="94"/>
-      <c r="G1" s="94"/>
-      <c r="H1" s="94"/>
-      <c r="I1" s="94"/>
-      <c r="J1" s="94"/>
-      <c r="K1" s="94"/>
-      <c r="L1" s="94"/>
-      <c r="M1" s="94"/>
-      <c r="N1" s="94"/>
-      <c r="O1" s="94"/>
-      <c r="P1" s="94"/>
-      <c r="Q1" s="94"/>
-      <c r="R1" s="94"/>
-      <c r="S1" s="94"/>
-      <c r="T1" s="94"/>
-      <c r="U1" s="94"/>
-      <c r="V1" s="94"/>
-      <c r="W1" s="94"/>
-      <c r="X1" s="94"/>
-      <c r="Y1" s="94"/>
-      <c r="Z1" s="94"/>
-      <c r="AA1" s="94"/>
-      <c r="AB1" s="94"/>
-      <c r="AC1" s="94"/>
+      <c r="A1" s="97" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="97"/>
+      <c r="C1" s="97"/>
+      <c r="D1" s="97"/>
+      <c r="E1" s="97"/>
+      <c r="F1" s="97"/>
+      <c r="G1" s="97"/>
+      <c r="H1" s="97"/>
+      <c r="I1" s="97"/>
+      <c r="J1" s="97"/>
+      <c r="K1" s="97"/>
+      <c r="L1" s="97"/>
+      <c r="M1" s="97"/>
+      <c r="N1" s="97"/>
+      <c r="O1" s="97"/>
+      <c r="P1" s="97"/>
+      <c r="Q1" s="97"/>
+      <c r="R1" s="97"/>
+      <c r="S1" s="97"/>
+      <c r="T1" s="97"/>
+      <c r="U1" s="97"/>
+      <c r="V1" s="97"/>
+      <c r="W1" s="97"/>
+      <c r="X1" s="97"/>
+      <c r="Y1" s="97"/>
+      <c r="Z1" s="97"/>
+      <c r="AA1" s="97"/>
+      <c r="AB1" s="97"/>
+      <c r="AC1" s="97"/>
     </row>
     <row r="2" spans="1:29" ht="18">
       <c r="A2" s="23" t="s">
@@ -3468,10 +3478,10 @@
       <c r="AC2" s="58"/>
     </row>
     <row r="3" spans="1:29">
-      <c r="A3" s="95" t="s">
+      <c r="A3" s="98" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="95"/>
+      <c r="B3" s="98"/>
       <c r="C3" s="59"/>
       <c r="D3" s="3">
         <v>4</v>
@@ -3754,38 +3764,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:33" ht="18">
-      <c r="A1" s="94" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="94"/>
-      <c r="C1" s="94"/>
-      <c r="D1" s="94"/>
-      <c r="E1" s="94"/>
-      <c r="F1" s="94"/>
-      <c r="G1" s="94"/>
-      <c r="H1" s="94"/>
-      <c r="I1" s="94"/>
-      <c r="J1" s="94"/>
-      <c r="K1" s="94"/>
-      <c r="L1" s="94"/>
-      <c r="M1" s="94"/>
-      <c r="N1" s="94"/>
-      <c r="O1" s="94"/>
-      <c r="P1" s="94"/>
-      <c r="Q1" s="94"/>
-      <c r="R1" s="94"/>
-      <c r="S1" s="94"/>
-      <c r="T1" s="94"/>
-      <c r="U1" s="94"/>
-      <c r="V1" s="94"/>
-      <c r="W1" s="94"/>
-      <c r="X1" s="94"/>
-      <c r="Y1" s="94"/>
-      <c r="Z1" s="94"/>
-      <c r="AA1" s="94"/>
-      <c r="AB1" s="94"/>
-      <c r="AC1" s="94"/>
-      <c r="AD1" s="94"/>
+      <c r="A1" s="97" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="97"/>
+      <c r="C1" s="97"/>
+      <c r="D1" s="97"/>
+      <c r="E1" s="97"/>
+      <c r="F1" s="97"/>
+      <c r="G1" s="97"/>
+      <c r="H1" s="97"/>
+      <c r="I1" s="97"/>
+      <c r="J1" s="97"/>
+      <c r="K1" s="97"/>
+      <c r="L1" s="97"/>
+      <c r="M1" s="97"/>
+      <c r="N1" s="97"/>
+      <c r="O1" s="97"/>
+      <c r="P1" s="97"/>
+      <c r="Q1" s="97"/>
+      <c r="R1" s="97"/>
+      <c r="S1" s="97"/>
+      <c r="T1" s="97"/>
+      <c r="U1" s="97"/>
+      <c r="V1" s="97"/>
+      <c r="W1" s="97"/>
+      <c r="X1" s="97"/>
+      <c r="Y1" s="97"/>
+      <c r="Z1" s="97"/>
+      <c r="AA1" s="97"/>
+      <c r="AB1" s="97"/>
+      <c r="AC1" s="97"/>
+      <c r="AD1" s="97"/>
     </row>
     <row r="2" spans="1:33" ht="18">
       <c r="A2" s="23" t="s">
@@ -3824,10 +3834,10 @@
       <c r="AD2" s="60"/>
     </row>
     <row r="3" spans="1:33" ht="15.75" thickBot="1">
-      <c r="A3" s="95" t="s">
+      <c r="A3" s="98" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="95"/>
+      <c r="B3" s="98"/>
       <c r="C3" s="61"/>
       <c r="D3" s="3">
         <v>2</v>
@@ -4440,37 +4450,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="18">
-      <c r="A1" s="94" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="94"/>
-      <c r="C1" s="94"/>
-      <c r="D1" s="94"/>
-      <c r="E1" s="94"/>
-      <c r="F1" s="94"/>
-      <c r="G1" s="94"/>
-      <c r="H1" s="94"/>
-      <c r="I1" s="94"/>
-      <c r="J1" s="94"/>
-      <c r="K1" s="94"/>
-      <c r="L1" s="94"/>
-      <c r="M1" s="94"/>
-      <c r="N1" s="94"/>
-      <c r="O1" s="94"/>
-      <c r="P1" s="94"/>
-      <c r="Q1" s="94"/>
-      <c r="R1" s="94"/>
-      <c r="S1" s="94"/>
-      <c r="T1" s="94"/>
-      <c r="U1" s="94"/>
-      <c r="V1" s="94"/>
-      <c r="W1" s="94"/>
-      <c r="X1" s="94"/>
-      <c r="Y1" s="94"/>
-      <c r="Z1" s="94"/>
-      <c r="AA1" s="94"/>
-      <c r="AB1" s="94"/>
-      <c r="AC1" s="94"/>
+      <c r="A1" s="97" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="97"/>
+      <c r="C1" s="97"/>
+      <c r="D1" s="97"/>
+      <c r="E1" s="97"/>
+      <c r="F1" s="97"/>
+      <c r="G1" s="97"/>
+      <c r="H1" s="97"/>
+      <c r="I1" s="97"/>
+      <c r="J1" s="97"/>
+      <c r="K1" s="97"/>
+      <c r="L1" s="97"/>
+      <c r="M1" s="97"/>
+      <c r="N1" s="97"/>
+      <c r="O1" s="97"/>
+      <c r="P1" s="97"/>
+      <c r="Q1" s="97"/>
+      <c r="R1" s="97"/>
+      <c r="S1" s="97"/>
+      <c r="T1" s="97"/>
+      <c r="U1" s="97"/>
+      <c r="V1" s="97"/>
+      <c r="W1" s="97"/>
+      <c r="X1" s="97"/>
+      <c r="Y1" s="97"/>
+      <c r="Z1" s="97"/>
+      <c r="AA1" s="97"/>
+      <c r="AB1" s="97"/>
+      <c r="AC1" s="97"/>
     </row>
     <row r="2" spans="1:29" ht="18">
       <c r="A2" s="23" t="s">
@@ -4508,10 +4518,10 @@
       <c r="AC2" s="62"/>
     </row>
     <row r="3" spans="1:29">
-      <c r="A3" s="95" t="s">
+      <c r="A3" s="98" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="95"/>
+      <c r="B3" s="98"/>
       <c r="C3" s="63"/>
       <c r="D3" s="3">
         <v>4</v>
@@ -4800,68 +4810,68 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:59" ht="18">
-      <c r="A1" s="94" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="94"/>
-      <c r="C1" s="94"/>
-      <c r="D1" s="94"/>
-      <c r="E1" s="94"/>
-      <c r="F1" s="94"/>
-      <c r="G1" s="94"/>
-      <c r="H1" s="94"/>
-      <c r="I1" s="94"/>
-      <c r="J1" s="94"/>
-      <c r="K1" s="94"/>
-      <c r="L1" s="94"/>
-      <c r="M1" s="94"/>
-      <c r="N1" s="94"/>
-      <c r="O1" s="94"/>
-      <c r="P1" s="94"/>
-      <c r="Q1" s="94"/>
-      <c r="R1" s="94"/>
-      <c r="S1" s="94"/>
-      <c r="T1" s="94"/>
-      <c r="U1" s="94"/>
-      <c r="V1" s="94"/>
-      <c r="W1" s="94"/>
-      <c r="X1" s="94"/>
-      <c r="Y1" s="94"/>
-      <c r="Z1" s="94"/>
-      <c r="AA1" s="94"/>
-      <c r="AB1" s="94"/>
-      <c r="AC1" s="94"/>
-      <c r="AD1" s="94" t="s">
-        <v>0</v>
-      </c>
-      <c r="AE1" s="94"/>
-      <c r="AF1" s="94"/>
-      <c r="AG1" s="94"/>
-      <c r="AH1" s="94"/>
-      <c r="AI1" s="94"/>
-      <c r="AJ1" s="94"/>
-      <c r="AK1" s="94"/>
-      <c r="AL1" s="94"/>
-      <c r="AM1" s="94"/>
-      <c r="AN1" s="94"/>
-      <c r="AO1" s="94"/>
-      <c r="AP1" s="94"/>
-      <c r="AQ1" s="94"/>
-      <c r="AR1" s="94"/>
-      <c r="AS1" s="94"/>
-      <c r="AT1" s="94"/>
-      <c r="AU1" s="94"/>
-      <c r="AV1" s="94"/>
-      <c r="AW1" s="94"/>
-      <c r="AX1" s="94"/>
-      <c r="AY1" s="94"/>
-      <c r="AZ1" s="94"/>
-      <c r="BA1" s="94"/>
-      <c r="BB1" s="94"/>
-      <c r="BC1" s="94"/>
-      <c r="BD1" s="94"/>
-      <c r="BE1" s="94"/>
-      <c r="BF1" s="94"/>
+      <c r="A1" s="97" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="97"/>
+      <c r="C1" s="97"/>
+      <c r="D1" s="97"/>
+      <c r="E1" s="97"/>
+      <c r="F1" s="97"/>
+      <c r="G1" s="97"/>
+      <c r="H1" s="97"/>
+      <c r="I1" s="97"/>
+      <c r="J1" s="97"/>
+      <c r="K1" s="97"/>
+      <c r="L1" s="97"/>
+      <c r="M1" s="97"/>
+      <c r="N1" s="97"/>
+      <c r="O1" s="97"/>
+      <c r="P1" s="97"/>
+      <c r="Q1" s="97"/>
+      <c r="R1" s="97"/>
+      <c r="S1" s="97"/>
+      <c r="T1" s="97"/>
+      <c r="U1" s="97"/>
+      <c r="V1" s="97"/>
+      <c r="W1" s="97"/>
+      <c r="X1" s="97"/>
+      <c r="Y1" s="97"/>
+      <c r="Z1" s="97"/>
+      <c r="AA1" s="97"/>
+      <c r="AB1" s="97"/>
+      <c r="AC1" s="97"/>
+      <c r="AD1" s="97" t="s">
+        <v>0</v>
+      </c>
+      <c r="AE1" s="97"/>
+      <c r="AF1" s="97"/>
+      <c r="AG1" s="97"/>
+      <c r="AH1" s="97"/>
+      <c r="AI1" s="97"/>
+      <c r="AJ1" s="97"/>
+      <c r="AK1" s="97"/>
+      <c r="AL1" s="97"/>
+      <c r="AM1" s="97"/>
+      <c r="AN1" s="97"/>
+      <c r="AO1" s="97"/>
+      <c r="AP1" s="97"/>
+      <c r="AQ1" s="97"/>
+      <c r="AR1" s="97"/>
+      <c r="AS1" s="97"/>
+      <c r="AT1" s="97"/>
+      <c r="AU1" s="97"/>
+      <c r="AV1" s="97"/>
+      <c r="AW1" s="97"/>
+      <c r="AX1" s="97"/>
+      <c r="AY1" s="97"/>
+      <c r="AZ1" s="97"/>
+      <c r="BA1" s="97"/>
+      <c r="BB1" s="97"/>
+      <c r="BC1" s="97"/>
+      <c r="BD1" s="97"/>
+      <c r="BE1" s="97"/>
+      <c r="BF1" s="97"/>
     </row>
     <row r="2" spans="1:59" ht="18">
       <c r="A2" s="23" t="s">
@@ -4932,10 +4942,10 @@
       <c r="BF2" s="64"/>
     </row>
     <row r="3" spans="1:59">
-      <c r="A3" s="95" t="s">
+      <c r="A3" s="98" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="95"/>
+      <c r="B3" s="98"/>
       <c r="C3" s="65"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -4975,10 +4985,10 @@
       <c r="AA3" s="6"/>
       <c r="AB3" s="6"/>
       <c r="AC3" s="6"/>
-      <c r="AD3" s="95" t="s">
+      <c r="AD3" s="98" t="s">
         <v>3</v>
       </c>
-      <c r="AE3" s="95"/>
+      <c r="AE3" s="98"/>
       <c r="AF3" s="65"/>
       <c r="AG3" s="3">
         <v>2</v>
@@ -5460,68 +5470,68 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:59" ht="18">
-      <c r="A1" s="94" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="94"/>
-      <c r="C1" s="94"/>
-      <c r="D1" s="94"/>
-      <c r="E1" s="94"/>
-      <c r="F1" s="94"/>
-      <c r="G1" s="94"/>
-      <c r="H1" s="94"/>
-      <c r="I1" s="94"/>
-      <c r="J1" s="94"/>
-      <c r="K1" s="94"/>
-      <c r="L1" s="94"/>
-      <c r="M1" s="94"/>
-      <c r="N1" s="94"/>
-      <c r="O1" s="94"/>
-      <c r="P1" s="94"/>
-      <c r="Q1" s="94"/>
-      <c r="R1" s="94"/>
-      <c r="S1" s="94"/>
-      <c r="T1" s="94"/>
-      <c r="U1" s="94"/>
-      <c r="V1" s="94"/>
-      <c r="W1" s="94"/>
-      <c r="X1" s="94"/>
-      <c r="Y1" s="94"/>
-      <c r="Z1" s="94"/>
-      <c r="AA1" s="94"/>
-      <c r="AB1" s="94"/>
-      <c r="AC1" s="94"/>
-      <c r="AD1" s="94" t="s">
-        <v>0</v>
-      </c>
-      <c r="AE1" s="94"/>
-      <c r="AF1" s="94"/>
-      <c r="AG1" s="94"/>
-      <c r="AH1" s="94"/>
-      <c r="AI1" s="94"/>
-      <c r="AJ1" s="94"/>
-      <c r="AK1" s="94"/>
-      <c r="AL1" s="94"/>
-      <c r="AM1" s="94"/>
-      <c r="AN1" s="94"/>
-      <c r="AO1" s="94"/>
-      <c r="AP1" s="94"/>
-      <c r="AQ1" s="94"/>
-      <c r="AR1" s="94"/>
-      <c r="AS1" s="94"/>
-      <c r="AT1" s="94"/>
-      <c r="AU1" s="94"/>
-      <c r="AV1" s="94"/>
-      <c r="AW1" s="94"/>
-      <c r="AX1" s="94"/>
-      <c r="AY1" s="94"/>
-      <c r="AZ1" s="94"/>
-      <c r="BA1" s="94"/>
-      <c r="BB1" s="94"/>
-      <c r="BC1" s="94"/>
-      <c r="BD1" s="94"/>
-      <c r="BE1" s="94"/>
-      <c r="BF1" s="94"/>
+      <c r="A1" s="97" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="97"/>
+      <c r="C1" s="97"/>
+      <c r="D1" s="97"/>
+      <c r="E1" s="97"/>
+      <c r="F1" s="97"/>
+      <c r="G1" s="97"/>
+      <c r="H1" s="97"/>
+      <c r="I1" s="97"/>
+      <c r="J1" s="97"/>
+      <c r="K1" s="97"/>
+      <c r="L1" s="97"/>
+      <c r="M1" s="97"/>
+      <c r="N1" s="97"/>
+      <c r="O1" s="97"/>
+      <c r="P1" s="97"/>
+      <c r="Q1" s="97"/>
+      <c r="R1" s="97"/>
+      <c r="S1" s="97"/>
+      <c r="T1" s="97"/>
+      <c r="U1" s="97"/>
+      <c r="V1" s="97"/>
+      <c r="W1" s="97"/>
+      <c r="X1" s="97"/>
+      <c r="Y1" s="97"/>
+      <c r="Z1" s="97"/>
+      <c r="AA1" s="97"/>
+      <c r="AB1" s="97"/>
+      <c r="AC1" s="97"/>
+      <c r="AD1" s="97" t="s">
+        <v>0</v>
+      </c>
+      <c r="AE1" s="97"/>
+      <c r="AF1" s="97"/>
+      <c r="AG1" s="97"/>
+      <c r="AH1" s="97"/>
+      <c r="AI1" s="97"/>
+      <c r="AJ1" s="97"/>
+      <c r="AK1" s="97"/>
+      <c r="AL1" s="97"/>
+      <c r="AM1" s="97"/>
+      <c r="AN1" s="97"/>
+      <c r="AO1" s="97"/>
+      <c r="AP1" s="97"/>
+      <c r="AQ1" s="97"/>
+      <c r="AR1" s="97"/>
+      <c r="AS1" s="97"/>
+      <c r="AT1" s="97"/>
+      <c r="AU1" s="97"/>
+      <c r="AV1" s="97"/>
+      <c r="AW1" s="97"/>
+      <c r="AX1" s="97"/>
+      <c r="AY1" s="97"/>
+      <c r="AZ1" s="97"/>
+      <c r="BA1" s="97"/>
+      <c r="BB1" s="97"/>
+      <c r="BC1" s="97"/>
+      <c r="BD1" s="97"/>
+      <c r="BE1" s="97"/>
+      <c r="BF1" s="97"/>
     </row>
     <row r="2" spans="1:59" ht="18">
       <c r="A2" s="23" t="s">
@@ -5592,10 +5602,10 @@
       <c r="BF2" s="67"/>
     </row>
     <row r="3" spans="1:59">
-      <c r="A3" s="95" t="s">
+      <c r="A3" s="98" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="95"/>
+      <c r="B3" s="98"/>
       <c r="C3" s="68"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -5635,10 +5645,10 @@
       <c r="AA3" s="6"/>
       <c r="AB3" s="6"/>
       <c r="AC3" s="6"/>
-      <c r="AD3" s="95" t="s">
+      <c r="AD3" s="98" t="s">
         <v>3</v>
       </c>
-      <c r="AE3" s="95"/>
+      <c r="AE3" s="98"/>
       <c r="AF3" s="68"/>
       <c r="AG3" s="3">
         <v>2</v>
@@ -6113,38 +6123,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:33" ht="18">
-      <c r="A1" s="94" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="94"/>
-      <c r="C1" s="94"/>
-      <c r="D1" s="94"/>
-      <c r="E1" s="94"/>
-      <c r="F1" s="94"/>
-      <c r="G1" s="94"/>
-      <c r="H1" s="94"/>
-      <c r="I1" s="94"/>
-      <c r="J1" s="94"/>
-      <c r="K1" s="94"/>
-      <c r="L1" s="94"/>
-      <c r="M1" s="94"/>
-      <c r="N1" s="94"/>
-      <c r="O1" s="94"/>
-      <c r="P1" s="94"/>
-      <c r="Q1" s="94"/>
-      <c r="R1" s="94"/>
-      <c r="S1" s="94"/>
-      <c r="T1" s="94"/>
-      <c r="U1" s="94"/>
-      <c r="V1" s="94"/>
-      <c r="W1" s="94"/>
-      <c r="X1" s="94"/>
-      <c r="Y1" s="94"/>
-      <c r="Z1" s="94"/>
-      <c r="AA1" s="94"/>
-      <c r="AB1" s="94"/>
-      <c r="AC1" s="94"/>
-      <c r="AD1" s="94"/>
+      <c r="A1" s="97" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="97"/>
+      <c r="C1" s="97"/>
+      <c r="D1" s="97"/>
+      <c r="E1" s="97"/>
+      <c r="F1" s="97"/>
+      <c r="G1" s="97"/>
+      <c r="H1" s="97"/>
+      <c r="I1" s="97"/>
+      <c r="J1" s="97"/>
+      <c r="K1" s="97"/>
+      <c r="L1" s="97"/>
+      <c r="M1" s="97"/>
+      <c r="N1" s="97"/>
+      <c r="O1" s="97"/>
+      <c r="P1" s="97"/>
+      <c r="Q1" s="97"/>
+      <c r="R1" s="97"/>
+      <c r="S1" s="97"/>
+      <c r="T1" s="97"/>
+      <c r="U1" s="97"/>
+      <c r="V1" s="97"/>
+      <c r="W1" s="97"/>
+      <c r="X1" s="97"/>
+      <c r="Y1" s="97"/>
+      <c r="Z1" s="97"/>
+      <c r="AA1" s="97"/>
+      <c r="AB1" s="97"/>
+      <c r="AC1" s="97"/>
+      <c r="AD1" s="97"/>
     </row>
     <row r="2" spans="1:33" ht="18">
       <c r="A2" s="23" t="s">
@@ -6183,10 +6193,10 @@
       <c r="AD2" s="70"/>
     </row>
     <row r="3" spans="1:33" ht="15.75" thickBot="1">
-      <c r="A3" s="95" t="s">
+      <c r="A3" s="98" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="95"/>
+      <c r="B3" s="98"/>
       <c r="C3" s="71"/>
       <c r="D3" s="3">
         <v>3</v>
@@ -7036,68 +7046,68 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:58" ht="18">
-      <c r="A1" s="94" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="94"/>
-      <c r="C1" s="94"/>
-      <c r="D1" s="94"/>
-      <c r="E1" s="94"/>
-      <c r="F1" s="94"/>
-      <c r="G1" s="94"/>
-      <c r="H1" s="94"/>
-      <c r="I1" s="94"/>
-      <c r="J1" s="94"/>
-      <c r="K1" s="94"/>
-      <c r="L1" s="94"/>
-      <c r="M1" s="94"/>
-      <c r="N1" s="94"/>
-      <c r="O1" s="94"/>
-      <c r="P1" s="94"/>
-      <c r="Q1" s="94"/>
-      <c r="R1" s="94"/>
-      <c r="S1" s="94"/>
-      <c r="T1" s="94"/>
-      <c r="U1" s="94"/>
-      <c r="V1" s="94"/>
-      <c r="W1" s="94"/>
-      <c r="X1" s="94"/>
-      <c r="Y1" s="94"/>
-      <c r="Z1" s="94"/>
-      <c r="AA1" s="94"/>
-      <c r="AB1" s="94"/>
-      <c r="AC1" s="94"/>
-      <c r="AD1" s="94" t="s">
-        <v>0</v>
-      </c>
-      <c r="AE1" s="94"/>
-      <c r="AF1" s="94"/>
-      <c r="AG1" s="94"/>
-      <c r="AH1" s="94"/>
-      <c r="AI1" s="94"/>
-      <c r="AJ1" s="94"/>
-      <c r="AK1" s="94"/>
-      <c r="AL1" s="94"/>
-      <c r="AM1" s="94"/>
-      <c r="AN1" s="94"/>
-      <c r="AO1" s="94"/>
-      <c r="AP1" s="94"/>
-      <c r="AQ1" s="94"/>
-      <c r="AR1" s="94"/>
-      <c r="AS1" s="94"/>
-      <c r="AT1" s="94"/>
-      <c r="AU1" s="94"/>
-      <c r="AV1" s="94"/>
-      <c r="AW1" s="94"/>
-      <c r="AX1" s="94"/>
-      <c r="AY1" s="94"/>
-      <c r="AZ1" s="94"/>
-      <c r="BA1" s="94"/>
-      <c r="BB1" s="94"/>
-      <c r="BC1" s="94"/>
-      <c r="BD1" s="94"/>
-      <c r="BE1" s="94"/>
-      <c r="BF1" s="94"/>
+      <c r="A1" s="97" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="97"/>
+      <c r="C1" s="97"/>
+      <c r="D1" s="97"/>
+      <c r="E1" s="97"/>
+      <c r="F1" s="97"/>
+      <c r="G1" s="97"/>
+      <c r="H1" s="97"/>
+      <c r="I1" s="97"/>
+      <c r="J1" s="97"/>
+      <c r="K1" s="97"/>
+      <c r="L1" s="97"/>
+      <c r="M1" s="97"/>
+      <c r="N1" s="97"/>
+      <c r="O1" s="97"/>
+      <c r="P1" s="97"/>
+      <c r="Q1" s="97"/>
+      <c r="R1" s="97"/>
+      <c r="S1" s="97"/>
+      <c r="T1" s="97"/>
+      <c r="U1" s="97"/>
+      <c r="V1" s="97"/>
+      <c r="W1" s="97"/>
+      <c r="X1" s="97"/>
+      <c r="Y1" s="97"/>
+      <c r="Z1" s="97"/>
+      <c r="AA1" s="97"/>
+      <c r="AB1" s="97"/>
+      <c r="AC1" s="97"/>
+      <c r="AD1" s="97" t="s">
+        <v>0</v>
+      </c>
+      <c r="AE1" s="97"/>
+      <c r="AF1" s="97"/>
+      <c r="AG1" s="97"/>
+      <c r="AH1" s="97"/>
+      <c r="AI1" s="97"/>
+      <c r="AJ1" s="97"/>
+      <c r="AK1" s="97"/>
+      <c r="AL1" s="97"/>
+      <c r="AM1" s="97"/>
+      <c r="AN1" s="97"/>
+      <c r="AO1" s="97"/>
+      <c r="AP1" s="97"/>
+      <c r="AQ1" s="97"/>
+      <c r="AR1" s="97"/>
+      <c r="AS1" s="97"/>
+      <c r="AT1" s="97"/>
+      <c r="AU1" s="97"/>
+      <c r="AV1" s="97"/>
+      <c r="AW1" s="97"/>
+      <c r="AX1" s="97"/>
+      <c r="AY1" s="97"/>
+      <c r="AZ1" s="97"/>
+      <c r="BA1" s="97"/>
+      <c r="BB1" s="97"/>
+      <c r="BC1" s="97"/>
+      <c r="BD1" s="97"/>
+      <c r="BE1" s="97"/>
+      <c r="BF1" s="97"/>
     </row>
     <row r="2" spans="1:58" ht="18">
       <c r="A2" s="23" t="s">
@@ -7168,10 +7178,10 @@
       <c r="BF2" s="36"/>
     </row>
     <row r="3" spans="1:58">
-      <c r="A3" s="95" t="s">
+      <c r="A3" s="98" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="95"/>
+      <c r="B3" s="98"/>
       <c r="C3" s="29"/>
       <c r="D3" s="3">
         <v>2</v>
@@ -7211,10 +7221,10 @@
       <c r="AA3" s="6"/>
       <c r="AB3" s="6"/>
       <c r="AC3" s="6"/>
-      <c r="AD3" s="95" t="s">
+      <c r="AD3" s="98" t="s">
         <v>3</v>
       </c>
-      <c r="AE3" s="95"/>
+      <c r="AE3" s="98"/>
       <c r="AF3" s="37"/>
       <c r="AG3" s="3">
         <v>2</v>
@@ -7690,37 +7700,37 @@
       <c r="A1" s="84" t="s">
         <v>112</v>
       </c>
-      <c r="B1" s="94" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="94"/>
-      <c r="D1" s="94"/>
-      <c r="E1" s="94"/>
-      <c r="F1" s="94"/>
-      <c r="G1" s="94"/>
-      <c r="H1" s="94"/>
-      <c r="I1" s="94"/>
-      <c r="J1" s="94"/>
-      <c r="K1" s="94"/>
-      <c r="L1" s="94"/>
-      <c r="M1" s="94"/>
-      <c r="N1" s="94"/>
-      <c r="O1" s="94"/>
-      <c r="P1" s="94"/>
-      <c r="Q1" s="94"/>
-      <c r="R1" s="94"/>
-      <c r="S1" s="94"/>
-      <c r="T1" s="94"/>
-      <c r="U1" s="94"/>
-      <c r="V1" s="94"/>
-      <c r="W1" s="94"/>
-      <c r="X1" s="94"/>
-      <c r="Y1" s="94"/>
-      <c r="Z1" s="94"/>
-      <c r="AA1" s="94"/>
-      <c r="AB1" s="94"/>
-      <c r="AC1" s="94"/>
-      <c r="AD1" s="94"/>
+      <c r="B1" s="97" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="97"/>
+      <c r="D1" s="97"/>
+      <c r="E1" s="97"/>
+      <c r="F1" s="97"/>
+      <c r="G1" s="97"/>
+      <c r="H1" s="97"/>
+      <c r="I1" s="97"/>
+      <c r="J1" s="97"/>
+      <c r="K1" s="97"/>
+      <c r="L1" s="97"/>
+      <c r="M1" s="97"/>
+      <c r="N1" s="97"/>
+      <c r="O1" s="97"/>
+      <c r="P1" s="97"/>
+      <c r="Q1" s="97"/>
+      <c r="R1" s="97"/>
+      <c r="S1" s="97"/>
+      <c r="T1" s="97"/>
+      <c r="U1" s="97"/>
+      <c r="V1" s="97"/>
+      <c r="W1" s="97"/>
+      <c r="X1" s="97"/>
+      <c r="Y1" s="97"/>
+      <c r="Z1" s="97"/>
+      <c r="AA1" s="97"/>
+      <c r="AB1" s="97"/>
+      <c r="AC1" s="97"/>
+      <c r="AD1" s="97"/>
     </row>
     <row r="2" spans="1:33" ht="18">
       <c r="A2" s="85"/>
@@ -7760,10 +7770,10 @@
     </row>
     <row r="3" spans="1:33" ht="15.75" thickBot="1">
       <c r="A3" s="85"/>
-      <c r="B3" s="95" t="s">
+      <c r="B3" s="98" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="95"/>
+      <c r="C3" s="98"/>
       <c r="D3" s="3">
         <v>2</v>
       </c>
@@ -7986,7 +7996,7 @@
         <f>IF($D$3=1,ROUND(((V5*X5)/2),2),0)</f>
         <v>0</v>
       </c>
-      <c r="AA5" s="24">
+      <c r="AA5" s="92">
         <f>IF($D$3=2,ROUND(((V5*X5)),2),0)</f>
         <v>90.09</v>
       </c>
@@ -9074,36 +9084,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:31" ht="18">
-      <c r="A1" s="94" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="94"/>
-      <c r="C1" s="94"/>
-      <c r="D1" s="94"/>
-      <c r="E1" s="94"/>
-      <c r="F1" s="94"/>
-      <c r="G1" s="94"/>
-      <c r="H1" s="94"/>
-      <c r="I1" s="94"/>
-      <c r="J1" s="94"/>
-      <c r="K1" s="94"/>
-      <c r="L1" s="94"/>
-      <c r="M1" s="94"/>
-      <c r="N1" s="94"/>
-      <c r="O1" s="94"/>
-      <c r="P1" s="94"/>
-      <c r="Q1" s="94"/>
-      <c r="R1" s="94"/>
-      <c r="S1" s="94"/>
-      <c r="T1" s="94"/>
-      <c r="U1" s="94"/>
-      <c r="V1" s="94"/>
-      <c r="W1" s="94"/>
-      <c r="X1" s="94"/>
-      <c r="Y1" s="94"/>
-      <c r="Z1" s="94"/>
-      <c r="AA1" s="94"/>
-      <c r="AB1" s="94"/>
+      <c r="A1" s="97" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="97"/>
+      <c r="C1" s="97"/>
+      <c r="D1" s="97"/>
+      <c r="E1" s="97"/>
+      <c r="F1" s="97"/>
+      <c r="G1" s="97"/>
+      <c r="H1" s="97"/>
+      <c r="I1" s="97"/>
+      <c r="J1" s="97"/>
+      <c r="K1" s="97"/>
+      <c r="L1" s="97"/>
+      <c r="M1" s="97"/>
+      <c r="N1" s="97"/>
+      <c r="O1" s="97"/>
+      <c r="P1" s="97"/>
+      <c r="Q1" s="97"/>
+      <c r="R1" s="97"/>
+      <c r="S1" s="97"/>
+      <c r="T1" s="97"/>
+      <c r="U1" s="97"/>
+      <c r="V1" s="97"/>
+      <c r="W1" s="97"/>
+      <c r="X1" s="97"/>
+      <c r="Y1" s="97"/>
+      <c r="Z1" s="97"/>
+      <c r="AA1" s="97"/>
+      <c r="AB1" s="97"/>
     </row>
     <row r="2" spans="1:31" ht="18">
       <c r="A2" s="23" t="s">
@@ -9140,10 +9150,10 @@
       <c r="AB2" s="80"/>
     </row>
     <row r="3" spans="1:31" ht="15.75" thickBot="1">
-      <c r="A3" s="95" t="s">
+      <c r="A3" s="98" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="95"/>
+      <c r="B3" s="98"/>
       <c r="C3" s="81"/>
       <c r="D3" s="3">
         <v>2</v>
@@ -9956,37 +9966,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:32" ht="18">
-      <c r="A1" s="94" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="94"/>
-      <c r="C1" s="94"/>
-      <c r="D1" s="94"/>
-      <c r="E1" s="94"/>
-      <c r="F1" s="94"/>
-      <c r="G1" s="94"/>
-      <c r="H1" s="94"/>
-      <c r="I1" s="94"/>
-      <c r="J1" s="94"/>
-      <c r="K1" s="94"/>
-      <c r="L1" s="94"/>
-      <c r="M1" s="94"/>
-      <c r="N1" s="94"/>
-      <c r="O1" s="94"/>
-      <c r="P1" s="94"/>
-      <c r="Q1" s="94"/>
-      <c r="R1" s="94"/>
-      <c r="S1" s="94"/>
-      <c r="T1" s="94"/>
-      <c r="U1" s="94"/>
-      <c r="V1" s="94"/>
-      <c r="W1" s="94"/>
-      <c r="X1" s="94"/>
-      <c r="Y1" s="94"/>
-      <c r="Z1" s="94"/>
-      <c r="AA1" s="94"/>
-      <c r="AB1" s="94"/>
-      <c r="AC1" s="94"/>
+      <c r="A1" s="97" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="97"/>
+      <c r="C1" s="97"/>
+      <c r="D1" s="97"/>
+      <c r="E1" s="97"/>
+      <c r="F1" s="97"/>
+      <c r="G1" s="97"/>
+      <c r="H1" s="97"/>
+      <c r="I1" s="97"/>
+      <c r="J1" s="97"/>
+      <c r="K1" s="97"/>
+      <c r="L1" s="97"/>
+      <c r="M1" s="97"/>
+      <c r="N1" s="97"/>
+      <c r="O1" s="97"/>
+      <c r="P1" s="97"/>
+      <c r="Q1" s="97"/>
+      <c r="R1" s="97"/>
+      <c r="S1" s="97"/>
+      <c r="T1" s="97"/>
+      <c r="U1" s="97"/>
+      <c r="V1" s="97"/>
+      <c r="W1" s="97"/>
+      <c r="X1" s="97"/>
+      <c r="Y1" s="97"/>
+      <c r="Z1" s="97"/>
+      <c r="AA1" s="97"/>
+      <c r="AB1" s="97"/>
+      <c r="AC1" s="97"/>
     </row>
     <row r="2" spans="1:32" ht="18">
       <c r="A2" s="23" t="s">
@@ -10024,10 +10034,10 @@
       <c r="AC2" s="87"/>
     </row>
     <row r="3" spans="1:32" ht="15.75" thickBot="1">
-      <c r="A3" s="95" t="s">
+      <c r="A3" s="98" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="95"/>
+      <c r="B3" s="98"/>
       <c r="C3" s="3">
         <v>2</v>
       </c>
@@ -10632,68 +10642,68 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:59" ht="18">
-      <c r="B1" s="94" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="94"/>
-      <c r="D1" s="94"/>
-      <c r="E1" s="94"/>
-      <c r="F1" s="94"/>
-      <c r="G1" s="94"/>
-      <c r="H1" s="94"/>
-      <c r="I1" s="94"/>
-      <c r="J1" s="94"/>
-      <c r="K1" s="94"/>
-      <c r="L1" s="94"/>
-      <c r="M1" s="94"/>
-      <c r="N1" s="94"/>
-      <c r="O1" s="94"/>
-      <c r="P1" s="94"/>
-      <c r="Q1" s="94"/>
-      <c r="R1" s="94"/>
-      <c r="S1" s="94"/>
-      <c r="T1" s="94"/>
-      <c r="U1" s="94"/>
-      <c r="V1" s="94"/>
-      <c r="W1" s="94"/>
-      <c r="X1" s="94"/>
-      <c r="Y1" s="94"/>
-      <c r="Z1" s="94"/>
-      <c r="AA1" s="94"/>
-      <c r="AB1" s="94"/>
-      <c r="AC1" s="94"/>
-      <c r="AD1" s="94"/>
-      <c r="AE1" s="94" t="s">
-        <v>0</v>
-      </c>
-      <c r="AF1" s="94"/>
-      <c r="AG1" s="94"/>
-      <c r="AH1" s="94"/>
-      <c r="AI1" s="94"/>
-      <c r="AJ1" s="94"/>
-      <c r="AK1" s="94"/>
-      <c r="AL1" s="94"/>
-      <c r="AM1" s="94"/>
-      <c r="AN1" s="94"/>
-      <c r="AO1" s="94"/>
-      <c r="AP1" s="94"/>
-      <c r="AQ1" s="94"/>
-      <c r="AR1" s="94"/>
-      <c r="AS1" s="94"/>
-      <c r="AT1" s="94"/>
-      <c r="AU1" s="94"/>
-      <c r="AV1" s="94"/>
-      <c r="AW1" s="94"/>
-      <c r="AX1" s="94"/>
-      <c r="AY1" s="94"/>
-      <c r="AZ1" s="94"/>
-      <c r="BA1" s="94"/>
-      <c r="BB1" s="94"/>
-      <c r="BC1" s="94"/>
-      <c r="BD1" s="94"/>
-      <c r="BE1" s="94"/>
-      <c r="BF1" s="94"/>
-      <c r="BG1" s="94"/>
+      <c r="B1" s="97" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="97"/>
+      <c r="D1" s="97"/>
+      <c r="E1" s="97"/>
+      <c r="F1" s="97"/>
+      <c r="G1" s="97"/>
+      <c r="H1" s="97"/>
+      <c r="I1" s="97"/>
+      <c r="J1" s="97"/>
+      <c r="K1" s="97"/>
+      <c r="L1" s="97"/>
+      <c r="M1" s="97"/>
+      <c r="N1" s="97"/>
+      <c r="O1" s="97"/>
+      <c r="P1" s="97"/>
+      <c r="Q1" s="97"/>
+      <c r="R1" s="97"/>
+      <c r="S1" s="97"/>
+      <c r="T1" s="97"/>
+      <c r="U1" s="97"/>
+      <c r="V1" s="97"/>
+      <c r="W1" s="97"/>
+      <c r="X1" s="97"/>
+      <c r="Y1" s="97"/>
+      <c r="Z1" s="97"/>
+      <c r="AA1" s="97"/>
+      <c r="AB1" s="97"/>
+      <c r="AC1" s="97"/>
+      <c r="AD1" s="97"/>
+      <c r="AE1" s="97" t="s">
+        <v>0</v>
+      </c>
+      <c r="AF1" s="97"/>
+      <c r="AG1" s="97"/>
+      <c r="AH1" s="97"/>
+      <c r="AI1" s="97"/>
+      <c r="AJ1" s="97"/>
+      <c r="AK1" s="97"/>
+      <c r="AL1" s="97"/>
+      <c r="AM1" s="97"/>
+      <c r="AN1" s="97"/>
+      <c r="AO1" s="97"/>
+      <c r="AP1" s="97"/>
+      <c r="AQ1" s="97"/>
+      <c r="AR1" s="97"/>
+      <c r="AS1" s="97"/>
+      <c r="AT1" s="97"/>
+      <c r="AU1" s="97"/>
+      <c r="AV1" s="97"/>
+      <c r="AW1" s="97"/>
+      <c r="AX1" s="97"/>
+      <c r="AY1" s="97"/>
+      <c r="AZ1" s="97"/>
+      <c r="BA1" s="97"/>
+      <c r="BB1" s="97"/>
+      <c r="BC1" s="97"/>
+      <c r="BD1" s="97"/>
+      <c r="BE1" s="97"/>
+      <c r="BF1" s="97"/>
+      <c r="BG1" s="97"/>
     </row>
     <row r="2" spans="1:59" ht="18">
       <c r="B2" s="23" t="s">
@@ -10764,10 +10774,10 @@
       <c r="BG2" s="88"/>
     </row>
     <row r="3" spans="1:59">
-      <c r="B3" s="95" t="s">
+      <c r="B3" s="98" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="95"/>
+      <c r="C3" s="98"/>
       <c r="D3" s="89"/>
       <c r="E3" s="3">
         <v>2</v>
@@ -10807,10 +10817,10 @@
       <c r="AB3" s="6"/>
       <c r="AC3" s="6"/>
       <c r="AD3" s="6"/>
-      <c r="AE3" s="95" t="s">
+      <c r="AE3" s="98" t="s">
         <v>3</v>
       </c>
-      <c r="AF3" s="95"/>
+      <c r="AF3" s="98"/>
       <c r="AG3" s="89"/>
       <c r="AH3" s="3">
         <v>2</v>
@@ -11290,37 +11300,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:32" ht="18">
-      <c r="B1" s="94" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="94"/>
-      <c r="D1" s="94"/>
-      <c r="E1" s="94"/>
-      <c r="F1" s="94"/>
-      <c r="G1" s="94"/>
-      <c r="H1" s="94"/>
-      <c r="I1" s="94"/>
-      <c r="J1" s="94"/>
-      <c r="K1" s="94"/>
-      <c r="L1" s="94"/>
-      <c r="M1" s="94"/>
-      <c r="N1" s="94"/>
-      <c r="O1" s="94"/>
-      <c r="P1" s="94"/>
-      <c r="Q1" s="94"/>
-      <c r="R1" s="94"/>
-      <c r="S1" s="94"/>
-      <c r="T1" s="94"/>
-      <c r="U1" s="94"/>
-      <c r="V1" s="94"/>
-      <c r="W1" s="94"/>
-      <c r="X1" s="94"/>
-      <c r="Y1" s="94"/>
-      <c r="Z1" s="94"/>
-      <c r="AA1" s="94"/>
-      <c r="AB1" s="94"/>
-      <c r="AC1" s="94"/>
-      <c r="AD1" s="94"/>
+      <c r="B1" s="97" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="97"/>
+      <c r="D1" s="97"/>
+      <c r="E1" s="97"/>
+      <c r="F1" s="97"/>
+      <c r="G1" s="97"/>
+      <c r="H1" s="97"/>
+      <c r="I1" s="97"/>
+      <c r="J1" s="97"/>
+      <c r="K1" s="97"/>
+      <c r="L1" s="97"/>
+      <c r="M1" s="97"/>
+      <c r="N1" s="97"/>
+      <c r="O1" s="97"/>
+      <c r="P1" s="97"/>
+      <c r="Q1" s="97"/>
+      <c r="R1" s="97"/>
+      <c r="S1" s="97"/>
+      <c r="T1" s="97"/>
+      <c r="U1" s="97"/>
+      <c r="V1" s="97"/>
+      <c r="W1" s="97"/>
+      <c r="X1" s="97"/>
+      <c r="Y1" s="97"/>
+      <c r="Z1" s="97"/>
+      <c r="AA1" s="97"/>
+      <c r="AB1" s="97"/>
+      <c r="AC1" s="97"/>
+      <c r="AD1" s="97"/>
     </row>
     <row r="2" spans="1:32" ht="16.5" customHeight="1">
       <c r="B2" s="23" t="s">
@@ -11358,10 +11368,10 @@
       <c r="AD2" s="90"/>
     </row>
     <row r="3" spans="1:32">
-      <c r="B3" s="95" t="s">
+      <c r="B3" s="98" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="95"/>
+      <c r="C3" s="98"/>
       <c r="E3">
         <v>2</v>
       </c>
@@ -11866,37 +11876,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:33" ht="18">
-      <c r="B1" s="94" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="94"/>
-      <c r="D1" s="94"/>
-      <c r="E1" s="94"/>
-      <c r="F1" s="94"/>
-      <c r="G1" s="94"/>
-      <c r="H1" s="94"/>
-      <c r="I1" s="94"/>
-      <c r="J1" s="94"/>
-      <c r="K1" s="94"/>
-      <c r="L1" s="94"/>
-      <c r="M1" s="94"/>
-      <c r="N1" s="94"/>
-      <c r="O1" s="94"/>
-      <c r="P1" s="94"/>
-      <c r="Q1" s="94"/>
-      <c r="R1" s="94"/>
-      <c r="S1" s="94"/>
-      <c r="T1" s="94"/>
-      <c r="U1" s="94"/>
-      <c r="V1" s="94"/>
-      <c r="W1" s="94"/>
-      <c r="X1" s="94"/>
-      <c r="Y1" s="94"/>
-      <c r="Z1" s="94"/>
-      <c r="AA1" s="94"/>
-      <c r="AB1" s="94"/>
-      <c r="AC1" s="94"/>
-      <c r="AD1" s="94"/>
+      <c r="B1" s="97" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="97"/>
+      <c r="D1" s="97"/>
+      <c r="E1" s="97"/>
+      <c r="F1" s="97"/>
+      <c r="G1" s="97"/>
+      <c r="H1" s="97"/>
+      <c r="I1" s="97"/>
+      <c r="J1" s="97"/>
+      <c r="K1" s="97"/>
+      <c r="L1" s="97"/>
+      <c r="M1" s="97"/>
+      <c r="N1" s="97"/>
+      <c r="O1" s="97"/>
+      <c r="P1" s="97"/>
+      <c r="Q1" s="97"/>
+      <c r="R1" s="97"/>
+      <c r="S1" s="97"/>
+      <c r="T1" s="97"/>
+      <c r="U1" s="97"/>
+      <c r="V1" s="97"/>
+      <c r="W1" s="97"/>
+      <c r="X1" s="97"/>
+      <c r="Y1" s="97"/>
+      <c r="Z1" s="97"/>
+      <c r="AA1" s="97"/>
+      <c r="AB1" s="97"/>
+      <c r="AC1" s="97"/>
+      <c r="AD1" s="97"/>
     </row>
     <row r="2" spans="1:33" ht="18">
       <c r="B2" s="23" t="s">
@@ -11934,10 +11944,10 @@
       <c r="AD2" s="91"/>
     </row>
     <row r="3" spans="1:33" ht="15.75" thickBot="1">
-      <c r="B3" s="95" t="s">
+      <c r="B3" s="98" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="95"/>
+      <c r="C3" s="98"/>
       <c r="D3" s="3">
         <v>2</v>
       </c>
@@ -12543,37 +12553,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="18">
-      <c r="A1" s="94" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="94"/>
-      <c r="C1" s="94"/>
-      <c r="D1" s="94"/>
-      <c r="E1" s="94"/>
-      <c r="F1" s="94"/>
-      <c r="G1" s="94"/>
-      <c r="H1" s="94"/>
-      <c r="I1" s="94"/>
-      <c r="J1" s="94"/>
-      <c r="K1" s="94"/>
-      <c r="L1" s="94"/>
-      <c r="M1" s="94"/>
-      <c r="N1" s="94"/>
-      <c r="O1" s="94"/>
-      <c r="P1" s="94"/>
-      <c r="Q1" s="94"/>
-      <c r="R1" s="94"/>
-      <c r="S1" s="94"/>
-      <c r="T1" s="94"/>
-      <c r="U1" s="94"/>
-      <c r="V1" s="94"/>
-      <c r="W1" s="94"/>
-      <c r="X1" s="94"/>
-      <c r="Y1" s="94"/>
-      <c r="Z1" s="94"/>
-      <c r="AA1" s="94"/>
-      <c r="AB1" s="94"/>
-      <c r="AC1" s="94"/>
+      <c r="A1" s="97" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="97"/>
+      <c r="C1" s="97"/>
+      <c r="D1" s="97"/>
+      <c r="E1" s="97"/>
+      <c r="F1" s="97"/>
+      <c r="G1" s="97"/>
+      <c r="H1" s="97"/>
+      <c r="I1" s="97"/>
+      <c r="J1" s="97"/>
+      <c r="K1" s="97"/>
+      <c r="L1" s="97"/>
+      <c r="M1" s="97"/>
+      <c r="N1" s="97"/>
+      <c r="O1" s="97"/>
+      <c r="P1" s="97"/>
+      <c r="Q1" s="97"/>
+      <c r="R1" s="97"/>
+      <c r="S1" s="97"/>
+      <c r="T1" s="97"/>
+      <c r="U1" s="97"/>
+      <c r="V1" s="97"/>
+      <c r="W1" s="97"/>
+      <c r="X1" s="97"/>
+      <c r="Y1" s="97"/>
+      <c r="Z1" s="97"/>
+      <c r="AA1" s="97"/>
+      <c r="AB1" s="97"/>
+      <c r="AC1" s="97"/>
     </row>
     <row r="2" spans="1:29" ht="18">
       <c r="A2" s="23" t="s">
@@ -12611,10 +12621,10 @@
       <c r="AC2" s="28"/>
     </row>
     <row r="3" spans="1:29">
-      <c r="A3" s="95" t="s">
+      <c r="A3" s="98" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="95"/>
+      <c r="B3" s="98"/>
       <c r="C3" s="29"/>
       <c r="D3" s="3">
         <v>4</v>
@@ -12876,6 +12886,1142 @@
 
 <file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:AE8"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="2" max="2" width="20.5703125" customWidth="1"/>
+    <col min="3" max="3" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="29.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.28515625" customWidth="1"/>
+    <col min="6" max="6" width="16.28515625" customWidth="1"/>
+    <col min="7" max="7" width="24.42578125" customWidth="1"/>
+    <col min="8" max="8" width="20.28515625" customWidth="1"/>
+    <col min="9" max="9" width="20" customWidth="1"/>
+    <col min="13" max="13" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="13.7109375" customWidth="1"/>
+    <col min="18" max="18" width="13" customWidth="1"/>
+    <col min="19" max="19" width="14.42578125" customWidth="1"/>
+    <col min="20" max="20" width="18.42578125" customWidth="1"/>
+    <col min="21" max="21" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:31" ht="18">
+      <c r="A1" s="97" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="97"/>
+      <c r="C1" s="97"/>
+      <c r="D1" s="97"/>
+      <c r="E1" s="97"/>
+      <c r="F1" s="97"/>
+      <c r="G1" s="97"/>
+      <c r="H1" s="97"/>
+      <c r="I1" s="97"/>
+      <c r="J1" s="97"/>
+      <c r="K1" s="97"/>
+      <c r="L1" s="97"/>
+      <c r="M1" s="97"/>
+      <c r="N1" s="97"/>
+      <c r="O1" s="97"/>
+      <c r="P1" s="97"/>
+      <c r="Q1" s="97"/>
+      <c r="R1" s="97"/>
+      <c r="S1" s="97"/>
+      <c r="T1" s="97"/>
+      <c r="U1" s="97"/>
+      <c r="V1" s="97"/>
+      <c r="W1" s="97"/>
+      <c r="X1" s="97"/>
+      <c r="Y1" s="97"/>
+      <c r="Z1" s="97"/>
+      <c r="AA1" s="97"/>
+      <c r="AB1" s="97"/>
+      <c r="AC1" s="97"/>
+    </row>
+    <row r="2" spans="1:31" ht="16.5" customHeight="1">
+      <c r="A2" s="23" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="23" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" s="94"/>
+      <c r="D2" s="94"/>
+      <c r="E2" s="94"/>
+      <c r="F2" s="94"/>
+      <c r="G2" s="94"/>
+      <c r="H2" s="94"/>
+      <c r="I2" s="94"/>
+      <c r="J2" s="94"/>
+      <c r="K2" s="94"/>
+      <c r="L2" s="94"/>
+      <c r="M2" s="94"/>
+      <c r="N2" s="94"/>
+      <c r="O2" s="94"/>
+      <c r="P2" s="94"/>
+      <c r="Q2" s="94"/>
+      <c r="R2" s="94"/>
+      <c r="S2" s="94"/>
+      <c r="T2" s="94"/>
+      <c r="U2" s="94"/>
+      <c r="V2" s="94"/>
+      <c r="W2" s="94"/>
+      <c r="X2" s="94"/>
+      <c r="Y2" s="94"/>
+      <c r="Z2" s="94"/>
+      <c r="AA2" s="94"/>
+      <c r="AB2" s="94"/>
+      <c r="AC2" s="94"/>
+    </row>
+    <row r="3" spans="1:31">
+      <c r="A3" s="98" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="98"/>
+      <c r="D3">
+        <v>2</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="F3" s="5"/>
+      <c r="G3" s="5"/>
+      <c r="H3" s="5"/>
+      <c r="I3" s="6"/>
+      <c r="J3" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="K3" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="L3" s="7"/>
+      <c r="M3" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="N3" s="7">
+        <v>1</v>
+      </c>
+      <c r="O3" s="7"/>
+      <c r="P3" s="7"/>
+      <c r="Q3" s="7"/>
+      <c r="R3" s="7"/>
+      <c r="S3" s="6"/>
+      <c r="T3" s="6"/>
+      <c r="U3" s="6"/>
+      <c r="V3" s="6"/>
+      <c r="W3" s="6"/>
+      <c r="X3" s="6"/>
+      <c r="Y3" s="6"/>
+      <c r="Z3" s="6"/>
+      <c r="AA3" s="6"/>
+      <c r="AB3" s="6"/>
+      <c r="AC3" s="6"/>
+    </row>
+    <row r="4" spans="1:31" ht="42.75">
+      <c r="A4" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="E4" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="F4" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="G4" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="H4" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="I4" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="J4" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="K4" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="L4" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="M4" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="N4" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="O4" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="P4" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q4" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="R4" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="S4" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="T4" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="U4" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="V4" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="W4" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="X4" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y4" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="Z4" s="16" t="s">
+        <v>30</v>
+      </c>
+      <c r="AA4" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="AB4" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="AC4" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="AD4" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="AE4" s="10" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="5" spans="1:31">
+      <c r="A5" s="9">
+        <v>1</v>
+      </c>
+      <c r="B5" s="27" t="s">
+        <v>44</v>
+      </c>
+      <c r="C5" s="9">
+        <v>0</v>
+      </c>
+      <c r="D5" s="27" t="s">
+        <v>44</v>
+      </c>
+      <c r="E5" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="F5" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="G5" s="24">
+        <v>2</v>
+      </c>
+      <c r="H5" s="9">
+        <v>250.25</v>
+      </c>
+      <c r="I5" s="8">
+        <v>500.5</v>
+      </c>
+      <c r="J5" s="25">
+        <v>0</v>
+      </c>
+      <c r="K5" s="25">
+        <v>0</v>
+      </c>
+      <c r="L5" s="25">
+        <v>0</v>
+      </c>
+      <c r="M5" s="8">
+        <v>500.5</v>
+      </c>
+      <c r="N5" s="8">
+        <f>ROUND(J5*M5%,2)</f>
+        <v>0</v>
+      </c>
+      <c r="O5" s="8">
+        <f>I5-N5</f>
+        <v>500.5</v>
+      </c>
+      <c r="P5" s="8">
+        <f>ROUND(K5*O5%,2)</f>
+        <v>0</v>
+      </c>
+      <c r="Q5" s="8">
+        <f>O5-P5</f>
+        <v>500.5</v>
+      </c>
+      <c r="R5" s="8">
+        <f>ROUND(L5*Q5%,2)</f>
+        <v>0</v>
+      </c>
+      <c r="S5" s="26">
+        <f>N5+P5+R5</f>
+        <v>0</v>
+      </c>
+      <c r="T5" s="26">
+        <v>0</v>
+      </c>
+      <c r="U5" s="8">
+        <f>(I5-S5)</f>
+        <v>500.5</v>
+      </c>
+      <c r="V5" s="24">
+        <v>88363222</v>
+      </c>
+      <c r="W5" s="18">
+        <v>0.18</v>
+      </c>
+      <c r="X5" s="24">
+        <f>IF($D$3=1,ROUND(((U5*W5)/2),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="Y5" s="24">
+        <f>IF($D$3=1,ROUND(((U5*W5)/2),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="Z5" s="92">
+        <f>IF($D$3=2,ROUND(((U5*W5)),2),0)</f>
+        <v>90.09</v>
+      </c>
+      <c r="AA5" s="24">
+        <v>0</v>
+      </c>
+      <c r="AB5" s="24">
+        <f>X5+Y5+Z5</f>
+        <v>90.09</v>
+      </c>
+      <c r="AC5" s="24">
+        <f>U5+AB5</f>
+        <v>590.59</v>
+      </c>
+      <c r="AD5" s="46" t="s">
+        <v>42</v>
+      </c>
+      <c r="AE5" s="46" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="6" spans="1:31" ht="16.5" customHeight="1">
+      <c r="A6" s="9">
+        <v>2</v>
+      </c>
+      <c r="B6" s="45" t="s">
+        <v>51</v>
+      </c>
+      <c r="C6" s="9">
+        <v>0</v>
+      </c>
+      <c r="D6" s="45" t="s">
+        <v>50</v>
+      </c>
+      <c r="E6" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="F6" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="G6" s="24">
+        <v>1</v>
+      </c>
+      <c r="H6" s="9">
+        <v>3458</v>
+      </c>
+      <c r="I6" s="8">
+        <v>3458</v>
+      </c>
+      <c r="J6" s="25">
+        <v>0</v>
+      </c>
+      <c r="K6" s="25">
+        <v>0</v>
+      </c>
+      <c r="L6" s="25">
+        <v>0</v>
+      </c>
+      <c r="M6" s="8">
+        <v>3458</v>
+      </c>
+      <c r="N6" s="8">
+        <f t="shared" ref="N6:N7" si="0">ROUND(J6*M6%,2)</f>
+        <v>0</v>
+      </c>
+      <c r="O6" s="8">
+        <f t="shared" ref="O6:O7" si="1">I6-N6</f>
+        <v>3458</v>
+      </c>
+      <c r="P6" s="8">
+        <f t="shared" ref="P6:P7" si="2">ROUND(K6*O6%,2)</f>
+        <v>0</v>
+      </c>
+      <c r="Q6" s="8">
+        <f t="shared" ref="Q6:Q7" si="3">O6-P6</f>
+        <v>3458</v>
+      </c>
+      <c r="R6" s="8">
+        <f t="shared" ref="R6:R7" si="4">ROUND(L6*Q6%,2)</f>
+        <v>0</v>
+      </c>
+      <c r="S6" s="26">
+        <f t="shared" ref="S6:S7" si="5">N6+P6+R6</f>
+        <v>0</v>
+      </c>
+      <c r="T6" s="26">
+        <v>0</v>
+      </c>
+      <c r="U6" s="8">
+        <f>(I6-S6)</f>
+        <v>3458</v>
+      </c>
+      <c r="V6" s="24">
+        <v>88363222</v>
+      </c>
+      <c r="W6" s="18">
+        <v>0.18</v>
+      </c>
+      <c r="X6" s="24">
+        <f>IF($D$3=1,ROUND(((U6*W6)/2),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="Y6" s="24">
+        <f>IF($D$3=1,ROUND(((U6*W6)/2),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="Z6" s="92">
+        <f t="shared" ref="Z6:Z7" si="6">IF($D$3=2,ROUND(((U6*W6)),2),0)</f>
+        <v>622.44000000000005</v>
+      </c>
+      <c r="AA6" s="24">
+        <v>0</v>
+      </c>
+      <c r="AB6" s="24">
+        <f>X6+Y6+Z6</f>
+        <v>622.44000000000005</v>
+      </c>
+      <c r="AC6" s="24">
+        <f>U6+AB6</f>
+        <v>4080.44</v>
+      </c>
+      <c r="AD6" s="46" t="s">
+        <v>53</v>
+      </c>
+      <c r="AE6" s="46" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="7" spans="1:31">
+      <c r="A7" s="9">
+        <v>3</v>
+      </c>
+      <c r="B7" s="27" t="s">
+        <v>52</v>
+      </c>
+      <c r="C7" s="9">
+        <v>0</v>
+      </c>
+      <c r="D7" s="27" t="s">
+        <v>52</v>
+      </c>
+      <c r="E7" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="F7" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="G7" s="24">
+        <v>3</v>
+      </c>
+      <c r="H7" s="9">
+        <v>675</v>
+      </c>
+      <c r="I7" s="8">
+        <v>2025</v>
+      </c>
+      <c r="J7" s="25">
+        <v>0</v>
+      </c>
+      <c r="K7" s="25">
+        <v>0</v>
+      </c>
+      <c r="L7" s="25">
+        <v>0</v>
+      </c>
+      <c r="M7" s="8">
+        <v>2025</v>
+      </c>
+      <c r="N7" s="8">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="O7" s="8">
+        <f t="shared" si="1"/>
+        <v>2025</v>
+      </c>
+      <c r="P7" s="8">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="Q7" s="8">
+        <f t="shared" si="3"/>
+        <v>2025</v>
+      </c>
+      <c r="R7" s="8">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="S7" s="26">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="T7" s="26">
+        <v>0</v>
+      </c>
+      <c r="U7" s="8">
+        <f>(I7-S7)</f>
+        <v>2025</v>
+      </c>
+      <c r="V7" s="24">
+        <v>88363222</v>
+      </c>
+      <c r="W7" s="18">
+        <v>0.18</v>
+      </c>
+      <c r="X7" s="24">
+        <f>IF($D$3=1,ROUND(((U7*W7)/2),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="Y7" s="24">
+        <f>IF($D$3=1,ROUND(((U7*W7)/2),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="Z7" s="92">
+        <f t="shared" si="6"/>
+        <v>364.5</v>
+      </c>
+      <c r="AA7" s="24">
+        <v>0</v>
+      </c>
+      <c r="AB7" s="24">
+        <f>X7+Y7+Z7</f>
+        <v>364.5</v>
+      </c>
+      <c r="AC7" s="24">
+        <f>U7+AB7</f>
+        <v>2389.5</v>
+      </c>
+      <c r="AD7" s="46" t="s">
+        <v>54</v>
+      </c>
+      <c r="AE7" s="46" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="8" spans="1:31">
+      <c r="AE8" s="46"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:AC1"/>
+    <mergeCell ref="A3:B3"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:AF8"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="3" max="3" width="20.5703125" customWidth="1"/>
+    <col min="4" max="4" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="29.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.28515625" customWidth="1"/>
+    <col min="7" max="7" width="16.28515625" customWidth="1"/>
+    <col min="8" max="8" width="24.42578125" customWidth="1"/>
+    <col min="9" max="9" width="20.28515625" customWidth="1"/>
+    <col min="10" max="10" width="20" customWidth="1"/>
+    <col min="14" max="14" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="13.7109375" customWidth="1"/>
+    <col min="19" max="19" width="13" customWidth="1"/>
+    <col min="20" max="20" width="14.42578125" customWidth="1"/>
+    <col min="21" max="21" width="18.42578125" customWidth="1"/>
+    <col min="22" max="22" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="11.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:32" ht="18">
+      <c r="B1" s="97" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="97"/>
+      <c r="D1" s="97"/>
+      <c r="E1" s="97"/>
+      <c r="F1" s="97"/>
+      <c r="G1" s="97"/>
+      <c r="H1" s="97"/>
+      <c r="I1" s="97"/>
+      <c r="J1" s="97"/>
+      <c r="K1" s="97"/>
+      <c r="L1" s="97"/>
+      <c r="M1" s="97"/>
+      <c r="N1" s="97"/>
+      <c r="O1" s="97"/>
+      <c r="P1" s="97"/>
+      <c r="Q1" s="97"/>
+      <c r="R1" s="97"/>
+      <c r="S1" s="97"/>
+      <c r="T1" s="97"/>
+      <c r="U1" s="97"/>
+      <c r="V1" s="97"/>
+      <c r="W1" s="97"/>
+      <c r="X1" s="97"/>
+      <c r="Y1" s="97"/>
+      <c r="Z1" s="97"/>
+      <c r="AA1" s="97"/>
+      <c r="AB1" s="97"/>
+      <c r="AC1" s="97"/>
+      <c r="AD1" s="97"/>
+    </row>
+    <row r="2" spans="1:32" ht="16.5" customHeight="1">
+      <c r="B2" s="23" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="23" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" s="95"/>
+      <c r="E2" s="95"/>
+      <c r="F2" s="95"/>
+      <c r="G2" s="95"/>
+      <c r="H2" s="95"/>
+      <c r="I2" s="95"/>
+      <c r="J2" s="95"/>
+      <c r="K2" s="95"/>
+      <c r="L2" s="95"/>
+      <c r="M2" s="95"/>
+      <c r="N2" s="95"/>
+      <c r="O2" s="95"/>
+      <c r="P2" s="95"/>
+      <c r="Q2" s="95"/>
+      <c r="R2" s="95"/>
+      <c r="S2" s="95"/>
+      <c r="T2" s="95"/>
+      <c r="U2" s="95"/>
+      <c r="V2" s="95"/>
+      <c r="W2" s="95"/>
+      <c r="X2" s="95"/>
+      <c r="Y2" s="95"/>
+      <c r="Z2" s="95"/>
+      <c r="AA2" s="95"/>
+      <c r="AB2" s="95"/>
+      <c r="AC2" s="95"/>
+      <c r="AD2" s="95"/>
+    </row>
+    <row r="3" spans="1:32">
+      <c r="B3" s="98" t="s">
+        <v>3</v>
+      </c>
+      <c r="C3" s="98"/>
+      <c r="E3">
+        <v>2</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="G3" s="5"/>
+      <c r="H3" s="5"/>
+      <c r="I3" s="5"/>
+      <c r="J3" s="6"/>
+      <c r="K3" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="L3" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="M3" s="7"/>
+      <c r="N3" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="O3" s="7">
+        <v>1</v>
+      </c>
+      <c r="P3" s="7"/>
+      <c r="Q3" s="7"/>
+      <c r="R3" s="7"/>
+      <c r="S3" s="7"/>
+      <c r="T3" s="6"/>
+      <c r="U3" s="6"/>
+      <c r="V3" s="6"/>
+      <c r="W3" s="6"/>
+      <c r="X3" s="6"/>
+      <c r="Y3" s="6"/>
+      <c r="Z3" s="6"/>
+      <c r="AA3" s="6"/>
+      <c r="AB3" s="6"/>
+      <c r="AC3" s="6"/>
+      <c r="AD3" s="6"/>
+    </row>
+    <row r="4" spans="1:32" ht="42.75">
+      <c r="A4" s="10" t="s">
+        <v>113</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="D4" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="E4" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="F4" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="G4" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="H4" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="I4" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="J4" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="K4" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="L4" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="M4" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="N4" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="O4" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="P4" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="Q4" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="R4" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="S4" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="T4" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="U4" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="V4" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="W4" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="X4" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y4" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z4" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="AA4" s="16" t="s">
+        <v>30</v>
+      </c>
+      <c r="AB4" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="AC4" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="AD4" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="AE4" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="AF4" s="10" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="5" spans="1:32">
+      <c r="A5" s="46"/>
+      <c r="B5" s="9">
+        <v>1</v>
+      </c>
+      <c r="C5" s="27" t="s">
+        <v>44</v>
+      </c>
+      <c r="D5" s="9">
+        <v>0</v>
+      </c>
+      <c r="E5" s="27" t="s">
+        <v>44</v>
+      </c>
+      <c r="F5" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="G5" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="H5" s="24">
+        <v>2</v>
+      </c>
+      <c r="I5" s="9">
+        <v>250.25</v>
+      </c>
+      <c r="J5" s="8">
+        <v>500.5</v>
+      </c>
+      <c r="K5" s="25">
+        <v>0</v>
+      </c>
+      <c r="L5" s="25">
+        <v>0</v>
+      </c>
+      <c r="M5" s="25">
+        <v>0</v>
+      </c>
+      <c r="N5" s="8">
+        <v>500.5</v>
+      </c>
+      <c r="O5" s="8">
+        <f>ROUND(K5*N5%,2)</f>
+        <v>0</v>
+      </c>
+      <c r="P5" s="8">
+        <f>J5-O5</f>
+        <v>500.5</v>
+      </c>
+      <c r="Q5" s="8">
+        <f>ROUND(L5*P5%,2)</f>
+        <v>0</v>
+      </c>
+      <c r="R5" s="8">
+        <f>P5-Q5</f>
+        <v>500.5</v>
+      </c>
+      <c r="S5" s="8">
+        <f>ROUND(M5*R5%,2)</f>
+        <v>0</v>
+      </c>
+      <c r="T5" s="26">
+        <f>O5+Q5+S5</f>
+        <v>0</v>
+      </c>
+      <c r="U5" s="26">
+        <v>0</v>
+      </c>
+      <c r="V5" s="8">
+        <f>(J5-T5)</f>
+        <v>500.5</v>
+      </c>
+      <c r="W5" s="24">
+        <v>88363222</v>
+      </c>
+      <c r="X5" s="18">
+        <v>0.18</v>
+      </c>
+      <c r="Y5" s="24">
+        <f>IF($E$3=1,ROUND(((V5*X5)/2),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="Z5" s="24">
+        <f>IF($E$3=1,ROUND(((V5*X5)/2),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="AA5" s="42">
+        <f>IF($E$3=2,ROUND(((V5*X5)),2),0)</f>
+        <v>90.09</v>
+      </c>
+      <c r="AB5" s="24">
+        <v>0</v>
+      </c>
+      <c r="AC5" s="24">
+        <f>Y5+Z5+AA5</f>
+        <v>90.09</v>
+      </c>
+      <c r="AD5" s="24">
+        <f>V5+AC5</f>
+        <v>590.59</v>
+      </c>
+      <c r="AE5" s="46" t="s">
+        <v>42</v>
+      </c>
+      <c r="AF5" s="46" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="6" spans="1:32" ht="16.5" customHeight="1">
+      <c r="A6" s="46"/>
+      <c r="B6" s="9">
+        <v>2</v>
+      </c>
+      <c r="C6" s="45" t="s">
+        <v>51</v>
+      </c>
+      <c r="D6" s="9">
+        <v>0</v>
+      </c>
+      <c r="E6" s="45" t="s">
+        <v>50</v>
+      </c>
+      <c r="F6" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="G6" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="H6" s="24">
+        <v>1</v>
+      </c>
+      <c r="I6" s="9">
+        <v>3458</v>
+      </c>
+      <c r="J6" s="8">
+        <v>3458</v>
+      </c>
+      <c r="K6" s="25">
+        <v>0</v>
+      </c>
+      <c r="L6" s="25">
+        <v>0</v>
+      </c>
+      <c r="M6" s="25">
+        <v>0</v>
+      </c>
+      <c r="N6" s="8">
+        <v>3458</v>
+      </c>
+      <c r="O6" s="8">
+        <f t="shared" ref="O6:O7" si="0">ROUND(K6*N6%,2)</f>
+        <v>0</v>
+      </c>
+      <c r="P6" s="8">
+        <f t="shared" ref="P6:P7" si="1">J6-O6</f>
+        <v>3458</v>
+      </c>
+      <c r="Q6" s="8">
+        <f t="shared" ref="Q6:Q7" si="2">ROUND(L6*P6%,2)</f>
+        <v>0</v>
+      </c>
+      <c r="R6" s="8">
+        <f t="shared" ref="R6:R7" si="3">P6-Q6</f>
+        <v>3458</v>
+      </c>
+      <c r="S6" s="8">
+        <f t="shared" ref="S6:S7" si="4">ROUND(M6*R6%,2)</f>
+        <v>0</v>
+      </c>
+      <c r="T6" s="26">
+        <f t="shared" ref="T6:T7" si="5">O6+Q6+S6</f>
+        <v>0</v>
+      </c>
+      <c r="U6" s="26">
+        <v>0</v>
+      </c>
+      <c r="V6" s="8">
+        <f>(J6-T6)</f>
+        <v>3458</v>
+      </c>
+      <c r="W6" s="24">
+        <v>88363222</v>
+      </c>
+      <c r="X6" s="18">
+        <v>0.18</v>
+      </c>
+      <c r="Y6" s="24">
+        <f>IF($E$3=1,ROUND(((V6*X6)/2),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="Z6" s="24">
+        <f>IF($E$3=1,ROUND(((V6*X6)/2),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="AA6" s="42">
+        <f t="shared" ref="AA6:AA7" si="6">IF($E$3=2,ROUND(((V6*X6)),2),0)</f>
+        <v>622.44000000000005</v>
+      </c>
+      <c r="AB6" s="24">
+        <v>0</v>
+      </c>
+      <c r="AC6" s="24">
+        <f>Y6+Z6+AA6</f>
+        <v>622.44000000000005</v>
+      </c>
+      <c r="AD6" s="24">
+        <f>V6+AC6</f>
+        <v>4080.44</v>
+      </c>
+      <c r="AE6" s="46" t="s">
+        <v>53</v>
+      </c>
+      <c r="AF6" s="46" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="7" spans="1:32">
+      <c r="A7" s="46"/>
+      <c r="B7" s="9">
+        <v>3</v>
+      </c>
+      <c r="C7" s="27" t="s">
+        <v>52</v>
+      </c>
+      <c r="D7" s="9">
+        <v>0</v>
+      </c>
+      <c r="E7" s="27" t="s">
+        <v>52</v>
+      </c>
+      <c r="F7" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="G7" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="H7" s="24">
+        <v>3</v>
+      </c>
+      <c r="I7" s="9">
+        <v>675</v>
+      </c>
+      <c r="J7" s="8">
+        <v>2025</v>
+      </c>
+      <c r="K7" s="25">
+        <v>0</v>
+      </c>
+      <c r="L7" s="25">
+        <v>0</v>
+      </c>
+      <c r="M7" s="25">
+        <v>0</v>
+      </c>
+      <c r="N7" s="8">
+        <v>2025</v>
+      </c>
+      <c r="O7" s="8">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="P7" s="8">
+        <f t="shared" si="1"/>
+        <v>2025</v>
+      </c>
+      <c r="Q7" s="8">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="R7" s="8">
+        <f t="shared" si="3"/>
+        <v>2025</v>
+      </c>
+      <c r="S7" s="8">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="T7" s="26">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="U7" s="26">
+        <v>0</v>
+      </c>
+      <c r="V7" s="8">
+        <f>(J7-T7)</f>
+        <v>2025</v>
+      </c>
+      <c r="W7" s="24">
+        <v>88363222</v>
+      </c>
+      <c r="X7" s="18">
+        <v>0.18</v>
+      </c>
+      <c r="Y7" s="24">
+        <f>IF($E$3=1,ROUND(((V7*X7)/2),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="Z7" s="24">
+        <f>IF($E$3=1,ROUND(((V7*X7)/2),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="AA7" s="96">
+        <f t="shared" si="6"/>
+        <v>364.5</v>
+      </c>
+      <c r="AB7" s="24">
+        <v>0</v>
+      </c>
+      <c r="AC7" s="24">
+        <f>Y7+Z7+AA7</f>
+        <v>364.5</v>
+      </c>
+      <c r="AD7" s="24">
+        <f>V7+AC7</f>
+        <v>2389.5</v>
+      </c>
+      <c r="AE7" s="46" t="s">
+        <v>54</v>
+      </c>
+      <c r="AF7" s="46" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="8" spans="1:32">
+      <c r="AF8" s="46"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B1:AD1"/>
+    <mergeCell ref="B3:C3"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData/>
@@ -12883,7 +14029,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -12915,37 +14061,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="18">
-      <c r="A1" s="94" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="94"/>
-      <c r="C1" s="94"/>
-      <c r="D1" s="94"/>
-      <c r="E1" s="94"/>
-      <c r="F1" s="94"/>
-      <c r="G1" s="94"/>
-      <c r="H1" s="94"/>
-      <c r="I1" s="94"/>
-      <c r="J1" s="94"/>
-      <c r="K1" s="94"/>
-      <c r="L1" s="94"/>
-      <c r="M1" s="94"/>
-      <c r="N1" s="94"/>
-      <c r="O1" s="94"/>
-      <c r="P1" s="94"/>
-      <c r="Q1" s="94"/>
-      <c r="R1" s="94"/>
-      <c r="S1" s="94"/>
-      <c r="T1" s="94"/>
-      <c r="U1" s="94"/>
-      <c r="V1" s="94"/>
-      <c r="W1" s="94"/>
-      <c r="X1" s="94"/>
-      <c r="Y1" s="94"/>
-      <c r="Z1" s="94"/>
-      <c r="AA1" s="94"/>
-      <c r="AB1" s="94"/>
-      <c r="AC1" s="94"/>
+      <c r="A1" s="97" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="97"/>
+      <c r="C1" s="97"/>
+      <c r="D1" s="97"/>
+      <c r="E1" s="97"/>
+      <c r="F1" s="97"/>
+      <c r="G1" s="97"/>
+      <c r="H1" s="97"/>
+      <c r="I1" s="97"/>
+      <c r="J1" s="97"/>
+      <c r="K1" s="97"/>
+      <c r="L1" s="97"/>
+      <c r="M1" s="97"/>
+      <c r="N1" s="97"/>
+      <c r="O1" s="97"/>
+      <c r="P1" s="97"/>
+      <c r="Q1" s="97"/>
+      <c r="R1" s="97"/>
+      <c r="S1" s="97"/>
+      <c r="T1" s="97"/>
+      <c r="U1" s="97"/>
+      <c r="V1" s="97"/>
+      <c r="W1" s="97"/>
+      <c r="X1" s="97"/>
+      <c r="Y1" s="97"/>
+      <c r="Z1" s="97"/>
+      <c r="AA1" s="97"/>
+      <c r="AB1" s="97"/>
+      <c r="AC1" s="97"/>
     </row>
     <row r="2" spans="1:29" ht="18">
       <c r="A2" s="23" t="s">
@@ -12983,10 +14129,10 @@
       <c r="AC2" s="28"/>
     </row>
     <row r="3" spans="1:29">
-      <c r="A3" s="95" t="s">
+      <c r="A3" s="98" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="95"/>
+      <c r="B3" s="98"/>
       <c r="C3" s="29"/>
       <c r="D3" s="3">
         <v>3</v>
@@ -13268,37 +14414,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="18">
-      <c r="A1" s="94" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="94"/>
-      <c r="C1" s="94"/>
-      <c r="D1" s="94"/>
-      <c r="E1" s="94"/>
-      <c r="F1" s="94"/>
-      <c r="G1" s="94"/>
-      <c r="H1" s="94"/>
-      <c r="I1" s="94"/>
-      <c r="J1" s="94"/>
-      <c r="K1" s="94"/>
-      <c r="L1" s="94"/>
-      <c r="M1" s="94"/>
-      <c r="N1" s="94"/>
-      <c r="O1" s="94"/>
-      <c r="P1" s="94"/>
-      <c r="Q1" s="94"/>
-      <c r="R1" s="94"/>
-      <c r="S1" s="94"/>
-      <c r="T1" s="94"/>
-      <c r="U1" s="94"/>
-      <c r="V1" s="94"/>
-      <c r="W1" s="94"/>
-      <c r="X1" s="94"/>
-      <c r="Y1" s="94"/>
-      <c r="Z1" s="94"/>
-      <c r="AA1" s="94"/>
-      <c r="AB1" s="94"/>
-      <c r="AC1" s="94"/>
+      <c r="A1" s="97" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="97"/>
+      <c r="C1" s="97"/>
+      <c r="D1" s="97"/>
+      <c r="E1" s="97"/>
+      <c r="F1" s="97"/>
+      <c r="G1" s="97"/>
+      <c r="H1" s="97"/>
+      <c r="I1" s="97"/>
+      <c r="J1" s="97"/>
+      <c r="K1" s="97"/>
+      <c r="L1" s="97"/>
+      <c r="M1" s="97"/>
+      <c r="N1" s="97"/>
+      <c r="O1" s="97"/>
+      <c r="P1" s="97"/>
+      <c r="Q1" s="97"/>
+      <c r="R1" s="97"/>
+      <c r="S1" s="97"/>
+      <c r="T1" s="97"/>
+      <c r="U1" s="97"/>
+      <c r="V1" s="97"/>
+      <c r="W1" s="97"/>
+      <c r="X1" s="97"/>
+      <c r="Y1" s="97"/>
+      <c r="Z1" s="97"/>
+      <c r="AA1" s="97"/>
+      <c r="AB1" s="97"/>
+      <c r="AC1" s="97"/>
     </row>
     <row r="2" spans="1:29" ht="18">
       <c r="A2" s="23" t="s">
@@ -13336,10 +14482,10 @@
       <c r="AC2" s="28"/>
     </row>
     <row r="3" spans="1:29">
-      <c r="A3" s="95" t="s">
+      <c r="A3" s="98" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="95"/>
+      <c r="B3" s="98"/>
       <c r="C3" s="29"/>
       <c r="D3" s="3">
         <v>5</v>
@@ -13623,37 +14769,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="18">
-      <c r="A1" s="94" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="94"/>
-      <c r="C1" s="94"/>
-      <c r="D1" s="94"/>
-      <c r="E1" s="94"/>
-      <c r="F1" s="94"/>
-      <c r="G1" s="94"/>
-      <c r="H1" s="94"/>
-      <c r="I1" s="94"/>
-      <c r="J1" s="94"/>
-      <c r="K1" s="94"/>
-      <c r="L1" s="94"/>
-      <c r="M1" s="94"/>
-      <c r="N1" s="94"/>
-      <c r="O1" s="94"/>
-      <c r="P1" s="94"/>
-      <c r="Q1" s="94"/>
-      <c r="R1" s="94"/>
-      <c r="S1" s="94"/>
-      <c r="T1" s="94"/>
-      <c r="U1" s="94"/>
-      <c r="V1" s="94"/>
-      <c r="W1" s="94"/>
-      <c r="X1" s="94"/>
-      <c r="Y1" s="94"/>
-      <c r="Z1" s="94"/>
-      <c r="AA1" s="94"/>
-      <c r="AB1" s="94"/>
-      <c r="AC1" s="94"/>
+      <c r="A1" s="97" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="97"/>
+      <c r="C1" s="97"/>
+      <c r="D1" s="97"/>
+      <c r="E1" s="97"/>
+      <c r="F1" s="97"/>
+      <c r="G1" s="97"/>
+      <c r="H1" s="97"/>
+      <c r="I1" s="97"/>
+      <c r="J1" s="97"/>
+      <c r="K1" s="97"/>
+      <c r="L1" s="97"/>
+      <c r="M1" s="97"/>
+      <c r="N1" s="97"/>
+      <c r="O1" s="97"/>
+      <c r="P1" s="97"/>
+      <c r="Q1" s="97"/>
+      <c r="R1" s="97"/>
+      <c r="S1" s="97"/>
+      <c r="T1" s="97"/>
+      <c r="U1" s="97"/>
+      <c r="V1" s="97"/>
+      <c r="W1" s="97"/>
+      <c r="X1" s="97"/>
+      <c r="Y1" s="97"/>
+      <c r="Z1" s="97"/>
+      <c r="AA1" s="97"/>
+      <c r="AB1" s="97"/>
+      <c r="AC1" s="97"/>
     </row>
     <row r="2" spans="1:29" ht="18">
       <c r="A2" s="23" t="s">
@@ -13691,10 +14837,10 @@
       <c r="AC2" s="32"/>
     </row>
     <row r="3" spans="1:29">
-      <c r="A3" s="95" t="s">
+      <c r="A3" s="98" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="95"/>
+      <c r="B3" s="98"/>
       <c r="C3" s="33"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -13976,37 +15122,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="18">
-      <c r="A1" s="94" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="94"/>
-      <c r="C1" s="94"/>
-      <c r="D1" s="94"/>
-      <c r="E1" s="94"/>
-      <c r="F1" s="94"/>
-      <c r="G1" s="94"/>
-      <c r="H1" s="94"/>
-      <c r="I1" s="94"/>
-      <c r="J1" s="94"/>
-      <c r="K1" s="94"/>
-      <c r="L1" s="94"/>
-      <c r="M1" s="94"/>
-      <c r="N1" s="94"/>
-      <c r="O1" s="94"/>
-      <c r="P1" s="94"/>
-      <c r="Q1" s="94"/>
-      <c r="R1" s="94"/>
-      <c r="S1" s="94"/>
-      <c r="T1" s="94"/>
-      <c r="U1" s="94"/>
-      <c r="V1" s="94"/>
-      <c r="W1" s="94"/>
-      <c r="X1" s="94"/>
-      <c r="Y1" s="94"/>
-      <c r="Z1" s="94"/>
-      <c r="AA1" s="94"/>
-      <c r="AB1" s="94"/>
-      <c r="AC1" s="94"/>
+      <c r="A1" s="97" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="97"/>
+      <c r="C1" s="97"/>
+      <c r="D1" s="97"/>
+      <c r="E1" s="97"/>
+      <c r="F1" s="97"/>
+      <c r="G1" s="97"/>
+      <c r="H1" s="97"/>
+      <c r="I1" s="97"/>
+      <c r="J1" s="97"/>
+      <c r="K1" s="97"/>
+      <c r="L1" s="97"/>
+      <c r="M1" s="97"/>
+      <c r="N1" s="97"/>
+      <c r="O1" s="97"/>
+      <c r="P1" s="97"/>
+      <c r="Q1" s="97"/>
+      <c r="R1" s="97"/>
+      <c r="S1" s="97"/>
+      <c r="T1" s="97"/>
+      <c r="U1" s="97"/>
+      <c r="V1" s="97"/>
+      <c r="W1" s="97"/>
+      <c r="X1" s="97"/>
+      <c r="Y1" s="97"/>
+      <c r="Z1" s="97"/>
+      <c r="AA1" s="97"/>
+      <c r="AB1" s="97"/>
+      <c r="AC1" s="97"/>
     </row>
     <row r="2" spans="1:29" ht="18">
       <c r="A2" s="23" t="s">
@@ -14044,10 +15190,10 @@
       <c r="AC2" s="34"/>
     </row>
     <row r="3" spans="1:29">
-      <c r="A3" s="95" t="s">
+      <c r="A3" s="98" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="95"/>
+      <c r="B3" s="98"/>
       <c r="C3" s="35"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -14327,38 +15473,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:30" ht="18">
-      <c r="A1" s="94" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="94"/>
-      <c r="C1" s="94"/>
-      <c r="D1" s="94"/>
-      <c r="E1" s="94"/>
-      <c r="F1" s="94"/>
-      <c r="G1" s="94"/>
-      <c r="H1" s="94"/>
-      <c r="I1" s="94"/>
-      <c r="J1" s="94"/>
-      <c r="K1" s="94"/>
-      <c r="L1" s="94"/>
-      <c r="M1" s="94"/>
-      <c r="N1" s="94"/>
-      <c r="O1" s="94"/>
-      <c r="P1" s="94"/>
-      <c r="Q1" s="94"/>
-      <c r="R1" s="94"/>
-      <c r="S1" s="94"/>
-      <c r="T1" s="94"/>
-      <c r="U1" s="94"/>
-      <c r="V1" s="94"/>
-      <c r="W1" s="94"/>
-      <c r="X1" s="94"/>
-      <c r="Y1" s="94"/>
-      <c r="Z1" s="94"/>
-      <c r="AA1" s="94"/>
-      <c r="AB1" s="94"/>
-      <c r="AC1" s="94"/>
-      <c r="AD1" s="94"/>
+      <c r="A1" s="97" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="97"/>
+      <c r="C1" s="97"/>
+      <c r="D1" s="97"/>
+      <c r="E1" s="97"/>
+      <c r="F1" s="97"/>
+      <c r="G1" s="97"/>
+      <c r="H1" s="97"/>
+      <c r="I1" s="97"/>
+      <c r="J1" s="97"/>
+      <c r="K1" s="97"/>
+      <c r="L1" s="97"/>
+      <c r="M1" s="97"/>
+      <c r="N1" s="97"/>
+      <c r="O1" s="97"/>
+      <c r="P1" s="97"/>
+      <c r="Q1" s="97"/>
+      <c r="R1" s="97"/>
+      <c r="S1" s="97"/>
+      <c r="T1" s="97"/>
+      <c r="U1" s="97"/>
+      <c r="V1" s="97"/>
+      <c r="W1" s="97"/>
+      <c r="X1" s="97"/>
+      <c r="Y1" s="97"/>
+      <c r="Z1" s="97"/>
+      <c r="AA1" s="97"/>
+      <c r="AB1" s="97"/>
+      <c r="AC1" s="97"/>
+      <c r="AD1" s="97"/>
     </row>
     <row r="2" spans="1:30" ht="18">
       <c r="A2" s="23" t="s">
@@ -14397,10 +15543,10 @@
       <c r="AD2" s="36"/>
     </row>
     <row r="3" spans="1:30">
-      <c r="A3" s="95" t="s">
+      <c r="A3" s="98" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="95"/>
+      <c r="B3" s="98"/>
       <c r="C3" s="83"/>
       <c r="D3" s="37"/>
       <c r="E3" s="3">
@@ -14703,37 +15849,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:33" ht="18">
-      <c r="A1" s="94" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="94"/>
-      <c r="C1" s="94"/>
-      <c r="D1" s="94"/>
-      <c r="E1" s="94"/>
-      <c r="F1" s="94"/>
-      <c r="G1" s="94"/>
-      <c r="H1" s="94"/>
-      <c r="I1" s="94"/>
-      <c r="J1" s="94"/>
-      <c r="K1" s="94"/>
-      <c r="L1" s="94"/>
-      <c r="M1" s="94"/>
-      <c r="N1" s="94"/>
-      <c r="O1" s="94"/>
-      <c r="P1" s="94"/>
-      <c r="Q1" s="94"/>
-      <c r="R1" s="94"/>
-      <c r="S1" s="94"/>
-      <c r="T1" s="94"/>
-      <c r="U1" s="94"/>
-      <c r="V1" s="94"/>
-      <c r="W1" s="94"/>
-      <c r="X1" s="94"/>
-      <c r="Y1" s="94"/>
-      <c r="Z1" s="94"/>
-      <c r="AA1" s="94"/>
-      <c r="AB1" s="94"/>
-      <c r="AC1" s="94"/>
+      <c r="A1" s="97" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="97"/>
+      <c r="C1" s="97"/>
+      <c r="D1" s="97"/>
+      <c r="E1" s="97"/>
+      <c r="F1" s="97"/>
+      <c r="G1" s="97"/>
+      <c r="H1" s="97"/>
+      <c r="I1" s="97"/>
+      <c r="J1" s="97"/>
+      <c r="K1" s="97"/>
+      <c r="L1" s="97"/>
+      <c r="M1" s="97"/>
+      <c r="N1" s="97"/>
+      <c r="O1" s="97"/>
+      <c r="P1" s="97"/>
+      <c r="Q1" s="97"/>
+      <c r="R1" s="97"/>
+      <c r="S1" s="97"/>
+      <c r="T1" s="97"/>
+      <c r="U1" s="97"/>
+      <c r="V1" s="97"/>
+      <c r="W1" s="97"/>
+      <c r="X1" s="97"/>
+      <c r="Y1" s="97"/>
+      <c r="Z1" s="97"/>
+      <c r="AA1" s="97"/>
+      <c r="AB1" s="97"/>
+      <c r="AC1" s="97"/>
       <c r="AD1" s="93"/>
       <c r="AE1" s="93"/>
     </row>
@@ -14775,10 +15921,10 @@
       <c r="AE2" s="93"/>
     </row>
     <row r="3" spans="1:33">
-      <c r="A3" s="95" t="s">
+      <c r="A3" s="98" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="95"/>
+      <c r="B3" s="98"/>
       <c r="D3">
         <v>2</v>
       </c>

</xml_diff>